<commit_message>
v2 4 mei 26 - fixing CRRT
</commit_message>
<xml_diff>
--- a/peritonitis-prediction/PeritonitisPrediction_Database.xlsx
+++ b/peritonitis-prediction/PeritonitisPrediction_Database.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z36"/>
+  <dimension ref="A1:Z42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4936,6 +4936,798 @@
         </is>
       </c>
     </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-05-04 18:33:43</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>8044AAE1</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>&gt;2 yo</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>&lt;12 mo</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Good service</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>Studies</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>No ESI</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>Normal Nutrition</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>Glomerular</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>Coiled/swan neck</t>
+        </is>
+      </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>Double</t>
+        </is>
+      </c>
+      <c r="P37" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>Patients</t>
+        </is>
+      </c>
+      <c r="S37" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T37" t="inlineStr">
+        <is>
+          <t>Lateral/downward</t>
+        </is>
+      </c>
+      <c r="U37" t="inlineStr">
+        <is>
+          <t>Stunting</t>
+        </is>
+      </c>
+      <c r="V37" t="inlineStr">
+        <is>
+          <t>95.45%</t>
+        </is>
+      </c>
+      <c r="W37" t="inlineStr">
+        <is>
+          <t>Survivor</t>
+        </is>
+      </c>
+      <c r="X37" t="inlineStr">
+        <is>
+          <t>Age, Gender, Duration of PD, Place of Residence, Housing, Socioeconomic, Education, Peritonitis in ESI, Nutrition, Cause of ESRD, Type of Catheter (Shape), Type of Catheter (Cuff), Catheter Placement, Gastrostomy/Intraperitoneal Device, Performed CAPD, Starting PD &lt;2 weeks after placement, Catheter Orientation</t>
+        </is>
+      </c>
+      <c r="Y37" t="inlineStr">
+        <is>
+          <t>Stunting</t>
+        </is>
+      </c>
+      <c r="Z37" t="inlineStr">
+        <is>
+          <t>Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-05-04 18:36:35</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>8044AAE1</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>&gt;2 yo</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>&lt;12 mo</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Good service</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>Studies</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>No ESI</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>Normal Nutrition</t>
+        </is>
+      </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>Glomerular</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>Coiled/swan neck</t>
+        </is>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>Double</t>
+        </is>
+      </c>
+      <c r="P38" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R38" t="inlineStr">
+        <is>
+          <t>Patients</t>
+        </is>
+      </c>
+      <c r="S38" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T38" t="inlineStr">
+        <is>
+          <t>Lateral/downward</t>
+        </is>
+      </c>
+      <c r="U38" t="inlineStr">
+        <is>
+          <t>Stunting</t>
+        </is>
+      </c>
+      <c r="V38" t="inlineStr">
+        <is>
+          <t>95.45%</t>
+        </is>
+      </c>
+      <c r="W38" t="inlineStr">
+        <is>
+          <t>Survivor</t>
+        </is>
+      </c>
+      <c r="X38" t="inlineStr">
+        <is>
+          <t>Age, Gender, Duration of PD, Place of Residence, Housing, Socioeconomic, Education, Peritonitis in ESI, Nutrition, Cause of ESRD, Type of Catheter (Shape), Type of Catheter (Cuff), Catheter Placement, Gastrostomy/Intraperitoneal Device, Performed CAPD, Starting PD &lt;2 weeks after placement, Catheter Orientation</t>
+        </is>
+      </c>
+      <c r="Y38" t="inlineStr">
+        <is>
+          <t>Stunting</t>
+        </is>
+      </c>
+      <c r="Z38" t="inlineStr">
+        <is>
+          <t>Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-05-04 18:36:38</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>8044AAE1</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>&gt;2 yo</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>&lt;12 mo</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Good service</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>Studies</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>No ESI</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>Normal Nutrition</t>
+        </is>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>Glomerular</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>Coiled/swan neck</t>
+        </is>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>Double</t>
+        </is>
+      </c>
+      <c r="P39" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R39" t="inlineStr">
+        <is>
+          <t>Patients</t>
+        </is>
+      </c>
+      <c r="S39" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T39" t="inlineStr">
+        <is>
+          <t>Lateral/downward</t>
+        </is>
+      </c>
+      <c r="U39" t="inlineStr">
+        <is>
+          <t>Stunting</t>
+        </is>
+      </c>
+      <c r="V39" t="inlineStr">
+        <is>
+          <t>95.45%</t>
+        </is>
+      </c>
+      <c r="W39" t="inlineStr">
+        <is>
+          <t>Survivor</t>
+        </is>
+      </c>
+      <c r="X39" t="inlineStr">
+        <is>
+          <t>Age, Gender, Duration of PD, Place of Residence, Housing, Socioeconomic, Education, Peritonitis in ESI, Nutrition, Cause of ESRD, Type of Catheter (Shape), Type of Catheter (Cuff), Catheter Placement, Gastrostomy/Intraperitoneal Device, Performed CAPD, Starting PD &lt;2 weeks after placement, Catheter Orientation</t>
+        </is>
+      </c>
+      <c r="Y39" t="inlineStr">
+        <is>
+          <t>Stunting</t>
+        </is>
+      </c>
+      <c r="Z39" t="inlineStr">
+        <is>
+          <t>Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-05-04 18:36:54</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>8044AAE1</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>&gt;2 yo</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>&lt;12 mo</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Good service</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>Studies</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>No ESI</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>Normal Nutrition</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>Glomerular</t>
+        </is>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>Coiled/swan neck</t>
+        </is>
+      </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>Double</t>
+        </is>
+      </c>
+      <c r="P40" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="Q40" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t>Patients</t>
+        </is>
+      </c>
+      <c r="S40" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T40" t="inlineStr">
+        <is>
+          <t>Lateral/downward</t>
+        </is>
+      </c>
+      <c r="U40" t="inlineStr">
+        <is>
+          <t>Stunting</t>
+        </is>
+      </c>
+      <c r="V40" t="inlineStr">
+        <is>
+          <t>95.45%</t>
+        </is>
+      </c>
+      <c r="W40" t="inlineStr">
+        <is>
+          <t>Survivor</t>
+        </is>
+      </c>
+      <c r="X40" t="inlineStr">
+        <is>
+          <t>Age, Gender, Duration of PD, Place of Residence, Housing, Socioeconomic, Education, Peritonitis in ESI, Nutrition, Cause of ESRD, Type of Catheter (Shape), Type of Catheter (Cuff), Catheter Placement, Gastrostomy/Intraperitoneal Device, Performed CAPD, Starting PD &lt;2 weeks after placement, Catheter Orientation</t>
+        </is>
+      </c>
+      <c r="Y40" t="inlineStr">
+        <is>
+          <t>Stunting</t>
+        </is>
+      </c>
+      <c r="Z40" t="inlineStr">
+        <is>
+          <t>Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-05-04 18:37:06</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>8044AAE1</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>&gt;2 yo</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>&lt;12 mo</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Good service</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>Studies</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>No ESI</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>Normal Nutrition</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>Glomerular</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>Coiled/swan neck</t>
+        </is>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>Double</t>
+        </is>
+      </c>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>Patients</t>
+        </is>
+      </c>
+      <c r="S41" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T41" t="inlineStr">
+        <is>
+          <t>Lateral/downward</t>
+        </is>
+      </c>
+      <c r="U41" t="inlineStr">
+        <is>
+          <t>Stunting</t>
+        </is>
+      </c>
+      <c r="V41" t="inlineStr">
+        <is>
+          <t>95.45%</t>
+        </is>
+      </c>
+      <c r="W41" t="inlineStr">
+        <is>
+          <t>Survivor</t>
+        </is>
+      </c>
+      <c r="X41" t="inlineStr">
+        <is>
+          <t>Age, Gender, Duration of PD, Place of Residence, Housing, Socioeconomic, Education, Peritonitis in ESI, Nutrition, Cause of ESRD, Type of Catheter (Shape), Type of Catheter (Cuff), Catheter Placement, Gastrostomy/Intraperitoneal Device, Performed CAPD, Starting PD &lt;2 weeks after placement, Catheter Orientation</t>
+        </is>
+      </c>
+      <c r="Y41" t="inlineStr">
+        <is>
+          <t>Stunting</t>
+        </is>
+      </c>
+      <c r="Z41" t="inlineStr">
+        <is>
+          <t>Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2026-05-04 18:37:18</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>8044AAE1</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>&gt;2 yo</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>&lt;12 mo</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Good service</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>Studies</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>No ESI</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>Normal Nutrition</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>Glomerular</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>Coiled/swan neck</t>
+        </is>
+      </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>Double</t>
+        </is>
+      </c>
+      <c r="P42" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R42" t="inlineStr">
+        <is>
+          <t>Patients</t>
+        </is>
+      </c>
+      <c r="S42" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T42" t="inlineStr">
+        <is>
+          <t>Lateral/downward</t>
+        </is>
+      </c>
+      <c r="U42" t="inlineStr">
+        <is>
+          <t>Stunting</t>
+        </is>
+      </c>
+      <c r="V42" t="inlineStr">
+        <is>
+          <t>95.45%</t>
+        </is>
+      </c>
+      <c r="W42" t="inlineStr">
+        <is>
+          <t>Survivor</t>
+        </is>
+      </c>
+      <c r="X42" t="inlineStr">
+        <is>
+          <t>Age, Gender, Duration of PD, Place of Residence, Housing, Socioeconomic, Education, Peritonitis in ESI, Nutrition, Cause of ESRD, Type of Catheter (Shape), Type of Catheter (Cuff), Catheter Placement, Gastrostomy/Intraperitoneal Device, Performed CAPD, Starting PD &lt;2 weeks after placement, Catheter Orientation</t>
+        </is>
+      </c>
+      <c r="Y42" t="inlineStr">
+        <is>
+          <t>Stunting</t>
+        </is>
+      </c>
+      <c r="Z42" t="inlineStr">
+        <is>
+          <t>Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
v1 5 mei 26 - connection to gsheets with GCP
</commit_message>
<xml_diff>
--- a/peritonitis-prediction/PeritonitisPrediction_Database.xlsx
+++ b/peritonitis-prediction/PeritonitisPrediction_Database.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z42"/>
+  <dimension ref="A1:Z48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5728,6 +5728,790 @@
         </is>
       </c>
     </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2026-05-05 15:10:32</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>CE0F6C28</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>&gt;2 yo</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>&lt;12 mo</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Good service</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>Studies</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>No ESI</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>Normal Nutrition</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>Glomerular</t>
+        </is>
+      </c>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>Coiled/swan neck</t>
+        </is>
+      </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>Double</t>
+        </is>
+      </c>
+      <c r="P43" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="Q43" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R43" t="inlineStr">
+        <is>
+          <t>Patients</t>
+        </is>
+      </c>
+      <c r="S43" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T43" t="inlineStr">
+        <is>
+          <t>Lateral/downward</t>
+        </is>
+      </c>
+      <c r="U43" t="inlineStr">
+        <is>
+          <t>No stunting</t>
+        </is>
+      </c>
+      <c r="V43" t="inlineStr">
+        <is>
+          <t>100.00%</t>
+        </is>
+      </c>
+      <c r="W43" t="inlineStr">
+        <is>
+          <t>Survivor</t>
+        </is>
+      </c>
+      <c r="X43" t="inlineStr">
+        <is>
+          <t>Age, Gender, Duration of PD, Place of Residence, Housing, Socioeconomic, Education, Peritonitis in ESI, Nutrition, Cause of ESRD, Type of Catheter (Shape), Type of Catheter (Cuff), Catheter Placement, Gastrostomy/Intraperitoneal Device, Performed CAPD, Starting PD &lt;2 weeks after placement, Catheter Orientation, Stunting</t>
+        </is>
+      </c>
+      <c r="Y43" t="inlineStr"/>
+      <c r="Z43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-05-05 15:19:00</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>A2B9C8D2</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>&gt;2 yo</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>&lt;12 mo</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Good service</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>Studies</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>No ESI</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>Normal Nutrition</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>Glomerular</t>
+        </is>
+      </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>Coiled/swan neck</t>
+        </is>
+      </c>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>Double</t>
+        </is>
+      </c>
+      <c r="P44" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="Q44" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R44" t="inlineStr">
+        <is>
+          <t>Patients</t>
+        </is>
+      </c>
+      <c r="S44" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T44" t="inlineStr">
+        <is>
+          <t>Lateral/downward</t>
+        </is>
+      </c>
+      <c r="U44" t="inlineStr">
+        <is>
+          <t>Stunting</t>
+        </is>
+      </c>
+      <c r="V44" t="inlineStr">
+        <is>
+          <t>95.45%</t>
+        </is>
+      </c>
+      <c r="W44" t="inlineStr">
+        <is>
+          <t>Survivor</t>
+        </is>
+      </c>
+      <c r="X44" t="inlineStr">
+        <is>
+          <t>Age, Gender, Duration of PD, Place of Residence, Housing, Socioeconomic, Education, Peritonitis in ESI, Nutrition, Cause of ESRD, Type of Catheter (Shape), Type of Catheter (Cuff), Catheter Placement, Gastrostomy/Intraperitoneal Device, Performed CAPD, Starting PD &lt;2 weeks after placement, Catheter Orientation</t>
+        </is>
+      </c>
+      <c r="Y44" t="inlineStr">
+        <is>
+          <t>Stunting</t>
+        </is>
+      </c>
+      <c r="Z44" t="inlineStr">
+        <is>
+          <t>Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-05-05 15:23:28</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>A2B9C8D2</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>&gt;2 yo</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>&lt;12 mo</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Good service</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>Studies</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>No ESI</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>Normal Nutrition</t>
+        </is>
+      </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>Glomerular</t>
+        </is>
+      </c>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>Coiled/swan neck</t>
+        </is>
+      </c>
+      <c r="O45" t="inlineStr">
+        <is>
+          <t>Double</t>
+        </is>
+      </c>
+      <c r="P45" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="Q45" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R45" t="inlineStr">
+        <is>
+          <t>Patients</t>
+        </is>
+      </c>
+      <c r="S45" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T45" t="inlineStr">
+        <is>
+          <t>Lateral/downward</t>
+        </is>
+      </c>
+      <c r="U45" t="inlineStr">
+        <is>
+          <t>Stunting</t>
+        </is>
+      </c>
+      <c r="V45" t="inlineStr">
+        <is>
+          <t>95.45%</t>
+        </is>
+      </c>
+      <c r="W45" t="inlineStr">
+        <is>
+          <t>Survivor</t>
+        </is>
+      </c>
+      <c r="X45" t="inlineStr">
+        <is>
+          <t>Age, Gender, Duration of PD, Place of Residence, Housing, Socioeconomic, Education, Peritonitis in ESI, Nutrition, Cause of ESRD, Type of Catheter (Shape), Type of Catheter (Cuff), Catheter Placement, Gastrostomy/Intraperitoneal Device, Performed CAPD, Starting PD &lt;2 weeks after placement, Catheter Orientation</t>
+        </is>
+      </c>
+      <c r="Y45" t="inlineStr">
+        <is>
+          <t>Stunting</t>
+        </is>
+      </c>
+      <c r="Z45" t="inlineStr">
+        <is>
+          <t>Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2026-05-05 15:27:04</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>A2B9C8D2</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>&gt;2 yo</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>&lt;12 mo</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>Good service</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>Studies</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>No ESI</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>Normal Nutrition</t>
+        </is>
+      </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>Glomerular</t>
+        </is>
+      </c>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>Coiled/swan neck</t>
+        </is>
+      </c>
+      <c r="O46" t="inlineStr">
+        <is>
+          <t>Double</t>
+        </is>
+      </c>
+      <c r="P46" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="Q46" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R46" t="inlineStr">
+        <is>
+          <t>Patients</t>
+        </is>
+      </c>
+      <c r="S46" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T46" t="inlineStr">
+        <is>
+          <t>Lateral/downward</t>
+        </is>
+      </c>
+      <c r="U46" t="inlineStr">
+        <is>
+          <t>Stunting</t>
+        </is>
+      </c>
+      <c r="V46" t="inlineStr">
+        <is>
+          <t>95.45%</t>
+        </is>
+      </c>
+      <c r="W46" t="inlineStr">
+        <is>
+          <t>Survivor</t>
+        </is>
+      </c>
+      <c r="X46" t="inlineStr">
+        <is>
+          <t>Age, Gender, Duration of PD, Place of Residence, Housing, Socioeconomic, Education, Peritonitis in ESI, Nutrition, Cause of ESRD, Type of Catheter (Shape), Type of Catheter (Cuff), Catheter Placement, Gastrostomy/Intraperitoneal Device, Performed CAPD, Starting PD &lt;2 weeks after placement, Catheter Orientation</t>
+        </is>
+      </c>
+      <c r="Y46" t="inlineStr">
+        <is>
+          <t>Stunting</t>
+        </is>
+      </c>
+      <c r="Z46" t="inlineStr">
+        <is>
+          <t>Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-05-05 15:27:43</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>A2B9C8D2</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>&gt;2 yo</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>&lt;12 mo</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Good service</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>Studies</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>ESI</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>Normal Nutrition</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>Glomerular</t>
+        </is>
+      </c>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>Coiled/swan neck</t>
+        </is>
+      </c>
+      <c r="O47" t="inlineStr">
+        <is>
+          <t>Double</t>
+        </is>
+      </c>
+      <c r="P47" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="Q47" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R47" t="inlineStr">
+        <is>
+          <t>Patients</t>
+        </is>
+      </c>
+      <c r="S47" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T47" t="inlineStr">
+        <is>
+          <t>Lateral/downward</t>
+        </is>
+      </c>
+      <c r="U47" t="inlineStr">
+        <is>
+          <t>Stunting</t>
+        </is>
+      </c>
+      <c r="V47" t="inlineStr">
+        <is>
+          <t>86.36%</t>
+        </is>
+      </c>
+      <c r="W47" t="inlineStr">
+        <is>
+          <t>Survivor</t>
+        </is>
+      </c>
+      <c r="X47" t="inlineStr">
+        <is>
+          <t>Age, Gender, Duration of PD, Place of Residence, Housing, Socioeconomic, Education, Nutrition, Cause of ESRD, Type of Catheter (Shape), Type of Catheter (Cuff), Catheter Placement, Gastrostomy/Intraperitoneal Device, Performed CAPD, Starting PD &lt;2 weeks after placement, Catheter Orientation</t>
+        </is>
+      </c>
+      <c r="Y47" t="inlineStr">
+        <is>
+          <t>Peritonitis in ESI, Stunting</t>
+        </is>
+      </c>
+      <c r="Z47" t="inlineStr">
+        <is>
+          <t>Peritonitis in ESI: Perlu penanganan agresif dan segera terhadap infeksi area keluar kateter (Exit Site Infection) agar kuman tidak masuk ke rongga perut. | Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2026-05-05 15:31:42</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>A2B9C8D2</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>&gt;2 yo</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>&lt;12 mo</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>Good service</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>Studies</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>ESI</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>Normal Nutrition</t>
+        </is>
+      </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>Glomerular</t>
+        </is>
+      </c>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>Coiled/swan neck</t>
+        </is>
+      </c>
+      <c r="O48" t="inlineStr">
+        <is>
+          <t>Double</t>
+        </is>
+      </c>
+      <c r="P48" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="Q48" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R48" t="inlineStr">
+        <is>
+          <t>Patients</t>
+        </is>
+      </c>
+      <c r="S48" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T48" t="inlineStr">
+        <is>
+          <t>Lateral/downward</t>
+        </is>
+      </c>
+      <c r="U48" t="inlineStr">
+        <is>
+          <t>Stunting</t>
+        </is>
+      </c>
+      <c r="V48" t="inlineStr">
+        <is>
+          <t>86.36%</t>
+        </is>
+      </c>
+      <c r="W48" t="inlineStr">
+        <is>
+          <t>Survivor</t>
+        </is>
+      </c>
+      <c r="X48" t="inlineStr">
+        <is>
+          <t>Age, Gender, Duration of PD, Place of Residence, Housing, Socioeconomic, Education, Nutrition, Cause of ESRD, Type of Catheter (Shape), Type of Catheter (Cuff), Catheter Placement, Gastrostomy/Intraperitoneal Device, Performed CAPD, Starting PD &lt;2 weeks after placement, Catheter Orientation</t>
+        </is>
+      </c>
+      <c r="Y48" t="inlineStr">
+        <is>
+          <t>Peritonitis in ESI, Stunting</t>
+        </is>
+      </c>
+      <c r="Z48" t="inlineStr">
+        <is>
+          <t>Peritonitis in ESI: Perlu penanganan agresif dan segera terhadap infeksi area keluar kateter (Exit Site Infection) agar kuman tidak masuk ke rongga perut. | Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
v1 6 mei 26 - update MRF explanatoins
</commit_message>
<xml_diff>
--- a/peritonitis-prediction/PeritonitisPrediction_Database.xlsx
+++ b/peritonitis-prediction/PeritonitisPrediction_Database.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z48"/>
+  <dimension ref="A1:Z51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6512,6 +6512,402 @@
         </is>
       </c>
     </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2026-05-05 23:55:59</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>1F62B632</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>&gt;2 yo</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>&lt;12 mo</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>Good service</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>Studies</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>No ESI</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>Normal Nutrition</t>
+        </is>
+      </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>Glomerular</t>
+        </is>
+      </c>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>Coiled/swan neck</t>
+        </is>
+      </c>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>Double</t>
+        </is>
+      </c>
+      <c r="P49" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="Q49" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R49" t="inlineStr">
+        <is>
+          <t>Patients</t>
+        </is>
+      </c>
+      <c r="S49" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T49" t="inlineStr">
+        <is>
+          <t>Lateral/downward</t>
+        </is>
+      </c>
+      <c r="U49" t="inlineStr">
+        <is>
+          <t>Stunting</t>
+        </is>
+      </c>
+      <c r="V49" t="inlineStr">
+        <is>
+          <t>95.45%</t>
+        </is>
+      </c>
+      <c r="W49" t="inlineStr">
+        <is>
+          <t>Survivor</t>
+        </is>
+      </c>
+      <c r="X49" t="inlineStr">
+        <is>
+          <t>Age, Gender, Duration of PD, Place of Residence, Housing, Socioeconomic, Education, Peritonitis in ESI, Nutrition, Cause of ESRD, Type of Catheter (Shape), Type of Catheter (Cuff), Catheter Placement, Gastrostomy/Intraperitoneal Device, Performed CAPD, Starting PD &lt;2 weeks after placement, Catheter Orientation</t>
+        </is>
+      </c>
+      <c r="Y49" t="inlineStr">
+        <is>
+          <t>Stunting</t>
+        </is>
+      </c>
+      <c r="Z49" t="inlineStr">
+        <is>
+          <t>Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2026-05-05 23:56:26</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>1F62B632</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>&gt;2 yo</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>&lt;12 mo</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>Fair/poor service</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>Studies</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>No ESI</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>Normal Nutrition</t>
+        </is>
+      </c>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>Glomerular</t>
+        </is>
+      </c>
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>Coiled/swan neck</t>
+        </is>
+      </c>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>Double</t>
+        </is>
+      </c>
+      <c r="P50" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="Q50" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R50" t="inlineStr">
+        <is>
+          <t>Patients</t>
+        </is>
+      </c>
+      <c r="S50" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T50" t="inlineStr">
+        <is>
+          <t>Lateral/downward</t>
+        </is>
+      </c>
+      <c r="U50" t="inlineStr">
+        <is>
+          <t>Stunting</t>
+        </is>
+      </c>
+      <c r="V50" t="inlineStr">
+        <is>
+          <t>90.91%</t>
+        </is>
+      </c>
+      <c r="W50" t="inlineStr">
+        <is>
+          <t>Survivor</t>
+        </is>
+      </c>
+      <c r="X50" t="inlineStr">
+        <is>
+          <t>Age, Gender, Duration of PD, Place of Residence, Socioeconomic, Education, Peritonitis in ESI, Nutrition, Cause of ESRD, Type of Catheter (Shape), Type of Catheter (Cuff), Catheter Placement, Gastrostomy/Intraperitoneal Device, Performed CAPD, Starting PD &lt;2 weeks after placement, Catheter Orientation</t>
+        </is>
+      </c>
+      <c r="Y50" t="inlineStr">
+        <is>
+          <t>Housing, Stunting</t>
+        </is>
+      </c>
+      <c r="Z50" t="inlineStr">
+        <is>
+          <t>Housing: Pastikan ada ruangan khusus yang bersih (minim debu/hewan peliharaan) untuk melakukan pertukaran cairan, serta ketersediaan wastafel dengan air mengalir di dalam ruangan tersebut untuk antisepsis tangan. [Sumber](https://www.scielo.br/j/jbn/a/hHtvqSXhwcCtvBnNqk9JBzk/?lang=en&amp;format=pdf) | Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2026-05-05 23:59:05</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>1F62B632</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>&gt;2 yo</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>&lt;12 mo</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>Fair/poor service</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>Studies</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>No ESI</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>Normal Nutrition</t>
+        </is>
+      </c>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>Glomerular</t>
+        </is>
+      </c>
+      <c r="N51" t="inlineStr">
+        <is>
+          <t>Coiled/swan neck</t>
+        </is>
+      </c>
+      <c r="O51" t="inlineStr">
+        <is>
+          <t>Double</t>
+        </is>
+      </c>
+      <c r="P51" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="Q51" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R51" t="inlineStr">
+        <is>
+          <t>Patients</t>
+        </is>
+      </c>
+      <c r="S51" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T51" t="inlineStr">
+        <is>
+          <t>Lateral/downward</t>
+        </is>
+      </c>
+      <c r="U51" t="inlineStr">
+        <is>
+          <t>Stunting</t>
+        </is>
+      </c>
+      <c r="V51" t="inlineStr">
+        <is>
+          <t>90.91%</t>
+        </is>
+      </c>
+      <c r="W51" t="inlineStr">
+        <is>
+          <t>Survivor</t>
+        </is>
+      </c>
+      <c r="X51" t="inlineStr">
+        <is>
+          <t>Age, Gender, Duration of PD, Place of Residence, Socioeconomic, Education, Peritonitis in ESI, Nutrition, Cause of ESRD, Type of Catheter (Shape), Type of Catheter (Cuff), Catheter Placement, Gastrostomy/Intraperitoneal Device, Performed CAPD, Starting PD &lt;2 weeks after placement, Catheter Orientation</t>
+        </is>
+      </c>
+      <c r="Y51" t="inlineStr">
+        <is>
+          <t>Housing, Stunting</t>
+        </is>
+      </c>
+      <c r="Z51" t="inlineStr">
+        <is>
+          <t>Housing: Pastikan ada ruangan khusus yang bersih (minim debu/hewan peliharaan) untuk melakukan pertukaran cairan, serta ketersediaan wastafel dengan air mengalir di dalam ruangan tersebut untuk antisepsis tangan. [Sumber](https://www.scielo.br/j/jbn/a/hHtvqSXhwcCtvBnNqk9JBzk/?lang=en&amp;format=pdf) | Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
v1 9 Mei 2026 - adding marks to significant variables, update XAI, adding knowledge warning
</commit_message>
<xml_diff>
--- a/peritonitis-prediction/PeritonitisPrediction_Database.xlsx
+++ b/peritonitis-prediction/PeritonitisPrediction_Database.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z51"/>
+  <dimension ref="A1:Z82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6908,6 +6908,4090 @@
         </is>
       </c>
     </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2026-05-09 09:36:32</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>03C5B5BD</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>&gt;2 yo</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>&lt;12 mo</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>Good service</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>Studies</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>No ESI</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>Normal Nutrition</t>
+        </is>
+      </c>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>Glomerular</t>
+        </is>
+      </c>
+      <c r="N52" t="inlineStr">
+        <is>
+          <t>Coiled/swan neck</t>
+        </is>
+      </c>
+      <c r="O52" t="inlineStr">
+        <is>
+          <t>Double</t>
+        </is>
+      </c>
+      <c r="P52" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="Q52" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R52" t="inlineStr">
+        <is>
+          <t>Patients</t>
+        </is>
+      </c>
+      <c r="S52" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T52" t="inlineStr">
+        <is>
+          <t>Lateral/downward</t>
+        </is>
+      </c>
+      <c r="U52" t="inlineStr">
+        <is>
+          <t>Stunting</t>
+        </is>
+      </c>
+      <c r="V52" t="inlineStr">
+        <is>
+          <t>95.45%</t>
+        </is>
+      </c>
+      <c r="W52" t="inlineStr">
+        <is>
+          <t>Survivor</t>
+        </is>
+      </c>
+      <c r="X52" t="inlineStr">
+        <is>
+          <t>Age, Gender, Duration of PD, Place of Residence, Housing, Socioeconomic, Education, Peritonitis in ESI, Nutrition, Cause of ESRD, Type of Catheter (Shape), Type of Catheter (Cuff), Catheter Placement, Gastrostomy/Intraperitoneal Device, Performed CAPD, Starting PD &lt;2 weeks after placement, Catheter Orientation</t>
+        </is>
+      </c>
+      <c r="Y52" t="inlineStr">
+        <is>
+          <t>Stunting</t>
+        </is>
+      </c>
+      <c r="Z52" t="inlineStr">
+        <is>
+          <t>Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2026-05-09 09:36:50</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>03C5B5BD</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>&gt;2 yo</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>&lt;12 mo</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>Good service</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>Studies</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>No ESI</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>Poor nutrition</t>
+        </is>
+      </c>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>Glomerular</t>
+        </is>
+      </c>
+      <c r="N53" t="inlineStr">
+        <is>
+          <t>Coiled/swan neck</t>
+        </is>
+      </c>
+      <c r="O53" t="inlineStr">
+        <is>
+          <t>Double</t>
+        </is>
+      </c>
+      <c r="P53" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="Q53" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R53" t="inlineStr">
+        <is>
+          <t>Patients</t>
+        </is>
+      </c>
+      <c r="S53" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T53" t="inlineStr">
+        <is>
+          <t>Lateral/downward</t>
+        </is>
+      </c>
+      <c r="U53" t="inlineStr">
+        <is>
+          <t>Stunting</t>
+        </is>
+      </c>
+      <c r="V53" t="inlineStr">
+        <is>
+          <t>90.91%</t>
+        </is>
+      </c>
+      <c r="W53" t="inlineStr">
+        <is>
+          <t>Survivor</t>
+        </is>
+      </c>
+      <c r="X53" t="inlineStr">
+        <is>
+          <t>Age, Gender, Duration of PD, Place of Residence, Housing, Socioeconomic, Education, Peritonitis in ESI, Cause of ESRD, Type of Catheter (Shape), Type of Catheter (Cuff), Catheter Placement, Gastrostomy/Intraperitoneal Device, Performed CAPD, Starting PD &lt;2 weeks after placement, Catheter Orientation</t>
+        </is>
+      </c>
+      <c r="Y53" t="inlineStr">
+        <is>
+          <t>Nutrition, Stunting</t>
+        </is>
+      </c>
+      <c r="Z53" t="inlineStr">
+        <is>
+          <t>Nutrition: Berikan asupan protein tinggi sesuai target usia (biasanya 1.4–3.0 g/kg/hari untuk anak) guna mengejar pertumbuhan dan mengganti protein yang hilang saat dialisis. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC7352713/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) | Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2026-05-09 09:37:14</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>03C5B5BD</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>&gt;2 yo</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>&lt;12 mo</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>Good service</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>Studies</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>No ESI</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>Poor nutrition</t>
+        </is>
+      </c>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>Glomerular</t>
+        </is>
+      </c>
+      <c r="N54" t="inlineStr">
+        <is>
+          <t>Coiled/swan neck</t>
+        </is>
+      </c>
+      <c r="O54" t="inlineStr">
+        <is>
+          <t>Single cuff</t>
+        </is>
+      </c>
+      <c r="P54" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="Q54" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R54" t="inlineStr">
+        <is>
+          <t>Patients</t>
+        </is>
+      </c>
+      <c r="S54" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T54" t="inlineStr">
+        <is>
+          <t>Lateral/downward</t>
+        </is>
+      </c>
+      <c r="U54" t="inlineStr">
+        <is>
+          <t>Stunting</t>
+        </is>
+      </c>
+      <c r="V54" t="inlineStr">
+        <is>
+          <t>86.36%</t>
+        </is>
+      </c>
+      <c r="W54" t="inlineStr">
+        <is>
+          <t>Survivor</t>
+        </is>
+      </c>
+      <c r="X54" t="inlineStr">
+        <is>
+          <t>Age, Gender, Duration of PD, Place of Residence, Housing, Socioeconomic, Education, Peritonitis in ESI, Cause of ESRD, Type of Catheter (Shape), Catheter Placement, Gastrostomy/Intraperitoneal Device, Performed CAPD, Starting PD &lt;2 weeks after placement, Catheter Orientation</t>
+        </is>
+      </c>
+      <c r="Y54" t="inlineStr">
+        <is>
+          <t>Nutrition, Type of Catheter (Cuff), Stunting</t>
+        </is>
+      </c>
+      <c r="Z54" t="inlineStr">
+        <is>
+          <t>Nutrition: Berikan asupan protein tinggi sesuai target usia (biasanya 1.4–3.0 g/kg/hari untuk anak) guna mengejar pertumbuhan dan mengganti protein yang hilang saat dialisis. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC7352713/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) | Type of Catheter (Cuff): Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2026-05-09 09:39:55</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>03C5B5BD</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>&gt;2 yo</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>&lt;12 mo</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>Good service</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>Studies</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>ESI</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>Poor nutrition</t>
+        </is>
+      </c>
+      <c r="M55" t="inlineStr">
+        <is>
+          <t>Glomerular</t>
+        </is>
+      </c>
+      <c r="N55" t="inlineStr">
+        <is>
+          <t>Coiled/swan neck</t>
+        </is>
+      </c>
+      <c r="O55" t="inlineStr">
+        <is>
+          <t>Single cuff</t>
+        </is>
+      </c>
+      <c r="P55" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="Q55" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R55" t="inlineStr">
+        <is>
+          <t>Patients</t>
+        </is>
+      </c>
+      <c r="S55" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T55" t="inlineStr">
+        <is>
+          <t>Lateral/downward</t>
+        </is>
+      </c>
+      <c r="U55" t="inlineStr">
+        <is>
+          <t>Stunting</t>
+        </is>
+      </c>
+      <c r="V55" t="inlineStr">
+        <is>
+          <t>77.27%</t>
+        </is>
+      </c>
+      <c r="W55" t="inlineStr">
+        <is>
+          <t>Survivor</t>
+        </is>
+      </c>
+      <c r="X55" t="inlineStr">
+        <is>
+          <t>Age, Gender, Duration of PD, Place of Residence, Housing, Socioeconomic, Education, Cause of ESRD, Type of Catheter (Shape), Catheter Placement, Gastrostomy/Intraperitoneal Device, Performed CAPD, Starting PD &lt;2 weeks after placement, Catheter Orientation</t>
+        </is>
+      </c>
+      <c r="Y55" t="inlineStr">
+        <is>
+          <t>Peritonitis in ESI, Nutrition, Type of Catheter (Cuff), Stunting</t>
+        </is>
+      </c>
+      <c r="Z55" t="inlineStr">
+        <is>
+          <t>Peritonitis in ESI: Gunakan salep antibiotik topikal (seperti mupirocin atau gentamisin) pada exit site secara rutin dan pembersihan area dengan cairan antiseptik non-iritan. [Sumber](https://journals.eco-vector.com/2075-3594/article/view/637454) | Nutrition: Berikan asupan protein tinggi sesuai target usia (biasanya 1.4–3.0 g/kg/hari untuk anak) guna mengejar pertumbuhan dan mengganti protein yang hilang saat dialisis. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC7352713/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) | Type of Catheter (Cuff): Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2026-05-09 09:44:19</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>BBF800B7</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>&gt;2 yo</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>&lt;12 mo</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>Good service</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>Studies</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>No ESI</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>Normal Nutrition</t>
+        </is>
+      </c>
+      <c r="M56" t="inlineStr">
+        <is>
+          <t>Glomerular</t>
+        </is>
+      </c>
+      <c r="N56" t="inlineStr">
+        <is>
+          <t>Coiled/swan neck</t>
+        </is>
+      </c>
+      <c r="O56" t="inlineStr">
+        <is>
+          <t>Double</t>
+        </is>
+      </c>
+      <c r="P56" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="Q56" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R56" t="inlineStr">
+        <is>
+          <t>Patients</t>
+        </is>
+      </c>
+      <c r="S56" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T56" t="inlineStr">
+        <is>
+          <t>Lateral/downward</t>
+        </is>
+      </c>
+      <c r="U56" t="inlineStr">
+        <is>
+          <t>No stunting</t>
+        </is>
+      </c>
+      <c r="V56" t="inlineStr">
+        <is>
+          <t>100.00%</t>
+        </is>
+      </c>
+      <c r="W56" t="inlineStr">
+        <is>
+          <t>Survivor</t>
+        </is>
+      </c>
+      <c r="X56" t="inlineStr">
+        <is>
+          <t>Age, Gender, Duration of PD, Place of Residence, Housing, Socioeconomic, Education, Peritonitis in ESI, Nutrition, Cause of ESRD, Type of Catheter (Shape), Type of Catheter (Cuff), Catheter Placement, Gastrostomy/Intraperitoneal Device, Performed CAPD, Starting PD &lt;2 weeks after placement, Catheter Orientation, Stunting</t>
+        </is>
+      </c>
+      <c r="Y56" t="inlineStr"/>
+      <c r="Z56" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2026-05-09 09:44:25</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>BBF800B7</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>&gt;2 yo</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>&lt;12 mo</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>Good service</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>Studies</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>No ESI</t>
+        </is>
+      </c>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>Normal Nutrition</t>
+        </is>
+      </c>
+      <c r="M57" t="inlineStr">
+        <is>
+          <t>Glomerular</t>
+        </is>
+      </c>
+      <c r="N57" t="inlineStr">
+        <is>
+          <t>Coiled/swan neck</t>
+        </is>
+      </c>
+      <c r="O57" t="inlineStr">
+        <is>
+          <t>Double</t>
+        </is>
+      </c>
+      <c r="P57" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="Q57" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R57" t="inlineStr">
+        <is>
+          <t>Patients</t>
+        </is>
+      </c>
+      <c r="S57" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T57" t="inlineStr">
+        <is>
+          <t>Lateral/downward</t>
+        </is>
+      </c>
+      <c r="U57" t="inlineStr">
+        <is>
+          <t>Stunting</t>
+        </is>
+      </c>
+      <c r="V57" t="inlineStr">
+        <is>
+          <t>95.45%</t>
+        </is>
+      </c>
+      <c r="W57" t="inlineStr">
+        <is>
+          <t>Survivor</t>
+        </is>
+      </c>
+      <c r="X57" t="inlineStr">
+        <is>
+          <t>Age, Gender, Duration of PD, Place of Residence, Housing, Socioeconomic, Education, Peritonitis in ESI, Nutrition, Cause of ESRD, Type of Catheter (Shape), Type of Catheter (Cuff), Catheter Placement, Gastrostomy/Intraperitoneal Device, Performed CAPD, Starting PD &lt;2 weeks after placement, Catheter Orientation</t>
+        </is>
+      </c>
+      <c r="Y57" t="inlineStr">
+        <is>
+          <t>Stunting</t>
+        </is>
+      </c>
+      <c r="Z57" t="inlineStr">
+        <is>
+          <t>Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>2026-05-09 09:44:54</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>BBF800B7</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>&gt;2 yo</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>&lt;12 mo</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>Good service</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>Studies</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>No ESI</t>
+        </is>
+      </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>Normal Nutrition</t>
+        </is>
+      </c>
+      <c r="M58" t="inlineStr">
+        <is>
+          <t>Glomerular</t>
+        </is>
+      </c>
+      <c r="N58" t="inlineStr">
+        <is>
+          <t>Coiled/swan neck</t>
+        </is>
+      </c>
+      <c r="O58" t="inlineStr">
+        <is>
+          <t>Double</t>
+        </is>
+      </c>
+      <c r="P58" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="Q58" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R58" t="inlineStr">
+        <is>
+          <t>Patients</t>
+        </is>
+      </c>
+      <c r="S58" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T58" t="inlineStr">
+        <is>
+          <t>Lateral/downward</t>
+        </is>
+      </c>
+      <c r="U58" t="inlineStr">
+        <is>
+          <t>Stunting</t>
+        </is>
+      </c>
+      <c r="V58" t="inlineStr">
+        <is>
+          <t>95.45%</t>
+        </is>
+      </c>
+      <c r="W58" t="inlineStr">
+        <is>
+          <t>Survivor</t>
+        </is>
+      </c>
+      <c r="X58" t="inlineStr">
+        <is>
+          <t>Age, Gender, Duration of PD, Place of Residence, Housing, Socioeconomic, Education, Peritonitis in ESI, Nutrition, Cause of ESRD, Type of Catheter (Shape), Type of Catheter (Cuff), Catheter Placement, Gastrostomy/Intraperitoneal Device, Performed CAPD, Starting PD &lt;2 weeks after placement, Catheter Orientation</t>
+        </is>
+      </c>
+      <c r="Y58" t="inlineStr">
+        <is>
+          <t>Stunting</t>
+        </is>
+      </c>
+      <c r="Z58" t="inlineStr">
+        <is>
+          <t>Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2026-05-09 09:46:32</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>BBF800B7</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>&gt;2 yo</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>&lt;12 mo</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>Good service</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>Studies</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>No ESI</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>Normal Nutrition</t>
+        </is>
+      </c>
+      <c r="M59" t="inlineStr">
+        <is>
+          <t>Glomerular</t>
+        </is>
+      </c>
+      <c r="N59" t="inlineStr">
+        <is>
+          <t>Coiled/swan neck</t>
+        </is>
+      </c>
+      <c r="O59" t="inlineStr">
+        <is>
+          <t>Double</t>
+        </is>
+      </c>
+      <c r="P59" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="Q59" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R59" t="inlineStr">
+        <is>
+          <t>Patients</t>
+        </is>
+      </c>
+      <c r="S59" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T59" t="inlineStr">
+        <is>
+          <t>Lateral/downward</t>
+        </is>
+      </c>
+      <c r="U59" t="inlineStr">
+        <is>
+          <t>Stunting</t>
+        </is>
+      </c>
+      <c r="V59" t="inlineStr">
+        <is>
+          <t>95.45%</t>
+        </is>
+      </c>
+      <c r="W59" t="inlineStr">
+        <is>
+          <t>Survivor</t>
+        </is>
+      </c>
+      <c r="X59" t="inlineStr">
+        <is>
+          <t>Age, Gender, Duration of PD, Place of Residence, Housing, Socioeconomic, Education, Peritonitis in ESI, Nutrition, Cause of ESRD, Type of Catheter (Shape), Type of Catheter (Cuff), Catheter Placement, Gastrostomy/Intraperitoneal Device, Performed CAPD, Starting PD &lt;2 weeks after placement, Catheter Orientation</t>
+        </is>
+      </c>
+      <c r="Y59" t="inlineStr">
+        <is>
+          <t>Stunting</t>
+        </is>
+      </c>
+      <c r="Z59" t="inlineStr">
+        <is>
+          <t>Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>2026-05-09 09:46:38</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>BBF800B7</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>&gt;2 yo</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>&lt;12 mo</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>Good service</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>Studies</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>No ESI</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>Normal Nutrition</t>
+        </is>
+      </c>
+      <c r="M60" t="inlineStr">
+        <is>
+          <t>Glomerular</t>
+        </is>
+      </c>
+      <c r="N60" t="inlineStr">
+        <is>
+          <t>Coiled/swan neck</t>
+        </is>
+      </c>
+      <c r="O60" t="inlineStr">
+        <is>
+          <t>Double</t>
+        </is>
+      </c>
+      <c r="P60" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="Q60" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R60" t="inlineStr">
+        <is>
+          <t>Patients</t>
+        </is>
+      </c>
+      <c r="S60" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T60" t="inlineStr">
+        <is>
+          <t>Lateral/downward</t>
+        </is>
+      </c>
+      <c r="U60" t="inlineStr">
+        <is>
+          <t>Stunting</t>
+        </is>
+      </c>
+      <c r="V60" t="inlineStr">
+        <is>
+          <t>95.45%</t>
+        </is>
+      </c>
+      <c r="W60" t="inlineStr">
+        <is>
+          <t>Survivor</t>
+        </is>
+      </c>
+      <c r="X60" t="inlineStr">
+        <is>
+          <t>Age, Gender, Duration of PD, Place of Residence, Housing, Socioeconomic, Education, Peritonitis in ESI, Nutrition, Cause of ESRD, Type of Catheter (Shape), Type of Catheter (Cuff), Catheter Placement, Gastrostomy/Intraperitoneal Device, Performed CAPD, Starting PD &lt;2 weeks after placement, Catheter Orientation</t>
+        </is>
+      </c>
+      <c r="Y60" t="inlineStr">
+        <is>
+          <t>Stunting</t>
+        </is>
+      </c>
+      <c r="Z60" t="inlineStr">
+        <is>
+          <t>Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2026-05-09 09:46:52</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>BBF800B7</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>&gt;2 yo</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>&lt;12 mo</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>Good service</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>Studies</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>No ESI</t>
+        </is>
+      </c>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>Normal Nutrition</t>
+        </is>
+      </c>
+      <c r="M61" t="inlineStr">
+        <is>
+          <t>Glomerular</t>
+        </is>
+      </c>
+      <c r="N61" t="inlineStr">
+        <is>
+          <t>Coiled/swan neck</t>
+        </is>
+      </c>
+      <c r="O61" t="inlineStr">
+        <is>
+          <t>Double</t>
+        </is>
+      </c>
+      <c r="P61" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="Q61" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R61" t="inlineStr">
+        <is>
+          <t>Patients</t>
+        </is>
+      </c>
+      <c r="S61" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T61" t="inlineStr">
+        <is>
+          <t>Lateral/downward</t>
+        </is>
+      </c>
+      <c r="U61" t="inlineStr">
+        <is>
+          <t>Stunting</t>
+        </is>
+      </c>
+      <c r="V61" t="inlineStr">
+        <is>
+          <t>95.45%</t>
+        </is>
+      </c>
+      <c r="W61" t="inlineStr">
+        <is>
+          <t>Survivor</t>
+        </is>
+      </c>
+      <c r="X61" t="inlineStr">
+        <is>
+          <t>Age, Gender, Duration of PD, Place of Residence, Housing, Socioeconomic, Education, Peritonitis in ESI, Nutrition, Cause of ESRD, Type of Catheter (Shape), Type of Catheter (Cuff), Catheter Placement, Gastrostomy/Intraperitoneal Device, Performed CAPD, Starting PD &lt;2 weeks after placement, Catheter Orientation</t>
+        </is>
+      </c>
+      <c r="Y61" t="inlineStr">
+        <is>
+          <t>Stunting</t>
+        </is>
+      </c>
+      <c r="Z61" t="inlineStr">
+        <is>
+          <t>Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>2026-05-09 09:47:25</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>BBF800B7</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>&gt;2 yo</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>&lt;12 mo</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>Good service</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>Studies</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>No ESI</t>
+        </is>
+      </c>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>Poor nutrition</t>
+        </is>
+      </c>
+      <c r="M62" t="inlineStr">
+        <is>
+          <t>Glomerular</t>
+        </is>
+      </c>
+      <c r="N62" t="inlineStr">
+        <is>
+          <t>Coiled/swan neck</t>
+        </is>
+      </c>
+      <c r="O62" t="inlineStr">
+        <is>
+          <t>Double</t>
+        </is>
+      </c>
+      <c r="P62" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="Q62" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R62" t="inlineStr">
+        <is>
+          <t>Patients</t>
+        </is>
+      </c>
+      <c r="S62" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T62" t="inlineStr">
+        <is>
+          <t>Lateral/downward</t>
+        </is>
+      </c>
+      <c r="U62" t="inlineStr">
+        <is>
+          <t>Stunting</t>
+        </is>
+      </c>
+      <c r="V62" t="inlineStr">
+        <is>
+          <t>90.91%</t>
+        </is>
+      </c>
+      <c r="W62" t="inlineStr">
+        <is>
+          <t>Survivor</t>
+        </is>
+      </c>
+      <c r="X62" t="inlineStr">
+        <is>
+          <t>Age, Gender, Duration of PD, Place of Residence, Housing, Socioeconomic, Education, Peritonitis in ESI, Cause of ESRD, Type of Catheter (Shape), Type of Catheter (Cuff), Catheter Placement, Gastrostomy/Intraperitoneal Device, Performed CAPD, Starting PD &lt;2 weeks after placement, Catheter Orientation</t>
+        </is>
+      </c>
+      <c r="Y62" t="inlineStr">
+        <is>
+          <t>Nutrition, Stunting</t>
+        </is>
+      </c>
+      <c r="Z62" t="inlineStr">
+        <is>
+          <t>Nutrition: Berikan asupan protein tinggi sesuai target usia (biasanya 1.4–3.0 g/kg/hari untuk anak) guna mengejar pertumbuhan dan mengganti protein yang hilang saat dialisis. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC7352713/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) | Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>2026-05-09 11:24:48</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>BB96B24A</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>&gt;2 yo</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>&lt;12 mo</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>Good service</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>Studies</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>No ESI</t>
+        </is>
+      </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>Poor nutrition</t>
+        </is>
+      </c>
+      <c r="M63" t="inlineStr">
+        <is>
+          <t>Glomerular</t>
+        </is>
+      </c>
+      <c r="N63" t="inlineStr">
+        <is>
+          <t>Coiled/swan neck</t>
+        </is>
+      </c>
+      <c r="O63" t="inlineStr">
+        <is>
+          <t>Double</t>
+        </is>
+      </c>
+      <c r="P63" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="Q63" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R63" t="inlineStr">
+        <is>
+          <t>Patients</t>
+        </is>
+      </c>
+      <c r="S63" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T63" t="inlineStr">
+        <is>
+          <t>Lateral/downward</t>
+        </is>
+      </c>
+      <c r="U63" t="inlineStr">
+        <is>
+          <t>Stunting</t>
+        </is>
+      </c>
+      <c r="V63" t="inlineStr">
+        <is>
+          <t>90.91%</t>
+        </is>
+      </c>
+      <c r="W63" t="inlineStr">
+        <is>
+          <t>Survivor</t>
+        </is>
+      </c>
+      <c r="X63" t="inlineStr">
+        <is>
+          <t>Age, Gender, Duration of PD, Place of Residence, Housing, Socioeconomic, Education, Peritonitis in ESI, Cause of ESRD, Type of Catheter (Shape), Type of Catheter (Cuff), Catheter Placement, Gastrostomy/Intraperitoneal Device, Performed CAPD, Starting PD &lt;2 weeks after placement, Catheter Orientation</t>
+        </is>
+      </c>
+      <c r="Y63" t="inlineStr">
+        <is>
+          <t>Nutrition, Stunting</t>
+        </is>
+      </c>
+      <c r="Z63" t="inlineStr">
+        <is>
+          <t>Nutrition: Rekomendasi asupan protein tinggi (1,4–3,0 g/kg/hari) disesuaikan dengan usia anak untuk mengganti kehilangan protein selama dialisis dan mengejar pertumbuhan. Pemantauan nutrisi dilakukan setiap bulan pada bayi dan setiap 3–4 bulan pada anak yang lebih tua. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC7352713/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) | Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>2026-05-09 11:26:04</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>BB96B24A</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>&gt;2 yo</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>&lt;12 mo</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>Good service</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>Studies</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>No ESI</t>
+        </is>
+      </c>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>Poor nutrition</t>
+        </is>
+      </c>
+      <c r="M64" t="inlineStr">
+        <is>
+          <t>Glomerular</t>
+        </is>
+      </c>
+      <c r="N64" t="inlineStr">
+        <is>
+          <t>Coiled/swan neck</t>
+        </is>
+      </c>
+      <c r="O64" t="inlineStr">
+        <is>
+          <t>Double</t>
+        </is>
+      </c>
+      <c r="P64" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="Q64" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R64" t="inlineStr">
+        <is>
+          <t>Patients</t>
+        </is>
+      </c>
+      <c r="S64" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T64" t="inlineStr">
+        <is>
+          <t>Lateral/downward</t>
+        </is>
+      </c>
+      <c r="U64" t="inlineStr">
+        <is>
+          <t>Stunting</t>
+        </is>
+      </c>
+      <c r="V64" t="inlineStr">
+        <is>
+          <t>90.91%</t>
+        </is>
+      </c>
+      <c r="W64" t="inlineStr">
+        <is>
+          <t>Survivor</t>
+        </is>
+      </c>
+      <c r="X64" t="inlineStr">
+        <is>
+          <t>Age, Gender, Duration of PD, Place of Residence, Housing, Socioeconomic, Education, Peritonitis in ESI, Cause of ESRD, Type of Catheter (Shape), Type of Catheter (Cuff), Catheter Placement, Gastrostomy/Intraperitoneal Device, Performed CAPD, Starting PD &lt;2 weeks after placement, Catheter Orientation</t>
+        </is>
+      </c>
+      <c r="Y64" t="inlineStr">
+        <is>
+          <t>Nutrition, Stunting</t>
+        </is>
+      </c>
+      <c r="Z64" t="inlineStr">
+        <is>
+          <t>Nutrition: Rekomendasi asupan protein tinggi (1,4–3,0 g/kg/hari) disesuaikan dengan usia anak untuk mengganti kehilangan protein selama dialisis dan mengejar pertumbuhan. Pemantauan nutrisi dilakukan setiap bulan pada bayi dan setiap 3–4 bulan pada anak yang lebih tua. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC7352713/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) | Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>2026-05-09 11:26:10</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>BB96B24A</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>&gt;2 yo</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>&lt;12 mo</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>Good service</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>Studies</t>
+        </is>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>No ESI</t>
+        </is>
+      </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>Normal Nutrition</t>
+        </is>
+      </c>
+      <c r="M65" t="inlineStr">
+        <is>
+          <t>Glomerular</t>
+        </is>
+      </c>
+      <c r="N65" t="inlineStr">
+        <is>
+          <t>Coiled/swan neck</t>
+        </is>
+      </c>
+      <c r="O65" t="inlineStr">
+        <is>
+          <t>Double</t>
+        </is>
+      </c>
+      <c r="P65" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="Q65" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R65" t="inlineStr">
+        <is>
+          <t>Patients</t>
+        </is>
+      </c>
+      <c r="S65" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T65" t="inlineStr">
+        <is>
+          <t>Lateral/downward</t>
+        </is>
+      </c>
+      <c r="U65" t="inlineStr">
+        <is>
+          <t>Stunting</t>
+        </is>
+      </c>
+      <c r="V65" t="inlineStr">
+        <is>
+          <t>95.45%</t>
+        </is>
+      </c>
+      <c r="W65" t="inlineStr">
+        <is>
+          <t>Survivor</t>
+        </is>
+      </c>
+      <c r="X65" t="inlineStr">
+        <is>
+          <t>Age, Gender, Duration of PD, Place of Residence, Housing, Socioeconomic, Education, Peritonitis in ESI, Nutrition, Cause of ESRD, Type of Catheter (Shape), Type of Catheter (Cuff), Catheter Placement, Gastrostomy/Intraperitoneal Device, Performed CAPD, Starting PD &lt;2 weeks after placement, Catheter Orientation</t>
+        </is>
+      </c>
+      <c r="Y65" t="inlineStr">
+        <is>
+          <t>Stunting</t>
+        </is>
+      </c>
+      <c r="Z65" t="inlineStr">
+        <is>
+          <t>Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>2026-05-09 11:31:49</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>BB96B24A</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>&gt;2 yo</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>&lt;12 mo</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>Good service</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>Studies</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>No ESI</t>
+        </is>
+      </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>Normal Nutrition</t>
+        </is>
+      </c>
+      <c r="M66" t="inlineStr">
+        <is>
+          <t>Glomerular</t>
+        </is>
+      </c>
+      <c r="N66" t="inlineStr">
+        <is>
+          <t>Coiled/swan neck</t>
+        </is>
+      </c>
+      <c r="O66" t="inlineStr">
+        <is>
+          <t>Double</t>
+        </is>
+      </c>
+      <c r="P66" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="Q66" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R66" t="inlineStr">
+        <is>
+          <t>Patients</t>
+        </is>
+      </c>
+      <c r="S66" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T66" t="inlineStr">
+        <is>
+          <t>Lateral/downward</t>
+        </is>
+      </c>
+      <c r="U66" t="inlineStr">
+        <is>
+          <t>Stunting</t>
+        </is>
+      </c>
+      <c r="V66" t="inlineStr">
+        <is>
+          <t>95.45%</t>
+        </is>
+      </c>
+      <c r="W66" t="inlineStr">
+        <is>
+          <t>Survivor</t>
+        </is>
+      </c>
+      <c r="X66" t="inlineStr">
+        <is>
+          <t>Age, Gender, Duration of PD, Place of Residence, Housing, Socioeconomic, Education, Peritonitis in ESI, Nutrition, Cause of ESRD, Type of Catheter (Shape), Type of Catheter (Cuff), Catheter Placement, Gastrostomy/Intraperitoneal Device, Performed CAPD, Starting PD &lt;2 weeks after placement, Catheter Orientation</t>
+        </is>
+      </c>
+      <c r="Y66" t="inlineStr">
+        <is>
+          <t>Stunting</t>
+        </is>
+      </c>
+      <c r="Z66" t="inlineStr">
+        <is>
+          <t>Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>2026-05-09 11:39:22</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>BB96B24A</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>&lt;2 yo</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>&lt;12 mo</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>Good service</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>Studies</t>
+        </is>
+      </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>No ESI</t>
+        </is>
+      </c>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>Normal Nutrition</t>
+        </is>
+      </c>
+      <c r="M67" t="inlineStr">
+        <is>
+          <t>Glomerular</t>
+        </is>
+      </c>
+      <c r="N67" t="inlineStr">
+        <is>
+          <t>Coiled/swan neck</t>
+        </is>
+      </c>
+      <c r="O67" t="inlineStr">
+        <is>
+          <t>Double</t>
+        </is>
+      </c>
+      <c r="P67" t="inlineStr">
+        <is>
+          <t>Laparoscopic</t>
+        </is>
+      </c>
+      <c r="Q67" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R67" t="inlineStr">
+        <is>
+          <t>Patients</t>
+        </is>
+      </c>
+      <c r="S67" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T67" t="inlineStr">
+        <is>
+          <t>Lateral/downward</t>
+        </is>
+      </c>
+      <c r="U67" t="inlineStr">
+        <is>
+          <t>Stunting</t>
+        </is>
+      </c>
+      <c r="V67" t="inlineStr">
+        <is>
+          <t>77.27%</t>
+        </is>
+      </c>
+      <c r="W67" t="inlineStr">
+        <is>
+          <t>Survivor</t>
+        </is>
+      </c>
+      <c r="X67" t="inlineStr">
+        <is>
+          <t>Duration of PD*, Place of Residence, Housing, Socioeconomic, Education, Peritonitis in ESI*, Nutrition, Cause of ESRD*, Type of Catheter (Shape), Type of Catheter (Cuff), Gastrostomy/Intraperitoneal Device, Performed CAPD, Starting PD &lt;2 weeks after placement, Catheter Orientation</t>
+        </is>
+      </c>
+      <c r="Y67" t="inlineStr">
+        <is>
+          <t>Age*, Gender, Catheter Placement, Stunting</t>
+        </is>
+      </c>
+      <c r="Z67" t="inlineStr">
+        <is>
+          <t>Catheter Placement: Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>2026-05-09 11:40:01</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>BB96B24A</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>&lt;2 yo</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>&lt;12 mo</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>Good service</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>Studies</t>
+        </is>
+      </c>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>No ESI</t>
+        </is>
+      </c>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>Normal Nutrition</t>
+        </is>
+      </c>
+      <c r="M68" t="inlineStr">
+        <is>
+          <t>Glomerular</t>
+        </is>
+      </c>
+      <c r="N68" t="inlineStr">
+        <is>
+          <t>Coiled/swan neck</t>
+        </is>
+      </c>
+      <c r="O68" t="inlineStr">
+        <is>
+          <t>Double</t>
+        </is>
+      </c>
+      <c r="P68" t="inlineStr">
+        <is>
+          <t>Laparoscopic</t>
+        </is>
+      </c>
+      <c r="Q68" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R68" t="inlineStr">
+        <is>
+          <t>Patients</t>
+        </is>
+      </c>
+      <c r="S68" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T68" t="inlineStr">
+        <is>
+          <t>upward</t>
+        </is>
+      </c>
+      <c r="U68" t="inlineStr">
+        <is>
+          <t>Stunting</t>
+        </is>
+      </c>
+      <c r="V68" t="inlineStr">
+        <is>
+          <t>72.73%</t>
+        </is>
+      </c>
+      <c r="W68" t="inlineStr">
+        <is>
+          <t>Survivor</t>
+        </is>
+      </c>
+      <c r="X68" t="inlineStr">
+        <is>
+          <t>Duration of PD*, Place of Residence, Housing, Socioeconomic, Education, Peritonitis in ESI*, Nutrition, Cause of ESRD*, Type of Catheter (Shape), Type of Catheter (Cuff), Gastrostomy/Intraperitoneal Device, Performed CAPD, Starting PD &lt;2 weeks after placement</t>
+        </is>
+      </c>
+      <c r="Y68" t="inlineStr">
+        <is>
+          <t>Age*, Gender, Catheter Placement, Catheter Orientation, Stunting</t>
+        </is>
+      </c>
+      <c r="Z68" t="inlineStr">
+        <is>
+          <t>Catheter Placement: Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Catheter Orientation:  | Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>2026-05-09 11:45:17</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>BB96B24A</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>&gt;2 yo</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>&lt;12 mo</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>Good service</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>Illiterate</t>
+        </is>
+      </c>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>No ESI</t>
+        </is>
+      </c>
+      <c r="L69" t="inlineStr">
+        <is>
+          <t>Normal Nutrition</t>
+        </is>
+      </c>
+      <c r="M69" t="inlineStr">
+        <is>
+          <t>Non-glomerular</t>
+        </is>
+      </c>
+      <c r="N69" t="inlineStr">
+        <is>
+          <t>Straight</t>
+        </is>
+      </c>
+      <c r="O69" t="inlineStr">
+        <is>
+          <t>Double</t>
+        </is>
+      </c>
+      <c r="P69" t="inlineStr">
+        <is>
+          <t>Laparoscopic</t>
+        </is>
+      </c>
+      <c r="Q69" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R69" t="inlineStr">
+        <is>
+          <t>Patients</t>
+        </is>
+      </c>
+      <c r="S69" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T69" t="inlineStr">
+        <is>
+          <t>upward</t>
+        </is>
+      </c>
+      <c r="U69" t="inlineStr">
+        <is>
+          <t>Stunting</t>
+        </is>
+      </c>
+      <c r="V69" t="inlineStr">
+        <is>
+          <t>63.64%</t>
+        </is>
+      </c>
+      <c r="W69" t="inlineStr">
+        <is>
+          <t>Survivor</t>
+        </is>
+      </c>
+      <c r="X69" t="inlineStr">
+        <is>
+          <t>Age*, Duration of PD*, Place of Residence, Housing, Socioeconomic, Peritonitis in ESI*, Nutrition, Type of Catheter (Cuff), Gastrostomy/Intraperitoneal Device, Performed CAPD, Starting PD &lt;2 weeks after placement</t>
+        </is>
+      </c>
+      <c r="Y69" t="inlineStr">
+        <is>
+          <t>Gender, Education, Cause of ESRD*, Type of Catheter (Shape), Catheter Placement, Catheter Orientation, Stunting</t>
+        </is>
+      </c>
+      <c r="Z69" t="inlineStr">
+        <is>
+          <t>Type of Catheter (Shape): Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Catheter Placement: Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Catheter Orientation:  | Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>2026-05-09 11:45:43</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>BB96B24A</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>&gt;2 yo</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>&lt;12 mo</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>Good service</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>Illiterate</t>
+        </is>
+      </c>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>No ESI</t>
+        </is>
+      </c>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>Poor nutrition</t>
+        </is>
+      </c>
+      <c r="M70" t="inlineStr">
+        <is>
+          <t>Non-glomerular</t>
+        </is>
+      </c>
+      <c r="N70" t="inlineStr">
+        <is>
+          <t>Straight</t>
+        </is>
+      </c>
+      <c r="O70" t="inlineStr">
+        <is>
+          <t>Double</t>
+        </is>
+      </c>
+      <c r="P70" t="inlineStr">
+        <is>
+          <t>Laparoscopic</t>
+        </is>
+      </c>
+      <c r="Q70" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R70" t="inlineStr">
+        <is>
+          <t>Patients</t>
+        </is>
+      </c>
+      <c r="S70" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T70" t="inlineStr">
+        <is>
+          <t>upward</t>
+        </is>
+      </c>
+      <c r="U70" t="inlineStr">
+        <is>
+          <t>Stunting</t>
+        </is>
+      </c>
+      <c r="V70" t="inlineStr">
+        <is>
+          <t>59.09%</t>
+        </is>
+      </c>
+      <c r="W70" t="inlineStr">
+        <is>
+          <t>Survivor</t>
+        </is>
+      </c>
+      <c r="X70" t="inlineStr">
+        <is>
+          <t>Age*, Duration of PD*, Place of Residence, Housing, Socioeconomic, Peritonitis in ESI*, Type of Catheter (Cuff), Gastrostomy/Intraperitoneal Device, Performed CAPD, Starting PD &lt;2 weeks after placement</t>
+        </is>
+      </c>
+      <c r="Y70" t="inlineStr">
+        <is>
+          <t>Gender, Education, Nutrition, Cause of ESRD*, Type of Catheter (Shape), Catheter Placement, Catheter Orientation, Stunting</t>
+        </is>
+      </c>
+      <c r="Z70" t="inlineStr">
+        <is>
+          <t>Nutrition: Rekomendasi asupan protein tinggi (1,4–3,0 g/kg/hari) disesuaikan dengan usia anak untuk mengganti kehilangan protein selama dialisis dan mengejar pertumbuhan. Pemantauan nutrisi dilakukan setiap bulan pada bayi dan setiap 3–4 bulan pada anak yang lebih tua. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC7352713/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) | Type of Catheter (Shape): Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Catheter Placement: Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Catheter Orientation:  | Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>2026-05-09 11:45:51</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>BB96B24A</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>&gt;2 yo</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>&lt;12 mo</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>Good service</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>Poor/fair</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>Illiterate</t>
+        </is>
+      </c>
+      <c r="K71" t="inlineStr">
+        <is>
+          <t>No ESI</t>
+        </is>
+      </c>
+      <c r="L71" t="inlineStr">
+        <is>
+          <t>Poor nutrition</t>
+        </is>
+      </c>
+      <c r="M71" t="inlineStr">
+        <is>
+          <t>Non-glomerular</t>
+        </is>
+      </c>
+      <c r="N71" t="inlineStr">
+        <is>
+          <t>Straight</t>
+        </is>
+      </c>
+      <c r="O71" t="inlineStr">
+        <is>
+          <t>Double</t>
+        </is>
+      </c>
+      <c r="P71" t="inlineStr">
+        <is>
+          <t>Laparoscopic</t>
+        </is>
+      </c>
+      <c r="Q71" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="R71" t="inlineStr">
+        <is>
+          <t>Patients</t>
+        </is>
+      </c>
+      <c r="S71" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T71" t="inlineStr">
+        <is>
+          <t>upward</t>
+        </is>
+      </c>
+      <c r="U71" t="inlineStr">
+        <is>
+          <t>Stunting</t>
+        </is>
+      </c>
+      <c r="V71" t="inlineStr">
+        <is>
+          <t>50.00%</t>
+        </is>
+      </c>
+      <c r="W71" t="inlineStr">
+        <is>
+          <t>Survivor</t>
+        </is>
+      </c>
+      <c r="X71" t="inlineStr">
+        <is>
+          <t>Age*, Duration of PD*, Place of Residence, Housing, Peritonitis in ESI*, Type of Catheter (Cuff), Performed CAPD, Starting PD &lt;2 weeks after placement</t>
+        </is>
+      </c>
+      <c r="Y71" t="inlineStr">
+        <is>
+          <t>Gender, Socioeconomic, Education, Nutrition, Cause of ESRD*, Type of Catheter (Shape), Catheter Placement, Gastrostomy/Intraperitoneal Device, Catheter Orientation, Stunting</t>
+        </is>
+      </c>
+      <c r="Z71" t="inlineStr">
+        <is>
+          <t>Socioeconomic: Edukasi atau retraining intensif bagi keluarga (caregiver) mengenai prosedur aseptik sangat dianjurkan, terutama bagi keluarga dengan keterbatasan akses informasi. [Sumber](https://www.researchgate.net/publication/45276240_Peritonitis_in_children_on_peritoneal_dialysis_in_Cape_Town_South_Africa_Epidemiology_and_risks) | Nutrition: Rekomendasi asupan protein tinggi (1,4–3,0 g/kg/hari) disesuaikan dengan usia anak untuk mengganti kehilangan protein selama dialisis dan mengejar pertumbuhan. Pemantauan nutrisi dilakukan setiap bulan pada bayi dan setiap 3–4 bulan pada anak yang lebih tua. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC7352713/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) | Type of Catheter (Shape): Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Catheter Placement: Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Gastrostomy/Intraperitoneal Device:  | Catheter Orientation:  | Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>2026-05-09 11:45:57</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>BB96B24A</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>&gt;2 yo</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>&gt;12 mo</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>Good service</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>Poor/fair</t>
+        </is>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>Illiterate</t>
+        </is>
+      </c>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>No ESI</t>
+        </is>
+      </c>
+      <c r="L72" t="inlineStr">
+        <is>
+          <t>Poor nutrition</t>
+        </is>
+      </c>
+      <c r="M72" t="inlineStr">
+        <is>
+          <t>Non-glomerular</t>
+        </is>
+      </c>
+      <c r="N72" t="inlineStr">
+        <is>
+          <t>Straight</t>
+        </is>
+      </c>
+      <c r="O72" t="inlineStr">
+        <is>
+          <t>Double</t>
+        </is>
+      </c>
+      <c r="P72" t="inlineStr">
+        <is>
+          <t>Laparoscopic</t>
+        </is>
+      </c>
+      <c r="Q72" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="R72" t="inlineStr">
+        <is>
+          <t>Patients</t>
+        </is>
+      </c>
+      <c r="S72" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T72" t="inlineStr">
+        <is>
+          <t>upward</t>
+        </is>
+      </c>
+      <c r="U72" t="inlineStr">
+        <is>
+          <t>Stunting</t>
+        </is>
+      </c>
+      <c r="V72" t="inlineStr">
+        <is>
+          <t>40.91%</t>
+        </is>
+      </c>
+      <c r="W72" t="inlineStr">
+        <is>
+          <t>Non-Survivor</t>
+        </is>
+      </c>
+      <c r="X72" t="inlineStr">
+        <is>
+          <t>Age*, Place of Residence, Housing, Peritonitis in ESI*, Type of Catheter (Cuff), Performed CAPD, Starting PD &lt;2 weeks after placement</t>
+        </is>
+      </c>
+      <c r="Y72" t="inlineStr">
+        <is>
+          <t>Gender, Duration of PD*, Socioeconomic, Education, Nutrition, Cause of ESRD*, Type of Catheter (Shape), Catheter Placement, Gastrostomy/Intraperitoneal Device, Catheter Orientation, Stunting</t>
+        </is>
+      </c>
+      <c r="Z72" t="inlineStr">
+        <is>
+          <t>Socioeconomic: Edukasi atau retraining intensif bagi keluarga (caregiver) mengenai prosedur aseptik sangat dianjurkan, terutama bagi keluarga dengan keterbatasan akses informasi. [Sumber](https://www.researchgate.net/publication/45276240_Peritonitis_in_children_on_peritoneal_dialysis_in_Cape_Town_South_Africa_Epidemiology_and_risks) | Nutrition: Rekomendasi asupan protein tinggi (1,4–3,0 g/kg/hari) disesuaikan dengan usia anak untuk mengganti kehilangan protein selama dialisis dan mengejar pertumbuhan. Pemantauan nutrisi dilakukan setiap bulan pada bayi dan setiap 3–4 bulan pada anak yang lebih tua. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC7352713/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) | Type of Catheter (Shape): Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Catheter Placement: Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Gastrostomy/Intraperitoneal Device:  | Catheter Orientation:  | Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>2026-05-09 11:47:33</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>BB96B24A</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>&gt;2 yo</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>&gt;12 mo</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>Fair/poor service</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>Poor/fair</t>
+        </is>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>Illiterate</t>
+        </is>
+      </c>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>No ESI</t>
+        </is>
+      </c>
+      <c r="L73" t="inlineStr">
+        <is>
+          <t>Poor nutrition</t>
+        </is>
+      </c>
+      <c r="M73" t="inlineStr">
+        <is>
+          <t>Non-glomerular</t>
+        </is>
+      </c>
+      <c r="N73" t="inlineStr">
+        <is>
+          <t>Straight</t>
+        </is>
+      </c>
+      <c r="O73" t="inlineStr">
+        <is>
+          <t>Double</t>
+        </is>
+      </c>
+      <c r="P73" t="inlineStr">
+        <is>
+          <t>Laparoscopic</t>
+        </is>
+      </c>
+      <c r="Q73" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="R73" t="inlineStr">
+        <is>
+          <t>Patients</t>
+        </is>
+      </c>
+      <c r="S73" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T73" t="inlineStr">
+        <is>
+          <t>upward</t>
+        </is>
+      </c>
+      <c r="U73" t="inlineStr">
+        <is>
+          <t>Stunting</t>
+        </is>
+      </c>
+      <c r="V73" t="inlineStr">
+        <is>
+          <t>36.36%</t>
+        </is>
+      </c>
+      <c r="W73" t="inlineStr">
+        <is>
+          <t>Non-Survivor</t>
+        </is>
+      </c>
+      <c r="X73" t="inlineStr">
+        <is>
+          <t>Age*, Place of Residence, Peritonitis in ESI*, Type of Catheter (Cuff), Performed CAPD, Starting PD &lt;2 weeks after placement</t>
+        </is>
+      </c>
+      <c r="Y73" t="inlineStr">
+        <is>
+          <t>Gender, Duration of PD*, Housing, Socioeconomic, Education, Nutrition, Cause of ESRD*, Type of Catheter (Shape), Catheter Placement, Gastrostomy/Intraperitoneal Device, Catheter Orientation, Stunting</t>
+        </is>
+      </c>
+      <c r="Z73" t="inlineStr">
+        <is>
+          <t>Housing: Ruangan harus bersih dan bebas dari hewan peliharaan selama prosedur untuk menghindari risiko kontaminasi bakteri Pasteurella atau kerusakan mekanis pada selang. Ketersediaan wastafel untuk mencuci tangan secara benar sangat krusial dalam mengurangi risiko peritonitis. [🔗Sumber 1](https://freseniusmedicalcare.com/content/dam/home-products-education/steps2home-pd/Preventing_Peritonitis.pdf) [🔗Sumber 2](https://spnp-spp.pt/media/rqdpbrom/catheter-related-infections-and-peritonitis-in-pediatric-patients-receiving-peritoneal-dialysis-guideline-for-prevention-and-treatment-2012-1-_compressed-1.pdf) [Sumber 3](https://www.ouh.nhs.uk/media/agxhnni2/85713pdialysis.pdf) [Sumber 4](https://www.satellitehealthcare.com/blog/pets-and-peritoneal-dialysis-absolutely/) | Socioeconomic: Edukasi atau retraining intensif bagi keluarga (caregiver) mengenai prosedur aseptik sangat dianjurkan, terutama bagi keluarga dengan keterbatasan akses informasi. [Sumber](https://www.researchgate.net/publication/45276240_Peritonitis_in_children_on_peritoneal_dialysis_in_Cape_Town_South_Africa_Epidemiology_and_risks) | Nutrition: Rekomendasi asupan protein tinggi (1,4–3,0 g/kg/hari) disesuaikan dengan usia anak untuk mengganti kehilangan protein selama dialisis dan mengejar pertumbuhan. Pemantauan nutrisi dilakukan setiap bulan pada bayi dan setiap 3–4 bulan pada anak yang lebih tua. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC7352713/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) | Type of Catheter (Shape): Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Catheter Placement: Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Gastrostomy/Intraperitoneal Device:  | Catheter Orientation:  | Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>2026-05-09 11:49:39</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>BB96B24A</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>&gt;2 yo</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>&gt;12 mo</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>Fair/poor service</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>Poor/fair</t>
+        </is>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>Illiterate</t>
+        </is>
+      </c>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t>No ESI</t>
+        </is>
+      </c>
+      <c r="L74" t="inlineStr">
+        <is>
+          <t>Poor nutrition</t>
+        </is>
+      </c>
+      <c r="M74" t="inlineStr">
+        <is>
+          <t>Non-glomerular</t>
+        </is>
+      </c>
+      <c r="N74" t="inlineStr">
+        <is>
+          <t>Straight</t>
+        </is>
+      </c>
+      <c r="O74" t="inlineStr">
+        <is>
+          <t>Double</t>
+        </is>
+      </c>
+      <c r="P74" t="inlineStr">
+        <is>
+          <t>Laparoscopic</t>
+        </is>
+      </c>
+      <c r="Q74" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="R74" t="inlineStr">
+        <is>
+          <t>Patients</t>
+        </is>
+      </c>
+      <c r="S74" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T74" t="inlineStr">
+        <is>
+          <t>upward</t>
+        </is>
+      </c>
+      <c r="U74" t="inlineStr">
+        <is>
+          <t>Stunting</t>
+        </is>
+      </c>
+      <c r="V74" t="inlineStr">
+        <is>
+          <t>36.36%</t>
+        </is>
+      </c>
+      <c r="W74" t="inlineStr">
+        <is>
+          <t>Non-Survivor</t>
+        </is>
+      </c>
+      <c r="X74" t="inlineStr">
+        <is>
+          <t>Age*, Place of Residence, Peritonitis in ESI*, Type of Catheter (Cuff), Performed CAPD, Starting PD &lt;2 weeks after placement</t>
+        </is>
+      </c>
+      <c r="Y74" t="inlineStr">
+        <is>
+          <t>Gender, Duration of PD*, Housing, Socioeconomic, Education, Nutrition, Cause of ESRD*, Type of Catheter (Shape), Catheter Placement, Gastrostomy/Intraperitoneal Device, Catheter Orientation, Stunting</t>
+        </is>
+      </c>
+      <c r="Z74" t="inlineStr">
+        <is>
+          <t>Housing: Ruangan harus bersih dan bebas dari hewan peliharaan selama prosedur untuk menghindari risiko kontaminasi bakteri Pasteurella atau kerusakan mekanis pada selang. Ketersediaan wastafel untuk mencuci tangan secara benar sangat krusial dalam mengurangi risiko peritonitis. [🔗Sumber 1](https://freseniusmedicalcare.com/content/dam/home-products-education/steps2home-pd/Preventing_Peritonitis.pdf) [🔗Sumber 2](https://spnp-spp.pt/media/rqdpbrom/catheter-related-infections-and-peritonitis-in-pediatric-patients-receiving-peritoneal-dialysis-guideline-for-prevention-and-treatment-2012-1-_compressed-1.pdf) [Sumber 3](https://www.ouh.nhs.uk/media/agxhnni2/85713pdialysis.pdf) [Sumber 4](https://www.satellitehealthcare.com/blog/pets-and-peritoneal-dialysis-absolutely/) | Socioeconomic: Edukasi atau retraining intensif bagi keluarga (caregiver) mengenai prosedur aseptik sangat dianjurkan, terutama bagi keluarga dengan keterbatasan akses informasi. [Sumber](https://www.researchgate.net/publication/45276240_Peritonitis_in_children_on_peritoneal_dialysis_in_Cape_Town_South_Africa_Epidemiology_and_risks) | Nutrition: Rekomendasi asupan protein tinggi (1,4–3,0 g/kg/hari) disesuaikan dengan usia anak untuk mengganti kehilangan protein selama dialisis dan mengejar pertumbuhan. Pemantauan nutrisi dilakukan setiap bulan pada bayi dan setiap 3–4 bulan pada anak yang lebih tua. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC7352713/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) | Type of Catheter (Shape): Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Catheter Placement: Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Gastrostomy/Intraperitoneal Device:  | Catheter Orientation:  | Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>2026-05-09 11:53:50</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>BB96B24A</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>&gt;2 yo</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>&gt;12 mo</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>Fair/poor service</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>Poor/fair</t>
+        </is>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>Illiterate</t>
+        </is>
+      </c>
+      <c r="K75" t="inlineStr">
+        <is>
+          <t>No ESI</t>
+        </is>
+      </c>
+      <c r="L75" t="inlineStr">
+        <is>
+          <t>Poor nutrition</t>
+        </is>
+      </c>
+      <c r="M75" t="inlineStr">
+        <is>
+          <t>Non-glomerular</t>
+        </is>
+      </c>
+      <c r="N75" t="inlineStr">
+        <is>
+          <t>Straight</t>
+        </is>
+      </c>
+      <c r="O75" t="inlineStr">
+        <is>
+          <t>Double</t>
+        </is>
+      </c>
+      <c r="P75" t="inlineStr">
+        <is>
+          <t>Laparoscopic</t>
+        </is>
+      </c>
+      <c r="Q75" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="R75" t="inlineStr">
+        <is>
+          <t>Patients</t>
+        </is>
+      </c>
+      <c r="S75" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T75" t="inlineStr">
+        <is>
+          <t>upward</t>
+        </is>
+      </c>
+      <c r="U75" t="inlineStr">
+        <is>
+          <t>Stunting</t>
+        </is>
+      </c>
+      <c r="V75" t="inlineStr">
+        <is>
+          <t>36.36%</t>
+        </is>
+      </c>
+      <c r="W75" t="inlineStr">
+        <is>
+          <t>Non-Survivor</t>
+        </is>
+      </c>
+      <c r="X75" t="inlineStr">
+        <is>
+          <t>Age*, Place of Residence, Peritonitis in ESI*, Type of Catheter (Cuff), Performed CAPD, Starting PD &lt;2 weeks after placement</t>
+        </is>
+      </c>
+      <c r="Y75" t="inlineStr">
+        <is>
+          <t>Gender, Duration of PD*, Housing, Socioeconomic, Education, Nutrition, Cause of ESRD*, Type of Catheter (Shape), Catheter Placement, Gastrostomy/Intraperitoneal Device, Catheter Orientation, Stunting</t>
+        </is>
+      </c>
+      <c r="Z75" t="inlineStr">
+        <is>
+          <t>Housing: Ruangan harus bersih dan bebas dari hewan peliharaan selama prosedur untuk menghindari risiko kontaminasi bakteri Pasteurella atau kerusakan mekanis pada selang. Ketersediaan wastafel untuk mencuci tangan secara benar sangat krusial dalam mengurangi risiko peritonitis. [🔗Sumber 1](https://freseniusmedicalcare.com/content/dam/home-products-education/steps2home-pd/Preventing_Peritonitis.pdf) [🔗Sumber 2](https://spnp-spp.pt/media/rqdpbrom/catheter-related-infections-and-peritonitis-in-pediatric-patients-receiving-peritoneal-dialysis-guideline-for-prevention-and-treatment-2012-1-_compressed-1.pdf) [Sumber 3](https://www.ouh.nhs.uk/media/agxhnni2/85713pdialysis.pdf) [Sumber 4](https://www.satellitehealthcare.com/blog/pets-and-peritoneal-dialysis-absolutely/) | Socioeconomic: Edukasi atau retraining intensif bagi keluarga (caregiver) mengenai prosedur aseptik sangat dianjurkan, terutama bagi keluarga dengan keterbatasan akses informasi. [Sumber](https://www.researchgate.net/publication/45276240_Peritonitis_in_children_on_peritoneal_dialysis_in_Cape_Town_South_Africa_Epidemiology_and_risks) | Nutrition: Rekomendasi asupan protein tinggi (1,4–3,0 g/kg/hari) disesuaikan dengan usia anak untuk mengganti kehilangan protein selama dialisis dan mengejar pertumbuhan. Pemantauan nutrisi dilakukan setiap bulan pada bayi dan setiap 3–4 bulan pada anak yang lebih tua. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC7352713/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) | Type of Catheter (Shape): Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Catheter Placement: Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Gastrostomy/Intraperitoneal Device:  | Catheter Orientation:  | Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>2026-05-09 11:54:15</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>BB96B24A</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>&gt;2 yo</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>&gt;12 mo</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>Fair/poor service</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>Poor/fair</t>
+        </is>
+      </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>Illiterate</t>
+        </is>
+      </c>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t>No ESI</t>
+        </is>
+      </c>
+      <c r="L76" t="inlineStr">
+        <is>
+          <t>Poor nutrition</t>
+        </is>
+      </c>
+      <c r="M76" t="inlineStr">
+        <is>
+          <t>Non-glomerular</t>
+        </is>
+      </c>
+      <c r="N76" t="inlineStr">
+        <is>
+          <t>Straight</t>
+        </is>
+      </c>
+      <c r="O76" t="inlineStr">
+        <is>
+          <t>Double</t>
+        </is>
+      </c>
+      <c r="P76" t="inlineStr">
+        <is>
+          <t>Laparoscopic</t>
+        </is>
+      </c>
+      <c r="Q76" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="R76" t="inlineStr">
+        <is>
+          <t>Patients</t>
+        </is>
+      </c>
+      <c r="S76" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T76" t="inlineStr">
+        <is>
+          <t>upward</t>
+        </is>
+      </c>
+      <c r="U76" t="inlineStr">
+        <is>
+          <t>Stunting</t>
+        </is>
+      </c>
+      <c r="V76" t="inlineStr">
+        <is>
+          <t>36.36%</t>
+        </is>
+      </c>
+      <c r="W76" t="inlineStr">
+        <is>
+          <t>Non-Survivor</t>
+        </is>
+      </c>
+      <c r="X76" t="inlineStr">
+        <is>
+          <t>Age*, Place of Residence, Peritonitis in ESI*, Type of Catheter (Cuff), Performed CAPD, Starting PD &lt;2 weeks after placement</t>
+        </is>
+      </c>
+      <c r="Y76" t="inlineStr">
+        <is>
+          <t>Gender, Duration of PD*, Housing, Socioeconomic, Education, Nutrition, Cause of ESRD*, Type of Catheter (Shape), Catheter Placement, Gastrostomy/Intraperitoneal Device, Catheter Orientation, Stunting</t>
+        </is>
+      </c>
+      <c r="Z76" t="inlineStr">
+        <is>
+          <t>Housing: Ruangan harus bersih dan bebas dari hewan peliharaan selama prosedur untuk menghindari risiko kontaminasi bakteri Pasteurella atau kerusakan mekanis pada selang. Ketersediaan wastafel untuk mencuci tangan secara benar sangat krusial dalam mengurangi risiko peritonitis. [🔗Sumber 1](https://freseniusmedicalcare.com/content/dam/home-products-education/steps2home-pd/Preventing_Peritonitis.pdf) [🔗Sumber 2](https://spnp-spp.pt/media/rqdpbrom/catheter-related-infections-and-peritonitis-in-pediatric-patients-receiving-peritoneal-dialysis-guideline-for-prevention-and-treatment-2012-1-_compressed-1.pdf) [Sumber 3](https://www.ouh.nhs.uk/media/agxhnni2/85713pdialysis.pdf) [Sumber 4](https://www.satellitehealthcare.com/blog/pets-and-peritoneal-dialysis-absolutely/) | Socioeconomic: Edukasi atau retraining intensif bagi keluarga (caregiver) mengenai prosedur aseptik sangat dianjurkan, terutama bagi keluarga dengan keterbatasan akses informasi. [Sumber](https://www.researchgate.net/publication/45276240_Peritonitis_in_children_on_peritoneal_dialysis_in_Cape_Town_South_Africa_Epidemiology_and_risks) | Nutrition: Rekomendasi asupan protein tinggi (1,4–3,0 g/kg/hari) disesuaikan dengan usia anak untuk mengganti kehilangan protein selama dialisis dan mengejar pertumbuhan. Pemantauan nutrisi dilakukan setiap bulan pada bayi dan setiap 3–4 bulan pada anak yang lebih tua. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC7352713/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) | Type of Catheter (Shape): Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Catheter Placement: Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Gastrostomy/Intraperitoneal Device:  | Catheter Orientation:  | Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>2026-05-09 11:55:11</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>BB96B24A</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>&gt;2 yo</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>&gt;12 mo</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>Fair/poor service</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>Poor/fair</t>
+        </is>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>Illiterate</t>
+        </is>
+      </c>
+      <c r="K77" t="inlineStr">
+        <is>
+          <t>No ESI</t>
+        </is>
+      </c>
+      <c r="L77" t="inlineStr">
+        <is>
+          <t>Poor nutrition</t>
+        </is>
+      </c>
+      <c r="M77" t="inlineStr">
+        <is>
+          <t>Non-glomerular</t>
+        </is>
+      </c>
+      <c r="N77" t="inlineStr">
+        <is>
+          <t>Straight</t>
+        </is>
+      </c>
+      <c r="O77" t="inlineStr">
+        <is>
+          <t>Double</t>
+        </is>
+      </c>
+      <c r="P77" t="inlineStr">
+        <is>
+          <t>Laparoscopic</t>
+        </is>
+      </c>
+      <c r="Q77" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="R77" t="inlineStr">
+        <is>
+          <t>Patients</t>
+        </is>
+      </c>
+      <c r="S77" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T77" t="inlineStr">
+        <is>
+          <t>upward</t>
+        </is>
+      </c>
+      <c r="U77" t="inlineStr">
+        <is>
+          <t>Stunting</t>
+        </is>
+      </c>
+      <c r="V77" t="inlineStr">
+        <is>
+          <t>36.36%</t>
+        </is>
+      </c>
+      <c r="W77" t="inlineStr">
+        <is>
+          <t>Non-Survivor</t>
+        </is>
+      </c>
+      <c r="X77" t="inlineStr">
+        <is>
+          <t>Age*, Place of Residence, Peritonitis in ESI*, Type of Catheter (Cuff), Performed CAPD, Starting PD &lt;2 weeks after placement</t>
+        </is>
+      </c>
+      <c r="Y77" t="inlineStr">
+        <is>
+          <t>Gender, Duration of PD*, Housing, Socioeconomic, Education, Nutrition, Cause of ESRD*, Type of Catheter (Shape), Catheter Placement, Gastrostomy/Intraperitoneal Device, Catheter Orientation, Stunting</t>
+        </is>
+      </c>
+      <c r="Z77" t="inlineStr">
+        <is>
+          <t>Housing: Ruangan harus bersih dan bebas dari hewan peliharaan selama prosedur untuk menghindari risiko kontaminasi bakteri Pasteurella atau kerusakan mekanis pada selang. Ketersediaan wastafel untuk mencuci tangan secara benar sangat krusial dalam mengurangi risiko peritonitis. [🔗Sumber 1](https://freseniusmedicalcare.com/content/dam/home-products-education/steps2home-pd/Preventing_Peritonitis.pdf) [🔗Sumber 2](https://spnp-spp.pt/media/rqdpbrom/catheter-related-infections-and-peritonitis-in-pediatric-patients-receiving-peritoneal-dialysis-guideline-for-prevention-and-treatment-2012-1-_compressed-1.pdf) [Sumber 3](https://www.ouh.nhs.uk/media/agxhnni2/85713pdialysis.pdf) [Sumber 4](https://www.satellitehealthcare.com/blog/pets-and-peritoneal-dialysis-absolutely/) | Socioeconomic: Edukasi atau retraining intensif bagi keluarga (caregiver) mengenai prosedur aseptik sangat dianjurkan, terutama bagi keluarga dengan keterbatasan akses informasi. [Sumber](https://www.researchgate.net/publication/45276240_Peritonitis_in_children_on_peritoneal_dialysis_in_Cape_Town_South_Africa_Epidemiology_and_risks) | Nutrition: Rekomendasi asupan protein tinggi (1,4–3,0 g/kg/hari) disesuaikan dengan usia anak untuk mengganti kehilangan protein selama dialisis dan mengejar pertumbuhan. Pemantauan nutrisi dilakukan setiap bulan pada bayi dan setiap 3–4 bulan pada anak yang lebih tua. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC7352713/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) | Type of Catheter (Shape): Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Catheter Placement: Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Gastrostomy/Intraperitoneal Device:  | Catheter Orientation:  | Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>2026-05-09 11:55:36</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>BB96B24A</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>&gt;2 yo</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>&gt;12 mo</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>Fair/poor service</t>
+        </is>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>Poor/fair</t>
+        </is>
+      </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>Illiterate</t>
+        </is>
+      </c>
+      <c r="K78" t="inlineStr">
+        <is>
+          <t>No ESI</t>
+        </is>
+      </c>
+      <c r="L78" t="inlineStr">
+        <is>
+          <t>Poor nutrition</t>
+        </is>
+      </c>
+      <c r="M78" t="inlineStr">
+        <is>
+          <t>Non-glomerular</t>
+        </is>
+      </c>
+      <c r="N78" t="inlineStr">
+        <is>
+          <t>Straight</t>
+        </is>
+      </c>
+      <c r="O78" t="inlineStr">
+        <is>
+          <t>Double</t>
+        </is>
+      </c>
+      <c r="P78" t="inlineStr">
+        <is>
+          <t>Laparoscopic</t>
+        </is>
+      </c>
+      <c r="Q78" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="R78" t="inlineStr">
+        <is>
+          <t>Patients</t>
+        </is>
+      </c>
+      <c r="S78" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T78" t="inlineStr">
+        <is>
+          <t>upward</t>
+        </is>
+      </c>
+      <c r="U78" t="inlineStr">
+        <is>
+          <t>Stunting</t>
+        </is>
+      </c>
+      <c r="V78" t="inlineStr">
+        <is>
+          <t>36.36%</t>
+        </is>
+      </c>
+      <c r="W78" t="inlineStr">
+        <is>
+          <t>Non-Survivor</t>
+        </is>
+      </c>
+      <c r="X78" t="inlineStr">
+        <is>
+          <t>Age*, Place of Residence, Peritonitis in ESI*, Type of Catheter (Cuff), Performed CAPD, Starting PD &lt;2 weeks after placement</t>
+        </is>
+      </c>
+      <c r="Y78" t="inlineStr">
+        <is>
+          <t>Gender, Duration of PD*, Housing, Socioeconomic, Education, Nutrition, Cause of ESRD*, Type of Catheter (Shape), Catheter Placement, Gastrostomy/Intraperitoneal Device, Catheter Orientation, Stunting</t>
+        </is>
+      </c>
+      <c r="Z78" t="inlineStr">
+        <is>
+          <t>Housing: Ruangan harus bersih dan bebas dari hewan peliharaan selama prosedur untuk menghindari risiko kontaminasi bakteri Pasteurella atau kerusakan mekanis pada selang. Ketersediaan wastafel untuk mencuci tangan secara benar sangat krusial dalam mengurangi risiko peritonitis. [🔗Sumber 1](https://freseniusmedicalcare.com/content/dam/home-products-education/steps2home-pd/Preventing_Peritonitis.pdf) [🔗Sumber 2](https://spnp-spp.pt/media/rqdpbrom/catheter-related-infections-and-peritonitis-in-pediatric-patients-receiving-peritoneal-dialysis-guideline-for-prevention-and-treatment-2012-1-_compressed-1.pdf) [Sumber 3](https://www.ouh.nhs.uk/media/agxhnni2/85713pdialysis.pdf) [Sumber 4](https://www.satellitehealthcare.com/blog/pets-and-peritoneal-dialysis-absolutely/) | Socioeconomic: Edukasi atau retraining intensif bagi keluarga (caregiver) mengenai prosedur aseptik sangat dianjurkan, terutama bagi keluarga dengan keterbatasan akses informasi. [Sumber](https://www.researchgate.net/publication/45276240_Peritonitis_in_children_on_peritoneal_dialysis_in_Cape_Town_South_Africa_Epidemiology_and_risks) | Nutrition: Rekomendasi asupan protein tinggi (1,4–3,0 g/kg/hari) disesuaikan dengan usia anak untuk mengganti kehilangan protein selama dialisis dan mengejar pertumbuhan. Pemantauan nutrisi dilakukan setiap bulan pada bayi dan setiap 3–4 bulan pada anak yang lebih tua. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC7352713/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) | Type of Catheter (Shape): Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Catheter Placement: Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Gastrostomy/Intraperitoneal Device:  | Catheter Orientation:  | Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>2026-05-09 11:56:38</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>BB96B24A</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>&gt;2 yo</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>&gt;12 mo</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>Fair/poor service</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>Poor/fair</t>
+        </is>
+      </c>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>Illiterate</t>
+        </is>
+      </c>
+      <c r="K79" t="inlineStr">
+        <is>
+          <t>No ESI</t>
+        </is>
+      </c>
+      <c r="L79" t="inlineStr">
+        <is>
+          <t>Poor nutrition</t>
+        </is>
+      </c>
+      <c r="M79" t="inlineStr">
+        <is>
+          <t>Non-glomerular</t>
+        </is>
+      </c>
+      <c r="N79" t="inlineStr">
+        <is>
+          <t>Straight</t>
+        </is>
+      </c>
+      <c r="O79" t="inlineStr">
+        <is>
+          <t>Double</t>
+        </is>
+      </c>
+      <c r="P79" t="inlineStr">
+        <is>
+          <t>Laparoscopic</t>
+        </is>
+      </c>
+      <c r="Q79" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="R79" t="inlineStr">
+        <is>
+          <t>Patients</t>
+        </is>
+      </c>
+      <c r="S79" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T79" t="inlineStr">
+        <is>
+          <t>upward</t>
+        </is>
+      </c>
+      <c r="U79" t="inlineStr">
+        <is>
+          <t>Stunting</t>
+        </is>
+      </c>
+      <c r="V79" t="inlineStr">
+        <is>
+          <t>36.36%</t>
+        </is>
+      </c>
+      <c r="W79" t="inlineStr">
+        <is>
+          <t>Non-Survivor</t>
+        </is>
+      </c>
+      <c r="X79" t="inlineStr">
+        <is>
+          <t>Age*, Place of Residence, Peritonitis in ESI*, Type of Catheter (Cuff), Performed CAPD, Starting PD &lt;2 weeks after placement</t>
+        </is>
+      </c>
+      <c r="Y79" t="inlineStr">
+        <is>
+          <t>Gender, Duration of PD*, Housing, Socioeconomic, Education, Nutrition, Cause of ESRD*, Type of Catheter (Shape), Catheter Placement, Gastrostomy/Intraperitoneal Device, Catheter Orientation, Stunting</t>
+        </is>
+      </c>
+      <c r="Z79" t="inlineStr">
+        <is>
+          <t>Housing: Ruangan harus bersih dan bebas dari hewan peliharaan selama prosedur untuk menghindari risiko kontaminasi bakteri Pasteurella atau kerusakan mekanis pada selang. Ketersediaan wastafel untuk mencuci tangan secara benar sangat krusial dalam mengurangi risiko peritonitis. [🔗Sumber 1](https://freseniusmedicalcare.com/content/dam/home-products-education/steps2home-pd/Preventing_Peritonitis.pdf) [🔗Sumber 2](https://spnp-spp.pt/media/rqdpbrom/catheter-related-infections-and-peritonitis-in-pediatric-patients-receiving-peritoneal-dialysis-guideline-for-prevention-and-treatment-2012-1-_compressed-1.pdf) [Sumber 3](https://www.ouh.nhs.uk/media/agxhnni2/85713pdialysis.pdf) [Sumber 4](https://www.satellitehealthcare.com/blog/pets-and-peritoneal-dialysis-absolutely/) | Socioeconomic: Edukasi atau retraining intensif bagi keluarga (caregiver) mengenai prosedur aseptik sangat dianjurkan, terutama bagi keluarga dengan keterbatasan akses informasi. [Sumber](https://www.researchgate.net/publication/45276240_Peritonitis_in_children_on_peritoneal_dialysis_in_Cape_Town_South_Africa_Epidemiology_and_risks) | Nutrition: Rekomendasi asupan protein tinggi (1,4–3,0 g/kg/hari) disesuaikan dengan usia anak untuk mengganti kehilangan protein selama dialisis dan mengejar pertumbuhan. Pemantauan nutrisi dilakukan setiap bulan pada bayi dan setiap 3–4 bulan pada anak yang lebih tua. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC7352713/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) | Type of Catheter (Shape): Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Catheter Placement: Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Gastrostomy/Intraperitoneal Device:  | Catheter Orientation:  | Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>2026-05-09 11:56:51</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>BB96B24A</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>&gt;2 yo</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>&gt;12 mo</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>Fair/poor service</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>Poor/fair</t>
+        </is>
+      </c>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>Illiterate</t>
+        </is>
+      </c>
+      <c r="K80" t="inlineStr">
+        <is>
+          <t>No ESI</t>
+        </is>
+      </c>
+      <c r="L80" t="inlineStr">
+        <is>
+          <t>Poor nutrition</t>
+        </is>
+      </c>
+      <c r="M80" t="inlineStr">
+        <is>
+          <t>Non-glomerular</t>
+        </is>
+      </c>
+      <c r="N80" t="inlineStr">
+        <is>
+          <t>Straight</t>
+        </is>
+      </c>
+      <c r="O80" t="inlineStr">
+        <is>
+          <t>Double</t>
+        </is>
+      </c>
+      <c r="P80" t="inlineStr">
+        <is>
+          <t>Laparoscopic</t>
+        </is>
+      </c>
+      <c r="Q80" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="R80" t="inlineStr">
+        <is>
+          <t>Patients</t>
+        </is>
+      </c>
+      <c r="S80" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T80" t="inlineStr">
+        <is>
+          <t>upward</t>
+        </is>
+      </c>
+      <c r="U80" t="inlineStr">
+        <is>
+          <t>Stunting</t>
+        </is>
+      </c>
+      <c r="V80" t="inlineStr">
+        <is>
+          <t>36.36%</t>
+        </is>
+      </c>
+      <c r="W80" t="inlineStr">
+        <is>
+          <t>Non-Survivor</t>
+        </is>
+      </c>
+      <c r="X80" t="inlineStr">
+        <is>
+          <t>Age*, Place of Residence, Peritonitis in ESI*, Type of Catheter (Cuff), Performed CAPD, Starting PD &lt;2 weeks after placement</t>
+        </is>
+      </c>
+      <c r="Y80" t="inlineStr">
+        <is>
+          <t>Gender, Duration of PD*, Housing, Socioeconomic, Education, Nutrition, Cause of ESRD*, Type of Catheter (Shape), Catheter Placement, Gastrostomy/Intraperitoneal Device, Catheter Orientation, Stunting</t>
+        </is>
+      </c>
+      <c r="Z80" t="inlineStr">
+        <is>
+          <t>Housing: Ruangan harus bersih dan bebas dari hewan peliharaan selama prosedur untuk menghindari risiko kontaminasi bakteri Pasteurella atau kerusakan mekanis pada selang. Ketersediaan wastafel untuk mencuci tangan secara benar sangat krusial dalam mengurangi risiko peritonitis. [🔗Sumber 1](https://freseniusmedicalcare.com/content/dam/home-products-education/steps2home-pd/Preventing_Peritonitis.pdf) [🔗Sumber 2](https://spnp-spp.pt/media/rqdpbrom/catheter-related-infections-and-peritonitis-in-pediatric-patients-receiving-peritoneal-dialysis-guideline-for-prevention-and-treatment-2012-1-_compressed-1.pdf) [Sumber 3](https://www.ouh.nhs.uk/media/agxhnni2/85713pdialysis.pdf) [Sumber 4](https://www.satellitehealthcare.com/blog/pets-and-peritoneal-dialysis-absolutely/) | Socioeconomic: Edukasi atau retraining intensif bagi keluarga (caregiver) mengenai prosedur aseptik sangat dianjurkan, terutama bagi keluarga dengan keterbatasan akses informasi. [Sumber](https://www.researchgate.net/publication/45276240_Peritonitis_in_children_on_peritoneal_dialysis_in_Cape_Town_South_Africa_Epidemiology_and_risks) | Nutrition: Rekomendasi asupan protein tinggi (1,4–3,0 g/kg/hari) disesuaikan dengan usia anak untuk mengganti kehilangan protein selama dialisis dan mengejar pertumbuhan. Pemantauan nutrisi dilakukan setiap bulan pada bayi dan setiap 3–4 bulan pada anak yang lebih tua. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC7352713/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) | Type of Catheter (Shape): Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Catheter Placement: Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Gastrostomy/Intraperitoneal Device:  | Catheter Orientation:  | Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>2026-05-09 11:57:35</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>BB96B24A</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>&gt;2 yo</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>&gt;12 mo</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>Fair/poor service</t>
+        </is>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>Poor/fair</t>
+        </is>
+      </c>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>Illiterate</t>
+        </is>
+      </c>
+      <c r="K81" t="inlineStr">
+        <is>
+          <t>No ESI</t>
+        </is>
+      </c>
+      <c r="L81" t="inlineStr">
+        <is>
+          <t>Poor nutrition</t>
+        </is>
+      </c>
+      <c r="M81" t="inlineStr">
+        <is>
+          <t>Non-glomerular</t>
+        </is>
+      </c>
+      <c r="N81" t="inlineStr">
+        <is>
+          <t>Straight</t>
+        </is>
+      </c>
+      <c r="O81" t="inlineStr">
+        <is>
+          <t>Double</t>
+        </is>
+      </c>
+      <c r="P81" t="inlineStr">
+        <is>
+          <t>Laparoscopic</t>
+        </is>
+      </c>
+      <c r="Q81" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="R81" t="inlineStr">
+        <is>
+          <t>Patients</t>
+        </is>
+      </c>
+      <c r="S81" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T81" t="inlineStr">
+        <is>
+          <t>upward</t>
+        </is>
+      </c>
+      <c r="U81" t="inlineStr">
+        <is>
+          <t>Stunting</t>
+        </is>
+      </c>
+      <c r="V81" t="inlineStr">
+        <is>
+          <t>36.36%</t>
+        </is>
+      </c>
+      <c r="W81" t="inlineStr">
+        <is>
+          <t>Non-Survivor</t>
+        </is>
+      </c>
+      <c r="X81" t="inlineStr">
+        <is>
+          <t>Age*, Place of Residence, Peritonitis in ESI*, Type of Catheter (Cuff), Performed CAPD, Starting PD &lt;2 weeks after placement</t>
+        </is>
+      </c>
+      <c r="Y81" t="inlineStr">
+        <is>
+          <t>Gender, Duration of PD*, Housing, Socioeconomic, Education, Nutrition, Cause of ESRD*, Type of Catheter (Shape), Catheter Placement, Gastrostomy/Intraperitoneal Device, Catheter Orientation, Stunting</t>
+        </is>
+      </c>
+      <c r="Z81" t="inlineStr">
+        <is>
+          <t>Housing: Ruangan harus bersih dan bebas dari hewan peliharaan selama prosedur untuk menghindari risiko kontaminasi bakteri Pasteurella atau kerusakan mekanis pada selang. Ketersediaan wastafel untuk mencuci tangan secara benar sangat krusial dalam mengurangi risiko peritonitis. [🔗Sumber 1](https://freseniusmedicalcare.com/content/dam/home-products-education/steps2home-pd/Preventing_Peritonitis.pdf) [🔗Sumber 2](https://spnp-spp.pt/media/rqdpbrom/catheter-related-infections-and-peritonitis-in-pediatric-patients-receiving-peritoneal-dialysis-guideline-for-prevention-and-treatment-2012-1-_compressed-1.pdf) [Sumber 3](https://www.ouh.nhs.uk/media/agxhnni2/85713pdialysis.pdf) [Sumber 4](https://www.satellitehealthcare.com/blog/pets-and-peritoneal-dialysis-absolutely/) | Socioeconomic: Edukasi atau retraining intensif bagi keluarga (caregiver) mengenai prosedur aseptik sangat dianjurkan, terutama bagi keluarga dengan keterbatasan akses informasi. [Sumber](https://www.researchgate.net/publication/45276240_Peritonitis_in_children_on_peritoneal_dialysis_in_Cape_Town_South_Africa_Epidemiology_and_risks) | Nutrition: Rekomendasi asupan protein tinggi (1,4–3,0 g/kg/hari) disesuaikan dengan usia anak untuk mengganti kehilangan protein selama dialisis dan mengejar pertumbuhan. Pemantauan nutrisi dilakukan setiap bulan pada bayi dan setiap 3–4 bulan pada anak yang lebih tua. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC7352713/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) | Type of Catheter (Shape): Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Catheter Placement: Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Gastrostomy/Intraperitoneal Device:  | Catheter Orientation:  | Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>2026-05-09 11:59:28</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>BB96B24A</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>&gt;2 yo</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>&gt;12 mo</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>Fair/poor service</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>Poor/fair</t>
+        </is>
+      </c>
+      <c r="J82" t="inlineStr">
+        <is>
+          <t>Illiterate</t>
+        </is>
+      </c>
+      <c r="K82" t="inlineStr">
+        <is>
+          <t>No ESI</t>
+        </is>
+      </c>
+      <c r="L82" t="inlineStr">
+        <is>
+          <t>Poor nutrition</t>
+        </is>
+      </c>
+      <c r="M82" t="inlineStr">
+        <is>
+          <t>Non-glomerular</t>
+        </is>
+      </c>
+      <c r="N82" t="inlineStr">
+        <is>
+          <t>Straight</t>
+        </is>
+      </c>
+      <c r="O82" t="inlineStr">
+        <is>
+          <t>Double</t>
+        </is>
+      </c>
+      <c r="P82" t="inlineStr">
+        <is>
+          <t>Laparoscopic</t>
+        </is>
+      </c>
+      <c r="Q82" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="R82" t="inlineStr">
+        <is>
+          <t>Patients</t>
+        </is>
+      </c>
+      <c r="S82" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T82" t="inlineStr">
+        <is>
+          <t>upward</t>
+        </is>
+      </c>
+      <c r="U82" t="inlineStr">
+        <is>
+          <t>Stunting</t>
+        </is>
+      </c>
+      <c r="V82" t="inlineStr">
+        <is>
+          <t>36.36%</t>
+        </is>
+      </c>
+      <c r="W82" t="inlineStr">
+        <is>
+          <t>Non-Survivor</t>
+        </is>
+      </c>
+      <c r="X82" t="inlineStr">
+        <is>
+          <t>Age*, Place of Residence, Peritonitis in ESI*, Type of Catheter (Cuff), Performed CAPD, Starting PD &lt;2 weeks after placement</t>
+        </is>
+      </c>
+      <c r="Y82" t="inlineStr">
+        <is>
+          <t>Gender, Duration of PD*, Housing, Socioeconomic, Education, Nutrition, Cause of ESRD*, Type of Catheter (Shape), Catheter Placement, Gastrostomy/Intraperitoneal Device, Catheter Orientation, Stunting</t>
+        </is>
+      </c>
+      <c r="Z82" t="inlineStr">
+        <is>
+          <t>Housing: Ruangan harus bersih dan bebas dari hewan peliharaan selama prosedur untuk menghindari risiko kontaminasi bakteri Pasteurella atau kerusakan mekanis pada selang. Ketersediaan wastafel untuk mencuci tangan secara benar sangat krusial dalam mengurangi risiko peritonitis. [🔗Sumber 1](https://freseniusmedicalcare.com/content/dam/home-products-education/steps2home-pd/Preventing_Peritonitis.pdf) [🔗Sumber 2](https://spnp-spp.pt/media/rqdpbrom/catheter-related-infections-and-peritonitis-in-pediatric-patients-receiving-peritoneal-dialysis-guideline-for-prevention-and-treatment-2012-1-_compressed-1.pdf) [Sumber 3](https://www.ouh.nhs.uk/media/agxhnni2/85713pdialysis.pdf) [Sumber 4](https://www.satellitehealthcare.com/blog/pets-and-peritoneal-dialysis-absolutely/) | Socioeconomic: Edukasi atau retraining intensif bagi keluarga (caregiver) mengenai prosedur aseptik sangat dianjurkan, terutama bagi keluarga dengan keterbatasan akses informasi. [Sumber](https://www.researchgate.net/publication/45276240_Peritonitis_in_children_on_peritoneal_dialysis_in_Cape_Town_South_Africa_Epidemiology_and_risks) | Nutrition: Rekomendasi asupan protein tinggi (1,4–3,0 g/kg/hari) disesuaikan dengan usia anak untuk mengganti kehilangan protein selama dialisis dan mengejar pertumbuhan. Pemantauan nutrisi dilakukan setiap bulan pada bayi dan setiap 3–4 bulan pada anak yang lebih tua. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC7352713/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) | Type of Catheter (Shape): Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Catheter Placement: Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Gastrostomy/Intraperitoneal Device:  | Catheter Orientation:  | Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
v1 15 mei 26  - fixing peringatan, adding MRF variable 'catheter orientation'
</commit_message>
<xml_diff>
--- a/peritonitis-prediction/PeritonitisPrediction_Database.xlsx
+++ b/peritonitis-prediction/PeritonitisPrediction_Database.xlsx
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,136 +413,136 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z82"/>
+  <dimension ref="A1:Z92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Timestamp</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Patient_ID</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Module</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Age</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Gender</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Duration of PD</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Place of Residence</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Housing</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Socioeconomic</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Education</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Peritonitis in ESI</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Nutrition</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Cause of ESRD</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Type of Catheter (Shape)</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>Type of Catheter (Cuff)</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>Catheter Placement</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>Gastrostomy/Intraperitoneal Device</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>Performed CAPD</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>Starting PD &lt;2 weeks after placement</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>Catheter Orientation</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>Stunting</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>Survival Rate</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>Outcome</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>Supporting_Factors</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>Risk_Factors</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>Modifiable_Risk_Factors_Advice</t>
         </is>
@@ -10992,6 +10980,1270 @@
         </is>
       </c>
     </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>2026-05-12 09:22:57</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>B82D2CFF</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>&gt;2 yo</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>&lt;12 mo</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>Good service</t>
+        </is>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="J83" t="inlineStr">
+        <is>
+          <t>Studies</t>
+        </is>
+      </c>
+      <c r="K83" t="inlineStr">
+        <is>
+          <t>No ESI</t>
+        </is>
+      </c>
+      <c r="L83" t="inlineStr">
+        <is>
+          <t>Normal Nutrition</t>
+        </is>
+      </c>
+      <c r="M83" t="inlineStr">
+        <is>
+          <t>Glomerular</t>
+        </is>
+      </c>
+      <c r="N83" t="inlineStr">
+        <is>
+          <t>Coiled/swan neck</t>
+        </is>
+      </c>
+      <c r="O83" t="inlineStr">
+        <is>
+          <t>Double</t>
+        </is>
+      </c>
+      <c r="P83" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="Q83" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R83" t="inlineStr">
+        <is>
+          <t>Patients</t>
+        </is>
+      </c>
+      <c r="S83" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T83" t="inlineStr">
+        <is>
+          <t>Lateral/downward</t>
+        </is>
+      </c>
+      <c r="U83" t="inlineStr">
+        <is>
+          <t>Stunting</t>
+        </is>
+      </c>
+      <c r="V83" t="inlineStr">
+        <is>
+          <t>95.45%</t>
+        </is>
+      </c>
+      <c r="W83" t="inlineStr">
+        <is>
+          <t>Survivor</t>
+        </is>
+      </c>
+      <c r="X83" t="inlineStr">
+        <is>
+          <t>Age*, Gender, Duration of PD*, Place of Residence, Housing, Socioeconomic, Education, Peritonitis in ESI*, Nutrition, Cause of ESRD*, Type of Catheter (Shape), Type of Catheter (Cuff), Catheter Placement, Gastrostomy/Intraperitoneal Device, Performed CAPD, Starting PD &lt;2 weeks after placement, Catheter Orientation</t>
+        </is>
+      </c>
+      <c r="Y83" t="inlineStr">
+        <is>
+          <t>Stunting</t>
+        </is>
+      </c>
+      <c r="Z83" t="inlineStr">
+        <is>
+          <t>Stunting: Stunting pada anak dialisis bukan hanya disebabkan oleh asupan kalori yang rendah, tetapi juga oleh asidosis metabolik, anemia, osteodistrofi ginjal, dan resistensi terhadap hormon pertumbuhan. Intervensi pertama adalah memastikan kecukupan dialisis dan koreksi parameter metabolik seperti asidosis dan hiperparatiroidisme.Jika pertumbuhan masih belum optimal meskipun parameter metabolik telah terkendali dan asupan nutrisi sudah mencapai target, terapi dengan hormon pertumbuhan manusia rekombinan (rhGH) dapat dipertimbangkan. Selain itu, dukungan nutrisi intensif dan klirens dialisis yang adekuat pada pasien prepubertal dapat mempromosikan pertumbuhan normal tanpa selalu memerlukan rhGH. Pada anak yang mengalami stunting (tinggi badan &lt; persentil ke-2), perhitungan kebutuhan energi dan mikronutrien harus didasarkan pada height-age pasien, bukan chronological age-nya, untuk memberikan dukungan yang sesuai dengan ukuran tubuh aktualnya. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/)</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>2026-05-12 09:23:19</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>B82D2CFF</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>&gt;2 yo</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>&lt;12 mo</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>Good service</t>
+        </is>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>Studies</t>
+        </is>
+      </c>
+      <c r="K84" t="inlineStr">
+        <is>
+          <t>No ESI</t>
+        </is>
+      </c>
+      <c r="L84" t="inlineStr">
+        <is>
+          <t>Normal Nutrition</t>
+        </is>
+      </c>
+      <c r="M84" t="inlineStr">
+        <is>
+          <t>Glomerular</t>
+        </is>
+      </c>
+      <c r="N84" t="inlineStr">
+        <is>
+          <t>Coiled/swan neck</t>
+        </is>
+      </c>
+      <c r="O84" t="inlineStr">
+        <is>
+          <t>Double</t>
+        </is>
+      </c>
+      <c r="P84" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="Q84" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R84" t="inlineStr">
+        <is>
+          <t>Patients</t>
+        </is>
+      </c>
+      <c r="S84" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T84" t="inlineStr">
+        <is>
+          <t>Lateral/downward</t>
+        </is>
+      </c>
+      <c r="U84" t="inlineStr">
+        <is>
+          <t>Stunting</t>
+        </is>
+      </c>
+      <c r="V84" t="inlineStr">
+        <is>
+          <t>95.45%</t>
+        </is>
+      </c>
+      <c r="W84" t="inlineStr">
+        <is>
+          <t>Survivor</t>
+        </is>
+      </c>
+      <c r="X84" t="inlineStr">
+        <is>
+          <t>Age*, Gender, Duration of PD*, Place of Residence, Housing, Socioeconomic, Education, Peritonitis in ESI*, Nutrition, Cause of ESRD*, Type of Catheter (Shape), Type of Catheter (Cuff), Catheter Placement, Gastrostomy/Intraperitoneal Device, Performed CAPD, Starting PD &lt;2 weeks after placement, Catheter Orientation</t>
+        </is>
+      </c>
+      <c r="Y84" t="inlineStr">
+        <is>
+          <t>Stunting</t>
+        </is>
+      </c>
+      <c r="Z84" t="inlineStr">
+        <is>
+          <t>Stunting: Stunting pada anak dialisis bukan hanya disebabkan oleh asupan kalori yang rendah, tetapi juga oleh asidosis metabolik, anemia, osteodistrofi ginjal, dan resistensi terhadap hormon pertumbuhan. Intervensi pertama adalah memastikan kecukupan dialisis dan koreksi parameter metabolik seperti asidosis dan hiperparatiroidisme.Jika pertumbuhan masih belum optimal meskipun parameter metabolik telah terkendali dan asupan nutrisi sudah mencapai target, terapi dengan hormon pertumbuhan manusia rekombinan (rhGH) dapat dipertimbangkan. Selain itu, dukungan nutrisi intensif dan klirens dialisis yang adekuat pada pasien prepubertal dapat mempromosikan pertumbuhan normal tanpa selalu memerlukan rhGH. Pada anak yang mengalami stunting (tinggi badan &lt; persentil ke-2), perhitungan kebutuhan energi dan mikronutrien harus didasarkan pada height-age pasien, bukan chronological age-nya, untuk memberikan dukungan yang sesuai dengan ukuran tubuh aktualnya. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/)</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>2026-05-12 09:23:39</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>B82D2CFF</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>&gt;2 yo</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>&lt;12 mo</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>Good service</t>
+        </is>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>Studies</t>
+        </is>
+      </c>
+      <c r="K85" t="inlineStr">
+        <is>
+          <t>No ESI</t>
+        </is>
+      </c>
+      <c r="L85" t="inlineStr">
+        <is>
+          <t>Normal Nutrition</t>
+        </is>
+      </c>
+      <c r="M85" t="inlineStr">
+        <is>
+          <t>Glomerular</t>
+        </is>
+      </c>
+      <c r="N85" t="inlineStr">
+        <is>
+          <t>Coiled/swan neck</t>
+        </is>
+      </c>
+      <c r="O85" t="inlineStr">
+        <is>
+          <t>Double</t>
+        </is>
+      </c>
+      <c r="P85" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="Q85" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R85" t="inlineStr">
+        <is>
+          <t>Patients</t>
+        </is>
+      </c>
+      <c r="S85" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T85" t="inlineStr">
+        <is>
+          <t>Lateral/downward</t>
+        </is>
+      </c>
+      <c r="U85" t="inlineStr">
+        <is>
+          <t>Stunting</t>
+        </is>
+      </c>
+      <c r="V85" t="inlineStr">
+        <is>
+          <t>95.45%</t>
+        </is>
+      </c>
+      <c r="W85" t="inlineStr">
+        <is>
+          <t>Survivor</t>
+        </is>
+      </c>
+      <c r="X85" t="inlineStr">
+        <is>
+          <t>Age*, Gender, Duration of PD*, Place of Residence, Housing, Socioeconomic, Education, Peritonitis in ESI*, Nutrition, Cause of ESRD*, Type of Catheter (Shape), Type of Catheter (Cuff), Catheter Placement, Gastrostomy/Intraperitoneal Device, Performed CAPD, Starting PD &lt;2 weeks after placement, Catheter Orientation</t>
+        </is>
+      </c>
+      <c r="Y85" t="inlineStr">
+        <is>
+          <t>Stunting</t>
+        </is>
+      </c>
+      <c r="Z85" t="inlineStr">
+        <is>
+          <t>Stunting: Stunting pada anak dialisis bukan hanya disebabkan oleh asupan kalori yang rendah, tetapi juga oleh asidosis metabolik, anemia, osteodistrofi ginjal, dan resistensi terhadap hormon pertumbuhan. Intervensi pertama adalah memastikan kecukupan dialisis dan koreksi parameter metabolik seperti asidosis dan hiperparatiroidisme.Jika pertumbuhan masih belum optimal meskipun parameter metabolik telah terkendali dan asupan nutrisi sudah mencapai target, terapi dengan hormon pertumbuhan manusia rekombinan (rhGH) dapat dipertimbangkan. Selain itu, dukungan nutrisi intensif dan klirens dialisis yang adekuat pada pasien prepubertal dapat mempromosikan pertumbuhan normal tanpa selalu memerlukan rhGH. Pada anak yang mengalami stunting (tinggi badan &lt; persentil ke-2), perhitungan kebutuhan energi dan mikronutrien harus didasarkan pada height-age pasien, bukan chronological age-nya, untuk memberikan dukungan yang sesuai dengan ukuran tubuh aktualnya. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/)</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>2026-05-15 14:07:17</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>15964F63</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>&gt;2 yo</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>&lt;12 mo</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>Good service</t>
+        </is>
+      </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>Studies</t>
+        </is>
+      </c>
+      <c r="K86" t="inlineStr">
+        <is>
+          <t>No ESI</t>
+        </is>
+      </c>
+      <c r="L86" t="inlineStr">
+        <is>
+          <t>Normal Nutrition</t>
+        </is>
+      </c>
+      <c r="M86" t="inlineStr">
+        <is>
+          <t>Glomerular</t>
+        </is>
+      </c>
+      <c r="N86" t="inlineStr">
+        <is>
+          <t>Coiled/swan neck</t>
+        </is>
+      </c>
+      <c r="O86" t="inlineStr">
+        <is>
+          <t>Double</t>
+        </is>
+      </c>
+      <c r="P86" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="Q86" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R86" t="inlineStr">
+        <is>
+          <t>Patients</t>
+        </is>
+      </c>
+      <c r="S86" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T86" t="inlineStr">
+        <is>
+          <t>Lateral/downward</t>
+        </is>
+      </c>
+      <c r="U86" t="inlineStr">
+        <is>
+          <t>No stunting</t>
+        </is>
+      </c>
+      <c r="V86" t="inlineStr">
+        <is>
+          <t>100.00%</t>
+        </is>
+      </c>
+      <c r="W86" t="inlineStr">
+        <is>
+          <t>Survivor</t>
+        </is>
+      </c>
+      <c r="X86" t="inlineStr">
+        <is>
+          <t>Age*, Gender, Duration of PD*, Place of Residence, Housing, Socioeconomic, Education, Peritonitis in ESI*, Nutrition, Cause of ESRD*, Type of Catheter (Shape), Type of Catheter (Cuff), Catheter Placement, Gastrostomy/Intraperitoneal Device, Performed CAPD, Starting PD &lt;2 weeks after placement, Catheter Orientation, Stunting</t>
+        </is>
+      </c>
+      <c r="Y86" t="inlineStr"/>
+      <c r="Z86" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>2026-05-15 14:08:26</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>15964F63</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>&gt;2 yo</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>&lt;12 mo</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>Good service</t>
+        </is>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t>Studies</t>
+        </is>
+      </c>
+      <c r="K87" t="inlineStr">
+        <is>
+          <t>No ESI</t>
+        </is>
+      </c>
+      <c r="L87" t="inlineStr">
+        <is>
+          <t>Normal Nutrition</t>
+        </is>
+      </c>
+      <c r="M87" t="inlineStr">
+        <is>
+          <t>Glomerular</t>
+        </is>
+      </c>
+      <c r="N87" t="inlineStr">
+        <is>
+          <t>Coiled/swan neck</t>
+        </is>
+      </c>
+      <c r="O87" t="inlineStr">
+        <is>
+          <t>Double</t>
+        </is>
+      </c>
+      <c r="P87" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="Q87" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R87" t="inlineStr">
+        <is>
+          <t>Patients</t>
+        </is>
+      </c>
+      <c r="S87" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T87" t="inlineStr">
+        <is>
+          <t>Lateral/downward</t>
+        </is>
+      </c>
+      <c r="U87" t="inlineStr">
+        <is>
+          <t>No stunting</t>
+        </is>
+      </c>
+      <c r="V87" t="inlineStr">
+        <is>
+          <t>100.00%</t>
+        </is>
+      </c>
+      <c r="W87" t="inlineStr">
+        <is>
+          <t>Survivor</t>
+        </is>
+      </c>
+      <c r="X87" t="inlineStr">
+        <is>
+          <t>Age*, Gender, Duration of PD*, Place of Residence, Housing, Socioeconomic, Education, Peritonitis in ESI*, Nutrition, Cause of ESRD*, Type of Catheter (Shape), Type of Catheter (Cuff), Catheter Placement, Gastrostomy/Intraperitoneal Device, Performed CAPD, Starting PD &lt;2 weeks after placement, Catheter Orientation, Stunting</t>
+        </is>
+      </c>
+      <c r="Y87" t="inlineStr"/>
+      <c r="Z87" t="inlineStr"/>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>2026-05-15 14:09:58</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>15964F63</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>&gt;2 yo</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>&lt;12 mo</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>Good service</t>
+        </is>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>Studies</t>
+        </is>
+      </c>
+      <c r="K88" t="inlineStr">
+        <is>
+          <t>No ESI</t>
+        </is>
+      </c>
+      <c r="L88" t="inlineStr">
+        <is>
+          <t>Normal Nutrition</t>
+        </is>
+      </c>
+      <c r="M88" t="inlineStr">
+        <is>
+          <t>Glomerular</t>
+        </is>
+      </c>
+      <c r="N88" t="inlineStr">
+        <is>
+          <t>Coiled/swan neck</t>
+        </is>
+      </c>
+      <c r="O88" t="inlineStr">
+        <is>
+          <t>Double</t>
+        </is>
+      </c>
+      <c r="P88" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="Q88" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R88" t="inlineStr">
+        <is>
+          <t>Patients</t>
+        </is>
+      </c>
+      <c r="S88" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T88" t="inlineStr">
+        <is>
+          <t>Lateral/downward</t>
+        </is>
+      </c>
+      <c r="U88" t="inlineStr">
+        <is>
+          <t>No stunting</t>
+        </is>
+      </c>
+      <c r="V88" t="inlineStr">
+        <is>
+          <t>100.00%</t>
+        </is>
+      </c>
+      <c r="W88" t="inlineStr">
+        <is>
+          <t>Survivor</t>
+        </is>
+      </c>
+      <c r="X88" t="inlineStr">
+        <is>
+          <t>Age*, Gender, Duration of PD*, Place of Residence, Housing, Socioeconomic, Education, Peritonitis in ESI*, Nutrition, Cause of ESRD*, Type of Catheter (Shape), Type of Catheter (Cuff), Catheter Placement, Gastrostomy/Intraperitoneal Device, Performed CAPD, Starting PD &lt;2 weeks after placement, Catheter Orientation, Stunting</t>
+        </is>
+      </c>
+      <c r="Y88" t="inlineStr"/>
+      <c r="Z88" t="inlineStr"/>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>2026-05-15 14:15:16</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>15964F63</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>&gt;2 yo</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>&lt;12 mo</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>Good service</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>Studies</t>
+        </is>
+      </c>
+      <c r="K89" t="inlineStr">
+        <is>
+          <t>No ESI</t>
+        </is>
+      </c>
+      <c r="L89" t="inlineStr">
+        <is>
+          <t>Normal Nutrition</t>
+        </is>
+      </c>
+      <c r="M89" t="inlineStr">
+        <is>
+          <t>Glomerular</t>
+        </is>
+      </c>
+      <c r="N89" t="inlineStr">
+        <is>
+          <t>Coiled/swan neck</t>
+        </is>
+      </c>
+      <c r="O89" t="inlineStr">
+        <is>
+          <t>Double</t>
+        </is>
+      </c>
+      <c r="P89" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="Q89" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R89" t="inlineStr">
+        <is>
+          <t>Patients</t>
+        </is>
+      </c>
+      <c r="S89" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T89" t="inlineStr">
+        <is>
+          <t>Lateral/downward</t>
+        </is>
+      </c>
+      <c r="U89" t="inlineStr">
+        <is>
+          <t>No stunting</t>
+        </is>
+      </c>
+      <c r="V89" t="inlineStr">
+        <is>
+          <t>100.00%</t>
+        </is>
+      </c>
+      <c r="W89" t="inlineStr">
+        <is>
+          <t>Survivor</t>
+        </is>
+      </c>
+      <c r="X89" t="inlineStr">
+        <is>
+          <t>Age*, Gender, Duration of PD*, Place of Residence, Housing, Socioeconomic, Education, Peritonitis in ESI*, Nutrition, Cause of ESRD*, Type of Catheter (Shape), Type of Catheter (Cuff), Catheter Placement, Gastrostomy/Intraperitoneal Device, Performed CAPD, Starting PD &lt;2 weeks after placement, Catheter Orientation, Stunting</t>
+        </is>
+      </c>
+      <c r="Y89" t="inlineStr"/>
+      <c r="Z89" t="inlineStr"/>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>2026-05-15 14:16:20</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>15964F63</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>&gt;2 yo</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>&lt;12 mo</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>Good service</t>
+        </is>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>Studies</t>
+        </is>
+      </c>
+      <c r="K90" t="inlineStr">
+        <is>
+          <t>No ESI</t>
+        </is>
+      </c>
+      <c r="L90" t="inlineStr">
+        <is>
+          <t>Normal Nutrition</t>
+        </is>
+      </c>
+      <c r="M90" t="inlineStr">
+        <is>
+          <t>Glomerular</t>
+        </is>
+      </c>
+      <c r="N90" t="inlineStr">
+        <is>
+          <t>Coiled/swan neck</t>
+        </is>
+      </c>
+      <c r="O90" t="inlineStr">
+        <is>
+          <t>Double</t>
+        </is>
+      </c>
+      <c r="P90" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="Q90" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R90" t="inlineStr">
+        <is>
+          <t>Patients</t>
+        </is>
+      </c>
+      <c r="S90" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T90" t="inlineStr">
+        <is>
+          <t>Lateral/downward</t>
+        </is>
+      </c>
+      <c r="U90" t="inlineStr">
+        <is>
+          <t>No stunting</t>
+        </is>
+      </c>
+      <c r="V90" t="inlineStr">
+        <is>
+          <t>100.00%</t>
+        </is>
+      </c>
+      <c r="W90" t="inlineStr">
+        <is>
+          <t>Survivor</t>
+        </is>
+      </c>
+      <c r="X90" t="inlineStr">
+        <is>
+          <t>Age*, Gender, Duration of PD*, Place of Residence, Housing, Socioeconomic, Education, Peritonitis in ESI*, Nutrition, Cause of ESRD*, Type of Catheter (Shape), Type of Catheter (Cuff), Catheter Placement, Gastrostomy/Intraperitoneal Device, Performed CAPD, Starting PD &lt;2 weeks after placement, Catheter Orientation, Stunting</t>
+        </is>
+      </c>
+      <c r="Y90" t="inlineStr"/>
+      <c r="Z90" t="inlineStr"/>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>2026-05-15 14:17:05</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>15964F63</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>&gt;2 yo</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>&lt;12 mo</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>Good service</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>Studies</t>
+        </is>
+      </c>
+      <c r="K91" t="inlineStr">
+        <is>
+          <t>No ESI</t>
+        </is>
+      </c>
+      <c r="L91" t="inlineStr">
+        <is>
+          <t>Normal Nutrition</t>
+        </is>
+      </c>
+      <c r="M91" t="inlineStr">
+        <is>
+          <t>Glomerular</t>
+        </is>
+      </c>
+      <c r="N91" t="inlineStr">
+        <is>
+          <t>Coiled/swan neck</t>
+        </is>
+      </c>
+      <c r="O91" t="inlineStr">
+        <is>
+          <t>Double</t>
+        </is>
+      </c>
+      <c r="P91" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="Q91" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R91" t="inlineStr">
+        <is>
+          <t>Patients</t>
+        </is>
+      </c>
+      <c r="S91" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T91" t="inlineStr">
+        <is>
+          <t>Lateral/downward</t>
+        </is>
+      </c>
+      <c r="U91" t="inlineStr">
+        <is>
+          <t>No stunting</t>
+        </is>
+      </c>
+      <c r="V91" t="inlineStr">
+        <is>
+          <t>100.00%</t>
+        </is>
+      </c>
+      <c r="W91" t="inlineStr">
+        <is>
+          <t>Survivor</t>
+        </is>
+      </c>
+      <c r="X91" t="inlineStr">
+        <is>
+          <t>Age*, Gender, Duration of PD*, Place of Residence, Housing, Socioeconomic, Education, Peritonitis in ESI*, Nutrition, Cause of ESRD*, Type of Catheter (Shape), Type of Catheter (Cuff), Catheter Placement, Gastrostomy/Intraperitoneal Device, Performed CAPD, Starting PD &lt;2 weeks after placement, Catheter Orientation, Stunting</t>
+        </is>
+      </c>
+      <c r="Y91" t="inlineStr"/>
+      <c r="Z91" t="inlineStr"/>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>2026-05-15 14:17:29</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>15964F63</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>&gt;2 yo</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>&lt;12 mo</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>Good service</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>Studies</t>
+        </is>
+      </c>
+      <c r="K92" t="inlineStr">
+        <is>
+          <t>No ESI</t>
+        </is>
+      </c>
+      <c r="L92" t="inlineStr">
+        <is>
+          <t>Normal Nutrition</t>
+        </is>
+      </c>
+      <c r="M92" t="inlineStr">
+        <is>
+          <t>Glomerular</t>
+        </is>
+      </c>
+      <c r="N92" t="inlineStr">
+        <is>
+          <t>Coiled/swan neck</t>
+        </is>
+      </c>
+      <c r="O92" t="inlineStr">
+        <is>
+          <t>Double</t>
+        </is>
+      </c>
+      <c r="P92" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="Q92" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R92" t="inlineStr">
+        <is>
+          <t>Patients</t>
+        </is>
+      </c>
+      <c r="S92" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T92" t="inlineStr">
+        <is>
+          <t>Lateral/downward</t>
+        </is>
+      </c>
+      <c r="U92" t="inlineStr">
+        <is>
+          <t>No stunting</t>
+        </is>
+      </c>
+      <c r="V92" t="inlineStr">
+        <is>
+          <t>100.00%</t>
+        </is>
+      </c>
+      <c r="W92" t="inlineStr">
+        <is>
+          <t>Survivor</t>
+        </is>
+      </c>
+      <c r="X92" t="inlineStr">
+        <is>
+          <t>Age*, Gender, Duration of PD*, Place of Residence, Housing, Socioeconomic, Education, Peritonitis in ESI*, Nutrition, Cause of ESRD*, Type of Catheter (Shape), Type of Catheter (Cuff), Catheter Placement, Gastrostomy/Intraperitoneal Device, Performed CAPD, Starting PD &lt;2 weeks after placement, Catheter Orientation, Stunting</t>
+        </is>
+      </c>
+      <c r="Y92" t="inlineStr"/>
+      <c r="Z92" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
v1 19 mei 2026 - completing MRF explanations
</commit_message>
<xml_diff>
--- a/peritonitis-prediction/PeritonitisPrediction_Database.xlsx
+++ b/peritonitis-prediction/PeritonitisPrediction_Database.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z92"/>
+  <dimension ref="A1:AA104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -545,6 +545,11 @@
       <c r="Z1" t="inlineStr">
         <is>
           <t>Modifiable_Risk_Factors_Advice</t>
+        </is>
+      </c>
+      <c r="AA1" t="inlineStr">
+        <is>
+          <t>Starting PD &lt;2 weeks after catheter placement</t>
         </is>
       </c>
     </row>
@@ -655,6 +660,7 @@
       <c r="X2" t="inlineStr"/>
       <c r="Y2" t="inlineStr"/>
       <c r="Z2" t="inlineStr"/>
+      <c r="AA2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -763,6 +769,7 @@
       <c r="X3" t="inlineStr"/>
       <c r="Y3" t="inlineStr"/>
       <c r="Z3" t="inlineStr"/>
+      <c r="AA3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -871,6 +878,7 @@
       <c r="X4" t="inlineStr"/>
       <c r="Y4" t="inlineStr"/>
       <c r="Z4" t="inlineStr"/>
+      <c r="AA4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -983,6 +991,7 @@
       <c r="X5" t="inlineStr"/>
       <c r="Y5" t="inlineStr"/>
       <c r="Z5" t="inlineStr"/>
+      <c r="AA5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1103,6 +1112,7 @@
       <c r="X6" t="inlineStr"/>
       <c r="Y6" t="inlineStr"/>
       <c r="Z6" t="inlineStr"/>
+      <c r="AA6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1223,6 +1233,7 @@
       <c r="X7" t="inlineStr"/>
       <c r="Y7" t="inlineStr"/>
       <c r="Z7" t="inlineStr"/>
+      <c r="AA7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1343,6 +1354,7 @@
       <c r="X8" t="inlineStr"/>
       <c r="Y8" t="inlineStr"/>
       <c r="Z8" t="inlineStr"/>
+      <c r="AA8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1463,6 +1475,7 @@
       <c r="X9" t="inlineStr"/>
       <c r="Y9" t="inlineStr"/>
       <c r="Z9" t="inlineStr"/>
+      <c r="AA9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1583,6 +1596,7 @@
       <c r="X10" t="inlineStr"/>
       <c r="Y10" t="inlineStr"/>
       <c r="Z10" t="inlineStr"/>
+      <c r="AA10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1703,6 +1717,7 @@
       <c r="X11" t="inlineStr"/>
       <c r="Y11" t="inlineStr"/>
       <c r="Z11" t="inlineStr"/>
+      <c r="AA11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1823,6 +1838,7 @@
       <c r="X12" t="inlineStr"/>
       <c r="Y12" t="inlineStr"/>
       <c r="Z12" t="inlineStr"/>
+      <c r="AA12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1951,6 +1967,7 @@
         </is>
       </c>
       <c r="Z13" t="inlineStr"/>
+      <c r="AA13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2083,6 +2100,7 @@
           <t>Housing: Perlu perbaikan sanitasi dan fasilitas lingkungan tempat tinggal untuk mengurangi risiko kontaminasi kuman dari lingkungan. | Peritonitis in ESI: Perlu penanganan agresif dan segera terhadap infeksi area keluar kateter (Exit Site Infection) agar kuman tidak masuk ke rongga perut. | Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
+      <c r="AA14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2207,6 +2225,7 @@
       </c>
       <c r="Y15" t="inlineStr"/>
       <c r="Z15" t="inlineStr"/>
+      <c r="AA15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2331,6 +2350,7 @@
       </c>
       <c r="Y16" t="inlineStr"/>
       <c r="Z16" t="inlineStr"/>
+      <c r="AA16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2455,6 +2475,7 @@
       </c>
       <c r="Y17" t="inlineStr"/>
       <c r="Z17" t="inlineStr"/>
+      <c r="AA17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2587,6 +2608,7 @@
           <t>Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
+      <c r="AA18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2711,6 +2733,7 @@
       </c>
       <c r="Y19" t="inlineStr"/>
       <c r="Z19" t="inlineStr"/>
+      <c r="AA19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2843,6 +2866,7 @@
           <t>Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
+      <c r="AA20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2975,6 +2999,7 @@
           <t>Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
+      <c r="AA21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -3107,6 +3132,7 @@
           <t>Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
+      <c r="AA22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -3239,6 +3265,7 @@
           <t>Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
+      <c r="AA23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -3363,6 +3390,7 @@
       </c>
       <c r="Y24" t="inlineStr"/>
       <c r="Z24" t="inlineStr"/>
+      <c r="AA24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -3491,6 +3519,7 @@
         </is>
       </c>
       <c r="Z25" t="inlineStr"/>
+      <c r="AA25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -3619,6 +3648,7 @@
         </is>
       </c>
       <c r="Z26" t="inlineStr"/>
+      <c r="AA26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -3747,6 +3777,7 @@
         </is>
       </c>
       <c r="Z27" t="inlineStr"/>
+      <c r="AA27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -3875,6 +3906,7 @@
         </is>
       </c>
       <c r="Z28" t="inlineStr"/>
+      <c r="AA28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -4007,6 +4039,7 @@
           <t>Nutrition: Perlu peningkatan asupan nutrisi dan pemantauan status gizi secara berkala oleh ahli gizi anak untuk mencapai status gizi normal.</t>
         </is>
       </c>
+      <c r="AA29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -4139,6 +4172,7 @@
           <t>Nutrition: Perlu peningkatan asupan nutrisi dan pemantauan status gizi secara berkala oleh ahli gizi anak untuk mencapai status gizi normal. | Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
+      <c r="AA30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -4271,6 +4305,7 @@
           <t>Catheter Orientation:  | Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
+      <c r="AA31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -4403,6 +4438,7 @@
           <t>Catheter Orientation:  | Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
+      <c r="AA32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -4535,6 +4571,7 @@
           <t>Peritonitis in ESI: Perlu penanganan agresif dan segera terhadap infeksi area keluar kateter (Exit Site Infection) agar kuman tidak masuk ke rongga perut. | Catheter Orientation:  | Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
+      <c r="AA33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -4667,6 +4704,7 @@
           <t xml:space="preserve">Catheter Orientation: </t>
         </is>
       </c>
+      <c r="AA34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -4791,6 +4829,7 @@
       </c>
       <c r="Y35" t="inlineStr"/>
       <c r="Z35" t="inlineStr"/>
+      <c r="AA35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -4923,6 +4962,7 @@
           <t>Performed CAPD: Perlu pelatihan ulang yang intensif bagi orang yang melakukan dialisis (pasien/keluarga) mengenai prosedur aseptik yang benar. | Starting PD &lt;2 weeks after placement: Sebaiknya menunda dimulainya dialisis (jika kondisi klinis memungkinkan) minimal 2 minggu setelah operasi agar luka kateter sembuh sempurna. | Catheter Orientation:  | Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
+      <c r="AA36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -5055,6 +5095,7 @@
           <t>Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
+      <c r="AA37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -5187,6 +5228,7 @@
           <t>Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
+      <c r="AA38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -5319,6 +5361,7 @@
           <t>Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
+      <c r="AA39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -5451,6 +5494,7 @@
           <t>Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
+      <c r="AA40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -5583,6 +5627,7 @@
           <t>Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
+      <c r="AA41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -5715,6 +5760,7 @@
           <t>Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
+      <c r="AA42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -5839,6 +5885,7 @@
       </c>
       <c r="Y43" t="inlineStr"/>
       <c r="Z43" t="inlineStr"/>
+      <c r="AA43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -5971,6 +6018,7 @@
           <t>Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
+      <c r="AA44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -6103,6 +6151,7 @@
           <t>Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
+      <c r="AA45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -6235,6 +6284,7 @@
           <t>Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
+      <c r="AA46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -6367,6 +6417,7 @@
           <t>Peritonitis in ESI: Perlu penanganan agresif dan segera terhadap infeksi area keluar kateter (Exit Site Infection) agar kuman tidak masuk ke rongga perut. | Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
+      <c r="AA47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -6499,6 +6550,7 @@
           <t>Peritonitis in ESI: Perlu penanganan agresif dan segera terhadap infeksi area keluar kateter (Exit Site Infection) agar kuman tidak masuk ke rongga perut. | Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
+      <c r="AA48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -6631,6 +6683,7 @@
           <t>Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
+      <c r="AA49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -6763,6 +6816,7 @@
           <t>Housing: Pastikan ada ruangan khusus yang bersih (minim debu/hewan peliharaan) untuk melakukan pertukaran cairan, serta ketersediaan wastafel dengan air mengalir di dalam ruangan tersebut untuk antisepsis tangan. [Sumber](https://www.scielo.br/j/jbn/a/hHtvqSXhwcCtvBnNqk9JBzk/?lang=en&amp;format=pdf) | Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
+      <c r="AA50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -6895,6 +6949,7 @@
           <t>Housing: Pastikan ada ruangan khusus yang bersih (minim debu/hewan peliharaan) untuk melakukan pertukaran cairan, serta ketersediaan wastafel dengan air mengalir di dalam ruangan tersebut untuk antisepsis tangan. [Sumber](https://www.scielo.br/j/jbn/a/hHtvqSXhwcCtvBnNqk9JBzk/?lang=en&amp;format=pdf) | Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
+      <c r="AA51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -7027,6 +7082,7 @@
           <t>Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
+      <c r="AA52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -7159,6 +7215,7 @@
           <t>Nutrition: Berikan asupan protein tinggi sesuai target usia (biasanya 1.4–3.0 g/kg/hari untuk anak) guna mengejar pertumbuhan dan mengganti protein yang hilang saat dialisis. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC7352713/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) | Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
+      <c r="AA53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -7291,6 +7348,7 @@
           <t>Nutrition: Berikan asupan protein tinggi sesuai target usia (biasanya 1.4–3.0 g/kg/hari untuk anak) guna mengejar pertumbuhan dan mengganti protein yang hilang saat dialisis. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC7352713/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) | Type of Catheter (Cuff): Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
+      <c r="AA54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -7423,6 +7481,7 @@
           <t>Peritonitis in ESI: Gunakan salep antibiotik topikal (seperti mupirocin atau gentamisin) pada exit site secara rutin dan pembersihan area dengan cairan antiseptik non-iritan. [Sumber](https://journals.eco-vector.com/2075-3594/article/view/637454) | Nutrition: Berikan asupan protein tinggi sesuai target usia (biasanya 1.4–3.0 g/kg/hari untuk anak) guna mengejar pertumbuhan dan mengganti protein yang hilang saat dialisis. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC7352713/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) | Type of Catheter (Cuff): Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
+      <c r="AA55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -7547,6 +7606,7 @@
       </c>
       <c r="Y56" t="inlineStr"/>
       <c r="Z56" t="inlineStr"/>
+      <c r="AA56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -7679,6 +7739,7 @@
           <t>Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
+      <c r="AA57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -7811,6 +7872,7 @@
           <t>Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
+      <c r="AA58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -7943,6 +8005,7 @@
           <t>Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
+      <c r="AA59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -8075,6 +8138,7 @@
           <t>Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
+      <c r="AA60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -8207,6 +8271,7 @@
           <t>Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
+      <c r="AA61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -8339,6 +8404,7 @@
           <t>Nutrition: Berikan asupan protein tinggi sesuai target usia (biasanya 1.4–3.0 g/kg/hari untuk anak) guna mengejar pertumbuhan dan mengganti protein yang hilang saat dialisis. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC7352713/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) | Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
+      <c r="AA62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -8471,6 +8537,7 @@
           <t>Nutrition: Rekomendasi asupan protein tinggi (1,4–3,0 g/kg/hari) disesuaikan dengan usia anak untuk mengganti kehilangan protein selama dialisis dan mengejar pertumbuhan. Pemantauan nutrisi dilakukan setiap bulan pada bayi dan setiap 3–4 bulan pada anak yang lebih tua. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC7352713/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) | Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
+      <c r="AA63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -8603,6 +8670,7 @@
           <t>Nutrition: Rekomendasi asupan protein tinggi (1,4–3,0 g/kg/hari) disesuaikan dengan usia anak untuk mengganti kehilangan protein selama dialisis dan mengejar pertumbuhan. Pemantauan nutrisi dilakukan setiap bulan pada bayi dan setiap 3–4 bulan pada anak yang lebih tua. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC7352713/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) | Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
+      <c r="AA64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -8735,6 +8803,7 @@
           <t>Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
+      <c r="AA65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -8867,6 +8936,7 @@
           <t>Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
+      <c r="AA66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -8999,6 +9069,7 @@
           <t>Catheter Placement: Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
+      <c r="AA67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -9131,6 +9202,7 @@
           <t>Catheter Placement: Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Catheter Orientation:  | Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
+      <c r="AA68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -9263,6 +9335,7 @@
           <t>Type of Catheter (Shape): Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Catheter Placement: Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Catheter Orientation:  | Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
+      <c r="AA69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -9395,6 +9468,7 @@
           <t>Nutrition: Rekomendasi asupan protein tinggi (1,4–3,0 g/kg/hari) disesuaikan dengan usia anak untuk mengganti kehilangan protein selama dialisis dan mengejar pertumbuhan. Pemantauan nutrisi dilakukan setiap bulan pada bayi dan setiap 3–4 bulan pada anak yang lebih tua. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC7352713/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) | Type of Catheter (Shape): Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Catheter Placement: Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Catheter Orientation:  | Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
+      <c r="AA70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -9527,6 +9601,7 @@
           <t>Socioeconomic: Edukasi atau retraining intensif bagi keluarga (caregiver) mengenai prosedur aseptik sangat dianjurkan, terutama bagi keluarga dengan keterbatasan akses informasi. [Sumber](https://www.researchgate.net/publication/45276240_Peritonitis_in_children_on_peritoneal_dialysis_in_Cape_Town_South_Africa_Epidemiology_and_risks) | Nutrition: Rekomendasi asupan protein tinggi (1,4–3,0 g/kg/hari) disesuaikan dengan usia anak untuk mengganti kehilangan protein selama dialisis dan mengejar pertumbuhan. Pemantauan nutrisi dilakukan setiap bulan pada bayi dan setiap 3–4 bulan pada anak yang lebih tua. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC7352713/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) | Type of Catheter (Shape): Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Catheter Placement: Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Gastrostomy/Intraperitoneal Device:  | Catheter Orientation:  | Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
+      <c r="AA71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -9659,6 +9734,7 @@
           <t>Socioeconomic: Edukasi atau retraining intensif bagi keluarga (caregiver) mengenai prosedur aseptik sangat dianjurkan, terutama bagi keluarga dengan keterbatasan akses informasi. [Sumber](https://www.researchgate.net/publication/45276240_Peritonitis_in_children_on_peritoneal_dialysis_in_Cape_Town_South_Africa_Epidemiology_and_risks) | Nutrition: Rekomendasi asupan protein tinggi (1,4–3,0 g/kg/hari) disesuaikan dengan usia anak untuk mengganti kehilangan protein selama dialisis dan mengejar pertumbuhan. Pemantauan nutrisi dilakukan setiap bulan pada bayi dan setiap 3–4 bulan pada anak yang lebih tua. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC7352713/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) | Type of Catheter (Shape): Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Catheter Placement: Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Gastrostomy/Intraperitoneal Device:  | Catheter Orientation:  | Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
+      <c r="AA72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -9791,6 +9867,7 @@
           <t>Housing: Ruangan harus bersih dan bebas dari hewan peliharaan selama prosedur untuk menghindari risiko kontaminasi bakteri Pasteurella atau kerusakan mekanis pada selang. Ketersediaan wastafel untuk mencuci tangan secara benar sangat krusial dalam mengurangi risiko peritonitis. [🔗Sumber 1](https://freseniusmedicalcare.com/content/dam/home-products-education/steps2home-pd/Preventing_Peritonitis.pdf) [🔗Sumber 2](https://spnp-spp.pt/media/rqdpbrom/catheter-related-infections-and-peritonitis-in-pediatric-patients-receiving-peritoneal-dialysis-guideline-for-prevention-and-treatment-2012-1-_compressed-1.pdf) [Sumber 3](https://www.ouh.nhs.uk/media/agxhnni2/85713pdialysis.pdf) [Sumber 4](https://www.satellitehealthcare.com/blog/pets-and-peritoneal-dialysis-absolutely/) | Socioeconomic: Edukasi atau retraining intensif bagi keluarga (caregiver) mengenai prosedur aseptik sangat dianjurkan, terutama bagi keluarga dengan keterbatasan akses informasi. [Sumber](https://www.researchgate.net/publication/45276240_Peritonitis_in_children_on_peritoneal_dialysis_in_Cape_Town_South_Africa_Epidemiology_and_risks) | Nutrition: Rekomendasi asupan protein tinggi (1,4–3,0 g/kg/hari) disesuaikan dengan usia anak untuk mengganti kehilangan protein selama dialisis dan mengejar pertumbuhan. Pemantauan nutrisi dilakukan setiap bulan pada bayi dan setiap 3–4 bulan pada anak yang lebih tua. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC7352713/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) | Type of Catheter (Shape): Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Catheter Placement: Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Gastrostomy/Intraperitoneal Device:  | Catheter Orientation:  | Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
+      <c r="AA73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -9923,6 +10000,7 @@
           <t>Housing: Ruangan harus bersih dan bebas dari hewan peliharaan selama prosedur untuk menghindari risiko kontaminasi bakteri Pasteurella atau kerusakan mekanis pada selang. Ketersediaan wastafel untuk mencuci tangan secara benar sangat krusial dalam mengurangi risiko peritonitis. [🔗Sumber 1](https://freseniusmedicalcare.com/content/dam/home-products-education/steps2home-pd/Preventing_Peritonitis.pdf) [🔗Sumber 2](https://spnp-spp.pt/media/rqdpbrom/catheter-related-infections-and-peritonitis-in-pediatric-patients-receiving-peritoneal-dialysis-guideline-for-prevention-and-treatment-2012-1-_compressed-1.pdf) [Sumber 3](https://www.ouh.nhs.uk/media/agxhnni2/85713pdialysis.pdf) [Sumber 4](https://www.satellitehealthcare.com/blog/pets-and-peritoneal-dialysis-absolutely/) | Socioeconomic: Edukasi atau retraining intensif bagi keluarga (caregiver) mengenai prosedur aseptik sangat dianjurkan, terutama bagi keluarga dengan keterbatasan akses informasi. [Sumber](https://www.researchgate.net/publication/45276240_Peritonitis_in_children_on_peritoneal_dialysis_in_Cape_Town_South_Africa_Epidemiology_and_risks) | Nutrition: Rekomendasi asupan protein tinggi (1,4–3,0 g/kg/hari) disesuaikan dengan usia anak untuk mengganti kehilangan protein selama dialisis dan mengejar pertumbuhan. Pemantauan nutrisi dilakukan setiap bulan pada bayi dan setiap 3–4 bulan pada anak yang lebih tua. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC7352713/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) | Type of Catheter (Shape): Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Catheter Placement: Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Gastrostomy/Intraperitoneal Device:  | Catheter Orientation:  | Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
+      <c r="AA74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -10055,6 +10133,7 @@
           <t>Housing: Ruangan harus bersih dan bebas dari hewan peliharaan selama prosedur untuk menghindari risiko kontaminasi bakteri Pasteurella atau kerusakan mekanis pada selang. Ketersediaan wastafel untuk mencuci tangan secara benar sangat krusial dalam mengurangi risiko peritonitis. [🔗Sumber 1](https://freseniusmedicalcare.com/content/dam/home-products-education/steps2home-pd/Preventing_Peritonitis.pdf) [🔗Sumber 2](https://spnp-spp.pt/media/rqdpbrom/catheter-related-infections-and-peritonitis-in-pediatric-patients-receiving-peritoneal-dialysis-guideline-for-prevention-and-treatment-2012-1-_compressed-1.pdf) [Sumber 3](https://www.ouh.nhs.uk/media/agxhnni2/85713pdialysis.pdf) [Sumber 4](https://www.satellitehealthcare.com/blog/pets-and-peritoneal-dialysis-absolutely/) | Socioeconomic: Edukasi atau retraining intensif bagi keluarga (caregiver) mengenai prosedur aseptik sangat dianjurkan, terutama bagi keluarga dengan keterbatasan akses informasi. [Sumber](https://www.researchgate.net/publication/45276240_Peritonitis_in_children_on_peritoneal_dialysis_in_Cape_Town_South_Africa_Epidemiology_and_risks) | Nutrition: Rekomendasi asupan protein tinggi (1,4–3,0 g/kg/hari) disesuaikan dengan usia anak untuk mengganti kehilangan protein selama dialisis dan mengejar pertumbuhan. Pemantauan nutrisi dilakukan setiap bulan pada bayi dan setiap 3–4 bulan pada anak yang lebih tua. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC7352713/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) | Type of Catheter (Shape): Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Catheter Placement: Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Gastrostomy/Intraperitoneal Device:  | Catheter Orientation:  | Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
+      <c r="AA75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -10187,6 +10266,7 @@
           <t>Housing: Ruangan harus bersih dan bebas dari hewan peliharaan selama prosedur untuk menghindari risiko kontaminasi bakteri Pasteurella atau kerusakan mekanis pada selang. Ketersediaan wastafel untuk mencuci tangan secara benar sangat krusial dalam mengurangi risiko peritonitis. [🔗Sumber 1](https://freseniusmedicalcare.com/content/dam/home-products-education/steps2home-pd/Preventing_Peritonitis.pdf) [🔗Sumber 2](https://spnp-spp.pt/media/rqdpbrom/catheter-related-infections-and-peritonitis-in-pediatric-patients-receiving-peritoneal-dialysis-guideline-for-prevention-and-treatment-2012-1-_compressed-1.pdf) [Sumber 3](https://www.ouh.nhs.uk/media/agxhnni2/85713pdialysis.pdf) [Sumber 4](https://www.satellitehealthcare.com/blog/pets-and-peritoneal-dialysis-absolutely/) | Socioeconomic: Edukasi atau retraining intensif bagi keluarga (caregiver) mengenai prosedur aseptik sangat dianjurkan, terutama bagi keluarga dengan keterbatasan akses informasi. [Sumber](https://www.researchgate.net/publication/45276240_Peritonitis_in_children_on_peritoneal_dialysis_in_Cape_Town_South_Africa_Epidemiology_and_risks) | Nutrition: Rekomendasi asupan protein tinggi (1,4–3,0 g/kg/hari) disesuaikan dengan usia anak untuk mengganti kehilangan protein selama dialisis dan mengejar pertumbuhan. Pemantauan nutrisi dilakukan setiap bulan pada bayi dan setiap 3–4 bulan pada anak yang lebih tua. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC7352713/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) | Type of Catheter (Shape): Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Catheter Placement: Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Gastrostomy/Intraperitoneal Device:  | Catheter Orientation:  | Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
+      <c r="AA76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -10319,6 +10399,7 @@
           <t>Housing: Ruangan harus bersih dan bebas dari hewan peliharaan selama prosedur untuk menghindari risiko kontaminasi bakteri Pasteurella atau kerusakan mekanis pada selang. Ketersediaan wastafel untuk mencuci tangan secara benar sangat krusial dalam mengurangi risiko peritonitis. [🔗Sumber 1](https://freseniusmedicalcare.com/content/dam/home-products-education/steps2home-pd/Preventing_Peritonitis.pdf) [🔗Sumber 2](https://spnp-spp.pt/media/rqdpbrom/catheter-related-infections-and-peritonitis-in-pediatric-patients-receiving-peritoneal-dialysis-guideline-for-prevention-and-treatment-2012-1-_compressed-1.pdf) [Sumber 3](https://www.ouh.nhs.uk/media/agxhnni2/85713pdialysis.pdf) [Sumber 4](https://www.satellitehealthcare.com/blog/pets-and-peritoneal-dialysis-absolutely/) | Socioeconomic: Edukasi atau retraining intensif bagi keluarga (caregiver) mengenai prosedur aseptik sangat dianjurkan, terutama bagi keluarga dengan keterbatasan akses informasi. [Sumber](https://www.researchgate.net/publication/45276240_Peritonitis_in_children_on_peritoneal_dialysis_in_Cape_Town_South_Africa_Epidemiology_and_risks) | Nutrition: Rekomendasi asupan protein tinggi (1,4–3,0 g/kg/hari) disesuaikan dengan usia anak untuk mengganti kehilangan protein selama dialisis dan mengejar pertumbuhan. Pemantauan nutrisi dilakukan setiap bulan pada bayi dan setiap 3–4 bulan pada anak yang lebih tua. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC7352713/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) | Type of Catheter (Shape): Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Catheter Placement: Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Gastrostomy/Intraperitoneal Device:  | Catheter Orientation:  | Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
+      <c r="AA77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -10451,6 +10532,7 @@
           <t>Housing: Ruangan harus bersih dan bebas dari hewan peliharaan selama prosedur untuk menghindari risiko kontaminasi bakteri Pasteurella atau kerusakan mekanis pada selang. Ketersediaan wastafel untuk mencuci tangan secara benar sangat krusial dalam mengurangi risiko peritonitis. [🔗Sumber 1](https://freseniusmedicalcare.com/content/dam/home-products-education/steps2home-pd/Preventing_Peritonitis.pdf) [🔗Sumber 2](https://spnp-spp.pt/media/rqdpbrom/catheter-related-infections-and-peritonitis-in-pediatric-patients-receiving-peritoneal-dialysis-guideline-for-prevention-and-treatment-2012-1-_compressed-1.pdf) [Sumber 3](https://www.ouh.nhs.uk/media/agxhnni2/85713pdialysis.pdf) [Sumber 4](https://www.satellitehealthcare.com/blog/pets-and-peritoneal-dialysis-absolutely/) | Socioeconomic: Edukasi atau retraining intensif bagi keluarga (caregiver) mengenai prosedur aseptik sangat dianjurkan, terutama bagi keluarga dengan keterbatasan akses informasi. [Sumber](https://www.researchgate.net/publication/45276240_Peritonitis_in_children_on_peritoneal_dialysis_in_Cape_Town_South_Africa_Epidemiology_and_risks) | Nutrition: Rekomendasi asupan protein tinggi (1,4–3,0 g/kg/hari) disesuaikan dengan usia anak untuk mengganti kehilangan protein selama dialisis dan mengejar pertumbuhan. Pemantauan nutrisi dilakukan setiap bulan pada bayi dan setiap 3–4 bulan pada anak yang lebih tua. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC7352713/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) | Type of Catheter (Shape): Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Catheter Placement: Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Gastrostomy/Intraperitoneal Device:  | Catheter Orientation:  | Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
+      <c r="AA78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -10583,6 +10665,7 @@
           <t>Housing: Ruangan harus bersih dan bebas dari hewan peliharaan selama prosedur untuk menghindari risiko kontaminasi bakteri Pasteurella atau kerusakan mekanis pada selang. Ketersediaan wastafel untuk mencuci tangan secara benar sangat krusial dalam mengurangi risiko peritonitis. [🔗Sumber 1](https://freseniusmedicalcare.com/content/dam/home-products-education/steps2home-pd/Preventing_Peritonitis.pdf) [🔗Sumber 2](https://spnp-spp.pt/media/rqdpbrom/catheter-related-infections-and-peritonitis-in-pediatric-patients-receiving-peritoneal-dialysis-guideline-for-prevention-and-treatment-2012-1-_compressed-1.pdf) [Sumber 3](https://www.ouh.nhs.uk/media/agxhnni2/85713pdialysis.pdf) [Sumber 4](https://www.satellitehealthcare.com/blog/pets-and-peritoneal-dialysis-absolutely/) | Socioeconomic: Edukasi atau retraining intensif bagi keluarga (caregiver) mengenai prosedur aseptik sangat dianjurkan, terutama bagi keluarga dengan keterbatasan akses informasi. [Sumber](https://www.researchgate.net/publication/45276240_Peritonitis_in_children_on_peritoneal_dialysis_in_Cape_Town_South_Africa_Epidemiology_and_risks) | Nutrition: Rekomendasi asupan protein tinggi (1,4–3,0 g/kg/hari) disesuaikan dengan usia anak untuk mengganti kehilangan protein selama dialisis dan mengejar pertumbuhan. Pemantauan nutrisi dilakukan setiap bulan pada bayi dan setiap 3–4 bulan pada anak yang lebih tua. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC7352713/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) | Type of Catheter (Shape): Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Catheter Placement: Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Gastrostomy/Intraperitoneal Device:  | Catheter Orientation:  | Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
+      <c r="AA79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -10715,6 +10798,7 @@
           <t>Housing: Ruangan harus bersih dan bebas dari hewan peliharaan selama prosedur untuk menghindari risiko kontaminasi bakteri Pasteurella atau kerusakan mekanis pada selang. Ketersediaan wastafel untuk mencuci tangan secara benar sangat krusial dalam mengurangi risiko peritonitis. [🔗Sumber 1](https://freseniusmedicalcare.com/content/dam/home-products-education/steps2home-pd/Preventing_Peritonitis.pdf) [🔗Sumber 2](https://spnp-spp.pt/media/rqdpbrom/catheter-related-infections-and-peritonitis-in-pediatric-patients-receiving-peritoneal-dialysis-guideline-for-prevention-and-treatment-2012-1-_compressed-1.pdf) [Sumber 3](https://www.ouh.nhs.uk/media/agxhnni2/85713pdialysis.pdf) [Sumber 4](https://www.satellitehealthcare.com/blog/pets-and-peritoneal-dialysis-absolutely/) | Socioeconomic: Edukasi atau retraining intensif bagi keluarga (caregiver) mengenai prosedur aseptik sangat dianjurkan, terutama bagi keluarga dengan keterbatasan akses informasi. [Sumber](https://www.researchgate.net/publication/45276240_Peritonitis_in_children_on_peritoneal_dialysis_in_Cape_Town_South_Africa_Epidemiology_and_risks) | Nutrition: Rekomendasi asupan protein tinggi (1,4–3,0 g/kg/hari) disesuaikan dengan usia anak untuk mengganti kehilangan protein selama dialisis dan mengejar pertumbuhan. Pemantauan nutrisi dilakukan setiap bulan pada bayi dan setiap 3–4 bulan pada anak yang lebih tua. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC7352713/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) | Type of Catheter (Shape): Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Catheter Placement: Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Gastrostomy/Intraperitoneal Device:  | Catheter Orientation:  | Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
+      <c r="AA80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -10847,6 +10931,7 @@
           <t>Housing: Ruangan harus bersih dan bebas dari hewan peliharaan selama prosedur untuk menghindari risiko kontaminasi bakteri Pasteurella atau kerusakan mekanis pada selang. Ketersediaan wastafel untuk mencuci tangan secara benar sangat krusial dalam mengurangi risiko peritonitis. [🔗Sumber 1](https://freseniusmedicalcare.com/content/dam/home-products-education/steps2home-pd/Preventing_Peritonitis.pdf) [🔗Sumber 2](https://spnp-spp.pt/media/rqdpbrom/catheter-related-infections-and-peritonitis-in-pediatric-patients-receiving-peritoneal-dialysis-guideline-for-prevention-and-treatment-2012-1-_compressed-1.pdf) [Sumber 3](https://www.ouh.nhs.uk/media/agxhnni2/85713pdialysis.pdf) [Sumber 4](https://www.satellitehealthcare.com/blog/pets-and-peritoneal-dialysis-absolutely/) | Socioeconomic: Edukasi atau retraining intensif bagi keluarga (caregiver) mengenai prosedur aseptik sangat dianjurkan, terutama bagi keluarga dengan keterbatasan akses informasi. [Sumber](https://www.researchgate.net/publication/45276240_Peritonitis_in_children_on_peritoneal_dialysis_in_Cape_Town_South_Africa_Epidemiology_and_risks) | Nutrition: Rekomendasi asupan protein tinggi (1,4–3,0 g/kg/hari) disesuaikan dengan usia anak untuk mengganti kehilangan protein selama dialisis dan mengejar pertumbuhan. Pemantauan nutrisi dilakukan setiap bulan pada bayi dan setiap 3–4 bulan pada anak yang lebih tua. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC7352713/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) | Type of Catheter (Shape): Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Catheter Placement: Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Gastrostomy/Intraperitoneal Device:  | Catheter Orientation:  | Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
+      <c r="AA81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -10979,6 +11064,7 @@
           <t>Housing: Ruangan harus bersih dan bebas dari hewan peliharaan selama prosedur untuk menghindari risiko kontaminasi bakteri Pasteurella atau kerusakan mekanis pada selang. Ketersediaan wastafel untuk mencuci tangan secara benar sangat krusial dalam mengurangi risiko peritonitis. [🔗Sumber 1](https://freseniusmedicalcare.com/content/dam/home-products-education/steps2home-pd/Preventing_Peritonitis.pdf) [🔗Sumber 2](https://spnp-spp.pt/media/rqdpbrom/catheter-related-infections-and-peritonitis-in-pediatric-patients-receiving-peritoneal-dialysis-guideline-for-prevention-and-treatment-2012-1-_compressed-1.pdf) [Sumber 3](https://www.ouh.nhs.uk/media/agxhnni2/85713pdialysis.pdf) [Sumber 4](https://www.satellitehealthcare.com/blog/pets-and-peritoneal-dialysis-absolutely/) | Socioeconomic: Edukasi atau retraining intensif bagi keluarga (caregiver) mengenai prosedur aseptik sangat dianjurkan, terutama bagi keluarga dengan keterbatasan akses informasi. [Sumber](https://www.researchgate.net/publication/45276240_Peritonitis_in_children_on_peritoneal_dialysis_in_Cape_Town_South_Africa_Epidemiology_and_risks) | Nutrition: Rekomendasi asupan protein tinggi (1,4–3,0 g/kg/hari) disesuaikan dengan usia anak untuk mengganti kehilangan protein selama dialisis dan mengejar pertumbuhan. Pemantauan nutrisi dilakukan setiap bulan pada bayi dan setiap 3–4 bulan pada anak yang lebih tua. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC7352713/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) | Type of Catheter (Shape): Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Catheter Placement: Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Gastrostomy/Intraperitoneal Device:  | Catheter Orientation:  | Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
+      <c r="AA82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -11111,6 +11197,7 @@
           <t>Stunting: Stunting pada anak dialisis bukan hanya disebabkan oleh asupan kalori yang rendah, tetapi juga oleh asidosis metabolik, anemia, osteodistrofi ginjal, dan resistensi terhadap hormon pertumbuhan. Intervensi pertama adalah memastikan kecukupan dialisis dan koreksi parameter metabolik seperti asidosis dan hiperparatiroidisme.Jika pertumbuhan masih belum optimal meskipun parameter metabolik telah terkendali dan asupan nutrisi sudah mencapai target, terapi dengan hormon pertumbuhan manusia rekombinan (rhGH) dapat dipertimbangkan. Selain itu, dukungan nutrisi intensif dan klirens dialisis yang adekuat pada pasien prepubertal dapat mempromosikan pertumbuhan normal tanpa selalu memerlukan rhGH. Pada anak yang mengalami stunting (tinggi badan &lt; persentil ke-2), perhitungan kebutuhan energi dan mikronutrien harus didasarkan pada height-age pasien, bukan chronological age-nya, untuk memberikan dukungan yang sesuai dengan ukuran tubuh aktualnya. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/)</t>
         </is>
       </c>
+      <c r="AA83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -11243,6 +11330,7 @@
           <t>Stunting: Stunting pada anak dialisis bukan hanya disebabkan oleh asupan kalori yang rendah, tetapi juga oleh asidosis metabolik, anemia, osteodistrofi ginjal, dan resistensi terhadap hormon pertumbuhan. Intervensi pertama adalah memastikan kecukupan dialisis dan koreksi parameter metabolik seperti asidosis dan hiperparatiroidisme.Jika pertumbuhan masih belum optimal meskipun parameter metabolik telah terkendali dan asupan nutrisi sudah mencapai target, terapi dengan hormon pertumbuhan manusia rekombinan (rhGH) dapat dipertimbangkan. Selain itu, dukungan nutrisi intensif dan klirens dialisis yang adekuat pada pasien prepubertal dapat mempromosikan pertumbuhan normal tanpa selalu memerlukan rhGH. Pada anak yang mengalami stunting (tinggi badan &lt; persentil ke-2), perhitungan kebutuhan energi dan mikronutrien harus didasarkan pada height-age pasien, bukan chronological age-nya, untuk memberikan dukungan yang sesuai dengan ukuran tubuh aktualnya. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/)</t>
         </is>
       </c>
+      <c r="AA84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -11375,6 +11463,7 @@
           <t>Stunting: Stunting pada anak dialisis bukan hanya disebabkan oleh asupan kalori yang rendah, tetapi juga oleh asidosis metabolik, anemia, osteodistrofi ginjal, dan resistensi terhadap hormon pertumbuhan. Intervensi pertama adalah memastikan kecukupan dialisis dan koreksi parameter metabolik seperti asidosis dan hiperparatiroidisme.Jika pertumbuhan masih belum optimal meskipun parameter metabolik telah terkendali dan asupan nutrisi sudah mencapai target, terapi dengan hormon pertumbuhan manusia rekombinan (rhGH) dapat dipertimbangkan. Selain itu, dukungan nutrisi intensif dan klirens dialisis yang adekuat pada pasien prepubertal dapat mempromosikan pertumbuhan normal tanpa selalu memerlukan rhGH. Pada anak yang mengalami stunting (tinggi badan &lt; persentil ke-2), perhitungan kebutuhan energi dan mikronutrien harus didasarkan pada height-age pasien, bukan chronological age-nya, untuk memberikan dukungan yang sesuai dengan ukuran tubuh aktualnya. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/)</t>
         </is>
       </c>
+      <c r="AA85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -11499,6 +11588,7 @@
       </c>
       <c r="Y86" t="inlineStr"/>
       <c r="Z86" t="inlineStr"/>
+      <c r="AA86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -11623,6 +11713,7 @@
       </c>
       <c r="Y87" t="inlineStr"/>
       <c r="Z87" t="inlineStr"/>
+      <c r="AA87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -11747,6 +11838,7 @@
       </c>
       <c r="Y88" t="inlineStr"/>
       <c r="Z88" t="inlineStr"/>
+      <c r="AA88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -11871,6 +11963,7 @@
       </c>
       <c r="Y89" t="inlineStr"/>
       <c r="Z89" t="inlineStr"/>
+      <c r="AA89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -11995,6 +12088,7 @@
       </c>
       <c r="Y90" t="inlineStr"/>
       <c r="Z90" t="inlineStr"/>
+      <c r="AA90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -12119,6 +12213,7 @@
       </c>
       <c r="Y91" t="inlineStr"/>
       <c r="Z91" t="inlineStr"/>
+      <c r="AA91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -12243,6 +12338,1595 @@
       </c>
       <c r="Y92" t="inlineStr"/>
       <c r="Z92" t="inlineStr"/>
+      <c r="AA92" t="inlineStr"/>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>2026-05-15 17:53:27</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>CE0F6C28</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>&gt;2 yo</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>&lt;12 mo</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>Good service</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>Studies</t>
+        </is>
+      </c>
+      <c r="K93" t="inlineStr">
+        <is>
+          <t>ESI</t>
+        </is>
+      </c>
+      <c r="L93" t="inlineStr">
+        <is>
+          <t>Normal Nutrition</t>
+        </is>
+      </c>
+      <c r="M93" t="inlineStr">
+        <is>
+          <t>Glomerular</t>
+        </is>
+      </c>
+      <c r="N93" t="inlineStr">
+        <is>
+          <t>Coiled/swan neck</t>
+        </is>
+      </c>
+      <c r="O93" t="inlineStr">
+        <is>
+          <t>Double</t>
+        </is>
+      </c>
+      <c r="P93" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="Q93" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R93" t="inlineStr">
+        <is>
+          <t>Patients</t>
+        </is>
+      </c>
+      <c r="S93" t="inlineStr"/>
+      <c r="T93" t="inlineStr">
+        <is>
+          <t>Lateral/downward</t>
+        </is>
+      </c>
+      <c r="U93" t="inlineStr">
+        <is>
+          <t>No stunting</t>
+        </is>
+      </c>
+      <c r="V93" t="inlineStr">
+        <is>
+          <t>90.91%</t>
+        </is>
+      </c>
+      <c r="W93" t="inlineStr">
+        <is>
+          <t>Survivor</t>
+        </is>
+      </c>
+      <c r="X93" t="inlineStr">
+        <is>
+          <t>Age*, Gender, Duration of PD*, Place of Residence, Housing, Socioeconomic, Education, Nutrition, Cause of ESRD*, Type of Catheter (Shape), Type of Catheter (Cuff), Catheter Placement, Gastrostomy/Intraperitoneal Device, Performed CAPD, Starting PD &lt;2 weeks after catheter placement, Catheter Orientation, Stunting</t>
+        </is>
+      </c>
+      <c r="Y93" t="inlineStr">
+        <is>
+          <t>Peritonitis in ESI*</t>
+        </is>
+      </c>
+      <c r="Z93" t="inlineStr">
+        <is>
+          <t>Peritonitis in ESI: Penggunaan antibiotik topikal secara rutin pada tempat keluar kateter telat terbukti menurunkan angka infeksi. Aplikasi harian salep mupirocin atau gentamicin pada exit-site direkomendasikan untuk menekan kolonisasi Staphylococcus aureus dan Pseudomonas aeruginosa.Pembersihan area secara rutin dengan larutan antiseptik non-iritan (seperti chlorhexidine 0,05% atau sabun antibakteri ringan) juga merupakan bagian standar dari perawatan. Penilaian kondisi exit-site secara objektif menggunakan sistem skor (seperti Skor ISPD yang mencakup pembengkakan, kerak, kemerahan, nyeri, dan sekret) sangat membantu caregiver dalam mendeteksi infeksi secara dini. Immobilisasi kateter dengan menggunakan plester atau perangkat fiksasi sangat krusial karena trauma mekanis pada tempat keluar sering kali menjadi pintu masuk bagi bakteri. Jika ESI terjadi, terapi antibiotik oral atau intraperitoneal harus dimulai segera dan dilanjutkan selama minimal 2 minggu, atau 3 minggu jika disebabkan oleh Pseudomonas. Pengangkatan kateter mungkin diperlukan jika infeksi bersifat refrakter (tidak merespons pengobatan setelah 2 minggu) atau jika infeksi telah menyebar ke terowongan kateter (tunnel infection) yang menyebabkan peritonitis berulang. [Sumber 1](https://ispd.org/wp-content/uploads/2025/09/LI-ET-1.pdf) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC12640025/) [Sumber 3](https://pmc.ncbi.nlm.nih.gov/articles/PMC5033625/) [Sumber 4](https://www.chikd.org/journal/view.php?number=726) [Sumber 5](https://ispd.org/wp-content/uploads/ISPD-Catheter-related-Infection-Recommendations-2023-Update.pdf) [Sumber 6](https://www.bcrenal.ca/resource-gallery/Documents/PD_Procedures-Exit_Site_Care-Post-Operative_PD_Catheter_Insertion.pdf) [Sumber 7](https://davita.com/treatment-options/articles/preventing-catheter-infections-on-peritoneal-dialysis/) [Sumber 8](https://edren.org/ren/handbook/pd-handbook/protocol-for-the-management-of-pd-peritonitis-long-version/)</t>
+        </is>
+      </c>
+      <c r="AA93" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>2026-05-15 17:54:53</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>CE0F6C28</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>&gt;2 yo</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>&lt;12 mo</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>Good service</t>
+        </is>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>Studies</t>
+        </is>
+      </c>
+      <c r="K94" t="inlineStr">
+        <is>
+          <t>ESI</t>
+        </is>
+      </c>
+      <c r="L94" t="inlineStr">
+        <is>
+          <t>Normal Nutrition</t>
+        </is>
+      </c>
+      <c r="M94" t="inlineStr">
+        <is>
+          <t>Glomerular</t>
+        </is>
+      </c>
+      <c r="N94" t="inlineStr">
+        <is>
+          <t>Coiled/swan neck</t>
+        </is>
+      </c>
+      <c r="O94" t="inlineStr">
+        <is>
+          <t>Double</t>
+        </is>
+      </c>
+      <c r="P94" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="Q94" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R94" t="inlineStr">
+        <is>
+          <t>Patients</t>
+        </is>
+      </c>
+      <c r="S94" t="inlineStr"/>
+      <c r="T94" t="inlineStr">
+        <is>
+          <t>Lateral/downward</t>
+        </is>
+      </c>
+      <c r="U94" t="inlineStr">
+        <is>
+          <t>Stunting</t>
+        </is>
+      </c>
+      <c r="V94" t="inlineStr">
+        <is>
+          <t>86.36%</t>
+        </is>
+      </c>
+      <c r="W94" t="inlineStr">
+        <is>
+          <t>Survivor</t>
+        </is>
+      </c>
+      <c r="X94" t="inlineStr">
+        <is>
+          <t>Age*, Gender, Duration of PD*, Place of Residence, Housing, Socioeconomic, Education, Nutrition, Cause of ESRD*, Type of Catheter (Shape), Type of Catheter (Cuff), Catheter Placement, Gastrostomy/Intraperitoneal Device, Performed CAPD, Starting PD &lt;2 weeks after catheter placement, Catheter Orientation</t>
+        </is>
+      </c>
+      <c r="Y94" t="inlineStr">
+        <is>
+          <t>Peritonitis in ESI*, Stunting</t>
+        </is>
+      </c>
+      <c r="Z94" t="inlineStr">
+        <is>
+          <t>Peritonitis in ESI: Penggunaan antibiotik topikal secara rutin pada tempat keluar kateter telat terbukti menurunkan angka infeksi. Aplikasi harian salep mupirocin atau gentamicin pada exit-site direkomendasikan untuk menekan kolonisasi Staphylococcus aureus dan Pseudomonas aeruginosa.Pembersihan area secara rutin dengan larutan antiseptik non-iritan (seperti chlorhexidine 0,05% atau sabun antibakteri ringan) juga merupakan bagian standar dari perawatan. Penilaian kondisi exit-site secara objektif menggunakan sistem skor (seperti Skor ISPD yang mencakup pembengkakan, kerak, kemerahan, nyeri, dan sekret) sangat membantu caregiver dalam mendeteksi infeksi secara dini. Immobilisasi kateter dengan menggunakan plester atau perangkat fiksasi sangat krusial karena trauma mekanis pada tempat keluar sering kali menjadi pintu masuk bagi bakteri. Jika ESI terjadi, terapi antibiotik oral atau intraperitoneal harus dimulai segera dan dilanjutkan selama minimal 2 minggu, atau 3 minggu jika disebabkan oleh Pseudomonas. Pengangkatan kateter mungkin diperlukan jika infeksi bersifat refrakter (tidak merespons pengobatan setelah 2 minggu) atau jika infeksi telah menyebar ke terowongan kateter (tunnel infection) yang menyebabkan peritonitis berulang. [Sumber 1](https://ispd.org/wp-content/uploads/2025/09/LI-ET-1.pdf) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC12640025/) [Sumber 3](https://pmc.ncbi.nlm.nih.gov/articles/PMC5033625/) [Sumber 4](https://www.chikd.org/journal/view.php?number=726) [Sumber 5](https://ispd.org/wp-content/uploads/ISPD-Catheter-related-Infection-Recommendations-2023-Update.pdf) [Sumber 6](https://www.bcrenal.ca/resource-gallery/Documents/PD_Procedures-Exit_Site_Care-Post-Operative_PD_Catheter_Insertion.pdf) [Sumber 7](https://davita.com/treatment-options/articles/preventing-catheter-infections-on-peritoneal-dialysis/) [Sumber 8](https://edren.org/ren/handbook/pd-handbook/protocol-for-the-management-of-pd-peritonitis-long-version/) | Stunting: Stunting pada anak dialisis bukan hanya disebabkan oleh asupan kalori yang rendah, tetapi juga oleh asidosis metabolik, anemia, osteodistrofi ginjal, dan resistensi terhadap hormon pertumbuhan. Intervensi pertama adalah memastikan kecukupan dialisis dan koreksi parameter metabolik seperti asidosis dan hiperparatiroidisme.Jika pertumbuhan masih belum optimal meskipun parameter metabolik telah terkendali dan asupan nutrisi sudah mencapai target, terapi dengan hormon pertumbuhan manusia rekombinan (rhGH) dapat dipertimbangkan. Selain itu, dukungan nutrisi intensif dan klirens dialisis yang adekuat pada pasien prepubertal dapat mempromosikan pertumbuhan normal tanpa selalu memerlukan rhGH. Pada anak yang mengalami stunting (tinggi badan &lt; persentil ke-2), perhitungan kebutuhan energi dan mikronutrien harus didasarkan pada height-age pasien, bukan chronological age-nya, untuk memberikan dukungan yang sesuai dengan ukuran tubuh aktualnya. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/)</t>
+        </is>
+      </c>
+      <c r="AA94" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>2026-05-15 17:55:05</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>CE0F6C28</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>&lt;2 yo</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>&lt;12 mo</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>Good service</t>
+        </is>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>Studies</t>
+        </is>
+      </c>
+      <c r="K95" t="inlineStr">
+        <is>
+          <t>ESI</t>
+        </is>
+      </c>
+      <c r="L95" t="inlineStr">
+        <is>
+          <t>Normal Nutrition</t>
+        </is>
+      </c>
+      <c r="M95" t="inlineStr">
+        <is>
+          <t>Glomerular</t>
+        </is>
+      </c>
+      <c r="N95" t="inlineStr">
+        <is>
+          <t>Coiled/swan neck</t>
+        </is>
+      </c>
+      <c r="O95" t="inlineStr">
+        <is>
+          <t>Double</t>
+        </is>
+      </c>
+      <c r="P95" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="Q95" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R95" t="inlineStr">
+        <is>
+          <t>Patients</t>
+        </is>
+      </c>
+      <c r="S95" t="inlineStr"/>
+      <c r="T95" t="inlineStr">
+        <is>
+          <t>Lateral/downward</t>
+        </is>
+      </c>
+      <c r="U95" t="inlineStr">
+        <is>
+          <t>Stunting</t>
+        </is>
+      </c>
+      <c r="V95" t="inlineStr">
+        <is>
+          <t>77.27%</t>
+        </is>
+      </c>
+      <c r="W95" t="inlineStr">
+        <is>
+          <t>Survivor</t>
+        </is>
+      </c>
+      <c r="X95" t="inlineStr">
+        <is>
+          <t>Gender, Duration of PD*, Place of Residence, Housing, Socioeconomic, Education, Nutrition, Cause of ESRD*, Type of Catheter (Shape), Type of Catheter (Cuff), Catheter Placement, Gastrostomy/Intraperitoneal Device, Performed CAPD, Starting PD &lt;2 weeks after catheter placement, Catheter Orientation</t>
+        </is>
+      </c>
+      <c r="Y95" t="inlineStr">
+        <is>
+          <t>Age*, Peritonitis in ESI*, Stunting</t>
+        </is>
+      </c>
+      <c r="Z95" t="inlineStr">
+        <is>
+          <t>Peritonitis in ESI: Penggunaan antibiotik topikal secara rutin pada tempat keluar kateter telat terbukti menurunkan angka infeksi. Aplikasi harian salep mupirocin atau gentamicin pada exit-site direkomendasikan untuk menekan kolonisasi Staphylococcus aureus dan Pseudomonas aeruginosa.Pembersihan area secara rutin dengan larutan antiseptik non-iritan (seperti chlorhexidine 0,05% atau sabun antibakteri ringan) juga merupakan bagian standar dari perawatan. Penilaian kondisi exit-site secara objektif menggunakan sistem skor (seperti Skor ISPD yang mencakup pembengkakan, kerak, kemerahan, nyeri, dan sekret) sangat membantu caregiver dalam mendeteksi infeksi secara dini. Immobilisasi kateter dengan menggunakan plester atau perangkat fiksasi sangat krusial karena trauma mekanis pada tempat keluar sering kali menjadi pintu masuk bagi bakteri. Jika ESI terjadi, terapi antibiotik oral atau intraperitoneal harus dimulai segera dan dilanjutkan selama minimal 2 minggu, atau 3 minggu jika disebabkan oleh Pseudomonas. Pengangkatan kateter mungkin diperlukan jika infeksi bersifat refrakter (tidak merespons pengobatan setelah 2 minggu) atau jika infeksi telah menyebar ke terowongan kateter (tunnel infection) yang menyebabkan peritonitis berulang. [Sumber 1](https://ispd.org/wp-content/uploads/2025/09/LI-ET-1.pdf) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC12640025/) [Sumber 3](https://pmc.ncbi.nlm.nih.gov/articles/PMC5033625/) [Sumber 4](https://www.chikd.org/journal/view.php?number=726) [Sumber 5](https://ispd.org/wp-content/uploads/ISPD-Catheter-related-Infection-Recommendations-2023-Update.pdf) [Sumber 6](https://www.bcrenal.ca/resource-gallery/Documents/PD_Procedures-Exit_Site_Care-Post-Operative_PD_Catheter_Insertion.pdf) [Sumber 7](https://davita.com/treatment-options/articles/preventing-catheter-infections-on-peritoneal-dialysis/) [Sumber 8](https://edren.org/ren/handbook/pd-handbook/protocol-for-the-management-of-pd-peritonitis-long-version/) | Stunting: Stunting pada anak dialisis bukan hanya disebabkan oleh asupan kalori yang rendah, tetapi juga oleh asidosis metabolik, anemia, osteodistrofi ginjal, dan resistensi terhadap hormon pertumbuhan. Intervensi pertama adalah memastikan kecukupan dialisis dan koreksi parameter metabolik seperti asidosis dan hiperparatiroidisme.Jika pertumbuhan masih belum optimal meskipun parameter metabolik telah terkendali dan asupan nutrisi sudah mencapai target, terapi dengan hormon pertumbuhan manusia rekombinan (rhGH) dapat dipertimbangkan. Selain itu, dukungan nutrisi intensif dan klirens dialisis yang adekuat pada pasien prepubertal dapat mempromosikan pertumbuhan normal tanpa selalu memerlukan rhGH. Pada anak yang mengalami stunting (tinggi badan &lt; persentil ke-2), perhitungan kebutuhan energi dan mikronutrien harus didasarkan pada height-age pasien, bukan chronological age-nya, untuk memberikan dukungan yang sesuai dengan ukuran tubuh aktualnya. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/)</t>
+        </is>
+      </c>
+      <c r="AA95" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>2026-05-15 17:55:24</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>CE0F6C28</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>&lt;2 yo</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>&lt;12 mo</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>Good service</t>
+        </is>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>Studies</t>
+        </is>
+      </c>
+      <c r="K96" t="inlineStr">
+        <is>
+          <t>ESI</t>
+        </is>
+      </c>
+      <c r="L96" t="inlineStr">
+        <is>
+          <t>Normal Nutrition</t>
+        </is>
+      </c>
+      <c r="M96" t="inlineStr">
+        <is>
+          <t>Glomerular</t>
+        </is>
+      </c>
+      <c r="N96" t="inlineStr">
+        <is>
+          <t>Straight</t>
+        </is>
+      </c>
+      <c r="O96" t="inlineStr">
+        <is>
+          <t>Single cuff</t>
+        </is>
+      </c>
+      <c r="P96" t="inlineStr">
+        <is>
+          <t>Laparoscopic</t>
+        </is>
+      </c>
+      <c r="Q96" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R96" t="inlineStr">
+        <is>
+          <t>Patients</t>
+        </is>
+      </c>
+      <c r="S96" t="inlineStr"/>
+      <c r="T96" t="inlineStr">
+        <is>
+          <t>Lateral/downward</t>
+        </is>
+      </c>
+      <c r="U96" t="inlineStr">
+        <is>
+          <t>Stunting</t>
+        </is>
+      </c>
+      <c r="V96" t="inlineStr">
+        <is>
+          <t>63.64%</t>
+        </is>
+      </c>
+      <c r="W96" t="inlineStr">
+        <is>
+          <t>Survivor</t>
+        </is>
+      </c>
+      <c r="X96" t="inlineStr">
+        <is>
+          <t>Gender, Duration of PD*, Place of Residence, Housing, Socioeconomic, Education, Nutrition, Cause of ESRD*, Gastrostomy/Intraperitoneal Device, Performed CAPD, Starting PD &lt;2 weeks after catheter placement, Catheter Orientation</t>
+        </is>
+      </c>
+      <c r="Y96" t="inlineStr">
+        <is>
+          <t>Age*, Peritonitis in ESI*, Type of Catheter (Shape), Type of Catheter (Cuff), Catheter Placement, Stunting</t>
+        </is>
+      </c>
+      <c r="Z96" t="inlineStr">
+        <is>
+          <t>Peritonitis in ESI: Penggunaan antibiotik topikal secara rutin pada tempat keluar kateter telat terbukti menurunkan angka infeksi. Aplikasi harian salep mupirocin atau gentamicin pada exit-site direkomendasikan untuk menekan kolonisasi Staphylococcus aureus dan Pseudomonas aeruginosa.Pembersihan area secara rutin dengan larutan antiseptik non-iritan (seperti chlorhexidine 0,05% atau sabun antibakteri ringan) juga merupakan bagian standar dari perawatan. Penilaian kondisi exit-site secara objektif menggunakan sistem skor (seperti Skor ISPD yang mencakup pembengkakan, kerak, kemerahan, nyeri, dan sekret) sangat membantu caregiver dalam mendeteksi infeksi secara dini. Immobilisasi kateter dengan menggunakan plester atau perangkat fiksasi sangat krusial karena trauma mekanis pada tempat keluar sering kali menjadi pintu masuk bagi bakteri. Jika ESI terjadi, terapi antibiotik oral atau intraperitoneal harus dimulai segera dan dilanjutkan selama minimal 2 minggu, atau 3 minggu jika disebabkan oleh Pseudomonas. Pengangkatan kateter mungkin diperlukan jika infeksi bersifat refrakter (tidak merespons pengobatan setelah 2 minggu) atau jika infeksi telah menyebar ke terowongan kateter (tunnel infection) yang menyebabkan peritonitis berulang. [Sumber 1](https://ispd.org/wp-content/uploads/2025/09/LI-ET-1.pdf) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC12640025/) [Sumber 3](https://pmc.ncbi.nlm.nih.gov/articles/PMC5033625/) [Sumber 4](https://www.chikd.org/journal/view.php?number=726) [Sumber 5](https://ispd.org/wp-content/uploads/ISPD-Catheter-related-Infection-Recommendations-2023-Update.pdf) [Sumber 6](https://www.bcrenal.ca/resource-gallery/Documents/PD_Procedures-Exit_Site_Care-Post-Operative_PD_Catheter_Insertion.pdf) [Sumber 7](https://davita.com/treatment-options/articles/preventing-catheter-infections-on-peritoneal-dialysis/) [Sumber 8](https://edren.org/ren/handbook/pd-handbook/protocol-for-the-management-of-pd-peritonitis-long-version/) | Type of Catheter (Shape): Perdebatan mengenai efektivitas kateter straight dibandingkan dengan kateter coiled/curled masih berlangsung. Kateter coiled secara teoretis mengurangi nyeri saat pengisian cairan dan meminimalkan trauma pada organ visceral, tetapi beberapa data menunjukkan risiko malposisi yang lebih tinggi dibandingkan tipe lurus pada beberapa kelompok pasien. Di sisi lain, kateter straight lebih mudah ditempatkan pada bayi kecil yang memiliki ruang intra-abdominal terbatas. Secara keseluruhan, pedoman tidak menyatakan superioritas mutlak salah satu bentuk, dan pemilihan sering kali bergantung pada preferensi pusat dialisis dan anatomi pasien. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC9365012/) [Sumber 2](http://ispd.org/wp-content/uploads/7.-Dagmara-Borzych-Duzalka-Peritoneal-Dialysis-Catheters-Outcome-in-Children.-The-IPPN-Data.pdf) [Sumber 3](https://scholarlyexchange.childrensmercy.org/cgi/viewcontent.cgi?article=7522&amp;context=papers) [Sumber 4](https://kidney.wiki/peritoneal-dialysis/pd-access/) | Type of Catheter (Cuff): Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff)untuk populasi anak secara umum. Deep cuff berfungsi untuk menjangkar kateter di otot rektus dan mencegah kebocoran, sementara superficial cuff bertindak sebagai penghalang fisik terhadap migrasi bakteri ke arah rongga peritoneum. Namun, pada neonatus atau bayi dengan dinding perut yang sangat tipis, kateter single-cuff sering kali lebih dipilih untuk mencegah ekstrusi manset ke permukaan kulit. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC10223083/) [Sumber 2](http://ispd.org/wp-content/uploads/7.-Dagmara-Borzych-Duzalka-Peritoneal-Dialysis-Catheters-Outcome-in-Children.-The-IPPN-Data.pdf) [Sumber 3](https://kidney.wiki/peritoneal-dialysis/pd-access/) | Catheter Placement: Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Stunting: Stunting pada anak dialisis bukan hanya disebabkan oleh asupan kalori yang rendah, tetapi juga oleh asidosis metabolik, anemia, osteodistrofi ginjal, dan resistensi terhadap hormon pertumbuhan. Intervensi pertama adalah memastikan kecukupan dialisis dan koreksi parameter metabolik seperti asidosis dan hiperparatiroidisme.Jika pertumbuhan masih belum optimal meskipun parameter metabolik telah terkendali dan asupan nutrisi sudah mencapai target, terapi dengan hormon pertumbuhan manusia rekombinan (rhGH) dapat dipertimbangkan. Selain itu, dukungan nutrisi intensif dan klirens dialisis yang adekuat pada pasien prepubertal dapat mempromosikan pertumbuhan normal tanpa selalu memerlukan rhGH. Pada anak yang mengalami stunting (tinggi badan &lt; persentil ke-2), perhitungan kebutuhan energi dan mikronutrien harus didasarkan pada height-age pasien, bukan chronological age-nya, untuk memberikan dukungan yang sesuai dengan ukuran tubuh aktualnya. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/)</t>
+        </is>
+      </c>
+      <c r="AA96" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>2026-05-15 17:55:31</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>CE0F6C28</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>&lt;2 yo</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>&gt;12 mo</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>Good service</t>
+        </is>
+      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="J97" t="inlineStr">
+        <is>
+          <t>Studies</t>
+        </is>
+      </c>
+      <c r="K97" t="inlineStr">
+        <is>
+          <t>ESI</t>
+        </is>
+      </c>
+      <c r="L97" t="inlineStr">
+        <is>
+          <t>Normal Nutrition</t>
+        </is>
+      </c>
+      <c r="M97" t="inlineStr">
+        <is>
+          <t>Glomerular</t>
+        </is>
+      </c>
+      <c r="N97" t="inlineStr">
+        <is>
+          <t>Straight</t>
+        </is>
+      </c>
+      <c r="O97" t="inlineStr">
+        <is>
+          <t>Single cuff</t>
+        </is>
+      </c>
+      <c r="P97" t="inlineStr">
+        <is>
+          <t>Laparoscopic</t>
+        </is>
+      </c>
+      <c r="Q97" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R97" t="inlineStr">
+        <is>
+          <t>Patients</t>
+        </is>
+      </c>
+      <c r="S97" t="inlineStr"/>
+      <c r="T97" t="inlineStr">
+        <is>
+          <t>Lateral/downward</t>
+        </is>
+      </c>
+      <c r="U97" t="inlineStr">
+        <is>
+          <t>Stunting</t>
+        </is>
+      </c>
+      <c r="V97" t="inlineStr">
+        <is>
+          <t>54.55%</t>
+        </is>
+      </c>
+      <c r="W97" t="inlineStr">
+        <is>
+          <t>Survivor</t>
+        </is>
+      </c>
+      <c r="X97" t="inlineStr">
+        <is>
+          <t>Gender, Place of Residence, Housing, Socioeconomic, Education, Nutrition, Cause of ESRD*, Gastrostomy/Intraperitoneal Device, Performed CAPD, Starting PD &lt;2 weeks after catheter placement, Catheter Orientation</t>
+        </is>
+      </c>
+      <c r="Y97" t="inlineStr">
+        <is>
+          <t>Age*, Duration of PD*, Peritonitis in ESI*, Type of Catheter (Shape), Type of Catheter (Cuff), Catheter Placement, Stunting</t>
+        </is>
+      </c>
+      <c r="Z97" t="inlineStr">
+        <is>
+          <t>Peritonitis in ESI: Penggunaan antibiotik topikal secara rutin pada tempat keluar kateter telat terbukti menurunkan angka infeksi. Aplikasi harian salep mupirocin atau gentamicin pada exit-site direkomendasikan untuk menekan kolonisasi Staphylococcus aureus dan Pseudomonas aeruginosa.Pembersihan area secara rutin dengan larutan antiseptik non-iritan (seperti chlorhexidine 0,05% atau sabun antibakteri ringan) juga merupakan bagian standar dari perawatan. Penilaian kondisi exit-site secara objektif menggunakan sistem skor (seperti Skor ISPD yang mencakup pembengkakan, kerak, kemerahan, nyeri, dan sekret) sangat membantu caregiver dalam mendeteksi infeksi secara dini. Immobilisasi kateter dengan menggunakan plester atau perangkat fiksasi sangat krusial karena trauma mekanis pada tempat keluar sering kali menjadi pintu masuk bagi bakteri. Jika ESI terjadi, terapi antibiotik oral atau intraperitoneal harus dimulai segera dan dilanjutkan selama minimal 2 minggu, atau 3 minggu jika disebabkan oleh Pseudomonas. Pengangkatan kateter mungkin diperlukan jika infeksi bersifat refrakter (tidak merespons pengobatan setelah 2 minggu) atau jika infeksi telah menyebar ke terowongan kateter (tunnel infection) yang menyebabkan peritonitis berulang. [Sumber 1](https://ispd.org/wp-content/uploads/2025/09/LI-ET-1.pdf) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC12640025/) [Sumber 3](https://pmc.ncbi.nlm.nih.gov/articles/PMC5033625/) [Sumber 4](https://www.chikd.org/journal/view.php?number=726) [Sumber 5](https://ispd.org/wp-content/uploads/ISPD-Catheter-related-Infection-Recommendations-2023-Update.pdf) [Sumber 6](https://www.bcrenal.ca/resource-gallery/Documents/PD_Procedures-Exit_Site_Care-Post-Operative_PD_Catheter_Insertion.pdf) [Sumber 7](https://davita.com/treatment-options/articles/preventing-catheter-infections-on-peritoneal-dialysis/) [Sumber 8](https://edren.org/ren/handbook/pd-handbook/protocol-for-the-management-of-pd-peritonitis-long-version/) | Type of Catheter (Shape): Perdebatan mengenai efektivitas kateter straight dibandingkan dengan kateter coiled/curled masih berlangsung. Kateter coiled secara teoretis mengurangi nyeri saat pengisian cairan dan meminimalkan trauma pada organ visceral, tetapi beberapa data menunjukkan risiko malposisi yang lebih tinggi dibandingkan tipe lurus pada beberapa kelompok pasien. Di sisi lain, kateter straight lebih mudah ditempatkan pada bayi kecil yang memiliki ruang intra-abdominal terbatas. Secara keseluruhan, pedoman tidak menyatakan superioritas mutlak salah satu bentuk, dan pemilihan sering kali bergantung pada preferensi pusat dialisis dan anatomi pasien. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC9365012/) [Sumber 2](http://ispd.org/wp-content/uploads/7.-Dagmara-Borzych-Duzalka-Peritoneal-Dialysis-Catheters-Outcome-in-Children.-The-IPPN-Data.pdf) [Sumber 3](https://scholarlyexchange.childrensmercy.org/cgi/viewcontent.cgi?article=7522&amp;context=papers) [Sumber 4](https://kidney.wiki/peritoneal-dialysis/pd-access/) | Type of Catheter (Cuff): Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff)untuk populasi anak secara umum. Deep cuff berfungsi untuk menjangkar kateter di otot rektus dan mencegah kebocoran, sementara superficial cuff bertindak sebagai penghalang fisik terhadap migrasi bakteri ke arah rongga peritoneum. Namun, pada neonatus atau bayi dengan dinding perut yang sangat tipis, kateter single-cuff sering kali lebih dipilih untuk mencegah ekstrusi manset ke permukaan kulit. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC10223083/) [Sumber 2](http://ispd.org/wp-content/uploads/7.-Dagmara-Borzych-Duzalka-Peritoneal-Dialysis-Catheters-Outcome-in-Children.-The-IPPN-Data.pdf) [Sumber 3](https://kidney.wiki/peritoneal-dialysis/pd-access/) | Catheter Placement: Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Stunting: Stunting pada anak dialisis bukan hanya disebabkan oleh asupan kalori yang rendah, tetapi juga oleh asidosis metabolik, anemia, osteodistrofi ginjal, dan resistensi terhadap hormon pertumbuhan. Intervensi pertama adalah memastikan kecukupan dialisis dan koreksi parameter metabolik seperti asidosis dan hiperparatiroidisme.Jika pertumbuhan masih belum optimal meskipun parameter metabolik telah terkendali dan asupan nutrisi sudah mencapai target, terapi dengan hormon pertumbuhan manusia rekombinan (rhGH) dapat dipertimbangkan. Selain itu, dukungan nutrisi intensif dan klirens dialisis yang adekuat pada pasien prepubertal dapat mempromosikan pertumbuhan normal tanpa selalu memerlukan rhGH. Pada anak yang mengalami stunting (tinggi badan &lt; persentil ke-2), perhitungan kebutuhan energi dan mikronutrien harus didasarkan pada height-age pasien, bukan chronological age-nya, untuk memberikan dukungan yang sesuai dengan ukuran tubuh aktualnya. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/)</t>
+        </is>
+      </c>
+      <c r="AA97" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>2026-05-15 17:55:39</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>CE0F6C28</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>&lt;2 yo</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>&gt;12 mo</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>Good service</t>
+        </is>
+      </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t>Studies</t>
+        </is>
+      </c>
+      <c r="K98" t="inlineStr">
+        <is>
+          <t>ESI</t>
+        </is>
+      </c>
+      <c r="L98" t="inlineStr">
+        <is>
+          <t>Normal Nutrition</t>
+        </is>
+      </c>
+      <c r="M98" t="inlineStr">
+        <is>
+          <t>Glomerular</t>
+        </is>
+      </c>
+      <c r="N98" t="inlineStr">
+        <is>
+          <t>Straight</t>
+        </is>
+      </c>
+      <c r="O98" t="inlineStr">
+        <is>
+          <t>Single cuff</t>
+        </is>
+      </c>
+      <c r="P98" t="inlineStr">
+        <is>
+          <t>Laparoscopic</t>
+        </is>
+      </c>
+      <c r="Q98" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R98" t="inlineStr">
+        <is>
+          <t>Patients</t>
+        </is>
+      </c>
+      <c r="S98" t="inlineStr"/>
+      <c r="T98" t="inlineStr">
+        <is>
+          <t>Lateral/downward</t>
+        </is>
+      </c>
+      <c r="U98" t="inlineStr">
+        <is>
+          <t>Stunting</t>
+        </is>
+      </c>
+      <c r="V98" t="inlineStr">
+        <is>
+          <t>50.00%</t>
+        </is>
+      </c>
+      <c r="W98" t="inlineStr">
+        <is>
+          <t>Survivor</t>
+        </is>
+      </c>
+      <c r="X98" t="inlineStr">
+        <is>
+          <t>Gender, Place of Residence, Housing, Socioeconomic, Education, Nutrition, Cause of ESRD*, Gastrostomy/Intraperitoneal Device, Performed CAPD, Catheter Orientation</t>
+        </is>
+      </c>
+      <c r="Y98" t="inlineStr">
+        <is>
+          <t>Age*, Duration of PD*, Peritonitis in ESI*, Type of Catheter (Shape), Type of Catheter (Cuff), Catheter Placement, Starting PD &lt;2 weeks after catheter placement, Stunting</t>
+        </is>
+      </c>
+      <c r="Z98" t="inlineStr">
+        <is>
+          <t>Peritonitis in ESI: Penggunaan antibiotik topikal secara rutin pada tempat keluar kateter telat terbukti menurunkan angka infeksi. Aplikasi harian salep mupirocin atau gentamicin pada exit-site direkomendasikan untuk menekan kolonisasi Staphylococcus aureus dan Pseudomonas aeruginosa.Pembersihan area secara rutin dengan larutan antiseptik non-iritan (seperti chlorhexidine 0,05% atau sabun antibakteri ringan) juga merupakan bagian standar dari perawatan. Penilaian kondisi exit-site secara objektif menggunakan sistem skor (seperti Skor ISPD yang mencakup pembengkakan, kerak, kemerahan, nyeri, dan sekret) sangat membantu caregiver dalam mendeteksi infeksi secara dini. Immobilisasi kateter dengan menggunakan plester atau perangkat fiksasi sangat krusial karena trauma mekanis pada tempat keluar sering kali menjadi pintu masuk bagi bakteri. Jika ESI terjadi, terapi antibiotik oral atau intraperitoneal harus dimulai segera dan dilanjutkan selama minimal 2 minggu, atau 3 minggu jika disebabkan oleh Pseudomonas. Pengangkatan kateter mungkin diperlukan jika infeksi bersifat refrakter (tidak merespons pengobatan setelah 2 minggu) atau jika infeksi telah menyebar ke terowongan kateter (tunnel infection) yang menyebabkan peritonitis berulang. [Sumber 1](https://ispd.org/wp-content/uploads/2025/09/LI-ET-1.pdf) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC12640025/) [Sumber 3](https://pmc.ncbi.nlm.nih.gov/articles/PMC5033625/) [Sumber 4](https://www.chikd.org/journal/view.php?number=726) [Sumber 5](https://ispd.org/wp-content/uploads/ISPD-Catheter-related-Infection-Recommendations-2023-Update.pdf) [Sumber 6](https://www.bcrenal.ca/resource-gallery/Documents/PD_Procedures-Exit_Site_Care-Post-Operative_PD_Catheter_Insertion.pdf) [Sumber 7](https://davita.com/treatment-options/articles/preventing-catheter-infections-on-peritoneal-dialysis/) [Sumber 8](https://edren.org/ren/handbook/pd-handbook/protocol-for-the-management-of-pd-peritonitis-long-version/) | Type of Catheter (Shape): Perdebatan mengenai efektivitas kateter straight dibandingkan dengan kateter coiled/curled masih berlangsung. Kateter coiled secara teoretis mengurangi nyeri saat pengisian cairan dan meminimalkan trauma pada organ visceral, tetapi beberapa data menunjukkan risiko malposisi yang lebih tinggi dibandingkan tipe lurus pada beberapa kelompok pasien. Di sisi lain, kateter straight lebih mudah ditempatkan pada bayi kecil yang memiliki ruang intra-abdominal terbatas. Secara keseluruhan, pedoman tidak menyatakan superioritas mutlak salah satu bentuk, dan pemilihan sering kali bergantung pada preferensi pusat dialisis dan anatomi pasien. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC9365012/) [Sumber 2](http://ispd.org/wp-content/uploads/7.-Dagmara-Borzych-Duzalka-Peritoneal-Dialysis-Catheters-Outcome-in-Children.-The-IPPN-Data.pdf) [Sumber 3](https://scholarlyexchange.childrensmercy.org/cgi/viewcontent.cgi?article=7522&amp;context=papers) [Sumber 4](https://kidney.wiki/peritoneal-dialysis/pd-access/) | Type of Catheter (Cuff): Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff)untuk populasi anak secara umum. Deep cuff berfungsi untuk menjangkar kateter di otot rektus dan mencegah kebocoran, sementara superficial cuff bertindak sebagai penghalang fisik terhadap migrasi bakteri ke arah rongga peritoneum. Namun, pada neonatus atau bayi dengan dinding perut yang sangat tipis, kateter single-cuff sering kali lebih dipilih untuk mencegah ekstrusi manset ke permukaan kulit. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC10223083/) [Sumber 2](http://ispd.org/wp-content/uploads/7.-Dagmara-Borzych-Duzalka-Peritoneal-Dialysis-Catheters-Outcome-in-Children.-The-IPPN-Data.pdf) [Sumber 3](https://kidney.wiki/peritoneal-dialysis/pd-access/) | Catheter Placement: Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Starting PD &lt;2 weeks after catheter placement: Waktu antara pemasangan kateter dan dimulainya dialisis (break-in-period) merupakan faktor penting untuk mencegah komplikasi. Masa penyembuhan minimal 2 minggu sebelum dialysis dimulai. Namun, dalam kondisi klinis tertentu di mana pasien membutuhkan dialisis segera, urgent-start PD (dimulai dalam &lt;14 hari atau bahkan &lt;48 jam) menjadi alternatif yang baik untuk menghindari penggunakan kateter hemodialysis sementara. Pasien dengan break-in-period &lt; 7 hari memiliki risiko yang lebih tinggi terhadap komplikasi awal seperti kebocoran dialisat dan malposisi kateter. Namun, risiko tersebut tidak berkorelasi dengan penurunan kelangsungan hidup atau peningkatan risiko peritonitis jika dilakukan dengan protokol yang tepat. Pada kondisi urgent-start, risiko kebocoran dimitigasi dengan menggunakan volume pengisian rendah (10-20 ml/kg) dan posisi pasien supine untuk mengurangi tekanan intra-abdominal.[Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC3923692/) [Sumber 2](https://journals.plos.org/plosone/article?id=10.1371/journal.pone.0206426) [Sumber 3](https://www.sages.org/publications/guidelines/peritoneal-dialysis-access-guideline-update-2023/) [Sumber 4](https://www.frontiersin.org/journals/endocrinology/articles/10.3389/fendo.2022.936573/full) [Sumber 5](https://scholarlyexchange.childrensmercy.org/cgi/viewcontent.cgi?article=7522&amp;context=papers) [Sumber 6](https://pubmed.ncbi.nlm.nih.gov/33523772/) [Sumber 7](https://www.bcrenal.ca/resource-gallery/Documents/PD_Procedures-Exit_Site_Care-Post-Operative_PD_Catheter_Insertion.pdf) | Stunting: Stunting pada anak dialisis bukan hanya disebabkan oleh asupan kalori yang rendah, tetapi juga oleh asidosis metabolik, anemia, osteodistrofi ginjal, dan resistensi terhadap hormon pertumbuhan. Intervensi pertama adalah memastikan kecukupan dialisis dan koreksi parameter metabolik seperti asidosis dan hiperparatiroidisme.Jika pertumbuhan masih belum optimal meskipun parameter metabolik telah terkendali dan asupan nutrisi sudah mencapai target, terapi dengan hormon pertumbuhan manusia rekombinan (rhGH) dapat dipertimbangkan. Selain itu, dukungan nutrisi intensif dan klirens dialisis yang adekuat pada pasien prepubertal dapat mempromosikan pertumbuhan normal tanpa selalu memerlukan rhGH. Pada anak yang mengalami stunting (tinggi badan &lt; persentil ke-2), perhitungan kebutuhan energi dan mikronutrien harus didasarkan pada height-age pasien, bukan chronological age-nya, untuk memberikan dukungan yang sesuai dengan ukuran tubuh aktualnya. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/)</t>
+        </is>
+      </c>
+      <c r="AA98" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>2026-05-15 17:55:45</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>CE0F6C28</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>&lt;2 yo</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>&gt;12 mo</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>Good service</t>
+        </is>
+      </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="J99" t="inlineStr">
+        <is>
+          <t>Studies</t>
+        </is>
+      </c>
+      <c r="K99" t="inlineStr">
+        <is>
+          <t>ESI</t>
+        </is>
+      </c>
+      <c r="L99" t="inlineStr">
+        <is>
+          <t>Normal Nutrition</t>
+        </is>
+      </c>
+      <c r="M99" t="inlineStr">
+        <is>
+          <t>Glomerular</t>
+        </is>
+      </c>
+      <c r="N99" t="inlineStr">
+        <is>
+          <t>Straight</t>
+        </is>
+      </c>
+      <c r="O99" t="inlineStr">
+        <is>
+          <t>Single cuff</t>
+        </is>
+      </c>
+      <c r="P99" t="inlineStr">
+        <is>
+          <t>Laparoscopic</t>
+        </is>
+      </c>
+      <c r="Q99" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R99" t="inlineStr">
+        <is>
+          <t>Patients</t>
+        </is>
+      </c>
+      <c r="S99" t="inlineStr"/>
+      <c r="T99" t="inlineStr">
+        <is>
+          <t>Lateral/downward</t>
+        </is>
+      </c>
+      <c r="U99" t="inlineStr">
+        <is>
+          <t>Stunting</t>
+        </is>
+      </c>
+      <c r="V99" t="inlineStr">
+        <is>
+          <t>45.45%</t>
+        </is>
+      </c>
+      <c r="W99" t="inlineStr">
+        <is>
+          <t>Non-Survivor</t>
+        </is>
+      </c>
+      <c r="X99" t="inlineStr">
+        <is>
+          <t>Place of Residence, Housing, Socioeconomic, Education, Nutrition, Cause of ESRD*, Gastrostomy/Intraperitoneal Device, Performed CAPD, Catheter Orientation</t>
+        </is>
+      </c>
+      <c r="Y99" t="inlineStr">
+        <is>
+          <t>Age*, Gender, Duration of PD*, Peritonitis in ESI*, Type of Catheter (Shape), Type of Catheter (Cuff), Catheter Placement, Starting PD &lt;2 weeks after catheter placement, Stunting</t>
+        </is>
+      </c>
+      <c r="Z99" t="inlineStr">
+        <is>
+          <t>Peritonitis in ESI: Penggunaan antibiotik topikal secara rutin pada tempat keluar kateter telat terbukti menurunkan angka infeksi. Aplikasi harian salep mupirocin atau gentamicin pada exit-site direkomendasikan untuk menekan kolonisasi Staphylococcus aureus dan Pseudomonas aeruginosa.Pembersihan area secara rutin dengan larutan antiseptik non-iritan (seperti chlorhexidine 0,05% atau sabun antibakteri ringan) juga merupakan bagian standar dari perawatan. Penilaian kondisi exit-site secara objektif menggunakan sistem skor (seperti Skor ISPD yang mencakup pembengkakan, kerak, kemerahan, nyeri, dan sekret) sangat membantu caregiver dalam mendeteksi infeksi secara dini. Immobilisasi kateter dengan menggunakan plester atau perangkat fiksasi sangat krusial karena trauma mekanis pada tempat keluar sering kali menjadi pintu masuk bagi bakteri. Jika ESI terjadi, terapi antibiotik oral atau intraperitoneal harus dimulai segera dan dilanjutkan selama minimal 2 minggu, atau 3 minggu jika disebabkan oleh Pseudomonas. Pengangkatan kateter mungkin diperlukan jika infeksi bersifat refrakter (tidak merespons pengobatan setelah 2 minggu) atau jika infeksi telah menyebar ke terowongan kateter (tunnel infection) yang menyebabkan peritonitis berulang. [Sumber 1](https://ispd.org/wp-content/uploads/2025/09/LI-ET-1.pdf) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC12640025/) [Sumber 3](https://pmc.ncbi.nlm.nih.gov/articles/PMC5033625/) [Sumber 4](https://www.chikd.org/journal/view.php?number=726) [Sumber 5](https://ispd.org/wp-content/uploads/ISPD-Catheter-related-Infection-Recommendations-2023-Update.pdf) [Sumber 6](https://www.bcrenal.ca/resource-gallery/Documents/PD_Procedures-Exit_Site_Care-Post-Operative_PD_Catheter_Insertion.pdf) [Sumber 7](https://davita.com/treatment-options/articles/preventing-catheter-infections-on-peritoneal-dialysis/) [Sumber 8](https://edren.org/ren/handbook/pd-handbook/protocol-for-the-management-of-pd-peritonitis-long-version/) | Type of Catheter (Shape): Perdebatan mengenai efektivitas kateter straight dibandingkan dengan kateter coiled/curled masih berlangsung. Kateter coiled secara teoretis mengurangi nyeri saat pengisian cairan dan meminimalkan trauma pada organ visceral, tetapi beberapa data menunjukkan risiko malposisi yang lebih tinggi dibandingkan tipe lurus pada beberapa kelompok pasien. Di sisi lain, kateter straight lebih mudah ditempatkan pada bayi kecil yang memiliki ruang intra-abdominal terbatas. Secara keseluruhan, pedoman tidak menyatakan superioritas mutlak salah satu bentuk, dan pemilihan sering kali bergantung pada preferensi pusat dialisis dan anatomi pasien. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC9365012/) [Sumber 2](http://ispd.org/wp-content/uploads/7.-Dagmara-Borzych-Duzalka-Peritoneal-Dialysis-Catheters-Outcome-in-Children.-The-IPPN-Data.pdf) [Sumber 3](https://scholarlyexchange.childrensmercy.org/cgi/viewcontent.cgi?article=7522&amp;context=papers) [Sumber 4](https://kidney.wiki/peritoneal-dialysis/pd-access/) | Type of Catheter (Cuff): Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff)untuk populasi anak secara umum. Deep cuff berfungsi untuk menjangkar kateter di otot rektus dan mencegah kebocoran, sementara superficial cuff bertindak sebagai penghalang fisik terhadap migrasi bakteri ke arah rongga peritoneum. Namun, pada neonatus atau bayi dengan dinding perut yang sangat tipis, kateter single-cuff sering kali lebih dipilih untuk mencegah ekstrusi manset ke permukaan kulit. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC10223083/) [Sumber 2](http://ispd.org/wp-content/uploads/7.-Dagmara-Borzych-Duzalka-Peritoneal-Dialysis-Catheters-Outcome-in-Children.-The-IPPN-Data.pdf) [Sumber 3](https://kidney.wiki/peritoneal-dialysis/pd-access/) | Catheter Placement: Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Starting PD &lt;2 weeks after catheter placement: Waktu antara pemasangan kateter dan dimulainya dialisis (break-in-period) merupakan faktor penting untuk mencegah komplikasi. Masa penyembuhan minimal 2 minggu sebelum dialysis dimulai. Namun, dalam kondisi klinis tertentu di mana pasien membutuhkan dialisis segera, urgent-start PD (dimulai dalam &lt;14 hari atau bahkan &lt;48 jam) menjadi alternatif yang baik untuk menghindari penggunakan kateter hemodialysis sementara. Pasien dengan break-in-period &lt; 7 hari memiliki risiko yang lebih tinggi terhadap komplikasi awal seperti kebocoran dialisat dan malposisi kateter. Namun, risiko tersebut tidak berkorelasi dengan penurunan kelangsungan hidup atau peningkatan risiko peritonitis jika dilakukan dengan protokol yang tepat. Pada kondisi urgent-start, risiko kebocoran dimitigasi dengan menggunakan volume pengisian rendah (10-20 ml/kg) dan posisi pasien supine untuk mengurangi tekanan intra-abdominal.[Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC3923692/) [Sumber 2](https://journals.plos.org/plosone/article?id=10.1371/journal.pone.0206426) [Sumber 3](https://www.sages.org/publications/guidelines/peritoneal-dialysis-access-guideline-update-2023/) [Sumber 4](https://www.frontiersin.org/journals/endocrinology/articles/10.3389/fendo.2022.936573/full) [Sumber 5](https://scholarlyexchange.childrensmercy.org/cgi/viewcontent.cgi?article=7522&amp;context=papers) [Sumber 6](https://pubmed.ncbi.nlm.nih.gov/33523772/) [Sumber 7](https://www.bcrenal.ca/resource-gallery/Documents/PD_Procedures-Exit_Site_Care-Post-Operative_PD_Catheter_Insertion.pdf) | Stunting: Stunting pada anak dialisis bukan hanya disebabkan oleh asupan kalori yang rendah, tetapi juga oleh asidosis metabolik, anemia, osteodistrofi ginjal, dan resistensi terhadap hormon pertumbuhan. Intervensi pertama adalah memastikan kecukupan dialisis dan koreksi parameter metabolik seperti asidosis dan hiperparatiroidisme.Jika pertumbuhan masih belum optimal meskipun parameter metabolik telah terkendali dan asupan nutrisi sudah mencapai target, terapi dengan hormon pertumbuhan manusia rekombinan (rhGH) dapat dipertimbangkan. Selain itu, dukungan nutrisi intensif dan klirens dialisis yang adekuat pada pasien prepubertal dapat mempromosikan pertumbuhan normal tanpa selalu memerlukan rhGH. Pada anak yang mengalami stunting (tinggi badan &lt; persentil ke-2), perhitungan kebutuhan energi dan mikronutrien harus didasarkan pada height-age pasien, bukan chronological age-nya, untuk memberikan dukungan yang sesuai dengan ukuran tubuh aktualnya. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/)</t>
+        </is>
+      </c>
+      <c r="AA99" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>2026-05-18 22:53:23</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>47DD1EB1</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>&gt;2 yo</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>&lt;12 mo</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>Good service</t>
+        </is>
+      </c>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="J100" t="inlineStr">
+        <is>
+          <t>Studies</t>
+        </is>
+      </c>
+      <c r="K100" t="inlineStr">
+        <is>
+          <t>No ESI</t>
+        </is>
+      </c>
+      <c r="L100" t="inlineStr">
+        <is>
+          <t>Normal Nutrition</t>
+        </is>
+      </c>
+      <c r="M100" t="inlineStr">
+        <is>
+          <t>Glomerular</t>
+        </is>
+      </c>
+      <c r="N100" t="inlineStr">
+        <is>
+          <t>Coiled/swan neck</t>
+        </is>
+      </c>
+      <c r="O100" t="inlineStr">
+        <is>
+          <t>Double</t>
+        </is>
+      </c>
+      <c r="P100" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="Q100" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R100" t="inlineStr">
+        <is>
+          <t>Patients</t>
+        </is>
+      </c>
+      <c r="S100" t="inlineStr"/>
+      <c r="T100" t="inlineStr">
+        <is>
+          <t>Lateral/downward</t>
+        </is>
+      </c>
+      <c r="U100" t="inlineStr">
+        <is>
+          <t>No stunting</t>
+        </is>
+      </c>
+      <c r="V100" t="inlineStr">
+        <is>
+          <t>100.00%</t>
+        </is>
+      </c>
+      <c r="W100" t="inlineStr">
+        <is>
+          <t>Survivor</t>
+        </is>
+      </c>
+      <c r="X100" t="inlineStr">
+        <is>
+          <t>Age*, Gender, Duration of PD*, Place of Residence, Housing, Socioeconomic, Education, Peritonitis in ESI*, Nutrition, Cause of ESRD*, Type of Catheter (Shape), Type of Catheter (Cuff), Catheter Placement, Gastrostomy/Intraperitoneal Device, Performed CAPD, Starting PD &lt;2 weeks after catheter placement, Catheter Orientation, Stunting</t>
+        </is>
+      </c>
+      <c r="Y100" t="inlineStr"/>
+      <c r="Z100" t="inlineStr"/>
+      <c r="AA100" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>2026-05-18 22:53:29</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>47DD1EB1</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>&gt;2 yo</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>&lt;12 mo</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>Good service</t>
+        </is>
+      </c>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>Studies</t>
+        </is>
+      </c>
+      <c r="K101" t="inlineStr">
+        <is>
+          <t>No ESI</t>
+        </is>
+      </c>
+      <c r="L101" t="inlineStr">
+        <is>
+          <t>Normal Nutrition</t>
+        </is>
+      </c>
+      <c r="M101" t="inlineStr">
+        <is>
+          <t>Glomerular</t>
+        </is>
+      </c>
+      <c r="N101" t="inlineStr">
+        <is>
+          <t>Coiled/swan neck</t>
+        </is>
+      </c>
+      <c r="O101" t="inlineStr">
+        <is>
+          <t>Double</t>
+        </is>
+      </c>
+      <c r="P101" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="Q101" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R101" t="inlineStr">
+        <is>
+          <t>Patients</t>
+        </is>
+      </c>
+      <c r="S101" t="inlineStr"/>
+      <c r="T101" t="inlineStr">
+        <is>
+          <t>upward</t>
+        </is>
+      </c>
+      <c r="U101" t="inlineStr">
+        <is>
+          <t>No stunting</t>
+        </is>
+      </c>
+      <c r="V101" t="inlineStr">
+        <is>
+          <t>95.45%</t>
+        </is>
+      </c>
+      <c r="W101" t="inlineStr">
+        <is>
+          <t>Survivor</t>
+        </is>
+      </c>
+      <c r="X101" t="inlineStr">
+        <is>
+          <t>Age*, Gender, Duration of PD*, Place of Residence, Housing, Socioeconomic, Education, Peritonitis in ESI*, Nutrition, Cause of ESRD*, Type of Catheter (Shape), Type of Catheter (Cuff), Catheter Placement, Gastrostomy/Intraperitoneal Device, Performed CAPD, Starting PD &lt;2 weeks after catheter placement, Stunting</t>
+        </is>
+      </c>
+      <c r="Y101" t="inlineStr">
+        <is>
+          <t>Catheter Orientation</t>
+        </is>
+      </c>
+      <c r="Z101" t="inlineStr">
+        <is>
+          <t>Catheter Orientation: Posisi atau arah lubang keluar kateter (exit site) sangat memengaruhi risiko terjadinya infeksi. Data multisentrik dari SCOPE Collaborative menunjukkan bahwa orientasi kateter yang menghadap ke atas (Upward) dikaitkan dengan peningkatan risiko peritonitis hingga 4.2 kali lipat (Rate Ratio: 4.2; 95% CI: 1.49–11.89) dibandingkan orientasi lainnya. Secara anatomis, lubang keluar yang menghadap ke atas menciptakan bentuk cekungan yang dapat menampung keringat, air mandi, dan kotoran. Akibat gaya gravitasi, bakteri yang terkumpul di area ini akan mengendap dan bermigrasi ke dalam terowongan kateter. Oleh karena itu, lubang keluar kateter harus selalu diarahkan ke bawah (Downward) atau ke samping (Lateral) untuk mencegah penumpukan bakteri secara alami. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC5012476/) [Sumber 2](https://openurologyandnephrologyjournal.com/VOLUME/5/PAGE/4/) [Sumber 3](https://kidney.wiki/peritoneal-dialysis/pd-access/)</t>
+        </is>
+      </c>
+      <c r="AA101" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>2026-05-18 22:54:10</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>47DD1EB1</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>&gt;2 yo</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>&lt;12 mo</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>Good service</t>
+        </is>
+      </c>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t>Studies</t>
+        </is>
+      </c>
+      <c r="K102" t="inlineStr">
+        <is>
+          <t>No ESI</t>
+        </is>
+      </c>
+      <c r="L102" t="inlineStr">
+        <is>
+          <t>Normal Nutrition</t>
+        </is>
+      </c>
+      <c r="M102" t="inlineStr">
+        <is>
+          <t>Glomerular</t>
+        </is>
+      </c>
+      <c r="N102" t="inlineStr">
+        <is>
+          <t>Coiled/swan neck</t>
+        </is>
+      </c>
+      <c r="O102" t="inlineStr">
+        <is>
+          <t>Double</t>
+        </is>
+      </c>
+      <c r="P102" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="Q102" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R102" t="inlineStr">
+        <is>
+          <t>Patients</t>
+        </is>
+      </c>
+      <c r="S102" t="inlineStr"/>
+      <c r="T102" t="inlineStr">
+        <is>
+          <t>upward</t>
+        </is>
+      </c>
+      <c r="U102" t="inlineStr">
+        <is>
+          <t>No stunting</t>
+        </is>
+      </c>
+      <c r="V102" t="inlineStr">
+        <is>
+          <t>95.45%</t>
+        </is>
+      </c>
+      <c r="W102" t="inlineStr">
+        <is>
+          <t>Survivor</t>
+        </is>
+      </c>
+      <c r="X102" t="inlineStr">
+        <is>
+          <t>Age*, Gender, Duration of PD*, Place of Residence, Housing, Socioeconomic, Education, Peritonitis in ESI*, Nutrition, Cause of ESRD*, Type of Catheter (Shape), Type of Catheter (Cuff), Catheter Placement, Gastrostomy/Intraperitoneal Device, Performed CAPD, Starting PD &lt;2 weeks after catheter placement, Stunting</t>
+        </is>
+      </c>
+      <c r="Y102" t="inlineStr">
+        <is>
+          <t>Catheter Orientation</t>
+        </is>
+      </c>
+      <c r="Z102" t="inlineStr">
+        <is>
+          <t>Catheter Orientation: Posisi atau arah lubang keluar kateter (exit site) sangat memengaruhi risiko terjadinya infeksi. Data multisentrik dari SCOPE Collaborative menunjukkan bahwa orientasi kateter yang menghadap ke atas (Upward) dikaitkan dengan peningkatan risiko peritonitis hingga 4.2 kali lipat (Rate Ratio: 4.2; 95% CI: 1.49–11.89) dibandingkan orientasi lainnya. Secara anatomis, lubang keluar yang menghadap ke atas menciptakan bentuk cekungan yang dapat menampung keringat, air mandi, dan kotoran. Akibat gaya gravitasi, bakteri yang terkumpul di area ini akan mengendap dan bermigrasi ke dalam terowongan kateter. Oleh karena itu, lubang keluar kateter harus selalu diarahkan ke bawah (Downward) atau ke samping (Lateral) untuk mencegah penumpukan bakteri secara alami. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC5012476/) [Sumber 2](https://openurologyandnephrologyjournal.com/VOLUME/5/PAGE/4/) [Sumber 3](https://kidney.wiki/peritoneal-dialysis/pd-access/)</t>
+        </is>
+      </c>
+      <c r="AA102" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>2026-05-18 22:54:22</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>47DD1EB1</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>&gt;2 yo</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>&lt;12 mo</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>Good service</t>
+        </is>
+      </c>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="J103" t="inlineStr">
+        <is>
+          <t>Studies</t>
+        </is>
+      </c>
+      <c r="K103" t="inlineStr">
+        <is>
+          <t>No ESI</t>
+        </is>
+      </c>
+      <c r="L103" t="inlineStr">
+        <is>
+          <t>Normal Nutrition</t>
+        </is>
+      </c>
+      <c r="M103" t="inlineStr">
+        <is>
+          <t>Glomerular</t>
+        </is>
+      </c>
+      <c r="N103" t="inlineStr">
+        <is>
+          <t>Coiled/swan neck</t>
+        </is>
+      </c>
+      <c r="O103" t="inlineStr">
+        <is>
+          <t>Double</t>
+        </is>
+      </c>
+      <c r="P103" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="Q103" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R103" t="inlineStr">
+        <is>
+          <t>Patients</t>
+        </is>
+      </c>
+      <c r="S103" t="inlineStr"/>
+      <c r="T103" t="inlineStr">
+        <is>
+          <t>upward</t>
+        </is>
+      </c>
+      <c r="U103" t="inlineStr">
+        <is>
+          <t>No stunting</t>
+        </is>
+      </c>
+      <c r="V103" t="inlineStr">
+        <is>
+          <t>95.45%</t>
+        </is>
+      </c>
+      <c r="W103" t="inlineStr">
+        <is>
+          <t>Survivor</t>
+        </is>
+      </c>
+      <c r="X103" t="inlineStr">
+        <is>
+          <t>Age*, Gender, Duration of PD*, Place of Residence, Housing, Socioeconomic, Education, Peritonitis in ESI*, Nutrition, Cause of ESRD*, Type of Catheter (Shape), Type of Catheter (Cuff), Catheter Placement, Gastrostomy/Intraperitoneal Device, Performed CAPD, Starting PD &lt;2 weeks after catheter placement, Stunting</t>
+        </is>
+      </c>
+      <c r="Y103" t="inlineStr">
+        <is>
+          <t>Catheter Orientation</t>
+        </is>
+      </c>
+      <c r="Z103" t="inlineStr">
+        <is>
+          <t>Catheter Orientation: Posisi atau arah lubang keluar kateter (exit site) sangat memengaruhi risiko terjadinya infeksi. Data multisentrik dari SCOPE Collaborative menunjukkan bahwa orientasi kateter yang menghadap ke atas (Upward) dikaitkan dengan peningkatan risiko peritonitis hingga 4.2 kali lipat (Rate Ratio: 4.2; 95% CI: 1.49–11.89) dibandingkan orientasi lainnya. Secara anatomis, lubang keluar yang menghadap ke atas menciptakan bentuk cekungan yang dapat menampung keringat, air mandi, dan kotoran. Akibat gaya gravitasi, bakteri yang terkumpul di area ini akan mengendap dan bermigrasi ke dalam terowongan kateter. Oleh karena itu, lubang keluar kateter harus selalu diarahkan ke bawah (Downward) atau ke samping (Lateral) untuk mencegah penumpukan bakteri secara alami. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC5012476/) [Sumber 2](https://openurologyandnephrologyjournal.com/VOLUME/5/PAGE/4/) [Sumber 3](https://kidney.wiki/peritoneal-dialysis/pd-access/)</t>
+        </is>
+      </c>
+      <c r="AA103" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>2026-05-18 22:54:27</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>47DD1EB1</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>&gt;2 yo</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>&lt;12 mo</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>Good service</t>
+        </is>
+      </c>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>Studies</t>
+        </is>
+      </c>
+      <c r="K104" t="inlineStr">
+        <is>
+          <t>No ESI</t>
+        </is>
+      </c>
+      <c r="L104" t="inlineStr">
+        <is>
+          <t>Normal Nutrition</t>
+        </is>
+      </c>
+      <c r="M104" t="inlineStr">
+        <is>
+          <t>Glomerular</t>
+        </is>
+      </c>
+      <c r="N104" t="inlineStr">
+        <is>
+          <t>Coiled/swan neck</t>
+        </is>
+      </c>
+      <c r="O104" t="inlineStr">
+        <is>
+          <t>Double</t>
+        </is>
+      </c>
+      <c r="P104" t="inlineStr">
+        <is>
+          <t>Laparoscopic</t>
+        </is>
+      </c>
+      <c r="Q104" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R104" t="inlineStr">
+        <is>
+          <t>Patients</t>
+        </is>
+      </c>
+      <c r="S104" t="inlineStr"/>
+      <c r="T104" t="inlineStr">
+        <is>
+          <t>upward</t>
+        </is>
+      </c>
+      <c r="U104" t="inlineStr">
+        <is>
+          <t>No stunting</t>
+        </is>
+      </c>
+      <c r="V104" t="inlineStr">
+        <is>
+          <t>90.91%</t>
+        </is>
+      </c>
+      <c r="W104" t="inlineStr">
+        <is>
+          <t>Survivor</t>
+        </is>
+      </c>
+      <c r="X104" t="inlineStr">
+        <is>
+          <t>Age*, Gender, Duration of PD*, Place of Residence, Housing, Socioeconomic, Education, Peritonitis in ESI*, Nutrition, Cause of ESRD*, Type of Catheter (Shape), Type of Catheter (Cuff), Gastrostomy/Intraperitoneal Device, Performed CAPD, Starting PD &lt;2 weeks after catheter placement, Stunting</t>
+        </is>
+      </c>
+      <c r="Y104" t="inlineStr">
+        <is>
+          <t>Catheter Placement, Catheter Orientation</t>
+        </is>
+      </c>
+      <c r="Z104" t="inlineStr">
+        <is>
+          <t>Catheter Placement: Pedoman klinis terbaru dari Society of American Gastrointestinal and Endoscopic Surgeons (SAGES) menyarankan penggunaan teknik laparoskopi tingkat lanjut (Laparoscopic) dibandingkan teknik bedah terbuka (Open) untuk pemasangan kateter pada populasi pediatrik. Laparoscopic menawarkan akurasi catheter placement yang jauh lebih tinggi di dalam rongga abdomen karena visualisasi langsung, serta meminimalkan trauma mekanis pada jaringan perut. Lebih lanjut, Laparoscopic memungkinkan dokter untuk melakukan prosedur profilaksis penting seperti omentektomi atau omentopeksi untuk meminimalkan risiko omental wrapping (penyumbatan kateter oleh omentum), yang merupakan salah satu penyebab utama kegagalan mekanis kateter pada anak-anak. Laparoscopic juga terbukti mempermudah penyelamatan (salvage) jika terjadi malposisi atau disfungsi kateter tanpa harus melakukan pembedahan ulang yang invasif. [Sumber 1](https://www.sages.org/publications/guidelines/peritoneal-dialysis-access-guideline-update-2023/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC10223083/) [[3]](https://kidney.wiki/peritoneal-dialysis/pd-access/) | Catheter Orientation: Posisi atau arah lubang keluar kateter (exit site) sangat memengaruhi risiko terjadinya infeksi. Data multisentrik dari SCOPE Collaborative menunjukkan bahwa orientasi kateter yang menghadap ke atas (Upward) dikaitkan dengan peningkatan risiko peritonitis hingga 4.2 kali lipat (Rate Ratio: 4.2; 95% CI: 1.49–11.89) dibandingkan orientasi lainnya. Secara anatomis, lubang keluar yang menghadap ke atas menciptakan bentuk cekungan yang dapat menampung keringat, air mandi, dan kotoran. Akibat gaya gravitasi, bakteri yang terkumpul di area ini akan mengendap dan bermigrasi ke dalam terowongan kateter. Oleh karena itu, lubang keluar kateter harus selalu diarahkan ke bawah (Downward) atau ke samping (Lateral) untuk mencegah penumpukan bakteri secara alami. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC5012476/) [Sumber 2](https://openurologyandnephrologyjournal.com/VOLUME/5/PAGE/4/) [Sumber 3](https://kidney.wiki/peritoneal-dialysis/pd-access/)</t>
+        </is>
+      </c>
+      <c r="AA104" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
v3 19 mei 2026 - merombak semua istilah survival rate menjadi perinotitis risk rate
</commit_message>
<xml_diff>
--- a/peritonitis-prediction/PeritonitisPrediction_Database.xlsx
+++ b/peritonitis-prediction/PeritonitisPrediction_Database.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA104"/>
+  <dimension ref="A1:Z129"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -509,7 +509,7 @@
       </c>
       <c r="S1" t="inlineStr">
         <is>
-          <t>Starting PD &lt;2 weeks after placement</t>
+          <t>Starting PD &lt;2 weeks after catheter placement</t>
         </is>
       </c>
       <c r="T1" t="inlineStr">
@@ -524,17 +524,17 @@
       </c>
       <c r="V1" t="inlineStr">
         <is>
-          <t>Survival Rate</t>
+          <t>Peritonitis_Risk_Rate</t>
         </is>
       </c>
       <c r="W1" t="inlineStr">
         <is>
-          <t>Outcome</t>
+          <t>Category_Outcome</t>
         </is>
       </c>
       <c r="X1" t="inlineStr">
         <is>
-          <t>Supporting_Factors</t>
+          <t>Protective_Factors</t>
         </is>
       </c>
       <c r="Y1" t="inlineStr">
@@ -545,11 +545,6 @@
       <c r="Z1" t="inlineStr">
         <is>
           <t>Modifiable_Risk_Factors_Advice</t>
-        </is>
-      </c>
-      <c r="AA1" t="inlineStr">
-        <is>
-          <t>Starting PD &lt;2 weeks after catheter placement</t>
         </is>
       </c>
     </row>
@@ -660,7 +655,6 @@
       <c r="X2" t="inlineStr"/>
       <c r="Y2" t="inlineStr"/>
       <c r="Z2" t="inlineStr"/>
-      <c r="AA2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -769,7 +763,6 @@
       <c r="X3" t="inlineStr"/>
       <c r="Y3" t="inlineStr"/>
       <c r="Z3" t="inlineStr"/>
-      <c r="AA3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -878,7 +871,6 @@
       <c r="X4" t="inlineStr"/>
       <c r="Y4" t="inlineStr"/>
       <c r="Z4" t="inlineStr"/>
-      <c r="AA4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -991,7 +983,6 @@
       <c r="X5" t="inlineStr"/>
       <c r="Y5" t="inlineStr"/>
       <c r="Z5" t="inlineStr"/>
-      <c r="AA5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1112,7 +1103,6 @@
       <c r="X6" t="inlineStr"/>
       <c r="Y6" t="inlineStr"/>
       <c r="Z6" t="inlineStr"/>
-      <c r="AA6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1233,7 +1223,6 @@
       <c r="X7" t="inlineStr"/>
       <c r="Y7" t="inlineStr"/>
       <c r="Z7" t="inlineStr"/>
-      <c r="AA7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1354,7 +1343,6 @@
       <c r="X8" t="inlineStr"/>
       <c r="Y8" t="inlineStr"/>
       <c r="Z8" t="inlineStr"/>
-      <c r="AA8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1475,7 +1463,6 @@
       <c r="X9" t="inlineStr"/>
       <c r="Y9" t="inlineStr"/>
       <c r="Z9" t="inlineStr"/>
-      <c r="AA9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1596,7 +1583,6 @@
       <c r="X10" t="inlineStr"/>
       <c r="Y10" t="inlineStr"/>
       <c r="Z10" t="inlineStr"/>
-      <c r="AA10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1717,7 +1703,6 @@
       <c r="X11" t="inlineStr"/>
       <c r="Y11" t="inlineStr"/>
       <c r="Z11" t="inlineStr"/>
-      <c r="AA11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1838,7 +1823,6 @@
       <c r="X12" t="inlineStr"/>
       <c r="Y12" t="inlineStr"/>
       <c r="Z12" t="inlineStr"/>
-      <c r="AA12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1967,7 +1951,6 @@
         </is>
       </c>
       <c r="Z13" t="inlineStr"/>
-      <c r="AA13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2100,7 +2083,6 @@
           <t>Housing: Perlu perbaikan sanitasi dan fasilitas lingkungan tempat tinggal untuk mengurangi risiko kontaminasi kuman dari lingkungan. | Peritonitis in ESI: Perlu penanganan agresif dan segera terhadap infeksi area keluar kateter (Exit Site Infection) agar kuman tidak masuk ke rongga perut. | Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
-      <c r="AA14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2225,7 +2207,6 @@
       </c>
       <c r="Y15" t="inlineStr"/>
       <c r="Z15" t="inlineStr"/>
-      <c r="AA15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2350,7 +2331,6 @@
       </c>
       <c r="Y16" t="inlineStr"/>
       <c r="Z16" t="inlineStr"/>
-      <c r="AA16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2475,7 +2455,6 @@
       </c>
       <c r="Y17" t="inlineStr"/>
       <c r="Z17" t="inlineStr"/>
-      <c r="AA17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2608,7 +2587,6 @@
           <t>Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
-      <c r="AA18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2733,7 +2711,6 @@
       </c>
       <c r="Y19" t="inlineStr"/>
       <c r="Z19" t="inlineStr"/>
-      <c r="AA19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2866,7 +2843,6 @@
           <t>Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
-      <c r="AA20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2999,7 +2975,6 @@
           <t>Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
-      <c r="AA21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -3132,7 +3107,6 @@
           <t>Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
-      <c r="AA22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -3265,7 +3239,6 @@
           <t>Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
-      <c r="AA23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -3390,7 +3363,6 @@
       </c>
       <c r="Y24" t="inlineStr"/>
       <c r="Z24" t="inlineStr"/>
-      <c r="AA24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -3519,7 +3491,6 @@
         </is>
       </c>
       <c r="Z25" t="inlineStr"/>
-      <c r="AA25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -3648,7 +3619,6 @@
         </is>
       </c>
       <c r="Z26" t="inlineStr"/>
-      <c r="AA26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -3777,7 +3747,6 @@
         </is>
       </c>
       <c r="Z27" t="inlineStr"/>
-      <c r="AA27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -3906,7 +3875,6 @@
         </is>
       </c>
       <c r="Z28" t="inlineStr"/>
-      <c r="AA28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -4039,7 +4007,6 @@
           <t>Nutrition: Perlu peningkatan asupan nutrisi dan pemantauan status gizi secara berkala oleh ahli gizi anak untuk mencapai status gizi normal.</t>
         </is>
       </c>
-      <c r="AA29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -4172,7 +4139,6 @@
           <t>Nutrition: Perlu peningkatan asupan nutrisi dan pemantauan status gizi secara berkala oleh ahli gizi anak untuk mencapai status gizi normal. | Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
-      <c r="AA30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -4305,7 +4271,6 @@
           <t>Catheter Orientation:  | Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
-      <c r="AA31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -4438,7 +4403,6 @@
           <t>Catheter Orientation:  | Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
-      <c r="AA32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -4571,7 +4535,6 @@
           <t>Peritonitis in ESI: Perlu penanganan agresif dan segera terhadap infeksi area keluar kateter (Exit Site Infection) agar kuman tidak masuk ke rongga perut. | Catheter Orientation:  | Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
-      <c r="AA33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -4704,7 +4667,6 @@
           <t xml:space="preserve">Catheter Orientation: </t>
         </is>
       </c>
-      <c r="AA34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -4829,7 +4791,6 @@
       </c>
       <c r="Y35" t="inlineStr"/>
       <c r="Z35" t="inlineStr"/>
-      <c r="AA35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -4962,7 +4923,6 @@
           <t>Performed CAPD: Perlu pelatihan ulang yang intensif bagi orang yang melakukan dialisis (pasien/keluarga) mengenai prosedur aseptik yang benar. | Starting PD &lt;2 weeks after placement: Sebaiknya menunda dimulainya dialisis (jika kondisi klinis memungkinkan) minimal 2 minggu setelah operasi agar luka kateter sembuh sempurna. | Catheter Orientation:  | Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
-      <c r="AA36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -5095,7 +5055,6 @@
           <t>Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
-      <c r="AA37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -5228,7 +5187,6 @@
           <t>Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
-      <c r="AA38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -5361,7 +5319,6 @@
           <t>Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
-      <c r="AA39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -5494,7 +5451,6 @@
           <t>Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
-      <c r="AA40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -5627,7 +5583,6 @@
           <t>Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
-      <c r="AA41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -5760,7 +5715,6 @@
           <t>Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
-      <c r="AA42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -5885,7 +5839,6 @@
       </c>
       <c r="Y43" t="inlineStr"/>
       <c r="Z43" t="inlineStr"/>
-      <c r="AA43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -6018,7 +5971,6 @@
           <t>Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
-      <c r="AA44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -6151,7 +6103,6 @@
           <t>Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
-      <c r="AA45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -6284,7 +6235,6 @@
           <t>Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
-      <c r="AA46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -6417,7 +6367,6 @@
           <t>Peritonitis in ESI: Perlu penanganan agresif dan segera terhadap infeksi area keluar kateter (Exit Site Infection) agar kuman tidak masuk ke rongga perut. | Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
-      <c r="AA47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -6550,7 +6499,6 @@
           <t>Peritonitis in ESI: Perlu penanganan agresif dan segera terhadap infeksi area keluar kateter (Exit Site Infection) agar kuman tidak masuk ke rongga perut. | Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
-      <c r="AA48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -6683,7 +6631,6 @@
           <t>Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
-      <c r="AA49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -6816,7 +6763,6 @@
           <t>Housing: Pastikan ada ruangan khusus yang bersih (minim debu/hewan peliharaan) untuk melakukan pertukaran cairan, serta ketersediaan wastafel dengan air mengalir di dalam ruangan tersebut untuk antisepsis tangan. [Sumber](https://www.scielo.br/j/jbn/a/hHtvqSXhwcCtvBnNqk9JBzk/?lang=en&amp;format=pdf) | Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
-      <c r="AA50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -6949,7 +6895,6 @@
           <t>Housing: Pastikan ada ruangan khusus yang bersih (minim debu/hewan peliharaan) untuk melakukan pertukaran cairan, serta ketersediaan wastafel dengan air mengalir di dalam ruangan tersebut untuk antisepsis tangan. [Sumber](https://www.scielo.br/j/jbn/a/hHtvqSXhwcCtvBnNqk9JBzk/?lang=en&amp;format=pdf) | Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
-      <c r="AA51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -7082,7 +7027,6 @@
           <t>Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
-      <c r="AA52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -7215,7 +7159,6 @@
           <t>Nutrition: Berikan asupan protein tinggi sesuai target usia (biasanya 1.4–3.0 g/kg/hari untuk anak) guna mengejar pertumbuhan dan mengganti protein yang hilang saat dialisis. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC7352713/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) | Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
-      <c r="AA53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -7348,7 +7291,6 @@
           <t>Nutrition: Berikan asupan protein tinggi sesuai target usia (biasanya 1.4–3.0 g/kg/hari untuk anak) guna mengejar pertumbuhan dan mengganti protein yang hilang saat dialisis. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC7352713/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) | Type of Catheter (Cuff): Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
-      <c r="AA54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -7481,7 +7423,6 @@
           <t>Peritonitis in ESI: Gunakan salep antibiotik topikal (seperti mupirocin atau gentamisin) pada exit site secara rutin dan pembersihan area dengan cairan antiseptik non-iritan. [Sumber](https://journals.eco-vector.com/2075-3594/article/view/637454) | Nutrition: Berikan asupan protein tinggi sesuai target usia (biasanya 1.4–3.0 g/kg/hari untuk anak) guna mengejar pertumbuhan dan mengganti protein yang hilang saat dialisis. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC7352713/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) | Type of Catheter (Cuff): Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
-      <c r="AA55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -7606,7 +7547,6 @@
       </c>
       <c r="Y56" t="inlineStr"/>
       <c r="Z56" t="inlineStr"/>
-      <c r="AA56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -7739,7 +7679,6 @@
           <t>Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
-      <c r="AA57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -7872,7 +7811,6 @@
           <t>Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
-      <c r="AA58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -8005,7 +7943,6 @@
           <t>Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
-      <c r="AA59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -8138,7 +8075,6 @@
           <t>Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
-      <c r="AA60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -8271,7 +8207,6 @@
           <t>Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
-      <c r="AA61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -8404,7 +8339,6 @@
           <t>Nutrition: Berikan asupan protein tinggi sesuai target usia (biasanya 1.4–3.0 g/kg/hari untuk anak) guna mengejar pertumbuhan dan mengganti protein yang hilang saat dialisis. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC7352713/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) | Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
-      <c r="AA62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -8537,7 +8471,6 @@
           <t>Nutrition: Rekomendasi asupan protein tinggi (1,4–3,0 g/kg/hari) disesuaikan dengan usia anak untuk mengganti kehilangan protein selama dialisis dan mengejar pertumbuhan. Pemantauan nutrisi dilakukan setiap bulan pada bayi dan setiap 3–4 bulan pada anak yang lebih tua. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC7352713/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) | Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
-      <c r="AA63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -8670,7 +8603,6 @@
           <t>Nutrition: Rekomendasi asupan protein tinggi (1,4–3,0 g/kg/hari) disesuaikan dengan usia anak untuk mengganti kehilangan protein selama dialisis dan mengejar pertumbuhan. Pemantauan nutrisi dilakukan setiap bulan pada bayi dan setiap 3–4 bulan pada anak yang lebih tua. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC7352713/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) | Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
-      <c r="AA64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -8803,7 +8735,6 @@
           <t>Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
-      <c r="AA65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -8936,7 +8867,6 @@
           <t>Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
-      <c r="AA66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -9069,7 +8999,6 @@
           <t>Catheter Placement: Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
-      <c r="AA67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -9202,7 +9131,6 @@
           <t>Catheter Placement: Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Catheter Orientation:  | Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
-      <c r="AA68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -9335,7 +9263,6 @@
           <t>Type of Catheter (Shape): Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Catheter Placement: Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Catheter Orientation:  | Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
-      <c r="AA69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -9468,7 +9395,6 @@
           <t>Nutrition: Rekomendasi asupan protein tinggi (1,4–3,0 g/kg/hari) disesuaikan dengan usia anak untuk mengganti kehilangan protein selama dialisis dan mengejar pertumbuhan. Pemantauan nutrisi dilakukan setiap bulan pada bayi dan setiap 3–4 bulan pada anak yang lebih tua. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC7352713/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) | Type of Catheter (Shape): Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Catheter Placement: Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Catheter Orientation:  | Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
-      <c r="AA70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -9601,7 +9527,6 @@
           <t>Socioeconomic: Edukasi atau retraining intensif bagi keluarga (caregiver) mengenai prosedur aseptik sangat dianjurkan, terutama bagi keluarga dengan keterbatasan akses informasi. [Sumber](https://www.researchgate.net/publication/45276240_Peritonitis_in_children_on_peritoneal_dialysis_in_Cape_Town_South_Africa_Epidemiology_and_risks) | Nutrition: Rekomendasi asupan protein tinggi (1,4–3,0 g/kg/hari) disesuaikan dengan usia anak untuk mengganti kehilangan protein selama dialisis dan mengejar pertumbuhan. Pemantauan nutrisi dilakukan setiap bulan pada bayi dan setiap 3–4 bulan pada anak yang lebih tua. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC7352713/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) | Type of Catheter (Shape): Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Catheter Placement: Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Gastrostomy/Intraperitoneal Device:  | Catheter Orientation:  | Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
-      <c r="AA71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -9734,7 +9659,6 @@
           <t>Socioeconomic: Edukasi atau retraining intensif bagi keluarga (caregiver) mengenai prosedur aseptik sangat dianjurkan, terutama bagi keluarga dengan keterbatasan akses informasi. [Sumber](https://www.researchgate.net/publication/45276240_Peritonitis_in_children_on_peritoneal_dialysis_in_Cape_Town_South_Africa_Epidemiology_and_risks) | Nutrition: Rekomendasi asupan protein tinggi (1,4–3,0 g/kg/hari) disesuaikan dengan usia anak untuk mengganti kehilangan protein selama dialisis dan mengejar pertumbuhan. Pemantauan nutrisi dilakukan setiap bulan pada bayi dan setiap 3–4 bulan pada anak yang lebih tua. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC7352713/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) | Type of Catheter (Shape): Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Catheter Placement: Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Gastrostomy/Intraperitoneal Device:  | Catheter Orientation:  | Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
-      <c r="AA72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -9867,7 +9791,6 @@
           <t>Housing: Ruangan harus bersih dan bebas dari hewan peliharaan selama prosedur untuk menghindari risiko kontaminasi bakteri Pasteurella atau kerusakan mekanis pada selang. Ketersediaan wastafel untuk mencuci tangan secara benar sangat krusial dalam mengurangi risiko peritonitis. [🔗Sumber 1](https://freseniusmedicalcare.com/content/dam/home-products-education/steps2home-pd/Preventing_Peritonitis.pdf) [🔗Sumber 2](https://spnp-spp.pt/media/rqdpbrom/catheter-related-infections-and-peritonitis-in-pediatric-patients-receiving-peritoneal-dialysis-guideline-for-prevention-and-treatment-2012-1-_compressed-1.pdf) [Sumber 3](https://www.ouh.nhs.uk/media/agxhnni2/85713pdialysis.pdf) [Sumber 4](https://www.satellitehealthcare.com/blog/pets-and-peritoneal-dialysis-absolutely/) | Socioeconomic: Edukasi atau retraining intensif bagi keluarga (caregiver) mengenai prosedur aseptik sangat dianjurkan, terutama bagi keluarga dengan keterbatasan akses informasi. [Sumber](https://www.researchgate.net/publication/45276240_Peritonitis_in_children_on_peritoneal_dialysis_in_Cape_Town_South_Africa_Epidemiology_and_risks) | Nutrition: Rekomendasi asupan protein tinggi (1,4–3,0 g/kg/hari) disesuaikan dengan usia anak untuk mengganti kehilangan protein selama dialisis dan mengejar pertumbuhan. Pemantauan nutrisi dilakukan setiap bulan pada bayi dan setiap 3–4 bulan pada anak yang lebih tua. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC7352713/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) | Type of Catheter (Shape): Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Catheter Placement: Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Gastrostomy/Intraperitoneal Device:  | Catheter Orientation:  | Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
-      <c r="AA73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -10000,7 +9923,6 @@
           <t>Housing: Ruangan harus bersih dan bebas dari hewan peliharaan selama prosedur untuk menghindari risiko kontaminasi bakteri Pasteurella atau kerusakan mekanis pada selang. Ketersediaan wastafel untuk mencuci tangan secara benar sangat krusial dalam mengurangi risiko peritonitis. [🔗Sumber 1](https://freseniusmedicalcare.com/content/dam/home-products-education/steps2home-pd/Preventing_Peritonitis.pdf) [🔗Sumber 2](https://spnp-spp.pt/media/rqdpbrom/catheter-related-infections-and-peritonitis-in-pediatric-patients-receiving-peritoneal-dialysis-guideline-for-prevention-and-treatment-2012-1-_compressed-1.pdf) [Sumber 3](https://www.ouh.nhs.uk/media/agxhnni2/85713pdialysis.pdf) [Sumber 4](https://www.satellitehealthcare.com/blog/pets-and-peritoneal-dialysis-absolutely/) | Socioeconomic: Edukasi atau retraining intensif bagi keluarga (caregiver) mengenai prosedur aseptik sangat dianjurkan, terutama bagi keluarga dengan keterbatasan akses informasi. [Sumber](https://www.researchgate.net/publication/45276240_Peritonitis_in_children_on_peritoneal_dialysis_in_Cape_Town_South_Africa_Epidemiology_and_risks) | Nutrition: Rekomendasi asupan protein tinggi (1,4–3,0 g/kg/hari) disesuaikan dengan usia anak untuk mengganti kehilangan protein selama dialisis dan mengejar pertumbuhan. Pemantauan nutrisi dilakukan setiap bulan pada bayi dan setiap 3–4 bulan pada anak yang lebih tua. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC7352713/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) | Type of Catheter (Shape): Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Catheter Placement: Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Gastrostomy/Intraperitoneal Device:  | Catheter Orientation:  | Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
-      <c r="AA74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -10133,7 +10055,6 @@
           <t>Housing: Ruangan harus bersih dan bebas dari hewan peliharaan selama prosedur untuk menghindari risiko kontaminasi bakteri Pasteurella atau kerusakan mekanis pada selang. Ketersediaan wastafel untuk mencuci tangan secara benar sangat krusial dalam mengurangi risiko peritonitis. [🔗Sumber 1](https://freseniusmedicalcare.com/content/dam/home-products-education/steps2home-pd/Preventing_Peritonitis.pdf) [🔗Sumber 2](https://spnp-spp.pt/media/rqdpbrom/catheter-related-infections-and-peritonitis-in-pediatric-patients-receiving-peritoneal-dialysis-guideline-for-prevention-and-treatment-2012-1-_compressed-1.pdf) [Sumber 3](https://www.ouh.nhs.uk/media/agxhnni2/85713pdialysis.pdf) [Sumber 4](https://www.satellitehealthcare.com/blog/pets-and-peritoneal-dialysis-absolutely/) | Socioeconomic: Edukasi atau retraining intensif bagi keluarga (caregiver) mengenai prosedur aseptik sangat dianjurkan, terutama bagi keluarga dengan keterbatasan akses informasi. [Sumber](https://www.researchgate.net/publication/45276240_Peritonitis_in_children_on_peritoneal_dialysis_in_Cape_Town_South_Africa_Epidemiology_and_risks) | Nutrition: Rekomendasi asupan protein tinggi (1,4–3,0 g/kg/hari) disesuaikan dengan usia anak untuk mengganti kehilangan protein selama dialisis dan mengejar pertumbuhan. Pemantauan nutrisi dilakukan setiap bulan pada bayi dan setiap 3–4 bulan pada anak yang lebih tua. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC7352713/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) | Type of Catheter (Shape): Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Catheter Placement: Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Gastrostomy/Intraperitoneal Device:  | Catheter Orientation:  | Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
-      <c r="AA75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -10266,7 +10187,6 @@
           <t>Housing: Ruangan harus bersih dan bebas dari hewan peliharaan selama prosedur untuk menghindari risiko kontaminasi bakteri Pasteurella atau kerusakan mekanis pada selang. Ketersediaan wastafel untuk mencuci tangan secara benar sangat krusial dalam mengurangi risiko peritonitis. [🔗Sumber 1](https://freseniusmedicalcare.com/content/dam/home-products-education/steps2home-pd/Preventing_Peritonitis.pdf) [🔗Sumber 2](https://spnp-spp.pt/media/rqdpbrom/catheter-related-infections-and-peritonitis-in-pediatric-patients-receiving-peritoneal-dialysis-guideline-for-prevention-and-treatment-2012-1-_compressed-1.pdf) [Sumber 3](https://www.ouh.nhs.uk/media/agxhnni2/85713pdialysis.pdf) [Sumber 4](https://www.satellitehealthcare.com/blog/pets-and-peritoneal-dialysis-absolutely/) | Socioeconomic: Edukasi atau retraining intensif bagi keluarga (caregiver) mengenai prosedur aseptik sangat dianjurkan, terutama bagi keluarga dengan keterbatasan akses informasi. [Sumber](https://www.researchgate.net/publication/45276240_Peritonitis_in_children_on_peritoneal_dialysis_in_Cape_Town_South_Africa_Epidemiology_and_risks) | Nutrition: Rekomendasi asupan protein tinggi (1,4–3,0 g/kg/hari) disesuaikan dengan usia anak untuk mengganti kehilangan protein selama dialisis dan mengejar pertumbuhan. Pemantauan nutrisi dilakukan setiap bulan pada bayi dan setiap 3–4 bulan pada anak yang lebih tua. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC7352713/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) | Type of Catheter (Shape): Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Catheter Placement: Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Gastrostomy/Intraperitoneal Device:  | Catheter Orientation:  | Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
-      <c r="AA76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -10399,7 +10319,6 @@
           <t>Housing: Ruangan harus bersih dan bebas dari hewan peliharaan selama prosedur untuk menghindari risiko kontaminasi bakteri Pasteurella atau kerusakan mekanis pada selang. Ketersediaan wastafel untuk mencuci tangan secara benar sangat krusial dalam mengurangi risiko peritonitis. [🔗Sumber 1](https://freseniusmedicalcare.com/content/dam/home-products-education/steps2home-pd/Preventing_Peritonitis.pdf) [🔗Sumber 2](https://spnp-spp.pt/media/rqdpbrom/catheter-related-infections-and-peritonitis-in-pediatric-patients-receiving-peritoneal-dialysis-guideline-for-prevention-and-treatment-2012-1-_compressed-1.pdf) [Sumber 3](https://www.ouh.nhs.uk/media/agxhnni2/85713pdialysis.pdf) [Sumber 4](https://www.satellitehealthcare.com/blog/pets-and-peritoneal-dialysis-absolutely/) | Socioeconomic: Edukasi atau retraining intensif bagi keluarga (caregiver) mengenai prosedur aseptik sangat dianjurkan, terutama bagi keluarga dengan keterbatasan akses informasi. [Sumber](https://www.researchgate.net/publication/45276240_Peritonitis_in_children_on_peritoneal_dialysis_in_Cape_Town_South_Africa_Epidemiology_and_risks) | Nutrition: Rekomendasi asupan protein tinggi (1,4–3,0 g/kg/hari) disesuaikan dengan usia anak untuk mengganti kehilangan protein selama dialisis dan mengejar pertumbuhan. Pemantauan nutrisi dilakukan setiap bulan pada bayi dan setiap 3–4 bulan pada anak yang lebih tua. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC7352713/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) | Type of Catheter (Shape): Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Catheter Placement: Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Gastrostomy/Intraperitoneal Device:  | Catheter Orientation:  | Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
-      <c r="AA77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -10532,7 +10451,6 @@
           <t>Housing: Ruangan harus bersih dan bebas dari hewan peliharaan selama prosedur untuk menghindari risiko kontaminasi bakteri Pasteurella atau kerusakan mekanis pada selang. Ketersediaan wastafel untuk mencuci tangan secara benar sangat krusial dalam mengurangi risiko peritonitis. [🔗Sumber 1](https://freseniusmedicalcare.com/content/dam/home-products-education/steps2home-pd/Preventing_Peritonitis.pdf) [🔗Sumber 2](https://spnp-spp.pt/media/rqdpbrom/catheter-related-infections-and-peritonitis-in-pediatric-patients-receiving-peritoneal-dialysis-guideline-for-prevention-and-treatment-2012-1-_compressed-1.pdf) [Sumber 3](https://www.ouh.nhs.uk/media/agxhnni2/85713pdialysis.pdf) [Sumber 4](https://www.satellitehealthcare.com/blog/pets-and-peritoneal-dialysis-absolutely/) | Socioeconomic: Edukasi atau retraining intensif bagi keluarga (caregiver) mengenai prosedur aseptik sangat dianjurkan, terutama bagi keluarga dengan keterbatasan akses informasi. [Sumber](https://www.researchgate.net/publication/45276240_Peritonitis_in_children_on_peritoneal_dialysis_in_Cape_Town_South_Africa_Epidemiology_and_risks) | Nutrition: Rekomendasi asupan protein tinggi (1,4–3,0 g/kg/hari) disesuaikan dengan usia anak untuk mengganti kehilangan protein selama dialisis dan mengejar pertumbuhan. Pemantauan nutrisi dilakukan setiap bulan pada bayi dan setiap 3–4 bulan pada anak yang lebih tua. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC7352713/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) | Type of Catheter (Shape): Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Catheter Placement: Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Gastrostomy/Intraperitoneal Device:  | Catheter Orientation:  | Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
-      <c r="AA78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -10665,7 +10583,6 @@
           <t>Housing: Ruangan harus bersih dan bebas dari hewan peliharaan selama prosedur untuk menghindari risiko kontaminasi bakteri Pasteurella atau kerusakan mekanis pada selang. Ketersediaan wastafel untuk mencuci tangan secara benar sangat krusial dalam mengurangi risiko peritonitis. [🔗Sumber 1](https://freseniusmedicalcare.com/content/dam/home-products-education/steps2home-pd/Preventing_Peritonitis.pdf) [🔗Sumber 2](https://spnp-spp.pt/media/rqdpbrom/catheter-related-infections-and-peritonitis-in-pediatric-patients-receiving-peritoneal-dialysis-guideline-for-prevention-and-treatment-2012-1-_compressed-1.pdf) [Sumber 3](https://www.ouh.nhs.uk/media/agxhnni2/85713pdialysis.pdf) [Sumber 4](https://www.satellitehealthcare.com/blog/pets-and-peritoneal-dialysis-absolutely/) | Socioeconomic: Edukasi atau retraining intensif bagi keluarga (caregiver) mengenai prosedur aseptik sangat dianjurkan, terutama bagi keluarga dengan keterbatasan akses informasi. [Sumber](https://www.researchgate.net/publication/45276240_Peritonitis_in_children_on_peritoneal_dialysis_in_Cape_Town_South_Africa_Epidemiology_and_risks) | Nutrition: Rekomendasi asupan protein tinggi (1,4–3,0 g/kg/hari) disesuaikan dengan usia anak untuk mengganti kehilangan protein selama dialisis dan mengejar pertumbuhan. Pemantauan nutrisi dilakukan setiap bulan pada bayi dan setiap 3–4 bulan pada anak yang lebih tua. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC7352713/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) | Type of Catheter (Shape): Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Catheter Placement: Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Gastrostomy/Intraperitoneal Device:  | Catheter Orientation:  | Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
-      <c r="AA79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -10798,7 +10715,6 @@
           <t>Housing: Ruangan harus bersih dan bebas dari hewan peliharaan selama prosedur untuk menghindari risiko kontaminasi bakteri Pasteurella atau kerusakan mekanis pada selang. Ketersediaan wastafel untuk mencuci tangan secara benar sangat krusial dalam mengurangi risiko peritonitis. [🔗Sumber 1](https://freseniusmedicalcare.com/content/dam/home-products-education/steps2home-pd/Preventing_Peritonitis.pdf) [🔗Sumber 2](https://spnp-spp.pt/media/rqdpbrom/catheter-related-infections-and-peritonitis-in-pediatric-patients-receiving-peritoneal-dialysis-guideline-for-prevention-and-treatment-2012-1-_compressed-1.pdf) [Sumber 3](https://www.ouh.nhs.uk/media/agxhnni2/85713pdialysis.pdf) [Sumber 4](https://www.satellitehealthcare.com/blog/pets-and-peritoneal-dialysis-absolutely/) | Socioeconomic: Edukasi atau retraining intensif bagi keluarga (caregiver) mengenai prosedur aseptik sangat dianjurkan, terutama bagi keluarga dengan keterbatasan akses informasi. [Sumber](https://www.researchgate.net/publication/45276240_Peritonitis_in_children_on_peritoneal_dialysis_in_Cape_Town_South_Africa_Epidemiology_and_risks) | Nutrition: Rekomendasi asupan protein tinggi (1,4–3,0 g/kg/hari) disesuaikan dengan usia anak untuk mengganti kehilangan protein selama dialisis dan mengejar pertumbuhan. Pemantauan nutrisi dilakukan setiap bulan pada bayi dan setiap 3–4 bulan pada anak yang lebih tua. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC7352713/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) | Type of Catheter (Shape): Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Catheter Placement: Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Gastrostomy/Intraperitoneal Device:  | Catheter Orientation:  | Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
-      <c r="AA80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -10931,7 +10847,6 @@
           <t>Housing: Ruangan harus bersih dan bebas dari hewan peliharaan selama prosedur untuk menghindari risiko kontaminasi bakteri Pasteurella atau kerusakan mekanis pada selang. Ketersediaan wastafel untuk mencuci tangan secara benar sangat krusial dalam mengurangi risiko peritonitis. [🔗Sumber 1](https://freseniusmedicalcare.com/content/dam/home-products-education/steps2home-pd/Preventing_Peritonitis.pdf) [🔗Sumber 2](https://spnp-spp.pt/media/rqdpbrom/catheter-related-infections-and-peritonitis-in-pediatric-patients-receiving-peritoneal-dialysis-guideline-for-prevention-and-treatment-2012-1-_compressed-1.pdf) [Sumber 3](https://www.ouh.nhs.uk/media/agxhnni2/85713pdialysis.pdf) [Sumber 4](https://www.satellitehealthcare.com/blog/pets-and-peritoneal-dialysis-absolutely/) | Socioeconomic: Edukasi atau retraining intensif bagi keluarga (caregiver) mengenai prosedur aseptik sangat dianjurkan, terutama bagi keluarga dengan keterbatasan akses informasi. [Sumber](https://www.researchgate.net/publication/45276240_Peritonitis_in_children_on_peritoneal_dialysis_in_Cape_Town_South_Africa_Epidemiology_and_risks) | Nutrition: Rekomendasi asupan protein tinggi (1,4–3,0 g/kg/hari) disesuaikan dengan usia anak untuk mengganti kehilangan protein selama dialisis dan mengejar pertumbuhan. Pemantauan nutrisi dilakukan setiap bulan pada bayi dan setiap 3–4 bulan pada anak yang lebih tua. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC7352713/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) | Type of Catheter (Shape): Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Catheter Placement: Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Gastrostomy/Intraperitoneal Device:  | Catheter Orientation:  | Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
-      <c r="AA81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -11064,7 +10979,6 @@
           <t>Housing: Ruangan harus bersih dan bebas dari hewan peliharaan selama prosedur untuk menghindari risiko kontaminasi bakteri Pasteurella atau kerusakan mekanis pada selang. Ketersediaan wastafel untuk mencuci tangan secara benar sangat krusial dalam mengurangi risiko peritonitis. [🔗Sumber 1](https://freseniusmedicalcare.com/content/dam/home-products-education/steps2home-pd/Preventing_Peritonitis.pdf) [🔗Sumber 2](https://spnp-spp.pt/media/rqdpbrom/catheter-related-infections-and-peritonitis-in-pediatric-patients-receiving-peritoneal-dialysis-guideline-for-prevention-and-treatment-2012-1-_compressed-1.pdf) [Sumber 3](https://www.ouh.nhs.uk/media/agxhnni2/85713pdialysis.pdf) [Sumber 4](https://www.satellitehealthcare.com/blog/pets-and-peritoneal-dialysis-absolutely/) | Socioeconomic: Edukasi atau retraining intensif bagi keluarga (caregiver) mengenai prosedur aseptik sangat dianjurkan, terutama bagi keluarga dengan keterbatasan akses informasi. [Sumber](https://www.researchgate.net/publication/45276240_Peritonitis_in_children_on_peritoneal_dialysis_in_Cape_Town_South_Africa_Epidemiology_and_risks) | Nutrition: Rekomendasi asupan protein tinggi (1,4–3,0 g/kg/hari) disesuaikan dengan usia anak untuk mengganti kehilangan protein selama dialisis dan mengejar pertumbuhan. Pemantauan nutrisi dilakukan setiap bulan pada bayi dan setiap 3–4 bulan pada anak yang lebih tua. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC7352713/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) | Type of Catheter (Shape): Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Catheter Placement: Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Gastrostomy/Intraperitoneal Device:  | Catheter Orientation:  | Stunting: Perlu optimalisasi pertumbuhan melalui dukungan nutrisi agresif atau terapi hormon pertumbuhan sesuai saran dokter.</t>
         </is>
       </c>
-      <c r="AA82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -11197,7 +11111,6 @@
           <t>Stunting: Stunting pada anak dialisis bukan hanya disebabkan oleh asupan kalori yang rendah, tetapi juga oleh asidosis metabolik, anemia, osteodistrofi ginjal, dan resistensi terhadap hormon pertumbuhan. Intervensi pertama adalah memastikan kecukupan dialisis dan koreksi parameter metabolik seperti asidosis dan hiperparatiroidisme.Jika pertumbuhan masih belum optimal meskipun parameter metabolik telah terkendali dan asupan nutrisi sudah mencapai target, terapi dengan hormon pertumbuhan manusia rekombinan (rhGH) dapat dipertimbangkan. Selain itu, dukungan nutrisi intensif dan klirens dialisis yang adekuat pada pasien prepubertal dapat mempromosikan pertumbuhan normal tanpa selalu memerlukan rhGH. Pada anak yang mengalami stunting (tinggi badan &lt; persentil ke-2), perhitungan kebutuhan energi dan mikronutrien harus didasarkan pada height-age pasien, bukan chronological age-nya, untuk memberikan dukungan yang sesuai dengan ukuran tubuh aktualnya. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/)</t>
         </is>
       </c>
-      <c r="AA83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -11330,7 +11243,6 @@
           <t>Stunting: Stunting pada anak dialisis bukan hanya disebabkan oleh asupan kalori yang rendah, tetapi juga oleh asidosis metabolik, anemia, osteodistrofi ginjal, dan resistensi terhadap hormon pertumbuhan. Intervensi pertama adalah memastikan kecukupan dialisis dan koreksi parameter metabolik seperti asidosis dan hiperparatiroidisme.Jika pertumbuhan masih belum optimal meskipun parameter metabolik telah terkendali dan asupan nutrisi sudah mencapai target, terapi dengan hormon pertumbuhan manusia rekombinan (rhGH) dapat dipertimbangkan. Selain itu, dukungan nutrisi intensif dan klirens dialisis yang adekuat pada pasien prepubertal dapat mempromosikan pertumbuhan normal tanpa selalu memerlukan rhGH. Pada anak yang mengalami stunting (tinggi badan &lt; persentil ke-2), perhitungan kebutuhan energi dan mikronutrien harus didasarkan pada height-age pasien, bukan chronological age-nya, untuk memberikan dukungan yang sesuai dengan ukuran tubuh aktualnya. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/)</t>
         </is>
       </c>
-      <c r="AA84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -11463,7 +11375,6 @@
           <t>Stunting: Stunting pada anak dialisis bukan hanya disebabkan oleh asupan kalori yang rendah, tetapi juga oleh asidosis metabolik, anemia, osteodistrofi ginjal, dan resistensi terhadap hormon pertumbuhan. Intervensi pertama adalah memastikan kecukupan dialisis dan koreksi parameter metabolik seperti asidosis dan hiperparatiroidisme.Jika pertumbuhan masih belum optimal meskipun parameter metabolik telah terkendali dan asupan nutrisi sudah mencapai target, terapi dengan hormon pertumbuhan manusia rekombinan (rhGH) dapat dipertimbangkan. Selain itu, dukungan nutrisi intensif dan klirens dialisis yang adekuat pada pasien prepubertal dapat mempromosikan pertumbuhan normal tanpa selalu memerlukan rhGH. Pada anak yang mengalami stunting (tinggi badan &lt; persentil ke-2), perhitungan kebutuhan energi dan mikronutrien harus didasarkan pada height-age pasien, bukan chronological age-nya, untuk memberikan dukungan yang sesuai dengan ukuran tubuh aktualnya. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/)</t>
         </is>
       </c>
-      <c r="AA85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -11588,7 +11499,6 @@
       </c>
       <c r="Y86" t="inlineStr"/>
       <c r="Z86" t="inlineStr"/>
-      <c r="AA86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -11713,7 +11623,6 @@
       </c>
       <c r="Y87" t="inlineStr"/>
       <c r="Z87" t="inlineStr"/>
-      <c r="AA87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -11838,7 +11747,6 @@
       </c>
       <c r="Y88" t="inlineStr"/>
       <c r="Z88" t="inlineStr"/>
-      <c r="AA88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -11963,7 +11871,6 @@
       </c>
       <c r="Y89" t="inlineStr"/>
       <c r="Z89" t="inlineStr"/>
-      <c r="AA89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -12088,7 +11995,6 @@
       </c>
       <c r="Y90" t="inlineStr"/>
       <c r="Z90" t="inlineStr"/>
-      <c r="AA90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -12213,7 +12119,6 @@
       </c>
       <c r="Y91" t="inlineStr"/>
       <c r="Z91" t="inlineStr"/>
-      <c r="AA91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -12338,7 +12243,6 @@
       </c>
       <c r="Y92" t="inlineStr"/>
       <c r="Z92" t="inlineStr"/>
-      <c r="AA92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -12467,11 +12371,6 @@
           <t>Peritonitis in ESI: Penggunaan antibiotik topikal secara rutin pada tempat keluar kateter telat terbukti menurunkan angka infeksi. Aplikasi harian salep mupirocin atau gentamicin pada exit-site direkomendasikan untuk menekan kolonisasi Staphylococcus aureus dan Pseudomonas aeruginosa.Pembersihan area secara rutin dengan larutan antiseptik non-iritan (seperti chlorhexidine 0,05% atau sabun antibakteri ringan) juga merupakan bagian standar dari perawatan. Penilaian kondisi exit-site secara objektif menggunakan sistem skor (seperti Skor ISPD yang mencakup pembengkakan, kerak, kemerahan, nyeri, dan sekret) sangat membantu caregiver dalam mendeteksi infeksi secara dini. Immobilisasi kateter dengan menggunakan plester atau perangkat fiksasi sangat krusial karena trauma mekanis pada tempat keluar sering kali menjadi pintu masuk bagi bakteri. Jika ESI terjadi, terapi antibiotik oral atau intraperitoneal harus dimulai segera dan dilanjutkan selama minimal 2 minggu, atau 3 minggu jika disebabkan oleh Pseudomonas. Pengangkatan kateter mungkin diperlukan jika infeksi bersifat refrakter (tidak merespons pengobatan setelah 2 minggu) atau jika infeksi telah menyebar ke terowongan kateter (tunnel infection) yang menyebabkan peritonitis berulang. [Sumber 1](https://ispd.org/wp-content/uploads/2025/09/LI-ET-1.pdf) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC12640025/) [Sumber 3](https://pmc.ncbi.nlm.nih.gov/articles/PMC5033625/) [Sumber 4](https://www.chikd.org/journal/view.php?number=726) [Sumber 5](https://ispd.org/wp-content/uploads/ISPD-Catheter-related-Infection-Recommendations-2023-Update.pdf) [Sumber 6](https://www.bcrenal.ca/resource-gallery/Documents/PD_Procedures-Exit_Site_Care-Post-Operative_PD_Catheter_Insertion.pdf) [Sumber 7](https://davita.com/treatment-options/articles/preventing-catheter-infections-on-peritoneal-dialysis/) [Sumber 8](https://edren.org/ren/handbook/pd-handbook/protocol-for-the-management-of-pd-peritonitis-long-version/)</t>
         </is>
       </c>
-      <c r="AA93" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -12600,11 +12499,6 @@
           <t>Peritonitis in ESI: Penggunaan antibiotik topikal secara rutin pada tempat keluar kateter telat terbukti menurunkan angka infeksi. Aplikasi harian salep mupirocin atau gentamicin pada exit-site direkomendasikan untuk menekan kolonisasi Staphylococcus aureus dan Pseudomonas aeruginosa.Pembersihan area secara rutin dengan larutan antiseptik non-iritan (seperti chlorhexidine 0,05% atau sabun antibakteri ringan) juga merupakan bagian standar dari perawatan. Penilaian kondisi exit-site secara objektif menggunakan sistem skor (seperti Skor ISPD yang mencakup pembengkakan, kerak, kemerahan, nyeri, dan sekret) sangat membantu caregiver dalam mendeteksi infeksi secara dini. Immobilisasi kateter dengan menggunakan plester atau perangkat fiksasi sangat krusial karena trauma mekanis pada tempat keluar sering kali menjadi pintu masuk bagi bakteri. Jika ESI terjadi, terapi antibiotik oral atau intraperitoneal harus dimulai segera dan dilanjutkan selama minimal 2 minggu, atau 3 minggu jika disebabkan oleh Pseudomonas. Pengangkatan kateter mungkin diperlukan jika infeksi bersifat refrakter (tidak merespons pengobatan setelah 2 minggu) atau jika infeksi telah menyebar ke terowongan kateter (tunnel infection) yang menyebabkan peritonitis berulang. [Sumber 1](https://ispd.org/wp-content/uploads/2025/09/LI-ET-1.pdf) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC12640025/) [Sumber 3](https://pmc.ncbi.nlm.nih.gov/articles/PMC5033625/) [Sumber 4](https://www.chikd.org/journal/view.php?number=726) [Sumber 5](https://ispd.org/wp-content/uploads/ISPD-Catheter-related-Infection-Recommendations-2023-Update.pdf) [Sumber 6](https://www.bcrenal.ca/resource-gallery/Documents/PD_Procedures-Exit_Site_Care-Post-Operative_PD_Catheter_Insertion.pdf) [Sumber 7](https://davita.com/treatment-options/articles/preventing-catheter-infections-on-peritoneal-dialysis/) [Sumber 8](https://edren.org/ren/handbook/pd-handbook/protocol-for-the-management-of-pd-peritonitis-long-version/) | Stunting: Stunting pada anak dialisis bukan hanya disebabkan oleh asupan kalori yang rendah, tetapi juga oleh asidosis metabolik, anemia, osteodistrofi ginjal, dan resistensi terhadap hormon pertumbuhan. Intervensi pertama adalah memastikan kecukupan dialisis dan koreksi parameter metabolik seperti asidosis dan hiperparatiroidisme.Jika pertumbuhan masih belum optimal meskipun parameter metabolik telah terkendali dan asupan nutrisi sudah mencapai target, terapi dengan hormon pertumbuhan manusia rekombinan (rhGH) dapat dipertimbangkan. Selain itu, dukungan nutrisi intensif dan klirens dialisis yang adekuat pada pasien prepubertal dapat mempromosikan pertumbuhan normal tanpa selalu memerlukan rhGH. Pada anak yang mengalami stunting (tinggi badan &lt; persentil ke-2), perhitungan kebutuhan energi dan mikronutrien harus didasarkan pada height-age pasien, bukan chronological age-nya, untuk memberikan dukungan yang sesuai dengan ukuran tubuh aktualnya. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/)</t>
         </is>
       </c>
-      <c r="AA94" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -12733,11 +12627,6 @@
           <t>Peritonitis in ESI: Penggunaan antibiotik topikal secara rutin pada tempat keluar kateter telat terbukti menurunkan angka infeksi. Aplikasi harian salep mupirocin atau gentamicin pada exit-site direkomendasikan untuk menekan kolonisasi Staphylococcus aureus dan Pseudomonas aeruginosa.Pembersihan area secara rutin dengan larutan antiseptik non-iritan (seperti chlorhexidine 0,05% atau sabun antibakteri ringan) juga merupakan bagian standar dari perawatan. Penilaian kondisi exit-site secara objektif menggunakan sistem skor (seperti Skor ISPD yang mencakup pembengkakan, kerak, kemerahan, nyeri, dan sekret) sangat membantu caregiver dalam mendeteksi infeksi secara dini. Immobilisasi kateter dengan menggunakan plester atau perangkat fiksasi sangat krusial karena trauma mekanis pada tempat keluar sering kali menjadi pintu masuk bagi bakteri. Jika ESI terjadi, terapi antibiotik oral atau intraperitoneal harus dimulai segera dan dilanjutkan selama minimal 2 minggu, atau 3 minggu jika disebabkan oleh Pseudomonas. Pengangkatan kateter mungkin diperlukan jika infeksi bersifat refrakter (tidak merespons pengobatan setelah 2 minggu) atau jika infeksi telah menyebar ke terowongan kateter (tunnel infection) yang menyebabkan peritonitis berulang. [Sumber 1](https://ispd.org/wp-content/uploads/2025/09/LI-ET-1.pdf) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC12640025/) [Sumber 3](https://pmc.ncbi.nlm.nih.gov/articles/PMC5033625/) [Sumber 4](https://www.chikd.org/journal/view.php?number=726) [Sumber 5](https://ispd.org/wp-content/uploads/ISPD-Catheter-related-Infection-Recommendations-2023-Update.pdf) [Sumber 6](https://www.bcrenal.ca/resource-gallery/Documents/PD_Procedures-Exit_Site_Care-Post-Operative_PD_Catheter_Insertion.pdf) [Sumber 7](https://davita.com/treatment-options/articles/preventing-catheter-infections-on-peritoneal-dialysis/) [Sumber 8](https://edren.org/ren/handbook/pd-handbook/protocol-for-the-management-of-pd-peritonitis-long-version/) | Stunting: Stunting pada anak dialisis bukan hanya disebabkan oleh asupan kalori yang rendah, tetapi juga oleh asidosis metabolik, anemia, osteodistrofi ginjal, dan resistensi terhadap hormon pertumbuhan. Intervensi pertama adalah memastikan kecukupan dialisis dan koreksi parameter metabolik seperti asidosis dan hiperparatiroidisme.Jika pertumbuhan masih belum optimal meskipun parameter metabolik telah terkendali dan asupan nutrisi sudah mencapai target, terapi dengan hormon pertumbuhan manusia rekombinan (rhGH) dapat dipertimbangkan. Selain itu, dukungan nutrisi intensif dan klirens dialisis yang adekuat pada pasien prepubertal dapat mempromosikan pertumbuhan normal tanpa selalu memerlukan rhGH. Pada anak yang mengalami stunting (tinggi badan &lt; persentil ke-2), perhitungan kebutuhan energi dan mikronutrien harus didasarkan pada height-age pasien, bukan chronological age-nya, untuk memberikan dukungan yang sesuai dengan ukuran tubuh aktualnya. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/)</t>
         </is>
       </c>
-      <c r="AA95" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -12866,11 +12755,6 @@
           <t>Peritonitis in ESI: Penggunaan antibiotik topikal secara rutin pada tempat keluar kateter telat terbukti menurunkan angka infeksi. Aplikasi harian salep mupirocin atau gentamicin pada exit-site direkomendasikan untuk menekan kolonisasi Staphylococcus aureus dan Pseudomonas aeruginosa.Pembersihan area secara rutin dengan larutan antiseptik non-iritan (seperti chlorhexidine 0,05% atau sabun antibakteri ringan) juga merupakan bagian standar dari perawatan. Penilaian kondisi exit-site secara objektif menggunakan sistem skor (seperti Skor ISPD yang mencakup pembengkakan, kerak, kemerahan, nyeri, dan sekret) sangat membantu caregiver dalam mendeteksi infeksi secara dini. Immobilisasi kateter dengan menggunakan plester atau perangkat fiksasi sangat krusial karena trauma mekanis pada tempat keluar sering kali menjadi pintu masuk bagi bakteri. Jika ESI terjadi, terapi antibiotik oral atau intraperitoneal harus dimulai segera dan dilanjutkan selama minimal 2 minggu, atau 3 minggu jika disebabkan oleh Pseudomonas. Pengangkatan kateter mungkin diperlukan jika infeksi bersifat refrakter (tidak merespons pengobatan setelah 2 minggu) atau jika infeksi telah menyebar ke terowongan kateter (tunnel infection) yang menyebabkan peritonitis berulang. [Sumber 1](https://ispd.org/wp-content/uploads/2025/09/LI-ET-1.pdf) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC12640025/) [Sumber 3](https://pmc.ncbi.nlm.nih.gov/articles/PMC5033625/) [Sumber 4](https://www.chikd.org/journal/view.php?number=726) [Sumber 5](https://ispd.org/wp-content/uploads/ISPD-Catheter-related-Infection-Recommendations-2023-Update.pdf) [Sumber 6](https://www.bcrenal.ca/resource-gallery/Documents/PD_Procedures-Exit_Site_Care-Post-Operative_PD_Catheter_Insertion.pdf) [Sumber 7](https://davita.com/treatment-options/articles/preventing-catheter-infections-on-peritoneal-dialysis/) [Sumber 8](https://edren.org/ren/handbook/pd-handbook/protocol-for-the-management-of-pd-peritonitis-long-version/) | Type of Catheter (Shape): Perdebatan mengenai efektivitas kateter straight dibandingkan dengan kateter coiled/curled masih berlangsung. Kateter coiled secara teoretis mengurangi nyeri saat pengisian cairan dan meminimalkan trauma pada organ visceral, tetapi beberapa data menunjukkan risiko malposisi yang lebih tinggi dibandingkan tipe lurus pada beberapa kelompok pasien. Di sisi lain, kateter straight lebih mudah ditempatkan pada bayi kecil yang memiliki ruang intra-abdominal terbatas. Secara keseluruhan, pedoman tidak menyatakan superioritas mutlak salah satu bentuk, dan pemilihan sering kali bergantung pada preferensi pusat dialisis dan anatomi pasien. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC9365012/) [Sumber 2](http://ispd.org/wp-content/uploads/7.-Dagmara-Borzych-Duzalka-Peritoneal-Dialysis-Catheters-Outcome-in-Children.-The-IPPN-Data.pdf) [Sumber 3](https://scholarlyexchange.childrensmercy.org/cgi/viewcontent.cgi?article=7522&amp;context=papers) [Sumber 4](https://kidney.wiki/peritoneal-dialysis/pd-access/) | Type of Catheter (Cuff): Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff)untuk populasi anak secara umum. Deep cuff berfungsi untuk menjangkar kateter di otot rektus dan mencegah kebocoran, sementara superficial cuff bertindak sebagai penghalang fisik terhadap migrasi bakteri ke arah rongga peritoneum. Namun, pada neonatus atau bayi dengan dinding perut yang sangat tipis, kateter single-cuff sering kali lebih dipilih untuk mencegah ekstrusi manset ke permukaan kulit. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC10223083/) [Sumber 2](http://ispd.org/wp-content/uploads/7.-Dagmara-Borzych-Duzalka-Peritoneal-Dialysis-Catheters-Outcome-in-Children.-The-IPPN-Data.pdf) [Sumber 3](https://kidney.wiki/peritoneal-dialysis/pd-access/) | Catheter Placement: Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Stunting: Stunting pada anak dialisis bukan hanya disebabkan oleh asupan kalori yang rendah, tetapi juga oleh asidosis metabolik, anemia, osteodistrofi ginjal, dan resistensi terhadap hormon pertumbuhan. Intervensi pertama adalah memastikan kecukupan dialisis dan koreksi parameter metabolik seperti asidosis dan hiperparatiroidisme.Jika pertumbuhan masih belum optimal meskipun parameter metabolik telah terkendali dan asupan nutrisi sudah mencapai target, terapi dengan hormon pertumbuhan manusia rekombinan (rhGH) dapat dipertimbangkan. Selain itu, dukungan nutrisi intensif dan klirens dialisis yang adekuat pada pasien prepubertal dapat mempromosikan pertumbuhan normal tanpa selalu memerlukan rhGH. Pada anak yang mengalami stunting (tinggi badan &lt; persentil ke-2), perhitungan kebutuhan energi dan mikronutrien harus didasarkan pada height-age pasien, bukan chronological age-nya, untuk memberikan dukungan yang sesuai dengan ukuran tubuh aktualnya. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/)</t>
         </is>
       </c>
-      <c r="AA96" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -12999,11 +12883,6 @@
           <t>Peritonitis in ESI: Penggunaan antibiotik topikal secara rutin pada tempat keluar kateter telat terbukti menurunkan angka infeksi. Aplikasi harian salep mupirocin atau gentamicin pada exit-site direkomendasikan untuk menekan kolonisasi Staphylococcus aureus dan Pseudomonas aeruginosa.Pembersihan area secara rutin dengan larutan antiseptik non-iritan (seperti chlorhexidine 0,05% atau sabun antibakteri ringan) juga merupakan bagian standar dari perawatan. Penilaian kondisi exit-site secara objektif menggunakan sistem skor (seperti Skor ISPD yang mencakup pembengkakan, kerak, kemerahan, nyeri, dan sekret) sangat membantu caregiver dalam mendeteksi infeksi secara dini. Immobilisasi kateter dengan menggunakan plester atau perangkat fiksasi sangat krusial karena trauma mekanis pada tempat keluar sering kali menjadi pintu masuk bagi bakteri. Jika ESI terjadi, terapi antibiotik oral atau intraperitoneal harus dimulai segera dan dilanjutkan selama minimal 2 minggu, atau 3 minggu jika disebabkan oleh Pseudomonas. Pengangkatan kateter mungkin diperlukan jika infeksi bersifat refrakter (tidak merespons pengobatan setelah 2 minggu) atau jika infeksi telah menyebar ke terowongan kateter (tunnel infection) yang menyebabkan peritonitis berulang. [Sumber 1](https://ispd.org/wp-content/uploads/2025/09/LI-ET-1.pdf) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC12640025/) [Sumber 3](https://pmc.ncbi.nlm.nih.gov/articles/PMC5033625/) [Sumber 4](https://www.chikd.org/journal/view.php?number=726) [Sumber 5](https://ispd.org/wp-content/uploads/ISPD-Catheter-related-Infection-Recommendations-2023-Update.pdf) [Sumber 6](https://www.bcrenal.ca/resource-gallery/Documents/PD_Procedures-Exit_Site_Care-Post-Operative_PD_Catheter_Insertion.pdf) [Sumber 7](https://davita.com/treatment-options/articles/preventing-catheter-infections-on-peritoneal-dialysis/) [Sumber 8](https://edren.org/ren/handbook/pd-handbook/protocol-for-the-management-of-pd-peritonitis-long-version/) | Type of Catheter (Shape): Perdebatan mengenai efektivitas kateter straight dibandingkan dengan kateter coiled/curled masih berlangsung. Kateter coiled secara teoretis mengurangi nyeri saat pengisian cairan dan meminimalkan trauma pada organ visceral, tetapi beberapa data menunjukkan risiko malposisi yang lebih tinggi dibandingkan tipe lurus pada beberapa kelompok pasien. Di sisi lain, kateter straight lebih mudah ditempatkan pada bayi kecil yang memiliki ruang intra-abdominal terbatas. Secara keseluruhan, pedoman tidak menyatakan superioritas mutlak salah satu bentuk, dan pemilihan sering kali bergantung pada preferensi pusat dialisis dan anatomi pasien. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC9365012/) [Sumber 2](http://ispd.org/wp-content/uploads/7.-Dagmara-Borzych-Duzalka-Peritoneal-Dialysis-Catheters-Outcome-in-Children.-The-IPPN-Data.pdf) [Sumber 3](https://scholarlyexchange.childrensmercy.org/cgi/viewcontent.cgi?article=7522&amp;context=papers) [Sumber 4](https://kidney.wiki/peritoneal-dialysis/pd-access/) | Type of Catheter (Cuff): Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff)untuk populasi anak secara umum. Deep cuff berfungsi untuk menjangkar kateter di otot rektus dan mencegah kebocoran, sementara superficial cuff bertindak sebagai penghalang fisik terhadap migrasi bakteri ke arah rongga peritoneum. Namun, pada neonatus atau bayi dengan dinding perut yang sangat tipis, kateter single-cuff sering kali lebih dipilih untuk mencegah ekstrusi manset ke permukaan kulit. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC10223083/) [Sumber 2](http://ispd.org/wp-content/uploads/7.-Dagmara-Borzych-Duzalka-Peritoneal-Dialysis-Catheters-Outcome-in-Children.-The-IPPN-Data.pdf) [Sumber 3](https://kidney.wiki/peritoneal-dialysis/pd-access/) | Catheter Placement: Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Stunting: Stunting pada anak dialisis bukan hanya disebabkan oleh asupan kalori yang rendah, tetapi juga oleh asidosis metabolik, anemia, osteodistrofi ginjal, dan resistensi terhadap hormon pertumbuhan. Intervensi pertama adalah memastikan kecukupan dialisis dan koreksi parameter metabolik seperti asidosis dan hiperparatiroidisme.Jika pertumbuhan masih belum optimal meskipun parameter metabolik telah terkendali dan asupan nutrisi sudah mencapai target, terapi dengan hormon pertumbuhan manusia rekombinan (rhGH) dapat dipertimbangkan. Selain itu, dukungan nutrisi intensif dan klirens dialisis yang adekuat pada pasien prepubertal dapat mempromosikan pertumbuhan normal tanpa selalu memerlukan rhGH. Pada anak yang mengalami stunting (tinggi badan &lt; persentil ke-2), perhitungan kebutuhan energi dan mikronutrien harus didasarkan pada height-age pasien, bukan chronological age-nya, untuk memberikan dukungan yang sesuai dengan ukuran tubuh aktualnya. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/)</t>
         </is>
       </c>
-      <c r="AA97" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -13132,11 +13011,6 @@
           <t>Peritonitis in ESI: Penggunaan antibiotik topikal secara rutin pada tempat keluar kateter telat terbukti menurunkan angka infeksi. Aplikasi harian salep mupirocin atau gentamicin pada exit-site direkomendasikan untuk menekan kolonisasi Staphylococcus aureus dan Pseudomonas aeruginosa.Pembersihan area secara rutin dengan larutan antiseptik non-iritan (seperti chlorhexidine 0,05% atau sabun antibakteri ringan) juga merupakan bagian standar dari perawatan. Penilaian kondisi exit-site secara objektif menggunakan sistem skor (seperti Skor ISPD yang mencakup pembengkakan, kerak, kemerahan, nyeri, dan sekret) sangat membantu caregiver dalam mendeteksi infeksi secara dini. Immobilisasi kateter dengan menggunakan plester atau perangkat fiksasi sangat krusial karena trauma mekanis pada tempat keluar sering kali menjadi pintu masuk bagi bakteri. Jika ESI terjadi, terapi antibiotik oral atau intraperitoneal harus dimulai segera dan dilanjutkan selama minimal 2 minggu, atau 3 minggu jika disebabkan oleh Pseudomonas. Pengangkatan kateter mungkin diperlukan jika infeksi bersifat refrakter (tidak merespons pengobatan setelah 2 minggu) atau jika infeksi telah menyebar ke terowongan kateter (tunnel infection) yang menyebabkan peritonitis berulang. [Sumber 1](https://ispd.org/wp-content/uploads/2025/09/LI-ET-1.pdf) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC12640025/) [Sumber 3](https://pmc.ncbi.nlm.nih.gov/articles/PMC5033625/) [Sumber 4](https://www.chikd.org/journal/view.php?number=726) [Sumber 5](https://ispd.org/wp-content/uploads/ISPD-Catheter-related-Infection-Recommendations-2023-Update.pdf) [Sumber 6](https://www.bcrenal.ca/resource-gallery/Documents/PD_Procedures-Exit_Site_Care-Post-Operative_PD_Catheter_Insertion.pdf) [Sumber 7](https://davita.com/treatment-options/articles/preventing-catheter-infections-on-peritoneal-dialysis/) [Sumber 8](https://edren.org/ren/handbook/pd-handbook/protocol-for-the-management-of-pd-peritonitis-long-version/) | Type of Catheter (Shape): Perdebatan mengenai efektivitas kateter straight dibandingkan dengan kateter coiled/curled masih berlangsung. Kateter coiled secara teoretis mengurangi nyeri saat pengisian cairan dan meminimalkan trauma pada organ visceral, tetapi beberapa data menunjukkan risiko malposisi yang lebih tinggi dibandingkan tipe lurus pada beberapa kelompok pasien. Di sisi lain, kateter straight lebih mudah ditempatkan pada bayi kecil yang memiliki ruang intra-abdominal terbatas. Secara keseluruhan, pedoman tidak menyatakan superioritas mutlak salah satu bentuk, dan pemilihan sering kali bergantung pada preferensi pusat dialisis dan anatomi pasien. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC9365012/) [Sumber 2](http://ispd.org/wp-content/uploads/7.-Dagmara-Borzych-Duzalka-Peritoneal-Dialysis-Catheters-Outcome-in-Children.-The-IPPN-Data.pdf) [Sumber 3](https://scholarlyexchange.childrensmercy.org/cgi/viewcontent.cgi?article=7522&amp;context=papers) [Sumber 4](https://kidney.wiki/peritoneal-dialysis/pd-access/) | Type of Catheter (Cuff): Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff)untuk populasi anak secara umum. Deep cuff berfungsi untuk menjangkar kateter di otot rektus dan mencegah kebocoran, sementara superficial cuff bertindak sebagai penghalang fisik terhadap migrasi bakteri ke arah rongga peritoneum. Namun, pada neonatus atau bayi dengan dinding perut yang sangat tipis, kateter single-cuff sering kali lebih dipilih untuk mencegah ekstrusi manset ke permukaan kulit. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC10223083/) [Sumber 2](http://ispd.org/wp-content/uploads/7.-Dagmara-Borzych-Duzalka-Peritoneal-Dialysis-Catheters-Outcome-in-Children.-The-IPPN-Data.pdf) [Sumber 3](https://kidney.wiki/peritoneal-dialysis/pd-access/) | Catheter Placement: Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Starting PD &lt;2 weeks after catheter placement: Waktu antara pemasangan kateter dan dimulainya dialisis (break-in-period) merupakan faktor penting untuk mencegah komplikasi. Masa penyembuhan minimal 2 minggu sebelum dialysis dimulai. Namun, dalam kondisi klinis tertentu di mana pasien membutuhkan dialisis segera, urgent-start PD (dimulai dalam &lt;14 hari atau bahkan &lt;48 jam) menjadi alternatif yang baik untuk menghindari penggunakan kateter hemodialysis sementara. Pasien dengan break-in-period &lt; 7 hari memiliki risiko yang lebih tinggi terhadap komplikasi awal seperti kebocoran dialisat dan malposisi kateter. Namun, risiko tersebut tidak berkorelasi dengan penurunan kelangsungan hidup atau peningkatan risiko peritonitis jika dilakukan dengan protokol yang tepat. Pada kondisi urgent-start, risiko kebocoran dimitigasi dengan menggunakan volume pengisian rendah (10-20 ml/kg) dan posisi pasien supine untuk mengurangi tekanan intra-abdominal.[Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC3923692/) [Sumber 2](https://journals.plos.org/plosone/article?id=10.1371/journal.pone.0206426) [Sumber 3](https://www.sages.org/publications/guidelines/peritoneal-dialysis-access-guideline-update-2023/) [Sumber 4](https://www.frontiersin.org/journals/endocrinology/articles/10.3389/fendo.2022.936573/full) [Sumber 5](https://scholarlyexchange.childrensmercy.org/cgi/viewcontent.cgi?article=7522&amp;context=papers) [Sumber 6](https://pubmed.ncbi.nlm.nih.gov/33523772/) [Sumber 7](https://www.bcrenal.ca/resource-gallery/Documents/PD_Procedures-Exit_Site_Care-Post-Operative_PD_Catheter_Insertion.pdf) | Stunting: Stunting pada anak dialisis bukan hanya disebabkan oleh asupan kalori yang rendah, tetapi juga oleh asidosis metabolik, anemia, osteodistrofi ginjal, dan resistensi terhadap hormon pertumbuhan. Intervensi pertama adalah memastikan kecukupan dialisis dan koreksi parameter metabolik seperti asidosis dan hiperparatiroidisme.Jika pertumbuhan masih belum optimal meskipun parameter metabolik telah terkendali dan asupan nutrisi sudah mencapai target, terapi dengan hormon pertumbuhan manusia rekombinan (rhGH) dapat dipertimbangkan. Selain itu, dukungan nutrisi intensif dan klirens dialisis yang adekuat pada pasien prepubertal dapat mempromosikan pertumbuhan normal tanpa selalu memerlukan rhGH. Pada anak yang mengalami stunting (tinggi badan &lt; persentil ke-2), perhitungan kebutuhan energi dan mikronutrien harus didasarkan pada height-age pasien, bukan chronological age-nya, untuk memberikan dukungan yang sesuai dengan ukuran tubuh aktualnya. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/)</t>
         </is>
       </c>
-      <c r="AA98" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -13265,11 +13139,6 @@
           <t>Peritonitis in ESI: Penggunaan antibiotik topikal secara rutin pada tempat keluar kateter telat terbukti menurunkan angka infeksi. Aplikasi harian salep mupirocin atau gentamicin pada exit-site direkomendasikan untuk menekan kolonisasi Staphylococcus aureus dan Pseudomonas aeruginosa.Pembersihan area secara rutin dengan larutan antiseptik non-iritan (seperti chlorhexidine 0,05% atau sabun antibakteri ringan) juga merupakan bagian standar dari perawatan. Penilaian kondisi exit-site secara objektif menggunakan sistem skor (seperti Skor ISPD yang mencakup pembengkakan, kerak, kemerahan, nyeri, dan sekret) sangat membantu caregiver dalam mendeteksi infeksi secara dini. Immobilisasi kateter dengan menggunakan plester atau perangkat fiksasi sangat krusial karena trauma mekanis pada tempat keluar sering kali menjadi pintu masuk bagi bakteri. Jika ESI terjadi, terapi antibiotik oral atau intraperitoneal harus dimulai segera dan dilanjutkan selama minimal 2 minggu, atau 3 minggu jika disebabkan oleh Pseudomonas. Pengangkatan kateter mungkin diperlukan jika infeksi bersifat refrakter (tidak merespons pengobatan setelah 2 minggu) atau jika infeksi telah menyebar ke terowongan kateter (tunnel infection) yang menyebabkan peritonitis berulang. [Sumber 1](https://ispd.org/wp-content/uploads/2025/09/LI-ET-1.pdf) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC12640025/) [Sumber 3](https://pmc.ncbi.nlm.nih.gov/articles/PMC5033625/) [Sumber 4](https://www.chikd.org/journal/view.php?number=726) [Sumber 5](https://ispd.org/wp-content/uploads/ISPD-Catheter-related-Infection-Recommendations-2023-Update.pdf) [Sumber 6](https://www.bcrenal.ca/resource-gallery/Documents/PD_Procedures-Exit_Site_Care-Post-Operative_PD_Catheter_Insertion.pdf) [Sumber 7](https://davita.com/treatment-options/articles/preventing-catheter-infections-on-peritoneal-dialysis/) [Sumber 8](https://edren.org/ren/handbook/pd-handbook/protocol-for-the-management-of-pd-peritonitis-long-version/) | Type of Catheter (Shape): Perdebatan mengenai efektivitas kateter straight dibandingkan dengan kateter coiled/curled masih berlangsung. Kateter coiled secara teoretis mengurangi nyeri saat pengisian cairan dan meminimalkan trauma pada organ visceral, tetapi beberapa data menunjukkan risiko malposisi yang lebih tinggi dibandingkan tipe lurus pada beberapa kelompok pasien. Di sisi lain, kateter straight lebih mudah ditempatkan pada bayi kecil yang memiliki ruang intra-abdominal terbatas. Secara keseluruhan, pedoman tidak menyatakan superioritas mutlak salah satu bentuk, dan pemilihan sering kali bergantung pada preferensi pusat dialisis dan anatomi pasien. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC9365012/) [Sumber 2](http://ispd.org/wp-content/uploads/7.-Dagmara-Borzych-Duzalka-Peritoneal-Dialysis-Catheters-Outcome-in-Children.-The-IPPN-Data.pdf) [Sumber 3](https://scholarlyexchange.childrensmercy.org/cgi/viewcontent.cgi?article=7522&amp;context=papers) [Sumber 4](https://kidney.wiki/peritoneal-dialysis/pd-access/) | Type of Catheter (Cuff): Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff)untuk populasi anak secara umum. Deep cuff berfungsi untuk menjangkar kateter di otot rektus dan mencegah kebocoran, sementara superficial cuff bertindak sebagai penghalang fisik terhadap migrasi bakteri ke arah rongga peritoneum. Namun, pada neonatus atau bayi dengan dinding perut yang sangat tipis, kateter single-cuff sering kali lebih dipilih untuk mencegah ekstrusi manset ke permukaan kulit. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC10223083/) [Sumber 2](http://ispd.org/wp-content/uploads/7.-Dagmara-Borzych-Duzalka-Peritoneal-Dialysis-Catheters-Outcome-in-Children.-The-IPPN-Data.pdf) [Sumber 3](https://kidney.wiki/peritoneal-dialysis/pd-access/) | Catheter Placement: Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff untuk mencegah migrasi bakteri ke rongga perut. Letak exit site harus menghadap ke bawah atau ke samping (bukan ke atas) untuk mencegah masuknya air atau kotoran. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/37232412/) [Sumber 2](https://journals.eco-vector.com/2075-3594/article/view/637454) | Starting PD &lt;2 weeks after catheter placement: Waktu antara pemasangan kateter dan dimulainya dialisis (break-in-period) merupakan faktor penting untuk mencegah komplikasi. Masa penyembuhan minimal 2 minggu sebelum dialysis dimulai. Namun, dalam kondisi klinis tertentu di mana pasien membutuhkan dialisis segera, urgent-start PD (dimulai dalam &lt;14 hari atau bahkan &lt;48 jam) menjadi alternatif yang baik untuk menghindari penggunakan kateter hemodialysis sementara. Pasien dengan break-in-period &lt; 7 hari memiliki risiko yang lebih tinggi terhadap komplikasi awal seperti kebocoran dialisat dan malposisi kateter. Namun, risiko tersebut tidak berkorelasi dengan penurunan kelangsungan hidup atau peningkatan risiko peritonitis jika dilakukan dengan protokol yang tepat. Pada kondisi urgent-start, risiko kebocoran dimitigasi dengan menggunakan volume pengisian rendah (10-20 ml/kg) dan posisi pasien supine untuk mengurangi tekanan intra-abdominal.[Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC3923692/) [Sumber 2](https://journals.plos.org/plosone/article?id=10.1371/journal.pone.0206426) [Sumber 3](https://www.sages.org/publications/guidelines/peritoneal-dialysis-access-guideline-update-2023/) [Sumber 4](https://www.frontiersin.org/journals/endocrinology/articles/10.3389/fendo.2022.936573/full) [Sumber 5](https://scholarlyexchange.childrensmercy.org/cgi/viewcontent.cgi?article=7522&amp;context=papers) [Sumber 6](https://pubmed.ncbi.nlm.nih.gov/33523772/) [Sumber 7](https://www.bcrenal.ca/resource-gallery/Documents/PD_Procedures-Exit_Site_Care-Post-Operative_PD_Catheter_Insertion.pdf) | Stunting: Stunting pada anak dialisis bukan hanya disebabkan oleh asupan kalori yang rendah, tetapi juga oleh asidosis metabolik, anemia, osteodistrofi ginjal, dan resistensi terhadap hormon pertumbuhan. Intervensi pertama adalah memastikan kecukupan dialisis dan koreksi parameter metabolik seperti asidosis dan hiperparatiroidisme.Jika pertumbuhan masih belum optimal meskipun parameter metabolik telah terkendali dan asupan nutrisi sudah mencapai target, terapi dengan hormon pertumbuhan manusia rekombinan (rhGH) dapat dipertimbangkan. Selain itu, dukungan nutrisi intensif dan klirens dialisis yang adekuat pada pasien prepubertal dapat mempromosikan pertumbuhan normal tanpa selalu memerlukan rhGH. Pada anak yang mengalami stunting (tinggi badan &lt; persentil ke-2), perhitungan kebutuhan energi dan mikronutrien harus didasarkan pada height-age pasien, bukan chronological age-nya, untuk memberikan dukungan yang sesuai dengan ukuran tubuh aktualnya. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/)</t>
         </is>
       </c>
-      <c r="AA99" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -13390,11 +13259,6 @@
       </c>
       <c r="Y100" t="inlineStr"/>
       <c r="Z100" t="inlineStr"/>
-      <c r="AA100" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -13523,11 +13387,6 @@
           <t>Catheter Orientation: Posisi atau arah lubang keluar kateter (exit site) sangat memengaruhi risiko terjadinya infeksi. Data multisentrik dari SCOPE Collaborative menunjukkan bahwa orientasi kateter yang menghadap ke atas (Upward) dikaitkan dengan peningkatan risiko peritonitis hingga 4.2 kali lipat (Rate Ratio: 4.2; 95% CI: 1.49–11.89) dibandingkan orientasi lainnya. Secara anatomis, lubang keluar yang menghadap ke atas menciptakan bentuk cekungan yang dapat menampung keringat, air mandi, dan kotoran. Akibat gaya gravitasi, bakteri yang terkumpul di area ini akan mengendap dan bermigrasi ke dalam terowongan kateter. Oleh karena itu, lubang keluar kateter harus selalu diarahkan ke bawah (Downward) atau ke samping (Lateral) untuk mencegah penumpukan bakteri secara alami. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC5012476/) [Sumber 2](https://openurologyandnephrologyjournal.com/VOLUME/5/PAGE/4/) [Sumber 3](https://kidney.wiki/peritoneal-dialysis/pd-access/)</t>
         </is>
       </c>
-      <c r="AA101" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -13656,11 +13515,6 @@
           <t>Catheter Orientation: Posisi atau arah lubang keluar kateter (exit site) sangat memengaruhi risiko terjadinya infeksi. Data multisentrik dari SCOPE Collaborative menunjukkan bahwa orientasi kateter yang menghadap ke atas (Upward) dikaitkan dengan peningkatan risiko peritonitis hingga 4.2 kali lipat (Rate Ratio: 4.2; 95% CI: 1.49–11.89) dibandingkan orientasi lainnya. Secara anatomis, lubang keluar yang menghadap ke atas menciptakan bentuk cekungan yang dapat menampung keringat, air mandi, dan kotoran. Akibat gaya gravitasi, bakteri yang terkumpul di area ini akan mengendap dan bermigrasi ke dalam terowongan kateter. Oleh karena itu, lubang keluar kateter harus selalu diarahkan ke bawah (Downward) atau ke samping (Lateral) untuk mencegah penumpukan bakteri secara alami. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC5012476/) [Sumber 2](https://openurologyandnephrologyjournal.com/VOLUME/5/PAGE/4/) [Sumber 3](https://kidney.wiki/peritoneal-dialysis/pd-access/)</t>
         </is>
       </c>
-      <c r="AA102" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -13789,11 +13643,6 @@
           <t>Catheter Orientation: Posisi atau arah lubang keluar kateter (exit site) sangat memengaruhi risiko terjadinya infeksi. Data multisentrik dari SCOPE Collaborative menunjukkan bahwa orientasi kateter yang menghadap ke atas (Upward) dikaitkan dengan peningkatan risiko peritonitis hingga 4.2 kali lipat (Rate Ratio: 4.2; 95% CI: 1.49–11.89) dibandingkan orientasi lainnya. Secara anatomis, lubang keluar yang menghadap ke atas menciptakan bentuk cekungan yang dapat menampung keringat, air mandi, dan kotoran. Akibat gaya gravitasi, bakteri yang terkumpul di area ini akan mengendap dan bermigrasi ke dalam terowongan kateter. Oleh karena itu, lubang keluar kateter harus selalu diarahkan ke bawah (Downward) atau ke samping (Lateral) untuk mencegah penumpukan bakteri secara alami. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC5012476/) [Sumber 2](https://openurologyandnephrologyjournal.com/VOLUME/5/PAGE/4/) [Sumber 3](https://kidney.wiki/peritoneal-dialysis/pd-access/)</t>
         </is>
       </c>
-      <c r="AA103" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -13922,9 +13771,2964 @@
           <t>Catheter Placement: Pedoman klinis terbaru dari Society of American Gastrointestinal and Endoscopic Surgeons (SAGES) menyarankan penggunaan teknik laparoskopi tingkat lanjut (Laparoscopic) dibandingkan teknik bedah terbuka (Open) untuk pemasangan kateter pada populasi pediatrik. Laparoscopic menawarkan akurasi catheter placement yang jauh lebih tinggi di dalam rongga abdomen karena visualisasi langsung, serta meminimalkan trauma mekanis pada jaringan perut. Lebih lanjut, Laparoscopic memungkinkan dokter untuk melakukan prosedur profilaksis penting seperti omentektomi atau omentopeksi untuk meminimalkan risiko omental wrapping (penyumbatan kateter oleh omentum), yang merupakan salah satu penyebab utama kegagalan mekanis kateter pada anak-anak. Laparoscopic juga terbukti mempermudah penyelamatan (salvage) jika terjadi malposisi atau disfungsi kateter tanpa harus melakukan pembedahan ulang yang invasif. [Sumber 1](https://www.sages.org/publications/guidelines/peritoneal-dialysis-access-guideline-update-2023/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC10223083/) [[3]](https://kidney.wiki/peritoneal-dialysis/pd-access/) | Catheter Orientation: Posisi atau arah lubang keluar kateter (exit site) sangat memengaruhi risiko terjadinya infeksi. Data multisentrik dari SCOPE Collaborative menunjukkan bahwa orientasi kateter yang menghadap ke atas (Upward) dikaitkan dengan peningkatan risiko peritonitis hingga 4.2 kali lipat (Rate Ratio: 4.2; 95% CI: 1.49–11.89) dibandingkan orientasi lainnya. Secara anatomis, lubang keluar yang menghadap ke atas menciptakan bentuk cekungan yang dapat menampung keringat, air mandi, dan kotoran. Akibat gaya gravitasi, bakteri yang terkumpul di area ini akan mengendap dan bermigrasi ke dalam terowongan kateter. Oleh karena itu, lubang keluar kateter harus selalu diarahkan ke bawah (Downward) atau ke samping (Lateral) untuk mencegah penumpukan bakteri secara alami. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC5012476/) [Sumber 2](https://openurologyandnephrologyjournal.com/VOLUME/5/PAGE/4/) [Sumber 3](https://kidney.wiki/peritoneal-dialysis/pd-access/)</t>
         </is>
       </c>
-      <c r="AA104" t="inlineStr">
-        <is>
-          <t>No</t>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>2026-05-19 12:39:57</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>18F27E0F</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>&gt;2 yo</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>&lt;12 mo</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>Good service</t>
+        </is>
+      </c>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="J105" t="inlineStr">
+        <is>
+          <t>Studies</t>
+        </is>
+      </c>
+      <c r="K105" t="inlineStr">
+        <is>
+          <t>No ESI</t>
+        </is>
+      </c>
+      <c r="L105" t="inlineStr">
+        <is>
+          <t>Normal Nutrition</t>
+        </is>
+      </c>
+      <c r="M105" t="inlineStr">
+        <is>
+          <t>Glomerular</t>
+        </is>
+      </c>
+      <c r="N105" t="inlineStr">
+        <is>
+          <t>Coiled/swan neck</t>
+        </is>
+      </c>
+      <c r="O105" t="inlineStr">
+        <is>
+          <t>Double</t>
+        </is>
+      </c>
+      <c r="P105" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="Q105" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R105" t="inlineStr">
+        <is>
+          <t>Patients</t>
+        </is>
+      </c>
+      <c r="S105" t="inlineStr"/>
+      <c r="T105" t="inlineStr">
+        <is>
+          <t>Lateral/downward</t>
+        </is>
+      </c>
+      <c r="U105" t="inlineStr">
+        <is>
+          <t>No stunting</t>
+        </is>
+      </c>
+      <c r="V105" t="inlineStr"/>
+      <c r="W105" t="inlineStr"/>
+      <c r="X105" t="inlineStr"/>
+      <c r="Y105" t="inlineStr"/>
+      <c r="Z105" t="inlineStr"/>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>2026-05-19 12:40:15</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>18F27E0F</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>&lt;2 yo</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>&lt;12 mo</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>Good service</t>
+        </is>
+      </c>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="J106" t="inlineStr">
+        <is>
+          <t>Studies</t>
+        </is>
+      </c>
+      <c r="K106" t="inlineStr">
+        <is>
+          <t>No ESI</t>
+        </is>
+      </c>
+      <c r="L106" t="inlineStr">
+        <is>
+          <t>Normal Nutrition</t>
+        </is>
+      </c>
+      <c r="M106" t="inlineStr">
+        <is>
+          <t>Glomerular</t>
+        </is>
+      </c>
+      <c r="N106" t="inlineStr">
+        <is>
+          <t>Coiled/swan neck</t>
+        </is>
+      </c>
+      <c r="O106" t="inlineStr">
+        <is>
+          <t>Double</t>
+        </is>
+      </c>
+      <c r="P106" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="Q106" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R106" t="inlineStr">
+        <is>
+          <t>Patients</t>
+        </is>
+      </c>
+      <c r="S106" t="inlineStr"/>
+      <c r="T106" t="inlineStr">
+        <is>
+          <t>Lateral/downward</t>
+        </is>
+      </c>
+      <c r="U106" t="inlineStr">
+        <is>
+          <t>No stunting</t>
+        </is>
+      </c>
+      <c r="V106" t="inlineStr"/>
+      <c r="W106" t="inlineStr"/>
+      <c r="X106" t="inlineStr"/>
+      <c r="Y106" t="inlineStr">
+        <is>
+          <t>Age*, Gender</t>
+        </is>
+      </c>
+      <c r="Z106" t="inlineStr"/>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>2026-05-19 12:40:34</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>18F27E0F</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>&lt;2 yo</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>&lt;12 mo</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>Good service</t>
+        </is>
+      </c>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="J107" t="inlineStr">
+        <is>
+          <t>Studies</t>
+        </is>
+      </c>
+      <c r="K107" t="inlineStr">
+        <is>
+          <t>No ESI</t>
+        </is>
+      </c>
+      <c r="L107" t="inlineStr">
+        <is>
+          <t>Poor nutrition</t>
+        </is>
+      </c>
+      <c r="M107" t="inlineStr">
+        <is>
+          <t>Glomerular</t>
+        </is>
+      </c>
+      <c r="N107" t="inlineStr">
+        <is>
+          <t>Coiled/swan neck</t>
+        </is>
+      </c>
+      <c r="O107" t="inlineStr">
+        <is>
+          <t>Double</t>
+        </is>
+      </c>
+      <c r="P107" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="Q107" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R107" t="inlineStr">
+        <is>
+          <t>Patients</t>
+        </is>
+      </c>
+      <c r="S107" t="inlineStr"/>
+      <c r="T107" t="inlineStr">
+        <is>
+          <t>Lateral/downward</t>
+        </is>
+      </c>
+      <c r="U107" t="inlineStr">
+        <is>
+          <t>No stunting</t>
+        </is>
+      </c>
+      <c r="V107" t="inlineStr"/>
+      <c r="W107" t="inlineStr"/>
+      <c r="X107" t="inlineStr"/>
+      <c r="Y107" t="inlineStr">
+        <is>
+          <t>Age*, Gender, Nutrition</t>
+        </is>
+      </c>
+      <c r="Z107" t="inlineStr">
+        <is>
+          <t>Nutrition: Malnutrisi protein-kalori (cachexia) adalah masalah umum pada anak yang menjalani PD. Manajemen nutrisi bertujuan untuk mengejar pertumbuhan dan mengganti hilangnya protein serta asam amino ke dalam cairan dialysis.Penilaian status nutrisi harus dilakukan secara berkala, minimal setiap bulan pada bayi dan 3-4 bulan pada anak yang lebih tua, menggunakan parameter antropometri (berat badan, tinggi badan, lingkar kepala), biokimia (albumin urea), dan analisis bioimpedansi jika tersedia. Penanganannya juga harus multidisiplin dan mencakup memastikan asupan energi dan protein yang adekuat; kontrol metabolik yang optimal, dengan koreksi asidosis, anemia, dan hiperparatiroidisme; dosis dialisis yang optimal (atau setidaknya adekuat); dan, jika perlu, pemberian obat-obatan tertentu seperti hormon pertumbuhan manusia rekombinan. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/)</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>2026-05-19 12:40:45</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>18F27E0F</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>&lt;2 yo</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>&lt;12 mo</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>Good service</t>
+        </is>
+      </c>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>Studies</t>
+        </is>
+      </c>
+      <c r="K108" t="inlineStr">
+        <is>
+          <t>No ESI</t>
+        </is>
+      </c>
+      <c r="L108" t="inlineStr">
+        <is>
+          <t>Poor nutrition</t>
+        </is>
+      </c>
+      <c r="M108" t="inlineStr">
+        <is>
+          <t>Glomerular</t>
+        </is>
+      </c>
+      <c r="N108" t="inlineStr">
+        <is>
+          <t>Coiled/swan neck</t>
+        </is>
+      </c>
+      <c r="O108" t="inlineStr">
+        <is>
+          <t>Double</t>
+        </is>
+      </c>
+      <c r="P108" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="Q108" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R108" t="inlineStr">
+        <is>
+          <t>Patients</t>
+        </is>
+      </c>
+      <c r="S108" t="inlineStr"/>
+      <c r="T108" t="inlineStr">
+        <is>
+          <t>Lateral/downward</t>
+        </is>
+      </c>
+      <c r="U108" t="inlineStr">
+        <is>
+          <t>Stunting</t>
+        </is>
+      </c>
+      <c r="V108" t="inlineStr"/>
+      <c r="W108" t="inlineStr"/>
+      <c r="X108" t="inlineStr"/>
+      <c r="Y108" t="inlineStr">
+        <is>
+          <t>Age*, Gender, Nutrition, Stunting</t>
+        </is>
+      </c>
+      <c r="Z108" t="inlineStr">
+        <is>
+          <t>Nutrition: Malnutrisi protein-kalori (cachexia) adalah masalah umum pada anak yang menjalani PD. Manajemen nutrisi bertujuan untuk mengejar pertumbuhan dan mengganti hilangnya protein serta asam amino ke dalam cairan dialysis.Penilaian status nutrisi harus dilakukan secara berkala, minimal setiap bulan pada bayi dan 3-4 bulan pada anak yang lebih tua, menggunakan parameter antropometri (berat badan, tinggi badan, lingkar kepala), biokimia (albumin urea), dan analisis bioimpedansi jika tersedia. Penanganannya juga harus multidisiplin dan mencakup memastikan asupan energi dan protein yang adekuat; kontrol metabolik yang optimal, dengan koreksi asidosis, anemia, dan hiperparatiroidisme; dosis dialisis yang optimal (atau setidaknya adekuat); dan, jika perlu, pemberian obat-obatan tertentu seperti hormon pertumbuhan manusia rekombinan. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) | Stunting: Stunting pada anak dialisis bukan hanya disebabkan oleh asupan kalori yang rendah, tetapi juga oleh asidosis metabolik, anemia, osteodistrofi ginjal, dan resistensi terhadap hormon pertumbuhan. Intervensi pertama adalah memastikan kecukupan dialisis dan koreksi parameter metabolik seperti asidosis dan hiperparatiroidisme.Jika pertumbuhan masih belum optimal meskipun parameter metabolik telah terkendali dan asupan nutrisi sudah mencapai target, terapi dengan hormon pertumbuhan manusia rekombinan (rhGH) dapat dipertimbangkan. Selain itu, dukungan nutrisi intensif dan klirens dialisis yang adekuat pada pasien prepubertal dapat mempromosikan pertumbuhan normal tanpa selalu memerlukan rhGH. Pada anak yang mengalami stunting (tinggi badan &lt; persentil ke-2), perhitungan kebutuhan energi dan mikronutrien harus didasarkan pada height-age pasien, bukan chronological age-nya, untuk memberikan dukungan yang sesuai dengan ukuran tubuh aktualnya. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/)</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>2026-05-19 12:41:32</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>18F27E0F</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>&lt;2 yo</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>&lt;12 mo</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>Good service</t>
+        </is>
+      </c>
+      <c r="I109" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="J109" t="inlineStr">
+        <is>
+          <t>Studies</t>
+        </is>
+      </c>
+      <c r="K109" t="inlineStr">
+        <is>
+          <t>No ESI</t>
+        </is>
+      </c>
+      <c r="L109" t="inlineStr">
+        <is>
+          <t>Poor nutrition</t>
+        </is>
+      </c>
+      <c r="M109" t="inlineStr">
+        <is>
+          <t>Glomerular</t>
+        </is>
+      </c>
+      <c r="N109" t="inlineStr">
+        <is>
+          <t>Coiled/swan neck</t>
+        </is>
+      </c>
+      <c r="O109" t="inlineStr">
+        <is>
+          <t>Double</t>
+        </is>
+      </c>
+      <c r="P109" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="Q109" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R109" t="inlineStr">
+        <is>
+          <t>Patients</t>
+        </is>
+      </c>
+      <c r="S109" t="inlineStr"/>
+      <c r="T109" t="inlineStr">
+        <is>
+          <t>Lateral/downward</t>
+        </is>
+      </c>
+      <c r="U109" t="inlineStr">
+        <is>
+          <t>Stunting</t>
+        </is>
+      </c>
+      <c r="V109" t="inlineStr"/>
+      <c r="W109" t="inlineStr"/>
+      <c r="X109" t="inlineStr"/>
+      <c r="Y109" t="inlineStr">
+        <is>
+          <t>Age*, Gender, Nutrition, Stunting</t>
+        </is>
+      </c>
+      <c r="Z109" t="inlineStr">
+        <is>
+          <t>Nutrition: Malnutrisi protein-kalori (cachexia) adalah masalah umum pada anak yang menjalani PD. Manajemen nutrisi bertujuan untuk mengejar pertumbuhan dan mengganti hilangnya protein serta asam amino ke dalam cairan dialysis.Penilaian status nutrisi harus dilakukan secara berkala, minimal setiap bulan pada bayi dan 3-4 bulan pada anak yang lebih tua, menggunakan parameter antropometri (berat badan, tinggi badan, lingkar kepala), biokimia (albumin urea), dan analisis bioimpedansi jika tersedia. Penanganannya juga harus multidisiplin dan mencakup memastikan asupan energi dan protein yang adekuat; kontrol metabolik yang optimal, dengan koreksi asidosis, anemia, dan hiperparatiroidisme; dosis dialisis yang optimal (atau setidaknya adekuat); dan, jika perlu, pemberian obat-obatan tertentu seperti hormon pertumbuhan manusia rekombinan. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) | Stunting: Stunting pada anak dialisis bukan hanya disebabkan oleh asupan kalori yang rendah, tetapi juga oleh asidosis metabolik, anemia, osteodistrofi ginjal, dan resistensi terhadap hormon pertumbuhan. Intervensi pertama adalah memastikan kecukupan dialisis dan koreksi parameter metabolik seperti asidosis dan hiperparatiroidisme.Jika pertumbuhan masih belum optimal meskipun parameter metabolik telah terkendali dan asupan nutrisi sudah mencapai target, terapi dengan hormon pertumbuhan manusia rekombinan (rhGH) dapat dipertimbangkan. Selain itu, dukungan nutrisi intensif dan klirens dialisis yang adekuat pada pasien prepubertal dapat mempromosikan pertumbuhan normal tanpa selalu memerlukan rhGH. Pada anak yang mengalami stunting (tinggi badan &lt; persentil ke-2), perhitungan kebutuhan energi dan mikronutrien harus didasarkan pada height-age pasien, bukan chronological age-nya, untuk memberikan dukungan yang sesuai dengan ukuran tubuh aktualnya. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/)</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>2026-05-19 12:42:46</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>18F27E0F</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>&lt;2 yo</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>&lt;12 mo</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>Good service</t>
+        </is>
+      </c>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="J110" t="inlineStr">
+        <is>
+          <t>Studies</t>
+        </is>
+      </c>
+      <c r="K110" t="inlineStr">
+        <is>
+          <t>No ESI</t>
+        </is>
+      </c>
+      <c r="L110" t="inlineStr">
+        <is>
+          <t>Poor nutrition</t>
+        </is>
+      </c>
+      <c r="M110" t="inlineStr">
+        <is>
+          <t>Glomerular</t>
+        </is>
+      </c>
+      <c r="N110" t="inlineStr">
+        <is>
+          <t>Coiled/swan neck</t>
+        </is>
+      </c>
+      <c r="O110" t="inlineStr">
+        <is>
+          <t>Double</t>
+        </is>
+      </c>
+      <c r="P110" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="Q110" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R110" t="inlineStr">
+        <is>
+          <t>Patients</t>
+        </is>
+      </c>
+      <c r="S110" t="inlineStr"/>
+      <c r="T110" t="inlineStr">
+        <is>
+          <t>Lateral/downward</t>
+        </is>
+      </c>
+      <c r="U110" t="inlineStr">
+        <is>
+          <t>Stunting</t>
+        </is>
+      </c>
+      <c r="V110" t="inlineStr"/>
+      <c r="W110" t="inlineStr"/>
+      <c r="X110" t="inlineStr"/>
+      <c r="Y110" t="inlineStr">
+        <is>
+          <t>Age*, Gender, Nutrition, Stunting</t>
+        </is>
+      </c>
+      <c r="Z110" t="inlineStr">
+        <is>
+          <t>Nutrition: Malnutrisi protein-kalori (cachexia) adalah masalah umum pada anak yang menjalani PD. Manajemen nutrisi bertujuan untuk mengejar pertumbuhan dan mengganti hilangnya protein serta asam amino ke dalam cairan dialysis.Penilaian status nutrisi harus dilakukan secara berkala, minimal setiap bulan pada bayi dan 3-4 bulan pada anak yang lebih tua, menggunakan parameter antropometri (berat badan, tinggi badan, lingkar kepala), biokimia (albumin urea), dan analisis bioimpedansi jika tersedia. Penanganannya juga harus multidisiplin dan mencakup memastikan asupan energi dan protein yang adekuat; kontrol metabolik yang optimal, dengan koreksi asidosis, anemia, dan hiperparatiroidisme; dosis dialisis yang optimal (atau setidaknya adekuat); dan, jika perlu, pemberian obat-obatan tertentu seperti hormon pertumbuhan manusia rekombinan. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) | Stunting: Stunting pada anak dialisis bukan hanya disebabkan oleh asupan kalori yang rendah, tetapi juga oleh asidosis metabolik, anemia, osteodistrofi ginjal, dan resistensi terhadap hormon pertumbuhan. Intervensi pertama adalah memastikan kecukupan dialisis dan koreksi parameter metabolik seperti asidosis dan hiperparatiroidisme.Jika pertumbuhan masih belum optimal meskipun parameter metabolik telah terkendali dan asupan nutrisi sudah mencapai target, terapi dengan hormon pertumbuhan manusia rekombinan (rhGH) dapat dipertimbangkan. Selain itu, dukungan nutrisi intensif dan klirens dialisis yang adekuat pada pasien prepubertal dapat mempromosikan pertumbuhan normal tanpa selalu memerlukan rhGH. Pada anak yang mengalami stunting (tinggi badan &lt; persentil ke-2), perhitungan kebutuhan energi dan mikronutrien harus didasarkan pada height-age pasien, bukan chronological age-nya, untuk memberikan dukungan yang sesuai dengan ukuran tubuh aktualnya. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/)</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>2026-05-19 12:43:14</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>18F27E0F</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>&lt;2 yo</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>&gt;12 mo</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>Urban</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>Fair/poor service</t>
+        </is>
+      </c>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>Poor/fair</t>
+        </is>
+      </c>
+      <c r="J111" t="inlineStr">
+        <is>
+          <t>Illiterate</t>
+        </is>
+      </c>
+      <c r="K111" t="inlineStr">
+        <is>
+          <t>ESI</t>
+        </is>
+      </c>
+      <c r="L111" t="inlineStr">
+        <is>
+          <t>Poor nutrition</t>
+        </is>
+      </c>
+      <c r="M111" t="inlineStr">
+        <is>
+          <t>Non-glomerular</t>
+        </is>
+      </c>
+      <c r="N111" t="inlineStr">
+        <is>
+          <t>Straight</t>
+        </is>
+      </c>
+      <c r="O111" t="inlineStr">
+        <is>
+          <t>Single cuff</t>
+        </is>
+      </c>
+      <c r="P111" t="inlineStr">
+        <is>
+          <t>Laparoscopic</t>
+        </is>
+      </c>
+      <c r="Q111" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="R111" t="inlineStr">
+        <is>
+          <t>Parents/others</t>
+        </is>
+      </c>
+      <c r="S111" t="inlineStr"/>
+      <c r="T111" t="inlineStr">
+        <is>
+          <t>upward</t>
+        </is>
+      </c>
+      <c r="U111" t="inlineStr">
+        <is>
+          <t>Stunting</t>
+        </is>
+      </c>
+      <c r="V111" t="inlineStr"/>
+      <c r="W111" t="inlineStr"/>
+      <c r="X111" t="inlineStr"/>
+      <c r="Y111" t="inlineStr">
+        <is>
+          <t>Age*, Gender, Duration of PD*, Place of Residence, Housing, Socioeconomic, Education, Peritonitis in ESI*, Nutrition, Cause of ESRD*, Type of Catheter (Shape), Type of Catheter (Cuff), Catheter Placement, Gastrostomy/Intraperitoneal Device, Performed CAPD, Starting PD &lt;2 weeks after catheter placement, Catheter Orientation, Stunting</t>
+        </is>
+      </c>
+      <c r="Z111" t="inlineStr">
+        <is>
+          <t>Housing: Lingkungan rumah harus diadaptasi untuk memenuhi standar prosedur medis. Ruangan yang digunakan untuk pertukaran cairan harus bersih dan bebas debu untuk meminimalkan risiko infeksi, sebab partikel debu dapat menjadi vektor bagi patogen udara yang dapat mengontaminasi set transfer saat prosedur koneksi atau diskoneksi. Penyediaan wastafel di dalam atau dekat ruangan dialisis diperlukan untuk memastikan kepatuhan protokol antiseptic tangan sehingga menurunkan insiden peritonitis akibat touch contamination. Pencahayaan yang optimal di dalam ruangan diperlukan agar caregiver dapat memantau kejernihan cairan efluen serta memeriksa kondisi tempat keluar kateter dengan teliti. Hewan peliharaan tidak boleh berada di area perawatan saat proses koneksi atau diskoneksi berlangsung karena risiko paparan bakteri seperti Pasteurella multocida atau kerusakan fisik pada selang dialisis akibat gigitan atau cakaran. Selain itu, caregiverharus ditekankan untuk selalu mencuci tangan setelah berinteraksi dengan hewan dan sebelum memulai prosedur dialisis. [Sumber 1](https://www.freseniuskidneycare.com/treatment/home-dialysis/getting-prepared) [Sumber 2](https://www.ouh.nhs.uk/media/agxhnni2/85713pdialysis.pdf) [Sumber 3](https://www.kidney.org/kidney-topics/preparing-home-dialysis) [Sumber 4](https://spnp-spp.pt/media/rqdpbrom/catheter-related-infections-and-peritonitis-in-pediatric-patients-receiving-peritoneal-dialysis-guideline-for-prevention-and-treatment-2012-1-_compressed-1.pdf) [Sumber 5](https://freseniusmedicalcare.com/content/dam/home-products-education/steps2home-pd/Preventing_Peritonitis.pdf) [Sumber 6](https://www.satellitehealthcare.com/blog/pets-and-peritoneal-dialysis-absolutely/) | Socioeconomic: Deprivasi sosioekonomi berdampak pada hasil treatment yang lebih buruk. Hal ini kemungkinan disebabkan oleh keterbatasan akses terhadap fasilitas sanitasi yang memadai, tekanan psikologis pada pengasuh, serta keterbatasan informasi medis. Strategi bisa dilakukan melalui program pelatihan bagi keluarga (caregiver) dari perawat dialisis yang berpengalaman. Bagi keluarga dengan keterbatasan pendidikan atau ekonomi, dukungan teknis telepon 24 jam dan kunjungan rumah secara berkala oleh tim medis sosial sangat efektif dalam memastikan kepatuhan terhadap prosedur aseptik. Pelatihan ulang sangat dianjurkan, terutama setelah terjadinya peritonitis, untuk mengidentifikasi adanya penyimpangan dalam teknik pertukaran cairan. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC11835194/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC4934433/) [Sumber 3](https://pubmed.ncbi.nlm.nih.gov/23226378/) [Sumber 4](https://pubmed.ncbi.nlm.nih.gov/16091376/) [Sumber 6](https://spnp-spp.pt/media/rqdpbrom/catheter-related-infections-and-peritonitis-in-pediatric-patients-receiving-peritoneal-dialysis-guideline-for-prevention-and-treatment-2012-1-_compressed-1.pdf) [Sumber 7](https://pmc.ncbi.nlm.nih.gov/articles/PMC5691857/) [Sumber 8](https://pmc.ncbi.nlm.nih.gov/articles/PMC4335934/) [Sumber 9](https://www.kidney.org/kidney-topics/preparing-home-dialysis) | Peritonitis in ESI: Penggunaan antibiotik topikal secara rutin pada tempat keluar kateter telat terbukti menurunkan angka infeksi. Aplikasi harian salep mupirocin atau gentamicin pada exit-site direkomendasikan untuk menekan kolonisasi Staphylococcus aureus dan Pseudomonas aeruginosa.Pembersihan area secara rutin dengan larutan antiseptik non-iritan (seperti chlorhexidine 0,05% atau sabun antibakteri ringan) juga merupakan bagian standar dari perawatan. Penilaian kondisi exit-site secara objektif menggunakan sistem skor (seperti Skor ISPD yang mencakup pembengkakan, kerak, kemerahan, nyeri, dan sekret) sangat membantu caregiver dalam mendeteksi infeksi secara dini. Immobilisasi kateter dengan menggunakan plester atau perangkat fiksasi sangat krusial karena trauma mekanis pada tempat keluar sering kali menjadi pintu masuk bagi bakteri. Jika ESI terjadi, terapi antibiotik oral atau intraperitoneal harus dimulai segera dan dilanjutkan selama minimal 2 minggu, atau 3 minggu jika disebabkan oleh Pseudomonas. Pengangkatan kateter mungkin diperlukan jika infeksi bersifat refrakter (tidak merespons pengobatan setelah 2 minggu) atau jika infeksi telah menyebar ke terowongan kateter (tunnel infection) yang menyebabkan peritonitis berulang. [Sumber 1](https://ispd.org/wp-content/uploads/2025/09/LI-ET-1.pdf) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC12640025/) [Sumber 3](https://pmc.ncbi.nlm.nih.gov/articles/PMC5033625/) [Sumber 4](https://www.chikd.org/journal/view.php?number=726) [Sumber 5](https://ispd.org/wp-content/uploads/ISPD-Catheter-related-Infection-Recommendations-2023-Update.pdf) [Sumber 6](https://www.bcrenal.ca/resource-gallery/Documents/PD_Procedures-Exit_Site_Care-Post-Operative_PD_Catheter_Insertion.pdf) [Sumber 7](https://davita.com/treatment-options/articles/preventing-catheter-infections-on-peritoneal-dialysis/) [Sumber 8](https://edren.org/ren/handbook/pd-handbook/protocol-for-the-management-of-pd-peritonitis-long-version/) | Nutrition: Malnutrisi protein-kalori (cachexia) adalah masalah umum pada anak yang menjalani PD. Manajemen nutrisi bertujuan untuk mengejar pertumbuhan dan mengganti hilangnya protein serta asam amino ke dalam cairan dialysis.Penilaian status nutrisi harus dilakukan secara berkala, minimal setiap bulan pada bayi dan 3-4 bulan pada anak yang lebih tua, menggunakan parameter antropometri (berat badan, tinggi badan, lingkar kepala), biokimia (albumin urea), dan analisis bioimpedansi jika tersedia. Penanganannya juga harus multidisiplin dan mencakup memastikan asupan energi dan protein yang adekuat; kontrol metabolik yang optimal, dengan koreksi asidosis, anemia, dan hiperparatiroidisme; dosis dialisis yang optimal (atau setidaknya adekuat); dan, jika perlu, pemberian obat-obatan tertentu seperti hormon pertumbuhan manusia rekombinan. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) | Type of Catheter (Shape): Perdebatan mengenai efektivitas kateter straight dibandingkan dengan kateter coiled/curled masih berlangsung. Kateter coiled secara teoretis mengurangi nyeri saat pengisian cairan dan meminimalkan trauma pada organ visceral, tetapi beberapa data menunjukkan risiko malposisi yang lebih tinggi dibandingkan tipe lurus pada beberapa kelompok pasien. Di sisi lain, kateter straight lebih mudah ditempatkan pada bayi kecil yang memiliki ruang intra-abdominal terbatas. Secara keseluruhan, pedoman tidak menyatakan superioritas mutlak salah satu bentuk, dan pemilihan sering kali bergantung pada preferensi pusat dialisis dan anatomi pasien. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC9365012/) [Sumber 2](http://ispd.org/wp-content/uploads/7.-Dagmara-Borzych-Duzalka-Peritoneal-Dialysis-Catheters-Outcome-in-Children.-The-IPPN-Data.pdf) [Sumber 3](https://scholarlyexchange.childrensmercy.org/cgi/viewcontent.cgi?article=7522&amp;context=papers) [Sumber 4](https://kidney.wiki/peritoneal-dialysis/pd-access/) | Type of Catheter (Cuff): Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff)untuk populasi anak secara umum. Deep cuff berfungsi untuk menjangkar kateter di otot rektus dan mencegah kebocoran, sementara superficial cuff bertindak sebagai penghalang fisik terhadap migrasi bakteri ke arah rongga peritoneum. Namun, pada neonatus atau bayi dengan dinding perut yang sangat tipis, kateter single-cuff sering kali lebih dipilih untuk mencegah ekstrusi manset ke permukaan kulit. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC10223083/) [Sumber 2](http://ispd.org/wp-content/uploads/7.-Dagmara-Borzych-Duzalka-Peritoneal-Dialysis-Catheters-Outcome-in-Children.-The-IPPN-Data.pdf) [Sumber 3](https://kidney.wiki/peritoneal-dialysis/pd-access/) | Catheter Placement: Pedoman klinis terbaru dari Society of American Gastrointestinal and Endoscopic Surgeons (SAGES) menyarankan penggunaan teknik laparoskopi tingkat lanjut (Laparoscopic) dibandingkan teknik bedah terbuka (Open) untuk pemasangan kateter pada populasi pediatrik. Laparoscopic menawarkan akurasi catheter placement yang jauh lebih tinggi di dalam rongga abdomen karena visualisasi langsung, serta meminimalkan trauma mekanis pada jaringan perut. Lebih lanjut, Laparoscopic memungkinkan dokter untuk melakukan prosedur profilaksis penting seperti omentektomi atau omentopeksi untuk meminimalkan risiko omental wrapping (penyumbatan kateter oleh omentum), yang merupakan salah satu penyebab utama kegagalan mekanis kateter pada anak-anak. Laparoscopic juga terbukti mempermudah penyelamatan (salvage) jika terjadi malposisi atau disfungsi kateter tanpa harus melakukan pembedahan ulang yang invasif. [Sumber 1](https://www.sages.org/publications/guidelines/peritoneal-dialysis-access-guideline-update-2023/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC10223083/) [[3]](https://kidney.wiki/peritoneal-dialysis/pd-access/) | Gastrostomy/Intraperitoneal Device:  | Performed CAPD: Tidak ada perbedaan yang signifikan dalam tingkat kelangsungan hidup teknik, kematian, maupun episode peritonitis antara dialisis yang dilakukan sendiri oleh pasien (self-care) dengan dialisis yang dibantu oleh keluarga atau pengasuh (assisted/home-care). Namun, pada populasi anak (khususnya balita atau anak dengan keterbatasan fisik/kognitif), peran orang tua (Parent/Others) sangat mutlak diperlukan. Bagi orang tua yang memiliki tingkat pendidikan rendah atau keterbatasan ekonomi, dialisis tetap dapat berhasil dengan baik tanpa komplikasi besar asalkan diberikan pelatihan intensif secara 1:1, dukungan telepon 24 jam, dan kunjungan rumah berkala oleh perawat dialisis berpengalaman. Di sisi lain, bagi pasien remaja yang melakukan dialisis secara mandiri (Patient), tantangan psikososial seperti kejenuhan (burnout), perasaan terkekang (slavery feeling), dan depresi sering kali muncul, sehingga membutuhkan pengawasan ketat dari tim medis agar kepatuhan terhadap prosedur aseptik tetap terjaga. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/29456210/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC4335934/) [Sumber 3](https://www.ispd.org/wp-content/uploads/2025/12/Assisted-PD-PP-2024-with-VA_formatted.pdf) | Starting PD &lt;2 weeks after catheter placement: Waktu antara pemasangan kateter dan dimulainya dialisis (break-in-period) merupakan faktor penting untuk mencegah komplikasi. Masa penyembuhan minimal 2 minggu sebelum dialysis dimulai. Namun, dalam kondisi klinis tertentu di mana pasien membutuhkan dialisis segera, urgent-start PD (dimulai dalam &lt;14 hari atau bahkan &lt;48 jam) menjadi alternatif yang baik untuk menghindari penggunakan kateter hemodialysis sementara. Pasien dengan break-in-period &lt; 7 hari memiliki risiko yang lebih tinggi terhadap komplikasi awal seperti kebocoran dialisat dan malposisi kateter. Namun, risiko tersebut tidak berkorelasi dengan penurunan kelangsungan hidup atau peningkatan risiko peritonitis jika dilakukan dengan protokol yang tepat. Pada kondisi urgent-start, risiko kebocoran dimitigasi dengan menggunakan volume pengisian rendah (10-20 ml/kg) dan posisi pasien supine untuk mengurangi tekanan intra-abdominal.[Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC3923692/) [Sumber 2](https://journals.plos.org/plosone/article?id=10.1371/journal.pone.0206426) [Sumber 3](https://www.sages.org/publications/guidelines/peritoneal-dialysis-access-guideline-update-2023/) [Sumber 4](https://www.frontiersin.org/journals/endocrinology/articles/10.3389/fendo.2022.936573/full) [Sumber 5](https://scholarlyexchange.childrensmercy.org/cgi/viewcontent.cgi?article=7522&amp;context=papers) [Sumber 6](https://pubmed.ncbi.nlm.nih.gov/33523772/) [Sumber 7](https://www.bcrenal.ca/resource-gallery/Documents/PD_Procedures-Exit_Site_Care-Post-Operative_PD_Catheter_Insertion.pdf) | Catheter Orientation: Posisi atau arah lubang keluar kateter (exit site) sangat memengaruhi risiko terjadinya infeksi. Data multisentrik dari SCOPE Collaborative menunjukkan bahwa orientasi kateter yang menghadap ke atas (Upward) dikaitkan dengan peningkatan risiko peritonitis hingga 4.2 kali lipat (Rate Ratio: 4.2; 95% CI: 1.49–11.89) dibandingkan orientasi lainnya. Secara anatomis, lubang keluar yang menghadap ke atas menciptakan bentuk cekungan yang dapat menampung keringat, air mandi, dan kotoran. Akibat gaya gravitasi, bakteri yang terkumpul di area ini akan mengendap dan bermigrasi ke dalam terowongan kateter. Oleh karena itu, lubang keluar kateter harus selalu diarahkan ke bawah (Downward) atau ke samping (Lateral) untuk mencegah penumpukan bakteri secara alami. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC5012476/) [Sumber 2](https://openurologyandnephrologyjournal.com/VOLUME/5/PAGE/4/) [Sumber 3](https://kidney.wiki/peritoneal-dialysis/pd-access/) | Stunting: Stunting pada anak dialisis bukan hanya disebabkan oleh asupan kalori yang rendah, tetapi juga oleh asidosis metabolik, anemia, osteodistrofi ginjal, dan resistensi terhadap hormon pertumbuhan. Intervensi pertama adalah memastikan kecukupan dialisis dan koreksi parameter metabolik seperti asidosis dan hiperparatiroidisme.Jika pertumbuhan masih belum optimal meskipun parameter metabolik telah terkendali dan asupan nutrisi sudah mencapai target, terapi dengan hormon pertumbuhan manusia rekombinan (rhGH) dapat dipertimbangkan. Selain itu, dukungan nutrisi intensif dan klirens dialisis yang adekuat pada pasien prepubertal dapat mempromosikan pertumbuhan normal tanpa selalu memerlukan rhGH. Pada anak yang mengalami stunting (tinggi badan &lt; persentil ke-2), perhitungan kebutuhan energi dan mikronutrien harus didasarkan pada height-age pasien, bukan chronological age-nya, untuk memberikan dukungan yang sesuai dengan ukuran tubuh aktualnya. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/)</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>2026-05-19 12:43:33</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>18F27E0F</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>&lt;2 yo</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>&gt;12 mo</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>Urban</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>Fair/poor service</t>
+        </is>
+      </c>
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>Poor/fair</t>
+        </is>
+      </c>
+      <c r="J112" t="inlineStr">
+        <is>
+          <t>Illiterate</t>
+        </is>
+      </c>
+      <c r="K112" t="inlineStr">
+        <is>
+          <t>ESI</t>
+        </is>
+      </c>
+      <c r="L112" t="inlineStr">
+        <is>
+          <t>Poor nutrition</t>
+        </is>
+      </c>
+      <c r="M112" t="inlineStr">
+        <is>
+          <t>Non-glomerular</t>
+        </is>
+      </c>
+      <c r="N112" t="inlineStr">
+        <is>
+          <t>Straight</t>
+        </is>
+      </c>
+      <c r="O112" t="inlineStr">
+        <is>
+          <t>Single cuff</t>
+        </is>
+      </c>
+      <c r="P112" t="inlineStr">
+        <is>
+          <t>Laparoscopic</t>
+        </is>
+      </c>
+      <c r="Q112" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="R112" t="inlineStr">
+        <is>
+          <t>Parents/others</t>
+        </is>
+      </c>
+      <c r="S112" t="inlineStr"/>
+      <c r="T112" t="inlineStr">
+        <is>
+          <t>upward</t>
+        </is>
+      </c>
+      <c r="U112" t="inlineStr">
+        <is>
+          <t>No stunting</t>
+        </is>
+      </c>
+      <c r="V112" t="inlineStr"/>
+      <c r="W112" t="inlineStr"/>
+      <c r="X112" t="inlineStr"/>
+      <c r="Y112" t="inlineStr">
+        <is>
+          <t>Age*, Gender, Duration of PD*, Place of Residence, Housing, Socioeconomic, Education, Peritonitis in ESI*, Nutrition, Cause of ESRD*, Type of Catheter (Shape), Type of Catheter (Cuff), Catheter Placement, Gastrostomy/Intraperitoneal Device, Performed CAPD, Starting PD &lt;2 weeks after catheter placement, Catheter Orientation</t>
+        </is>
+      </c>
+      <c r="Z112" t="inlineStr">
+        <is>
+          <t>Housing: Lingkungan rumah harus diadaptasi untuk memenuhi standar prosedur medis. Ruangan yang digunakan untuk pertukaran cairan harus bersih dan bebas debu untuk meminimalkan risiko infeksi, sebab partikel debu dapat menjadi vektor bagi patogen udara yang dapat mengontaminasi set transfer saat prosedur koneksi atau diskoneksi. Penyediaan wastafel di dalam atau dekat ruangan dialisis diperlukan untuk memastikan kepatuhan protokol antiseptic tangan sehingga menurunkan insiden peritonitis akibat touch contamination. Pencahayaan yang optimal di dalam ruangan diperlukan agar caregiver dapat memantau kejernihan cairan efluen serta memeriksa kondisi tempat keluar kateter dengan teliti. Hewan peliharaan tidak boleh berada di area perawatan saat proses koneksi atau diskoneksi berlangsung karena risiko paparan bakteri seperti Pasteurella multocida atau kerusakan fisik pada selang dialisis akibat gigitan atau cakaran. Selain itu, caregiverharus ditekankan untuk selalu mencuci tangan setelah berinteraksi dengan hewan dan sebelum memulai prosedur dialisis. [Sumber 1](https://www.freseniuskidneycare.com/treatment/home-dialysis/getting-prepared) [Sumber 2](https://www.ouh.nhs.uk/media/agxhnni2/85713pdialysis.pdf) [Sumber 3](https://www.kidney.org/kidney-topics/preparing-home-dialysis) [Sumber 4](https://spnp-spp.pt/media/rqdpbrom/catheter-related-infections-and-peritonitis-in-pediatric-patients-receiving-peritoneal-dialysis-guideline-for-prevention-and-treatment-2012-1-_compressed-1.pdf) [Sumber 5](https://freseniusmedicalcare.com/content/dam/home-products-education/steps2home-pd/Preventing_Peritonitis.pdf) [Sumber 6](https://www.satellitehealthcare.com/blog/pets-and-peritoneal-dialysis-absolutely/) | Socioeconomic: Deprivasi sosioekonomi berdampak pada hasil treatment yang lebih buruk. Hal ini kemungkinan disebabkan oleh keterbatasan akses terhadap fasilitas sanitasi yang memadai, tekanan psikologis pada pengasuh, serta keterbatasan informasi medis. Strategi bisa dilakukan melalui program pelatihan bagi keluarga (caregiver) dari perawat dialisis yang berpengalaman. Bagi keluarga dengan keterbatasan pendidikan atau ekonomi, dukungan teknis telepon 24 jam dan kunjungan rumah secara berkala oleh tim medis sosial sangat efektif dalam memastikan kepatuhan terhadap prosedur aseptik. Pelatihan ulang sangat dianjurkan, terutama setelah terjadinya peritonitis, untuk mengidentifikasi adanya penyimpangan dalam teknik pertukaran cairan. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC11835194/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC4934433/) [Sumber 3](https://pubmed.ncbi.nlm.nih.gov/23226378/) [Sumber 4](https://pubmed.ncbi.nlm.nih.gov/16091376/) [Sumber 6](https://spnp-spp.pt/media/rqdpbrom/catheter-related-infections-and-peritonitis-in-pediatric-patients-receiving-peritoneal-dialysis-guideline-for-prevention-and-treatment-2012-1-_compressed-1.pdf) [Sumber 7](https://pmc.ncbi.nlm.nih.gov/articles/PMC5691857/) [Sumber 8](https://pmc.ncbi.nlm.nih.gov/articles/PMC4335934/) [Sumber 9](https://www.kidney.org/kidney-topics/preparing-home-dialysis) | Peritonitis in ESI: Penggunaan antibiotik topikal secara rutin pada tempat keluar kateter telat terbukti menurunkan angka infeksi. Aplikasi harian salep mupirocin atau gentamicin pada exit-site direkomendasikan untuk menekan kolonisasi Staphylococcus aureus dan Pseudomonas aeruginosa.Pembersihan area secara rutin dengan larutan antiseptik non-iritan (seperti chlorhexidine 0,05% atau sabun antibakteri ringan) juga merupakan bagian standar dari perawatan. Penilaian kondisi exit-site secara objektif menggunakan sistem skor (seperti Skor ISPD yang mencakup pembengkakan, kerak, kemerahan, nyeri, dan sekret) sangat membantu caregiver dalam mendeteksi infeksi secara dini. Immobilisasi kateter dengan menggunakan plester atau perangkat fiksasi sangat krusial karena trauma mekanis pada tempat keluar sering kali menjadi pintu masuk bagi bakteri. Jika ESI terjadi, terapi antibiotik oral atau intraperitoneal harus dimulai segera dan dilanjutkan selama minimal 2 minggu, atau 3 minggu jika disebabkan oleh Pseudomonas. Pengangkatan kateter mungkin diperlukan jika infeksi bersifat refrakter (tidak merespons pengobatan setelah 2 minggu) atau jika infeksi telah menyebar ke terowongan kateter (tunnel infection) yang menyebabkan peritonitis berulang. [Sumber 1](https://ispd.org/wp-content/uploads/2025/09/LI-ET-1.pdf) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC12640025/) [Sumber 3](https://pmc.ncbi.nlm.nih.gov/articles/PMC5033625/) [Sumber 4](https://www.chikd.org/journal/view.php?number=726) [Sumber 5](https://ispd.org/wp-content/uploads/ISPD-Catheter-related-Infection-Recommendations-2023-Update.pdf) [Sumber 6](https://www.bcrenal.ca/resource-gallery/Documents/PD_Procedures-Exit_Site_Care-Post-Operative_PD_Catheter_Insertion.pdf) [Sumber 7](https://davita.com/treatment-options/articles/preventing-catheter-infections-on-peritoneal-dialysis/) [Sumber 8](https://edren.org/ren/handbook/pd-handbook/protocol-for-the-management-of-pd-peritonitis-long-version/) | Nutrition: Malnutrisi protein-kalori (cachexia) adalah masalah umum pada anak yang menjalani PD. Manajemen nutrisi bertujuan untuk mengejar pertumbuhan dan mengganti hilangnya protein serta asam amino ke dalam cairan dialysis.Penilaian status nutrisi harus dilakukan secara berkala, minimal setiap bulan pada bayi dan 3-4 bulan pada anak yang lebih tua, menggunakan parameter antropometri (berat badan, tinggi badan, lingkar kepala), biokimia (albumin urea), dan analisis bioimpedansi jika tersedia. Penanganannya juga harus multidisiplin dan mencakup memastikan asupan energi dan protein yang adekuat; kontrol metabolik yang optimal, dengan koreksi asidosis, anemia, dan hiperparatiroidisme; dosis dialisis yang optimal (atau setidaknya adekuat); dan, jika perlu, pemberian obat-obatan tertentu seperti hormon pertumbuhan manusia rekombinan. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) | Type of Catheter (Shape): Perdebatan mengenai efektivitas kateter straight dibandingkan dengan kateter coiled/curled masih berlangsung. Kateter coiled secara teoretis mengurangi nyeri saat pengisian cairan dan meminimalkan trauma pada organ visceral, tetapi beberapa data menunjukkan risiko malposisi yang lebih tinggi dibandingkan tipe lurus pada beberapa kelompok pasien. Di sisi lain, kateter straight lebih mudah ditempatkan pada bayi kecil yang memiliki ruang intra-abdominal terbatas. Secara keseluruhan, pedoman tidak menyatakan superioritas mutlak salah satu bentuk, dan pemilihan sering kali bergantung pada preferensi pusat dialisis dan anatomi pasien. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC9365012/) [Sumber 2](http://ispd.org/wp-content/uploads/7.-Dagmara-Borzych-Duzalka-Peritoneal-Dialysis-Catheters-Outcome-in-Children.-The-IPPN-Data.pdf) [Sumber 3](https://scholarlyexchange.childrensmercy.org/cgi/viewcontent.cgi?article=7522&amp;context=papers) [Sumber 4](https://kidney.wiki/peritoneal-dialysis/pd-access/) | Type of Catheter (Cuff): Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff)untuk populasi anak secara umum. Deep cuff berfungsi untuk menjangkar kateter di otot rektus dan mencegah kebocoran, sementara superficial cuff bertindak sebagai penghalang fisik terhadap migrasi bakteri ke arah rongga peritoneum. Namun, pada neonatus atau bayi dengan dinding perut yang sangat tipis, kateter single-cuff sering kali lebih dipilih untuk mencegah ekstrusi manset ke permukaan kulit. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC10223083/) [Sumber 2](http://ispd.org/wp-content/uploads/7.-Dagmara-Borzych-Duzalka-Peritoneal-Dialysis-Catheters-Outcome-in-Children.-The-IPPN-Data.pdf) [Sumber 3](https://kidney.wiki/peritoneal-dialysis/pd-access/) | Catheter Placement: Pedoman klinis terbaru dari Society of American Gastrointestinal and Endoscopic Surgeons (SAGES) menyarankan penggunaan teknik laparoskopi tingkat lanjut (Laparoscopic) dibandingkan teknik bedah terbuka (Open) untuk pemasangan kateter pada populasi pediatrik. Laparoscopic menawarkan akurasi catheter placement yang jauh lebih tinggi di dalam rongga abdomen karena visualisasi langsung, serta meminimalkan trauma mekanis pada jaringan perut. Lebih lanjut, Laparoscopic memungkinkan dokter untuk melakukan prosedur profilaksis penting seperti omentektomi atau omentopeksi untuk meminimalkan risiko omental wrapping (penyumbatan kateter oleh omentum), yang merupakan salah satu penyebab utama kegagalan mekanis kateter pada anak-anak. Laparoscopic juga terbukti mempermudah penyelamatan (salvage) jika terjadi malposisi atau disfungsi kateter tanpa harus melakukan pembedahan ulang yang invasif. [Sumber 1](https://www.sages.org/publications/guidelines/peritoneal-dialysis-access-guideline-update-2023/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC10223083/) [[3]](https://kidney.wiki/peritoneal-dialysis/pd-access/) | Gastrostomy/Intraperitoneal Device:  | Performed CAPD: Tidak ada perbedaan yang signifikan dalam tingkat kelangsungan hidup teknik, kematian, maupun episode peritonitis antara dialisis yang dilakukan sendiri oleh pasien (self-care) dengan dialisis yang dibantu oleh keluarga atau pengasuh (assisted/home-care). Namun, pada populasi anak (khususnya balita atau anak dengan keterbatasan fisik/kognitif), peran orang tua (Parent/Others) sangat mutlak diperlukan. Bagi orang tua yang memiliki tingkat pendidikan rendah atau keterbatasan ekonomi, dialisis tetap dapat berhasil dengan baik tanpa komplikasi besar asalkan diberikan pelatihan intensif secara 1:1, dukungan telepon 24 jam, dan kunjungan rumah berkala oleh perawat dialisis berpengalaman. Di sisi lain, bagi pasien remaja yang melakukan dialisis secara mandiri (Patient), tantangan psikososial seperti kejenuhan (burnout), perasaan terkekang (slavery feeling), dan depresi sering kali muncul, sehingga membutuhkan pengawasan ketat dari tim medis agar kepatuhan terhadap prosedur aseptik tetap terjaga. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/29456210/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC4335934/) [Sumber 3](https://www.ispd.org/wp-content/uploads/2025/12/Assisted-PD-PP-2024-with-VA_formatted.pdf) | Starting PD &lt;2 weeks after catheter placement: Waktu antara pemasangan kateter dan dimulainya dialisis (break-in-period) merupakan faktor penting untuk mencegah komplikasi. Masa penyembuhan minimal 2 minggu sebelum dialysis dimulai. Namun, dalam kondisi klinis tertentu di mana pasien membutuhkan dialisis segera, urgent-start PD (dimulai dalam &lt;14 hari atau bahkan &lt;48 jam) menjadi alternatif yang baik untuk menghindari penggunakan kateter hemodialysis sementara. Pasien dengan break-in-period &lt; 7 hari memiliki risiko yang lebih tinggi terhadap komplikasi awal seperti kebocoran dialisat dan malposisi kateter. Namun, risiko tersebut tidak berkorelasi dengan penurunan kelangsungan hidup atau peningkatan risiko peritonitis jika dilakukan dengan protokol yang tepat. Pada kondisi urgent-start, risiko kebocoran dimitigasi dengan menggunakan volume pengisian rendah (10-20 ml/kg) dan posisi pasien supine untuk mengurangi tekanan intra-abdominal.[Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC3923692/) [Sumber 2](https://journals.plos.org/plosone/article?id=10.1371/journal.pone.0206426) [Sumber 3](https://www.sages.org/publications/guidelines/peritoneal-dialysis-access-guideline-update-2023/) [Sumber 4](https://www.frontiersin.org/journals/endocrinology/articles/10.3389/fendo.2022.936573/full) [Sumber 5](https://scholarlyexchange.childrensmercy.org/cgi/viewcontent.cgi?article=7522&amp;context=papers) [Sumber 6](https://pubmed.ncbi.nlm.nih.gov/33523772/) [Sumber 7](https://www.bcrenal.ca/resource-gallery/Documents/PD_Procedures-Exit_Site_Care-Post-Operative_PD_Catheter_Insertion.pdf) | Catheter Orientation: Posisi atau arah lubang keluar kateter (exit site) sangat memengaruhi risiko terjadinya infeksi. Data multisentrik dari SCOPE Collaborative menunjukkan bahwa orientasi kateter yang menghadap ke atas (Upward) dikaitkan dengan peningkatan risiko peritonitis hingga 4.2 kali lipat (Rate Ratio: 4.2; 95% CI: 1.49–11.89) dibandingkan orientasi lainnya. Secara anatomis, lubang keluar yang menghadap ke atas menciptakan bentuk cekungan yang dapat menampung keringat, air mandi, dan kotoran. Akibat gaya gravitasi, bakteri yang terkumpul di area ini akan mengendap dan bermigrasi ke dalam terowongan kateter. Oleh karena itu, lubang keluar kateter harus selalu diarahkan ke bawah (Downward) atau ke samping (Lateral) untuk mencegah penumpukan bakteri secara alami. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC5012476/) [Sumber 2](https://openurologyandnephrologyjournal.com/VOLUME/5/PAGE/4/) [Sumber 3](https://kidney.wiki/peritoneal-dialysis/pd-access/)</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>2026-05-19 12:44:13</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>18F27E0F</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>&lt;2 yo</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>&gt;12 mo</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>Urban</t>
+        </is>
+      </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>Fair/poor service</t>
+        </is>
+      </c>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>Poor/fair</t>
+        </is>
+      </c>
+      <c r="J113" t="inlineStr">
+        <is>
+          <t>Illiterate</t>
+        </is>
+      </c>
+      <c r="K113" t="inlineStr">
+        <is>
+          <t>ESI</t>
+        </is>
+      </c>
+      <c r="L113" t="inlineStr">
+        <is>
+          <t>Poor nutrition</t>
+        </is>
+      </c>
+      <c r="M113" t="inlineStr">
+        <is>
+          <t>Non-glomerular</t>
+        </is>
+      </c>
+      <c r="N113" t="inlineStr">
+        <is>
+          <t>Straight</t>
+        </is>
+      </c>
+      <c r="O113" t="inlineStr">
+        <is>
+          <t>Single cuff</t>
+        </is>
+      </c>
+      <c r="P113" t="inlineStr">
+        <is>
+          <t>Laparoscopic</t>
+        </is>
+      </c>
+      <c r="Q113" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="R113" t="inlineStr">
+        <is>
+          <t>Parents/others</t>
+        </is>
+      </c>
+      <c r="S113" t="inlineStr"/>
+      <c r="T113" t="inlineStr">
+        <is>
+          <t>upward</t>
+        </is>
+      </c>
+      <c r="U113" t="inlineStr">
+        <is>
+          <t>No stunting</t>
+        </is>
+      </c>
+      <c r="V113" t="inlineStr"/>
+      <c r="W113" t="inlineStr"/>
+      <c r="X113" t="inlineStr"/>
+      <c r="Y113" t="inlineStr">
+        <is>
+          <t>Age*, Gender, Duration of PD*, Place of Residence, Housing, Socioeconomic, Education, Peritonitis in ESI*, Nutrition, Cause of ESRD*, Type of Catheter (Shape), Type of Catheter (Cuff), Catheter Placement, Gastrostomy/Intraperitoneal Device, Performed CAPD, Starting PD &lt;2 weeks after catheter placement, Catheter Orientation</t>
+        </is>
+      </c>
+      <c r="Z113" t="inlineStr">
+        <is>
+          <t>Housing: Lingkungan rumah harus diadaptasi untuk memenuhi standar prosedur medis. Ruangan yang digunakan untuk pertukaran cairan harus bersih dan bebas debu untuk meminimalkan risiko infeksi, sebab partikel debu dapat menjadi vektor bagi patogen udara yang dapat mengontaminasi set transfer saat prosedur koneksi atau diskoneksi. Penyediaan wastafel di dalam atau dekat ruangan dialisis diperlukan untuk memastikan kepatuhan protokol antiseptic tangan sehingga menurunkan insiden peritonitis akibat touch contamination. Pencahayaan yang optimal di dalam ruangan diperlukan agar caregiver dapat memantau kejernihan cairan efluen serta memeriksa kondisi tempat keluar kateter dengan teliti. Hewan peliharaan tidak boleh berada di area perawatan saat proses koneksi atau diskoneksi berlangsung karena risiko paparan bakteri seperti Pasteurella multocida atau kerusakan fisik pada selang dialisis akibat gigitan atau cakaran. Selain itu, caregiverharus ditekankan untuk selalu mencuci tangan setelah berinteraksi dengan hewan dan sebelum memulai prosedur dialisis. [Sumber 1](https://www.freseniuskidneycare.com/treatment/home-dialysis/getting-prepared) [Sumber 2](https://www.ouh.nhs.uk/media/agxhnni2/85713pdialysis.pdf) [Sumber 3](https://www.kidney.org/kidney-topics/preparing-home-dialysis) [Sumber 4](https://spnp-spp.pt/media/rqdpbrom/catheter-related-infections-and-peritonitis-in-pediatric-patients-receiving-peritoneal-dialysis-guideline-for-prevention-and-treatment-2012-1-_compressed-1.pdf) [Sumber 5](https://freseniusmedicalcare.com/content/dam/home-products-education/steps2home-pd/Preventing_Peritonitis.pdf) [Sumber 6](https://www.satellitehealthcare.com/blog/pets-and-peritoneal-dialysis-absolutely/) | Socioeconomic: Deprivasi sosioekonomi berdampak pada hasil treatment yang lebih buruk. Hal ini kemungkinan disebabkan oleh keterbatasan akses terhadap fasilitas sanitasi yang memadai, tekanan psikologis pada pengasuh, serta keterbatasan informasi medis. Strategi bisa dilakukan melalui program pelatihan bagi keluarga (caregiver) dari perawat dialisis yang berpengalaman. Bagi keluarga dengan keterbatasan pendidikan atau ekonomi, dukungan teknis telepon 24 jam dan kunjungan rumah secara berkala oleh tim medis sosial sangat efektif dalam memastikan kepatuhan terhadap prosedur aseptik. Pelatihan ulang sangat dianjurkan, terutama setelah terjadinya peritonitis, untuk mengidentifikasi adanya penyimpangan dalam teknik pertukaran cairan. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC11835194/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC4934433/) [Sumber 3](https://pubmed.ncbi.nlm.nih.gov/23226378/) [Sumber 4](https://pubmed.ncbi.nlm.nih.gov/16091376/) [Sumber 6](https://spnp-spp.pt/media/rqdpbrom/catheter-related-infections-and-peritonitis-in-pediatric-patients-receiving-peritoneal-dialysis-guideline-for-prevention-and-treatment-2012-1-_compressed-1.pdf) [Sumber 7](https://pmc.ncbi.nlm.nih.gov/articles/PMC5691857/) [Sumber 8](https://pmc.ncbi.nlm.nih.gov/articles/PMC4335934/) [Sumber 9](https://www.kidney.org/kidney-topics/preparing-home-dialysis) | Peritonitis in ESI: Penggunaan antibiotik topikal secara rutin pada tempat keluar kateter telat terbukti menurunkan angka infeksi. Aplikasi harian salep mupirocin atau gentamicin pada exit-site direkomendasikan untuk menekan kolonisasi Staphylococcus aureus dan Pseudomonas aeruginosa.Pembersihan area secara rutin dengan larutan antiseptik non-iritan (seperti chlorhexidine 0,05% atau sabun antibakteri ringan) juga merupakan bagian standar dari perawatan. Penilaian kondisi exit-site secara objektif menggunakan sistem skor (seperti Skor ISPD yang mencakup pembengkakan, kerak, kemerahan, nyeri, dan sekret) sangat membantu caregiver dalam mendeteksi infeksi secara dini. Immobilisasi kateter dengan menggunakan plester atau perangkat fiksasi sangat krusial karena trauma mekanis pada tempat keluar sering kali menjadi pintu masuk bagi bakteri. Jika ESI terjadi, terapi antibiotik oral atau intraperitoneal harus dimulai segera dan dilanjutkan selama minimal 2 minggu, atau 3 minggu jika disebabkan oleh Pseudomonas. Pengangkatan kateter mungkin diperlukan jika infeksi bersifat refrakter (tidak merespons pengobatan setelah 2 minggu) atau jika infeksi telah menyebar ke terowongan kateter (tunnel infection) yang menyebabkan peritonitis berulang. [Sumber 1](https://ispd.org/wp-content/uploads/2025/09/LI-ET-1.pdf) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC12640025/) [Sumber 3](https://pmc.ncbi.nlm.nih.gov/articles/PMC5033625/) [Sumber 4](https://www.chikd.org/journal/view.php?number=726) [Sumber 5](https://ispd.org/wp-content/uploads/ISPD-Catheter-related-Infection-Recommendations-2023-Update.pdf) [Sumber 6](https://www.bcrenal.ca/resource-gallery/Documents/PD_Procedures-Exit_Site_Care-Post-Operative_PD_Catheter_Insertion.pdf) [Sumber 7](https://davita.com/treatment-options/articles/preventing-catheter-infections-on-peritoneal-dialysis/) [Sumber 8](https://edren.org/ren/handbook/pd-handbook/protocol-for-the-management-of-pd-peritonitis-long-version/) | Nutrition: Malnutrisi protein-kalori (cachexia) adalah masalah umum pada anak yang menjalani PD. Manajemen nutrisi bertujuan untuk mengejar pertumbuhan dan mengganti hilangnya protein serta asam amino ke dalam cairan dialysis.Penilaian status nutrisi harus dilakukan secara berkala, minimal setiap bulan pada bayi dan 3-4 bulan pada anak yang lebih tua, menggunakan parameter antropometri (berat badan, tinggi badan, lingkar kepala), biokimia (albumin urea), dan analisis bioimpedansi jika tersedia. Penanganannya juga harus multidisiplin dan mencakup memastikan asupan energi dan protein yang adekuat; kontrol metabolik yang optimal, dengan koreksi asidosis, anemia, dan hiperparatiroidisme; dosis dialisis yang optimal (atau setidaknya adekuat); dan, jika perlu, pemberian obat-obatan tertentu seperti hormon pertumbuhan manusia rekombinan. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) | Type of Catheter (Shape): Perdebatan mengenai efektivitas kateter straight dibandingkan dengan kateter coiled/curled masih berlangsung. Kateter coiled secara teoretis mengurangi nyeri saat pengisian cairan dan meminimalkan trauma pada organ visceral, tetapi beberapa data menunjukkan risiko malposisi yang lebih tinggi dibandingkan tipe lurus pada beberapa kelompok pasien. Di sisi lain, kateter straight lebih mudah ditempatkan pada bayi kecil yang memiliki ruang intra-abdominal terbatas. Secara keseluruhan, pedoman tidak menyatakan superioritas mutlak salah satu bentuk, dan pemilihan sering kali bergantung pada preferensi pusat dialisis dan anatomi pasien. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC9365012/) [Sumber 2](http://ispd.org/wp-content/uploads/7.-Dagmara-Borzych-Duzalka-Peritoneal-Dialysis-Catheters-Outcome-in-Children.-The-IPPN-Data.pdf) [Sumber 3](https://scholarlyexchange.childrensmercy.org/cgi/viewcontent.cgi?article=7522&amp;context=papers) [Sumber 4](https://kidney.wiki/peritoneal-dialysis/pd-access/) | Type of Catheter (Cuff): Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff)untuk populasi anak secara umum. Deep cuff berfungsi untuk menjangkar kateter di otot rektus dan mencegah kebocoran, sementara superficial cuff bertindak sebagai penghalang fisik terhadap migrasi bakteri ke arah rongga peritoneum. Namun, pada neonatus atau bayi dengan dinding perut yang sangat tipis, kateter single-cuff sering kali lebih dipilih untuk mencegah ekstrusi manset ke permukaan kulit. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC10223083/) [Sumber 2](http://ispd.org/wp-content/uploads/7.-Dagmara-Borzych-Duzalka-Peritoneal-Dialysis-Catheters-Outcome-in-Children.-The-IPPN-Data.pdf) [Sumber 3](https://kidney.wiki/peritoneal-dialysis/pd-access/) | Catheter Placement: Pedoman klinis terbaru dari Society of American Gastrointestinal and Endoscopic Surgeons (SAGES) menyarankan penggunaan teknik laparoskopi tingkat lanjut (Laparoscopic) dibandingkan teknik bedah terbuka (Open) untuk pemasangan kateter pada populasi pediatrik. Laparoscopic menawarkan akurasi catheter placement yang jauh lebih tinggi di dalam rongga abdomen karena visualisasi langsung, serta meminimalkan trauma mekanis pada jaringan perut. Lebih lanjut, Laparoscopic memungkinkan dokter untuk melakukan prosedur profilaksis penting seperti omentektomi atau omentopeksi untuk meminimalkan risiko omental wrapping (penyumbatan kateter oleh omentum), yang merupakan salah satu penyebab utama kegagalan mekanis kateter pada anak-anak. Laparoscopic juga terbukti mempermudah penyelamatan (salvage) jika terjadi malposisi atau disfungsi kateter tanpa harus melakukan pembedahan ulang yang invasif. [Sumber 1](https://www.sages.org/publications/guidelines/peritoneal-dialysis-access-guideline-update-2023/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC10223083/) [[3]](https://kidney.wiki/peritoneal-dialysis/pd-access/) | Gastrostomy/Intraperitoneal Device:  | Performed CAPD: Tidak ada perbedaan yang signifikan dalam tingkat kelangsungan hidup teknik, kematian, maupun episode peritonitis antara dialisis yang dilakukan sendiri oleh pasien (self-care) dengan dialisis yang dibantu oleh keluarga atau pengasuh (assisted/home-care). Namun, pada populasi anak (khususnya balita atau anak dengan keterbatasan fisik/kognitif), peran orang tua (Parent/Others) sangat mutlak diperlukan. Bagi orang tua yang memiliki tingkat pendidikan rendah atau keterbatasan ekonomi, dialisis tetap dapat berhasil dengan baik tanpa komplikasi besar asalkan diberikan pelatihan intensif secara 1:1, dukungan telepon 24 jam, dan kunjungan rumah berkala oleh perawat dialisis berpengalaman. Di sisi lain, bagi pasien remaja yang melakukan dialisis secara mandiri (Patient), tantangan psikososial seperti kejenuhan (burnout), perasaan terkekang (slavery feeling), dan depresi sering kali muncul, sehingga membutuhkan pengawasan ketat dari tim medis agar kepatuhan terhadap prosedur aseptik tetap terjaga. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/29456210/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC4335934/) [Sumber 3](https://www.ispd.org/wp-content/uploads/2025/12/Assisted-PD-PP-2024-with-VA_formatted.pdf) | Starting PD &lt;2 weeks after catheter placement: Waktu antara pemasangan kateter dan dimulainya dialisis (break-in-period) merupakan faktor penting untuk mencegah komplikasi. Masa penyembuhan minimal 2 minggu sebelum dialysis dimulai. Namun, dalam kondisi klinis tertentu di mana pasien membutuhkan dialisis segera, urgent-start PD (dimulai dalam &lt;14 hari atau bahkan &lt;48 jam) menjadi alternatif yang baik untuk menghindari penggunakan kateter hemodialysis sementara. Pasien dengan break-in-period &lt; 7 hari memiliki risiko yang lebih tinggi terhadap komplikasi awal seperti kebocoran dialisat dan malposisi kateter. Namun, risiko tersebut tidak berkorelasi dengan penurunan kelangsungan hidup atau peningkatan risiko peritonitis jika dilakukan dengan protokol yang tepat. Pada kondisi urgent-start, risiko kebocoran dimitigasi dengan menggunakan volume pengisian rendah (10-20 ml/kg) dan posisi pasien supine untuk mengurangi tekanan intra-abdominal.[Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC3923692/) [Sumber 2](https://journals.plos.org/plosone/article?id=10.1371/journal.pone.0206426) [Sumber 3](https://www.sages.org/publications/guidelines/peritoneal-dialysis-access-guideline-update-2023/) [Sumber 4](https://www.frontiersin.org/journals/endocrinology/articles/10.3389/fendo.2022.936573/full) [Sumber 5](https://scholarlyexchange.childrensmercy.org/cgi/viewcontent.cgi?article=7522&amp;context=papers) [Sumber 6](https://pubmed.ncbi.nlm.nih.gov/33523772/) [Sumber 7](https://www.bcrenal.ca/resource-gallery/Documents/PD_Procedures-Exit_Site_Care-Post-Operative_PD_Catheter_Insertion.pdf) | Catheter Orientation: Posisi atau arah lubang keluar kateter (exit site) sangat memengaruhi risiko terjadinya infeksi. Data multisentrik dari SCOPE Collaborative menunjukkan bahwa orientasi kateter yang menghadap ke atas (Upward) dikaitkan dengan peningkatan risiko peritonitis hingga 4.2 kali lipat (Rate Ratio: 4.2; 95% CI: 1.49–11.89) dibandingkan orientasi lainnya. Secara anatomis, lubang keluar yang menghadap ke atas menciptakan bentuk cekungan yang dapat menampung keringat, air mandi, dan kotoran. Akibat gaya gravitasi, bakteri yang terkumpul di area ini akan mengendap dan bermigrasi ke dalam terowongan kateter. Oleh karena itu, lubang keluar kateter harus selalu diarahkan ke bawah (Downward) atau ke samping (Lateral) untuk mencegah penumpukan bakteri secara alami. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC5012476/) [Sumber 2](https://openurologyandnephrologyjournal.com/VOLUME/5/PAGE/4/) [Sumber 3](https://kidney.wiki/peritoneal-dialysis/pd-access/)</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>2026-05-19 12:44:51</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>18F27E0F</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>&lt;2 yo</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>&gt;12 mo</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>Urban</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>Fair/poor service</t>
+        </is>
+      </c>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>Poor/fair</t>
+        </is>
+      </c>
+      <c r="J114" t="inlineStr">
+        <is>
+          <t>Illiterate</t>
+        </is>
+      </c>
+      <c r="K114" t="inlineStr">
+        <is>
+          <t>ESI</t>
+        </is>
+      </c>
+      <c r="L114" t="inlineStr">
+        <is>
+          <t>Poor nutrition</t>
+        </is>
+      </c>
+      <c r="M114" t="inlineStr">
+        <is>
+          <t>Non-glomerular</t>
+        </is>
+      </c>
+      <c r="N114" t="inlineStr">
+        <is>
+          <t>Straight</t>
+        </is>
+      </c>
+      <c r="O114" t="inlineStr">
+        <is>
+          <t>Single cuff</t>
+        </is>
+      </c>
+      <c r="P114" t="inlineStr">
+        <is>
+          <t>Laparoscopic</t>
+        </is>
+      </c>
+      <c r="Q114" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="R114" t="inlineStr">
+        <is>
+          <t>Parents/others</t>
+        </is>
+      </c>
+      <c r="S114" t="inlineStr"/>
+      <c r="T114" t="inlineStr">
+        <is>
+          <t>upward</t>
+        </is>
+      </c>
+      <c r="U114" t="inlineStr">
+        <is>
+          <t>No stunting</t>
+        </is>
+      </c>
+      <c r="V114" t="inlineStr"/>
+      <c r="W114" t="inlineStr"/>
+      <c r="X114" t="inlineStr"/>
+      <c r="Y114" t="inlineStr">
+        <is>
+          <t>Age*, Gender, Duration of PD*, Place of Residence, Housing, Socioeconomic, Education, Peritonitis in ESI*, Nutrition, Cause of ESRD*, Type of Catheter (Shape), Type of Catheter (Cuff), Catheter Placement, Gastrostomy/Intraperitoneal Device, Performed CAPD, Starting PD &lt;2 weeks after catheter placement, Catheter Orientation</t>
+        </is>
+      </c>
+      <c r="Z114" t="inlineStr">
+        <is>
+          <t>Housing: Lingkungan rumah harus diadaptasi untuk memenuhi standar prosedur medis. Ruangan yang digunakan untuk pertukaran cairan harus bersih dan bebas debu untuk meminimalkan risiko infeksi, sebab partikel debu dapat menjadi vektor bagi patogen udara yang dapat mengontaminasi set transfer saat prosedur koneksi atau diskoneksi. Penyediaan wastafel di dalam atau dekat ruangan dialisis diperlukan untuk memastikan kepatuhan protokol antiseptic tangan sehingga menurunkan insiden peritonitis akibat touch contamination. Pencahayaan yang optimal di dalam ruangan diperlukan agar caregiver dapat memantau kejernihan cairan efluen serta memeriksa kondisi tempat keluar kateter dengan teliti. Hewan peliharaan tidak boleh berada di area perawatan saat proses koneksi atau diskoneksi berlangsung karena risiko paparan bakteri seperti Pasteurella multocida atau kerusakan fisik pada selang dialisis akibat gigitan atau cakaran. Selain itu, caregiverharus ditekankan untuk selalu mencuci tangan setelah berinteraksi dengan hewan dan sebelum memulai prosedur dialisis. [Sumber 1](https://www.freseniuskidneycare.com/treatment/home-dialysis/getting-prepared) [Sumber 2](https://www.ouh.nhs.uk/media/agxhnni2/85713pdialysis.pdf) [Sumber 3](https://www.kidney.org/kidney-topics/preparing-home-dialysis) [Sumber 4](https://spnp-spp.pt/media/rqdpbrom/catheter-related-infections-and-peritonitis-in-pediatric-patients-receiving-peritoneal-dialysis-guideline-for-prevention-and-treatment-2012-1-_compressed-1.pdf) [Sumber 5](https://freseniusmedicalcare.com/content/dam/home-products-education/steps2home-pd/Preventing_Peritonitis.pdf) [Sumber 6](https://www.satellitehealthcare.com/blog/pets-and-peritoneal-dialysis-absolutely/) | Socioeconomic: Deprivasi sosioekonomi berdampak pada hasil treatment yang lebih buruk. Hal ini kemungkinan disebabkan oleh keterbatasan akses terhadap fasilitas sanitasi yang memadai, tekanan psikologis pada pengasuh, serta keterbatasan informasi medis. Strategi bisa dilakukan melalui program pelatihan bagi keluarga (caregiver) dari perawat dialisis yang berpengalaman. Bagi keluarga dengan keterbatasan pendidikan atau ekonomi, dukungan teknis telepon 24 jam dan kunjungan rumah secara berkala oleh tim medis sosial sangat efektif dalam memastikan kepatuhan terhadap prosedur aseptik. Pelatihan ulang sangat dianjurkan, terutama setelah terjadinya peritonitis, untuk mengidentifikasi adanya penyimpangan dalam teknik pertukaran cairan. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC11835194/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC4934433/) [Sumber 3](https://pubmed.ncbi.nlm.nih.gov/23226378/) [Sumber 4](https://pubmed.ncbi.nlm.nih.gov/16091376/) [Sumber 6](https://spnp-spp.pt/media/rqdpbrom/catheter-related-infections-and-peritonitis-in-pediatric-patients-receiving-peritoneal-dialysis-guideline-for-prevention-and-treatment-2012-1-_compressed-1.pdf) [Sumber 7](https://pmc.ncbi.nlm.nih.gov/articles/PMC5691857/) [Sumber 8](https://pmc.ncbi.nlm.nih.gov/articles/PMC4335934/) [Sumber 9](https://www.kidney.org/kidney-topics/preparing-home-dialysis) | Peritonitis in ESI: Penggunaan antibiotik topikal secara rutin pada tempat keluar kateter telat terbukti menurunkan angka infeksi. Aplikasi harian salep mupirocin atau gentamicin pada exit-site direkomendasikan untuk menekan kolonisasi Staphylococcus aureus dan Pseudomonas aeruginosa.Pembersihan area secara rutin dengan larutan antiseptik non-iritan (seperti chlorhexidine 0,05% atau sabun antibakteri ringan) juga merupakan bagian standar dari perawatan. Penilaian kondisi exit-site secara objektif menggunakan sistem skor (seperti Skor ISPD yang mencakup pembengkakan, kerak, kemerahan, nyeri, dan sekret) sangat membantu caregiver dalam mendeteksi infeksi secara dini. Immobilisasi kateter dengan menggunakan plester atau perangkat fiksasi sangat krusial karena trauma mekanis pada tempat keluar sering kali menjadi pintu masuk bagi bakteri. Jika ESI terjadi, terapi antibiotik oral atau intraperitoneal harus dimulai segera dan dilanjutkan selama minimal 2 minggu, atau 3 minggu jika disebabkan oleh Pseudomonas. Pengangkatan kateter mungkin diperlukan jika infeksi bersifat refrakter (tidak merespons pengobatan setelah 2 minggu) atau jika infeksi telah menyebar ke terowongan kateter (tunnel infection) yang menyebabkan peritonitis berulang. [Sumber 1](https://ispd.org/wp-content/uploads/2025/09/LI-ET-1.pdf) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC12640025/) [Sumber 3](https://pmc.ncbi.nlm.nih.gov/articles/PMC5033625/) [Sumber 4](https://www.chikd.org/journal/view.php?number=726) [Sumber 5](https://ispd.org/wp-content/uploads/ISPD-Catheter-related-Infection-Recommendations-2023-Update.pdf) [Sumber 6](https://www.bcrenal.ca/resource-gallery/Documents/PD_Procedures-Exit_Site_Care-Post-Operative_PD_Catheter_Insertion.pdf) [Sumber 7](https://davita.com/treatment-options/articles/preventing-catheter-infections-on-peritoneal-dialysis/) [Sumber 8](https://edren.org/ren/handbook/pd-handbook/protocol-for-the-management-of-pd-peritonitis-long-version/) | Nutrition: Malnutrisi protein-kalori (cachexia) adalah masalah umum pada anak yang menjalani PD. Manajemen nutrisi bertujuan untuk mengejar pertumbuhan dan mengganti hilangnya protein serta asam amino ke dalam cairan dialysis.Penilaian status nutrisi harus dilakukan secara berkala, minimal setiap bulan pada bayi dan 3-4 bulan pada anak yang lebih tua, menggunakan parameter antropometri (berat badan, tinggi badan, lingkar kepala), biokimia (albumin urea), dan analisis bioimpedansi jika tersedia. Penanganannya juga harus multidisiplin dan mencakup memastikan asupan energi dan protein yang adekuat; kontrol metabolik yang optimal, dengan koreksi asidosis, anemia, dan hiperparatiroidisme; dosis dialisis yang optimal (atau setidaknya adekuat); dan, jika perlu, pemberian obat-obatan tertentu seperti hormon pertumbuhan manusia rekombinan. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) | Type of Catheter (Shape): Perdebatan mengenai efektivitas kateter straight dibandingkan dengan kateter coiled/curled masih berlangsung. Kateter coiled secara teoretis mengurangi nyeri saat pengisian cairan dan meminimalkan trauma pada organ visceral, tetapi beberapa data menunjukkan risiko malposisi yang lebih tinggi dibandingkan tipe lurus pada beberapa kelompok pasien. Di sisi lain, kateter straight lebih mudah ditempatkan pada bayi kecil yang memiliki ruang intra-abdominal terbatas. Secara keseluruhan, pedoman tidak menyatakan superioritas mutlak salah satu bentuk, dan pemilihan sering kali bergantung pada preferensi pusat dialisis dan anatomi pasien. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC9365012/) [Sumber 2](http://ispd.org/wp-content/uploads/7.-Dagmara-Borzych-Duzalka-Peritoneal-Dialysis-Catheters-Outcome-in-Children.-The-IPPN-Data.pdf) [Sumber 3](https://scholarlyexchange.childrensmercy.org/cgi/viewcontent.cgi?article=7522&amp;context=papers) [Sumber 4](https://kidney.wiki/peritoneal-dialysis/pd-access/) | Type of Catheter (Cuff): Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff)untuk populasi anak secara umum. Deep cuff berfungsi untuk menjangkar kateter di otot rektus dan mencegah kebocoran, sementara superficial cuff bertindak sebagai penghalang fisik terhadap migrasi bakteri ke arah rongga peritoneum. Namun, pada neonatus atau bayi dengan dinding perut yang sangat tipis, kateter single-cuff sering kali lebih dipilih untuk mencegah ekstrusi manset ke permukaan kulit. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC10223083/) [Sumber 2](http://ispd.org/wp-content/uploads/7.-Dagmara-Borzych-Duzalka-Peritoneal-Dialysis-Catheters-Outcome-in-Children.-The-IPPN-Data.pdf) [Sumber 3](https://kidney.wiki/peritoneal-dialysis/pd-access/) | Catheter Placement: Pedoman klinis terbaru dari Society of American Gastrointestinal and Endoscopic Surgeons (SAGES) menyarankan penggunaan teknik laparoskopi tingkat lanjut (Laparoscopic) dibandingkan teknik bedah terbuka (Open) untuk pemasangan kateter pada populasi pediatrik. Laparoscopic menawarkan akurasi catheter placement yang jauh lebih tinggi di dalam rongga abdomen karena visualisasi langsung, serta meminimalkan trauma mekanis pada jaringan perut. Lebih lanjut, Laparoscopic memungkinkan dokter untuk melakukan prosedur profilaksis penting seperti omentektomi atau omentopeksi untuk meminimalkan risiko omental wrapping (penyumbatan kateter oleh omentum), yang merupakan salah satu penyebab utama kegagalan mekanis kateter pada anak-anak. Laparoscopic juga terbukti mempermudah penyelamatan (salvage) jika terjadi malposisi atau disfungsi kateter tanpa harus melakukan pembedahan ulang yang invasif. [Sumber 1](https://www.sages.org/publications/guidelines/peritoneal-dialysis-access-guideline-update-2023/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC10223083/) [[3]](https://kidney.wiki/peritoneal-dialysis/pd-access/) | Gastrostomy/Intraperitoneal Device:  | Performed CAPD: Tidak ada perbedaan yang signifikan dalam tingkat kelangsungan hidup teknik, kematian, maupun episode peritonitis antara dialisis yang dilakukan sendiri oleh pasien (self-care) dengan dialisis yang dibantu oleh keluarga atau pengasuh (assisted/home-care). Namun, pada populasi anak (khususnya balita atau anak dengan keterbatasan fisik/kognitif), peran orang tua (Parent/Others) sangat mutlak diperlukan. Bagi orang tua yang memiliki tingkat pendidikan rendah atau keterbatasan ekonomi, dialisis tetap dapat berhasil dengan baik tanpa komplikasi besar asalkan diberikan pelatihan intensif secara 1:1, dukungan telepon 24 jam, dan kunjungan rumah berkala oleh perawat dialisis berpengalaman. Di sisi lain, bagi pasien remaja yang melakukan dialisis secara mandiri (Patient), tantangan psikososial seperti kejenuhan (burnout), perasaan terkekang (slavery feeling), dan depresi sering kali muncul, sehingga membutuhkan pengawasan ketat dari tim medis agar kepatuhan terhadap prosedur aseptik tetap terjaga. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/29456210/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC4335934/) [Sumber 3](https://www.ispd.org/wp-content/uploads/2025/12/Assisted-PD-PP-2024-with-VA_formatted.pdf) | Starting PD &lt;2 weeks after catheter placement: Waktu antara pemasangan kateter dan dimulainya dialisis (break-in-period) merupakan faktor penting untuk mencegah komplikasi. Masa penyembuhan minimal 2 minggu sebelum dialysis dimulai. Namun, dalam kondisi klinis tertentu di mana pasien membutuhkan dialisis segera, urgent-start PD (dimulai dalam &lt;14 hari atau bahkan &lt;48 jam) menjadi alternatif yang baik untuk menghindari penggunakan kateter hemodialysis sementara. Pasien dengan break-in-period &lt; 7 hari memiliki risiko yang lebih tinggi terhadap komplikasi awal seperti kebocoran dialisat dan malposisi kateter. Namun, risiko tersebut tidak berkorelasi dengan penurunan kelangsungan hidup atau peningkatan risiko peritonitis jika dilakukan dengan protokol yang tepat. Pada kondisi urgent-start, risiko kebocoran dimitigasi dengan menggunakan volume pengisian rendah (10-20 ml/kg) dan posisi pasien supine untuk mengurangi tekanan intra-abdominal.[Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC3923692/) [Sumber 2](https://journals.plos.org/plosone/article?id=10.1371/journal.pone.0206426) [Sumber 3](https://www.sages.org/publications/guidelines/peritoneal-dialysis-access-guideline-update-2023/) [Sumber 4](https://www.frontiersin.org/journals/endocrinology/articles/10.3389/fendo.2022.936573/full) [Sumber 5](https://scholarlyexchange.childrensmercy.org/cgi/viewcontent.cgi?article=7522&amp;context=papers) [Sumber 6](https://pubmed.ncbi.nlm.nih.gov/33523772/) [Sumber 7](https://www.bcrenal.ca/resource-gallery/Documents/PD_Procedures-Exit_Site_Care-Post-Operative_PD_Catheter_Insertion.pdf) | Catheter Orientation: Posisi atau arah lubang keluar kateter (exit site) sangat memengaruhi risiko terjadinya infeksi. Data multisentrik dari SCOPE Collaborative menunjukkan bahwa orientasi kateter yang menghadap ke atas (Upward) dikaitkan dengan peningkatan risiko peritonitis hingga 4.2 kali lipat (Rate Ratio: 4.2; 95% CI: 1.49–11.89) dibandingkan orientasi lainnya. Secara anatomis, lubang keluar yang menghadap ke atas menciptakan bentuk cekungan yang dapat menampung keringat, air mandi, dan kotoran. Akibat gaya gravitasi, bakteri yang terkumpul di area ini akan mengendap dan bermigrasi ke dalam terowongan kateter. Oleh karena itu, lubang keluar kateter harus selalu diarahkan ke bawah (Downward) atau ke samping (Lateral) untuk mencegah penumpukan bakteri secara alami. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC5012476/) [Sumber 2](https://openurologyandnephrologyjournal.com/VOLUME/5/PAGE/4/) [Sumber 3](https://kidney.wiki/peritoneal-dialysis/pd-access/)</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>2026-05-19 12:45:01</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>18F27E0F</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>&lt;2 yo</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>&gt;12 mo</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>Urban</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>Fair/poor service</t>
+        </is>
+      </c>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>Poor/fair</t>
+        </is>
+      </c>
+      <c r="J115" t="inlineStr">
+        <is>
+          <t>Illiterate</t>
+        </is>
+      </c>
+      <c r="K115" t="inlineStr">
+        <is>
+          <t>ESI</t>
+        </is>
+      </c>
+      <c r="L115" t="inlineStr">
+        <is>
+          <t>Normal Nutrition</t>
+        </is>
+      </c>
+      <c r="M115" t="inlineStr">
+        <is>
+          <t>Non-glomerular</t>
+        </is>
+      </c>
+      <c r="N115" t="inlineStr">
+        <is>
+          <t>Straight</t>
+        </is>
+      </c>
+      <c r="O115" t="inlineStr">
+        <is>
+          <t>Single cuff</t>
+        </is>
+      </c>
+      <c r="P115" t="inlineStr">
+        <is>
+          <t>Laparoscopic</t>
+        </is>
+      </c>
+      <c r="Q115" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="R115" t="inlineStr">
+        <is>
+          <t>Parents/others</t>
+        </is>
+      </c>
+      <c r="S115" t="inlineStr"/>
+      <c r="T115" t="inlineStr">
+        <is>
+          <t>upward</t>
+        </is>
+      </c>
+      <c r="U115" t="inlineStr">
+        <is>
+          <t>No stunting</t>
+        </is>
+      </c>
+      <c r="V115" t="inlineStr"/>
+      <c r="W115" t="inlineStr"/>
+      <c r="X115" t="inlineStr"/>
+      <c r="Y115" t="inlineStr">
+        <is>
+          <t>Age*, Gender, Duration of PD*, Place of Residence, Housing, Socioeconomic, Education, Peritonitis in ESI*, Cause of ESRD*, Type of Catheter (Shape), Type of Catheter (Cuff), Catheter Placement, Gastrostomy/Intraperitoneal Device, Performed CAPD, Starting PD &lt;2 weeks after catheter placement, Catheter Orientation</t>
+        </is>
+      </c>
+      <c r="Z115" t="inlineStr">
+        <is>
+          <t>Housing: Lingkungan rumah harus diadaptasi untuk memenuhi standar prosedur medis. Ruangan yang digunakan untuk pertukaran cairan harus bersih dan bebas debu untuk meminimalkan risiko infeksi, sebab partikel debu dapat menjadi vektor bagi patogen udara yang dapat mengontaminasi set transfer saat prosedur koneksi atau diskoneksi. Penyediaan wastafel di dalam atau dekat ruangan dialisis diperlukan untuk memastikan kepatuhan protokol antiseptic tangan sehingga menurunkan insiden peritonitis akibat touch contamination. Pencahayaan yang optimal di dalam ruangan diperlukan agar caregiver dapat memantau kejernihan cairan efluen serta memeriksa kondisi tempat keluar kateter dengan teliti. Hewan peliharaan tidak boleh berada di area perawatan saat proses koneksi atau diskoneksi berlangsung karena risiko paparan bakteri seperti Pasteurella multocida atau kerusakan fisik pada selang dialisis akibat gigitan atau cakaran. Selain itu, caregiverharus ditekankan untuk selalu mencuci tangan setelah berinteraksi dengan hewan dan sebelum memulai prosedur dialisis. [Sumber 1](https://www.freseniuskidneycare.com/treatment/home-dialysis/getting-prepared) [Sumber 2](https://www.ouh.nhs.uk/media/agxhnni2/85713pdialysis.pdf) [Sumber 3](https://www.kidney.org/kidney-topics/preparing-home-dialysis) [Sumber 4](https://spnp-spp.pt/media/rqdpbrom/catheter-related-infections-and-peritonitis-in-pediatric-patients-receiving-peritoneal-dialysis-guideline-for-prevention-and-treatment-2012-1-_compressed-1.pdf) [Sumber 5](https://freseniusmedicalcare.com/content/dam/home-products-education/steps2home-pd/Preventing_Peritonitis.pdf) [Sumber 6](https://www.satellitehealthcare.com/blog/pets-and-peritoneal-dialysis-absolutely/) | Socioeconomic: Deprivasi sosioekonomi berdampak pada hasil treatment yang lebih buruk. Hal ini kemungkinan disebabkan oleh keterbatasan akses terhadap fasilitas sanitasi yang memadai, tekanan psikologis pada pengasuh, serta keterbatasan informasi medis. Strategi bisa dilakukan melalui program pelatihan bagi keluarga (caregiver) dari perawat dialisis yang berpengalaman. Bagi keluarga dengan keterbatasan pendidikan atau ekonomi, dukungan teknis telepon 24 jam dan kunjungan rumah secara berkala oleh tim medis sosial sangat efektif dalam memastikan kepatuhan terhadap prosedur aseptik. Pelatihan ulang sangat dianjurkan, terutama setelah terjadinya peritonitis, untuk mengidentifikasi adanya penyimpangan dalam teknik pertukaran cairan. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC11835194/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC4934433/) [Sumber 3](https://pubmed.ncbi.nlm.nih.gov/23226378/) [Sumber 4](https://pubmed.ncbi.nlm.nih.gov/16091376/) [Sumber 6](https://spnp-spp.pt/media/rqdpbrom/catheter-related-infections-and-peritonitis-in-pediatric-patients-receiving-peritoneal-dialysis-guideline-for-prevention-and-treatment-2012-1-_compressed-1.pdf) [Sumber 7](https://pmc.ncbi.nlm.nih.gov/articles/PMC5691857/) [Sumber 8](https://pmc.ncbi.nlm.nih.gov/articles/PMC4335934/) [Sumber 9](https://www.kidney.org/kidney-topics/preparing-home-dialysis) | Peritonitis in ESI: Penggunaan antibiotik topikal secara rutin pada tempat keluar kateter telat terbukti menurunkan angka infeksi. Aplikasi harian salep mupirocin atau gentamicin pada exit-site direkomendasikan untuk menekan kolonisasi Staphylococcus aureus dan Pseudomonas aeruginosa.Pembersihan area secara rutin dengan larutan antiseptik non-iritan (seperti chlorhexidine 0,05% atau sabun antibakteri ringan) juga merupakan bagian standar dari perawatan. Penilaian kondisi exit-site secara objektif menggunakan sistem skor (seperti Skor ISPD yang mencakup pembengkakan, kerak, kemerahan, nyeri, dan sekret) sangat membantu caregiver dalam mendeteksi infeksi secara dini. Immobilisasi kateter dengan menggunakan plester atau perangkat fiksasi sangat krusial karena trauma mekanis pada tempat keluar sering kali menjadi pintu masuk bagi bakteri. Jika ESI terjadi, terapi antibiotik oral atau intraperitoneal harus dimulai segera dan dilanjutkan selama minimal 2 minggu, atau 3 minggu jika disebabkan oleh Pseudomonas. Pengangkatan kateter mungkin diperlukan jika infeksi bersifat refrakter (tidak merespons pengobatan setelah 2 minggu) atau jika infeksi telah menyebar ke terowongan kateter (tunnel infection) yang menyebabkan peritonitis berulang. [Sumber 1](https://ispd.org/wp-content/uploads/2025/09/LI-ET-1.pdf) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC12640025/) [Sumber 3](https://pmc.ncbi.nlm.nih.gov/articles/PMC5033625/) [Sumber 4](https://www.chikd.org/journal/view.php?number=726) [Sumber 5](https://ispd.org/wp-content/uploads/ISPD-Catheter-related-Infection-Recommendations-2023-Update.pdf) [Sumber 6](https://www.bcrenal.ca/resource-gallery/Documents/PD_Procedures-Exit_Site_Care-Post-Operative_PD_Catheter_Insertion.pdf) [Sumber 7](https://davita.com/treatment-options/articles/preventing-catheter-infections-on-peritoneal-dialysis/) [Sumber 8](https://edren.org/ren/handbook/pd-handbook/protocol-for-the-management-of-pd-peritonitis-long-version/) | Type of Catheter (Shape): Perdebatan mengenai efektivitas kateter straight dibandingkan dengan kateter coiled/curled masih berlangsung. Kateter coiled secara teoretis mengurangi nyeri saat pengisian cairan dan meminimalkan trauma pada organ visceral, tetapi beberapa data menunjukkan risiko malposisi yang lebih tinggi dibandingkan tipe lurus pada beberapa kelompok pasien. Di sisi lain, kateter straight lebih mudah ditempatkan pada bayi kecil yang memiliki ruang intra-abdominal terbatas. Secara keseluruhan, pedoman tidak menyatakan superioritas mutlak salah satu bentuk, dan pemilihan sering kali bergantung pada preferensi pusat dialisis dan anatomi pasien. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC9365012/) [Sumber 2](http://ispd.org/wp-content/uploads/7.-Dagmara-Borzych-Duzalka-Peritoneal-Dialysis-Catheters-Outcome-in-Children.-The-IPPN-Data.pdf) [Sumber 3](https://scholarlyexchange.childrensmercy.org/cgi/viewcontent.cgi?article=7522&amp;context=papers) [Sumber 4](https://kidney.wiki/peritoneal-dialysis/pd-access/) | Type of Catheter (Cuff): Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff)untuk populasi anak secara umum. Deep cuff berfungsi untuk menjangkar kateter di otot rektus dan mencegah kebocoran, sementara superficial cuff bertindak sebagai penghalang fisik terhadap migrasi bakteri ke arah rongga peritoneum. Namun, pada neonatus atau bayi dengan dinding perut yang sangat tipis, kateter single-cuff sering kali lebih dipilih untuk mencegah ekstrusi manset ke permukaan kulit. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC10223083/) [Sumber 2](http://ispd.org/wp-content/uploads/7.-Dagmara-Borzych-Duzalka-Peritoneal-Dialysis-Catheters-Outcome-in-Children.-The-IPPN-Data.pdf) [Sumber 3](https://kidney.wiki/peritoneal-dialysis/pd-access/) | Catheter Placement: Pedoman klinis terbaru dari Society of American Gastrointestinal and Endoscopic Surgeons (SAGES) menyarankan penggunaan teknik laparoskopi tingkat lanjut (Laparoscopic) dibandingkan teknik bedah terbuka (Open) untuk pemasangan kateter pada populasi pediatrik. Laparoscopic menawarkan akurasi catheter placement yang jauh lebih tinggi di dalam rongga abdomen karena visualisasi langsung, serta meminimalkan trauma mekanis pada jaringan perut. Lebih lanjut, Laparoscopic memungkinkan dokter untuk melakukan prosedur profilaksis penting seperti omentektomi atau omentopeksi untuk meminimalkan risiko omental wrapping (penyumbatan kateter oleh omentum), yang merupakan salah satu penyebab utama kegagalan mekanis kateter pada anak-anak. Laparoscopic juga terbukti mempermudah penyelamatan (salvage) jika terjadi malposisi atau disfungsi kateter tanpa harus melakukan pembedahan ulang yang invasif. [Sumber 1](https://www.sages.org/publications/guidelines/peritoneal-dialysis-access-guideline-update-2023/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC10223083/) [[3]](https://kidney.wiki/peritoneal-dialysis/pd-access/) | Gastrostomy/Intraperitoneal Device:  | Performed CAPD: Tidak ada perbedaan yang signifikan dalam tingkat kelangsungan hidup teknik, kematian, maupun episode peritonitis antara dialisis yang dilakukan sendiri oleh pasien (self-care) dengan dialisis yang dibantu oleh keluarga atau pengasuh (assisted/home-care). Namun, pada populasi anak (khususnya balita atau anak dengan keterbatasan fisik/kognitif), peran orang tua (Parent/Others) sangat mutlak diperlukan. Bagi orang tua yang memiliki tingkat pendidikan rendah atau keterbatasan ekonomi, dialisis tetap dapat berhasil dengan baik tanpa komplikasi besar asalkan diberikan pelatihan intensif secara 1:1, dukungan telepon 24 jam, dan kunjungan rumah berkala oleh perawat dialisis berpengalaman. Di sisi lain, bagi pasien remaja yang melakukan dialisis secara mandiri (Patient), tantangan psikososial seperti kejenuhan (burnout), perasaan terkekang (slavery feeling), dan depresi sering kali muncul, sehingga membutuhkan pengawasan ketat dari tim medis agar kepatuhan terhadap prosedur aseptik tetap terjaga. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/29456210/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC4335934/) [Sumber 3](https://www.ispd.org/wp-content/uploads/2025/12/Assisted-PD-PP-2024-with-VA_formatted.pdf) | Starting PD &lt;2 weeks after catheter placement: Waktu antara pemasangan kateter dan dimulainya dialisis (break-in-period) merupakan faktor penting untuk mencegah komplikasi. Masa penyembuhan minimal 2 minggu sebelum dialysis dimulai. Namun, dalam kondisi klinis tertentu di mana pasien membutuhkan dialisis segera, urgent-start PD (dimulai dalam &lt;14 hari atau bahkan &lt;48 jam) menjadi alternatif yang baik untuk menghindari penggunakan kateter hemodialysis sementara. Pasien dengan break-in-period &lt; 7 hari memiliki risiko yang lebih tinggi terhadap komplikasi awal seperti kebocoran dialisat dan malposisi kateter. Namun, risiko tersebut tidak berkorelasi dengan penurunan kelangsungan hidup atau peningkatan risiko peritonitis jika dilakukan dengan protokol yang tepat. Pada kondisi urgent-start, risiko kebocoran dimitigasi dengan menggunakan volume pengisian rendah (10-20 ml/kg) dan posisi pasien supine untuk mengurangi tekanan intra-abdominal.[Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC3923692/) [Sumber 2](https://journals.plos.org/plosone/article?id=10.1371/journal.pone.0206426) [Sumber 3](https://www.sages.org/publications/guidelines/peritoneal-dialysis-access-guideline-update-2023/) [Sumber 4](https://www.frontiersin.org/journals/endocrinology/articles/10.3389/fendo.2022.936573/full) [Sumber 5](https://scholarlyexchange.childrensmercy.org/cgi/viewcontent.cgi?article=7522&amp;context=papers) [Sumber 6](https://pubmed.ncbi.nlm.nih.gov/33523772/) [Sumber 7](https://www.bcrenal.ca/resource-gallery/Documents/PD_Procedures-Exit_Site_Care-Post-Operative_PD_Catheter_Insertion.pdf) | Catheter Orientation: Posisi atau arah lubang keluar kateter (exit site) sangat memengaruhi risiko terjadinya infeksi. Data multisentrik dari SCOPE Collaborative menunjukkan bahwa orientasi kateter yang menghadap ke atas (Upward) dikaitkan dengan peningkatan risiko peritonitis hingga 4.2 kali lipat (Rate Ratio: 4.2; 95% CI: 1.49–11.89) dibandingkan orientasi lainnya. Secara anatomis, lubang keluar yang menghadap ke atas menciptakan bentuk cekungan yang dapat menampung keringat, air mandi, dan kotoran. Akibat gaya gravitasi, bakteri yang terkumpul di area ini akan mengendap dan bermigrasi ke dalam terowongan kateter. Oleh karena itu, lubang keluar kateter harus selalu diarahkan ke bawah (Downward) atau ke samping (Lateral) untuk mencegah penumpukan bakteri secara alami. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC5012476/) [Sumber 2](https://openurologyandnephrologyjournal.com/VOLUME/5/PAGE/4/) [Sumber 3](https://kidney.wiki/peritoneal-dialysis/pd-access/)</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>2026-05-19 12:45:07</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>18F27E0F</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>&lt;2 yo</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>&gt;12 mo</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>Fair/poor service</t>
+        </is>
+      </c>
+      <c r="I116" t="inlineStr">
+        <is>
+          <t>Poor/fair</t>
+        </is>
+      </c>
+      <c r="J116" t="inlineStr">
+        <is>
+          <t>Illiterate</t>
+        </is>
+      </c>
+      <c r="K116" t="inlineStr">
+        <is>
+          <t>ESI</t>
+        </is>
+      </c>
+      <c r="L116" t="inlineStr">
+        <is>
+          <t>Normal Nutrition</t>
+        </is>
+      </c>
+      <c r="M116" t="inlineStr">
+        <is>
+          <t>Non-glomerular</t>
+        </is>
+      </c>
+      <c r="N116" t="inlineStr">
+        <is>
+          <t>Straight</t>
+        </is>
+      </c>
+      <c r="O116" t="inlineStr">
+        <is>
+          <t>Single cuff</t>
+        </is>
+      </c>
+      <c r="P116" t="inlineStr">
+        <is>
+          <t>Laparoscopic</t>
+        </is>
+      </c>
+      <c r="Q116" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="R116" t="inlineStr">
+        <is>
+          <t>Parents/others</t>
+        </is>
+      </c>
+      <c r="S116" t="inlineStr"/>
+      <c r="T116" t="inlineStr">
+        <is>
+          <t>upward</t>
+        </is>
+      </c>
+      <c r="U116" t="inlineStr">
+        <is>
+          <t>No stunting</t>
+        </is>
+      </c>
+      <c r="V116" t="inlineStr"/>
+      <c r="W116" t="inlineStr"/>
+      <c r="X116" t="inlineStr"/>
+      <c r="Y116" t="inlineStr">
+        <is>
+          <t>Age*, Gender, Duration of PD*, Housing, Socioeconomic, Education, Peritonitis in ESI*, Cause of ESRD*, Type of Catheter (Shape), Type of Catheter (Cuff), Catheter Placement, Gastrostomy/Intraperitoneal Device, Performed CAPD, Starting PD &lt;2 weeks after catheter placement, Catheter Orientation</t>
+        </is>
+      </c>
+      <c r="Z116" t="inlineStr">
+        <is>
+          <t>Housing: Lingkungan rumah harus diadaptasi untuk memenuhi standar prosedur medis. Ruangan yang digunakan untuk pertukaran cairan harus bersih dan bebas debu untuk meminimalkan risiko infeksi, sebab partikel debu dapat menjadi vektor bagi patogen udara yang dapat mengontaminasi set transfer saat prosedur koneksi atau diskoneksi. Penyediaan wastafel di dalam atau dekat ruangan dialisis diperlukan untuk memastikan kepatuhan protokol antiseptic tangan sehingga menurunkan insiden peritonitis akibat touch contamination. Pencahayaan yang optimal di dalam ruangan diperlukan agar caregiver dapat memantau kejernihan cairan efluen serta memeriksa kondisi tempat keluar kateter dengan teliti. Hewan peliharaan tidak boleh berada di area perawatan saat proses koneksi atau diskoneksi berlangsung karena risiko paparan bakteri seperti Pasteurella multocida atau kerusakan fisik pada selang dialisis akibat gigitan atau cakaran. Selain itu, caregiverharus ditekankan untuk selalu mencuci tangan setelah berinteraksi dengan hewan dan sebelum memulai prosedur dialisis. [Sumber 1](https://www.freseniuskidneycare.com/treatment/home-dialysis/getting-prepared) [Sumber 2](https://www.ouh.nhs.uk/media/agxhnni2/85713pdialysis.pdf) [Sumber 3](https://www.kidney.org/kidney-topics/preparing-home-dialysis) [Sumber 4](https://spnp-spp.pt/media/rqdpbrom/catheter-related-infections-and-peritonitis-in-pediatric-patients-receiving-peritoneal-dialysis-guideline-for-prevention-and-treatment-2012-1-_compressed-1.pdf) [Sumber 5](https://freseniusmedicalcare.com/content/dam/home-products-education/steps2home-pd/Preventing_Peritonitis.pdf) [Sumber 6](https://www.satellitehealthcare.com/blog/pets-and-peritoneal-dialysis-absolutely/) | Socioeconomic: Deprivasi sosioekonomi berdampak pada hasil treatment yang lebih buruk. Hal ini kemungkinan disebabkan oleh keterbatasan akses terhadap fasilitas sanitasi yang memadai, tekanan psikologis pada pengasuh, serta keterbatasan informasi medis. Strategi bisa dilakukan melalui program pelatihan bagi keluarga (caregiver) dari perawat dialisis yang berpengalaman. Bagi keluarga dengan keterbatasan pendidikan atau ekonomi, dukungan teknis telepon 24 jam dan kunjungan rumah secara berkala oleh tim medis sosial sangat efektif dalam memastikan kepatuhan terhadap prosedur aseptik. Pelatihan ulang sangat dianjurkan, terutama setelah terjadinya peritonitis, untuk mengidentifikasi adanya penyimpangan dalam teknik pertukaran cairan. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC11835194/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC4934433/) [Sumber 3](https://pubmed.ncbi.nlm.nih.gov/23226378/) [Sumber 4](https://pubmed.ncbi.nlm.nih.gov/16091376/) [Sumber 6](https://spnp-spp.pt/media/rqdpbrom/catheter-related-infections-and-peritonitis-in-pediatric-patients-receiving-peritoneal-dialysis-guideline-for-prevention-and-treatment-2012-1-_compressed-1.pdf) [Sumber 7](https://pmc.ncbi.nlm.nih.gov/articles/PMC5691857/) [Sumber 8](https://pmc.ncbi.nlm.nih.gov/articles/PMC4335934/) [Sumber 9](https://www.kidney.org/kidney-topics/preparing-home-dialysis) | Peritonitis in ESI: Penggunaan antibiotik topikal secara rutin pada tempat keluar kateter telat terbukti menurunkan angka infeksi. Aplikasi harian salep mupirocin atau gentamicin pada exit-site direkomendasikan untuk menekan kolonisasi Staphylococcus aureus dan Pseudomonas aeruginosa.Pembersihan area secara rutin dengan larutan antiseptik non-iritan (seperti chlorhexidine 0,05% atau sabun antibakteri ringan) juga merupakan bagian standar dari perawatan. Penilaian kondisi exit-site secara objektif menggunakan sistem skor (seperti Skor ISPD yang mencakup pembengkakan, kerak, kemerahan, nyeri, dan sekret) sangat membantu caregiver dalam mendeteksi infeksi secara dini. Immobilisasi kateter dengan menggunakan plester atau perangkat fiksasi sangat krusial karena trauma mekanis pada tempat keluar sering kali menjadi pintu masuk bagi bakteri. Jika ESI terjadi, terapi antibiotik oral atau intraperitoneal harus dimulai segera dan dilanjutkan selama minimal 2 minggu, atau 3 minggu jika disebabkan oleh Pseudomonas. Pengangkatan kateter mungkin diperlukan jika infeksi bersifat refrakter (tidak merespons pengobatan setelah 2 minggu) atau jika infeksi telah menyebar ke terowongan kateter (tunnel infection) yang menyebabkan peritonitis berulang. [Sumber 1](https://ispd.org/wp-content/uploads/2025/09/LI-ET-1.pdf) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC12640025/) [Sumber 3](https://pmc.ncbi.nlm.nih.gov/articles/PMC5033625/) [Sumber 4](https://www.chikd.org/journal/view.php?number=726) [Sumber 5](https://ispd.org/wp-content/uploads/ISPD-Catheter-related-Infection-Recommendations-2023-Update.pdf) [Sumber 6](https://www.bcrenal.ca/resource-gallery/Documents/PD_Procedures-Exit_Site_Care-Post-Operative_PD_Catheter_Insertion.pdf) [Sumber 7](https://davita.com/treatment-options/articles/preventing-catheter-infections-on-peritoneal-dialysis/) [Sumber 8](https://edren.org/ren/handbook/pd-handbook/protocol-for-the-management-of-pd-peritonitis-long-version/) | Type of Catheter (Shape): Perdebatan mengenai efektivitas kateter straight dibandingkan dengan kateter coiled/curled masih berlangsung. Kateter coiled secara teoretis mengurangi nyeri saat pengisian cairan dan meminimalkan trauma pada organ visceral, tetapi beberapa data menunjukkan risiko malposisi yang lebih tinggi dibandingkan tipe lurus pada beberapa kelompok pasien. Di sisi lain, kateter straight lebih mudah ditempatkan pada bayi kecil yang memiliki ruang intra-abdominal terbatas. Secara keseluruhan, pedoman tidak menyatakan superioritas mutlak salah satu bentuk, dan pemilihan sering kali bergantung pada preferensi pusat dialisis dan anatomi pasien. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC9365012/) [Sumber 2](http://ispd.org/wp-content/uploads/7.-Dagmara-Borzych-Duzalka-Peritoneal-Dialysis-Catheters-Outcome-in-Children.-The-IPPN-Data.pdf) [Sumber 3](https://scholarlyexchange.childrensmercy.org/cgi/viewcontent.cgi?article=7522&amp;context=papers) [Sumber 4](https://kidney.wiki/peritoneal-dialysis/pd-access/) | Type of Catheter (Cuff): Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff)untuk populasi anak secara umum. Deep cuff berfungsi untuk menjangkar kateter di otot rektus dan mencegah kebocoran, sementara superficial cuff bertindak sebagai penghalang fisik terhadap migrasi bakteri ke arah rongga peritoneum. Namun, pada neonatus atau bayi dengan dinding perut yang sangat tipis, kateter single-cuff sering kali lebih dipilih untuk mencegah ekstrusi manset ke permukaan kulit. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC10223083/) [Sumber 2](http://ispd.org/wp-content/uploads/7.-Dagmara-Borzych-Duzalka-Peritoneal-Dialysis-Catheters-Outcome-in-Children.-The-IPPN-Data.pdf) [Sumber 3](https://kidney.wiki/peritoneal-dialysis/pd-access/) | Catheter Placement: Pedoman klinis terbaru dari Society of American Gastrointestinal and Endoscopic Surgeons (SAGES) menyarankan penggunaan teknik laparoskopi tingkat lanjut (Laparoscopic) dibandingkan teknik bedah terbuka (Open) untuk pemasangan kateter pada populasi pediatrik. Laparoscopic menawarkan akurasi catheter placement yang jauh lebih tinggi di dalam rongga abdomen karena visualisasi langsung, serta meminimalkan trauma mekanis pada jaringan perut. Lebih lanjut, Laparoscopic memungkinkan dokter untuk melakukan prosedur profilaksis penting seperti omentektomi atau omentopeksi untuk meminimalkan risiko omental wrapping (penyumbatan kateter oleh omentum), yang merupakan salah satu penyebab utama kegagalan mekanis kateter pada anak-anak. Laparoscopic juga terbukti mempermudah penyelamatan (salvage) jika terjadi malposisi atau disfungsi kateter tanpa harus melakukan pembedahan ulang yang invasif. [Sumber 1](https://www.sages.org/publications/guidelines/peritoneal-dialysis-access-guideline-update-2023/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC10223083/) [[3]](https://kidney.wiki/peritoneal-dialysis/pd-access/) | Gastrostomy/Intraperitoneal Device:  | Performed CAPD: Tidak ada perbedaan yang signifikan dalam tingkat kelangsungan hidup teknik, kematian, maupun episode peritonitis antara dialisis yang dilakukan sendiri oleh pasien (self-care) dengan dialisis yang dibantu oleh keluarga atau pengasuh (assisted/home-care). Namun, pada populasi anak (khususnya balita atau anak dengan keterbatasan fisik/kognitif), peran orang tua (Parent/Others) sangat mutlak diperlukan. Bagi orang tua yang memiliki tingkat pendidikan rendah atau keterbatasan ekonomi, dialisis tetap dapat berhasil dengan baik tanpa komplikasi besar asalkan diberikan pelatihan intensif secara 1:1, dukungan telepon 24 jam, dan kunjungan rumah berkala oleh perawat dialisis berpengalaman. Di sisi lain, bagi pasien remaja yang melakukan dialisis secara mandiri (Patient), tantangan psikososial seperti kejenuhan (burnout), perasaan terkekang (slavery feeling), dan depresi sering kali muncul, sehingga membutuhkan pengawasan ketat dari tim medis agar kepatuhan terhadap prosedur aseptik tetap terjaga. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/29456210/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC4335934/) [Sumber 3](https://www.ispd.org/wp-content/uploads/2025/12/Assisted-PD-PP-2024-with-VA_formatted.pdf) | Starting PD &lt;2 weeks after catheter placement: Waktu antara pemasangan kateter dan dimulainya dialisis (break-in-period) merupakan faktor penting untuk mencegah komplikasi. Masa penyembuhan minimal 2 minggu sebelum dialysis dimulai. Namun, dalam kondisi klinis tertentu di mana pasien membutuhkan dialisis segera, urgent-start PD (dimulai dalam &lt;14 hari atau bahkan &lt;48 jam) menjadi alternatif yang baik untuk menghindari penggunakan kateter hemodialysis sementara. Pasien dengan break-in-period &lt; 7 hari memiliki risiko yang lebih tinggi terhadap komplikasi awal seperti kebocoran dialisat dan malposisi kateter. Namun, risiko tersebut tidak berkorelasi dengan penurunan kelangsungan hidup atau peningkatan risiko peritonitis jika dilakukan dengan protokol yang tepat. Pada kondisi urgent-start, risiko kebocoran dimitigasi dengan menggunakan volume pengisian rendah (10-20 ml/kg) dan posisi pasien supine untuk mengurangi tekanan intra-abdominal.[Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC3923692/) [Sumber 2](https://journals.plos.org/plosone/article?id=10.1371/journal.pone.0206426) [Sumber 3](https://www.sages.org/publications/guidelines/peritoneal-dialysis-access-guideline-update-2023/) [Sumber 4](https://www.frontiersin.org/journals/endocrinology/articles/10.3389/fendo.2022.936573/full) [Sumber 5](https://scholarlyexchange.childrensmercy.org/cgi/viewcontent.cgi?article=7522&amp;context=papers) [Sumber 6](https://pubmed.ncbi.nlm.nih.gov/33523772/) [Sumber 7](https://www.bcrenal.ca/resource-gallery/Documents/PD_Procedures-Exit_Site_Care-Post-Operative_PD_Catheter_Insertion.pdf) | Catheter Orientation: Posisi atau arah lubang keluar kateter (exit site) sangat memengaruhi risiko terjadinya infeksi. Data multisentrik dari SCOPE Collaborative menunjukkan bahwa orientasi kateter yang menghadap ke atas (Upward) dikaitkan dengan peningkatan risiko peritonitis hingga 4.2 kali lipat (Rate Ratio: 4.2; 95% CI: 1.49–11.89) dibandingkan orientasi lainnya. Secara anatomis, lubang keluar yang menghadap ke atas menciptakan bentuk cekungan yang dapat menampung keringat, air mandi, dan kotoran. Akibat gaya gravitasi, bakteri yang terkumpul di area ini akan mengendap dan bermigrasi ke dalam terowongan kateter. Oleh karena itu, lubang keluar kateter harus selalu diarahkan ke bawah (Downward) atau ke samping (Lateral) untuk mencegah penumpukan bakteri secara alami. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC5012476/) [Sumber 2](https://openurologyandnephrologyjournal.com/VOLUME/5/PAGE/4/) [Sumber 3](https://kidney.wiki/peritoneal-dialysis/pd-access/)</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>2026-05-19 12:45:11</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>18F27E0F</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>&lt;2 yo</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>&gt;12 mo</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>Fair/poor service</t>
+        </is>
+      </c>
+      <c r="I117" t="inlineStr">
+        <is>
+          <t>Poor/fair</t>
+        </is>
+      </c>
+      <c r="J117" t="inlineStr">
+        <is>
+          <t>Studies</t>
+        </is>
+      </c>
+      <c r="K117" t="inlineStr">
+        <is>
+          <t>ESI</t>
+        </is>
+      </c>
+      <c r="L117" t="inlineStr">
+        <is>
+          <t>Normal Nutrition</t>
+        </is>
+      </c>
+      <c r="M117" t="inlineStr">
+        <is>
+          <t>Non-glomerular</t>
+        </is>
+      </c>
+      <c r="N117" t="inlineStr">
+        <is>
+          <t>Straight</t>
+        </is>
+      </c>
+      <c r="O117" t="inlineStr">
+        <is>
+          <t>Single cuff</t>
+        </is>
+      </c>
+      <c r="P117" t="inlineStr">
+        <is>
+          <t>Laparoscopic</t>
+        </is>
+      </c>
+      <c r="Q117" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="R117" t="inlineStr">
+        <is>
+          <t>Parents/others</t>
+        </is>
+      </c>
+      <c r="S117" t="inlineStr"/>
+      <c r="T117" t="inlineStr">
+        <is>
+          <t>upward</t>
+        </is>
+      </c>
+      <c r="U117" t="inlineStr">
+        <is>
+          <t>No stunting</t>
+        </is>
+      </c>
+      <c r="V117" t="inlineStr"/>
+      <c r="W117" t="inlineStr"/>
+      <c r="X117" t="inlineStr"/>
+      <c r="Y117" t="inlineStr">
+        <is>
+          <t>Age*, Gender, Duration of PD*, Housing, Socioeconomic, Peritonitis in ESI*, Cause of ESRD*, Type of Catheter (Shape), Type of Catheter (Cuff), Catheter Placement, Gastrostomy/Intraperitoneal Device, Performed CAPD, Starting PD &lt;2 weeks after catheter placement, Catheter Orientation</t>
+        </is>
+      </c>
+      <c r="Z117" t="inlineStr">
+        <is>
+          <t>Housing: Lingkungan rumah harus diadaptasi untuk memenuhi standar prosedur medis. Ruangan yang digunakan untuk pertukaran cairan harus bersih dan bebas debu untuk meminimalkan risiko infeksi, sebab partikel debu dapat menjadi vektor bagi patogen udara yang dapat mengontaminasi set transfer saat prosedur koneksi atau diskoneksi. Penyediaan wastafel di dalam atau dekat ruangan dialisis diperlukan untuk memastikan kepatuhan protokol antiseptic tangan sehingga menurunkan insiden peritonitis akibat touch contamination. Pencahayaan yang optimal di dalam ruangan diperlukan agar caregiver dapat memantau kejernihan cairan efluen serta memeriksa kondisi tempat keluar kateter dengan teliti. Hewan peliharaan tidak boleh berada di area perawatan saat proses koneksi atau diskoneksi berlangsung karena risiko paparan bakteri seperti Pasteurella multocida atau kerusakan fisik pada selang dialisis akibat gigitan atau cakaran. Selain itu, caregiverharus ditekankan untuk selalu mencuci tangan setelah berinteraksi dengan hewan dan sebelum memulai prosedur dialisis. [Sumber 1](https://www.freseniuskidneycare.com/treatment/home-dialysis/getting-prepared) [Sumber 2](https://www.ouh.nhs.uk/media/agxhnni2/85713pdialysis.pdf) [Sumber 3](https://www.kidney.org/kidney-topics/preparing-home-dialysis) [Sumber 4](https://spnp-spp.pt/media/rqdpbrom/catheter-related-infections-and-peritonitis-in-pediatric-patients-receiving-peritoneal-dialysis-guideline-for-prevention-and-treatment-2012-1-_compressed-1.pdf) [Sumber 5](https://freseniusmedicalcare.com/content/dam/home-products-education/steps2home-pd/Preventing_Peritonitis.pdf) [Sumber 6](https://www.satellitehealthcare.com/blog/pets-and-peritoneal-dialysis-absolutely/) | Socioeconomic: Deprivasi sosioekonomi berdampak pada hasil treatment yang lebih buruk. Hal ini kemungkinan disebabkan oleh keterbatasan akses terhadap fasilitas sanitasi yang memadai, tekanan psikologis pada pengasuh, serta keterbatasan informasi medis. Strategi bisa dilakukan melalui program pelatihan bagi keluarga (caregiver) dari perawat dialisis yang berpengalaman. Bagi keluarga dengan keterbatasan pendidikan atau ekonomi, dukungan teknis telepon 24 jam dan kunjungan rumah secara berkala oleh tim medis sosial sangat efektif dalam memastikan kepatuhan terhadap prosedur aseptik. Pelatihan ulang sangat dianjurkan, terutama setelah terjadinya peritonitis, untuk mengidentifikasi adanya penyimpangan dalam teknik pertukaran cairan. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC11835194/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC4934433/) [Sumber 3](https://pubmed.ncbi.nlm.nih.gov/23226378/) [Sumber 4](https://pubmed.ncbi.nlm.nih.gov/16091376/) [Sumber 6](https://spnp-spp.pt/media/rqdpbrom/catheter-related-infections-and-peritonitis-in-pediatric-patients-receiving-peritoneal-dialysis-guideline-for-prevention-and-treatment-2012-1-_compressed-1.pdf) [Sumber 7](https://pmc.ncbi.nlm.nih.gov/articles/PMC5691857/) [Sumber 8](https://pmc.ncbi.nlm.nih.gov/articles/PMC4335934/) [Sumber 9](https://www.kidney.org/kidney-topics/preparing-home-dialysis) | Peritonitis in ESI: Penggunaan antibiotik topikal secara rutin pada tempat keluar kateter telat terbukti menurunkan angka infeksi. Aplikasi harian salep mupirocin atau gentamicin pada exit-site direkomendasikan untuk menekan kolonisasi Staphylococcus aureus dan Pseudomonas aeruginosa.Pembersihan area secara rutin dengan larutan antiseptik non-iritan (seperti chlorhexidine 0,05% atau sabun antibakteri ringan) juga merupakan bagian standar dari perawatan. Penilaian kondisi exit-site secara objektif menggunakan sistem skor (seperti Skor ISPD yang mencakup pembengkakan, kerak, kemerahan, nyeri, dan sekret) sangat membantu caregiver dalam mendeteksi infeksi secara dini. Immobilisasi kateter dengan menggunakan plester atau perangkat fiksasi sangat krusial karena trauma mekanis pada tempat keluar sering kali menjadi pintu masuk bagi bakteri. Jika ESI terjadi, terapi antibiotik oral atau intraperitoneal harus dimulai segera dan dilanjutkan selama minimal 2 minggu, atau 3 minggu jika disebabkan oleh Pseudomonas. Pengangkatan kateter mungkin diperlukan jika infeksi bersifat refrakter (tidak merespons pengobatan setelah 2 minggu) atau jika infeksi telah menyebar ke terowongan kateter (tunnel infection) yang menyebabkan peritonitis berulang. [Sumber 1](https://ispd.org/wp-content/uploads/2025/09/LI-ET-1.pdf) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC12640025/) [Sumber 3](https://pmc.ncbi.nlm.nih.gov/articles/PMC5033625/) [Sumber 4](https://www.chikd.org/journal/view.php?number=726) [Sumber 5](https://ispd.org/wp-content/uploads/ISPD-Catheter-related-Infection-Recommendations-2023-Update.pdf) [Sumber 6](https://www.bcrenal.ca/resource-gallery/Documents/PD_Procedures-Exit_Site_Care-Post-Operative_PD_Catheter_Insertion.pdf) [Sumber 7](https://davita.com/treatment-options/articles/preventing-catheter-infections-on-peritoneal-dialysis/) [Sumber 8](https://edren.org/ren/handbook/pd-handbook/protocol-for-the-management-of-pd-peritonitis-long-version/) | Type of Catheter (Shape): Perdebatan mengenai efektivitas kateter straight dibandingkan dengan kateter coiled/curled masih berlangsung. Kateter coiled secara teoretis mengurangi nyeri saat pengisian cairan dan meminimalkan trauma pada organ visceral, tetapi beberapa data menunjukkan risiko malposisi yang lebih tinggi dibandingkan tipe lurus pada beberapa kelompok pasien. Di sisi lain, kateter straight lebih mudah ditempatkan pada bayi kecil yang memiliki ruang intra-abdominal terbatas. Secara keseluruhan, pedoman tidak menyatakan superioritas mutlak salah satu bentuk, dan pemilihan sering kali bergantung pada preferensi pusat dialisis dan anatomi pasien. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC9365012/) [Sumber 2](http://ispd.org/wp-content/uploads/7.-Dagmara-Borzych-Duzalka-Peritoneal-Dialysis-Catheters-Outcome-in-Children.-The-IPPN-Data.pdf) [Sumber 3](https://scholarlyexchange.childrensmercy.org/cgi/viewcontent.cgi?article=7522&amp;context=papers) [Sumber 4](https://kidney.wiki/peritoneal-dialysis/pd-access/) | Type of Catheter (Cuff): Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff)untuk populasi anak secara umum. Deep cuff berfungsi untuk menjangkar kateter di otot rektus dan mencegah kebocoran, sementara superficial cuff bertindak sebagai penghalang fisik terhadap migrasi bakteri ke arah rongga peritoneum. Namun, pada neonatus atau bayi dengan dinding perut yang sangat tipis, kateter single-cuff sering kali lebih dipilih untuk mencegah ekstrusi manset ke permukaan kulit. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC10223083/) [Sumber 2](http://ispd.org/wp-content/uploads/7.-Dagmara-Borzych-Duzalka-Peritoneal-Dialysis-Catheters-Outcome-in-Children.-The-IPPN-Data.pdf) [Sumber 3](https://kidney.wiki/peritoneal-dialysis/pd-access/) | Catheter Placement: Pedoman klinis terbaru dari Society of American Gastrointestinal and Endoscopic Surgeons (SAGES) menyarankan penggunaan teknik laparoskopi tingkat lanjut (Laparoscopic) dibandingkan teknik bedah terbuka (Open) untuk pemasangan kateter pada populasi pediatrik. Laparoscopic menawarkan akurasi catheter placement yang jauh lebih tinggi di dalam rongga abdomen karena visualisasi langsung, serta meminimalkan trauma mekanis pada jaringan perut. Lebih lanjut, Laparoscopic memungkinkan dokter untuk melakukan prosedur profilaksis penting seperti omentektomi atau omentopeksi untuk meminimalkan risiko omental wrapping (penyumbatan kateter oleh omentum), yang merupakan salah satu penyebab utama kegagalan mekanis kateter pada anak-anak. Laparoscopic juga terbukti mempermudah penyelamatan (salvage) jika terjadi malposisi atau disfungsi kateter tanpa harus melakukan pembedahan ulang yang invasif. [Sumber 1](https://www.sages.org/publications/guidelines/peritoneal-dialysis-access-guideline-update-2023/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC10223083/) [[3]](https://kidney.wiki/peritoneal-dialysis/pd-access/) | Gastrostomy/Intraperitoneal Device:  | Performed CAPD: Tidak ada perbedaan yang signifikan dalam tingkat kelangsungan hidup teknik, kematian, maupun episode peritonitis antara dialisis yang dilakukan sendiri oleh pasien (self-care) dengan dialisis yang dibantu oleh keluarga atau pengasuh (assisted/home-care). Namun, pada populasi anak (khususnya balita atau anak dengan keterbatasan fisik/kognitif), peran orang tua (Parent/Others) sangat mutlak diperlukan. Bagi orang tua yang memiliki tingkat pendidikan rendah atau keterbatasan ekonomi, dialisis tetap dapat berhasil dengan baik tanpa komplikasi besar asalkan diberikan pelatihan intensif secara 1:1, dukungan telepon 24 jam, dan kunjungan rumah berkala oleh perawat dialisis berpengalaman. Di sisi lain, bagi pasien remaja yang melakukan dialisis secara mandiri (Patient), tantangan psikososial seperti kejenuhan (burnout), perasaan terkekang (slavery feeling), dan depresi sering kali muncul, sehingga membutuhkan pengawasan ketat dari tim medis agar kepatuhan terhadap prosedur aseptik tetap terjaga. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/29456210/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC4335934/) [Sumber 3](https://www.ispd.org/wp-content/uploads/2025/12/Assisted-PD-PP-2024-with-VA_formatted.pdf) | Starting PD &lt;2 weeks after catheter placement: Waktu antara pemasangan kateter dan dimulainya dialisis (break-in-period) merupakan faktor penting untuk mencegah komplikasi. Masa penyembuhan minimal 2 minggu sebelum dialysis dimulai. Namun, dalam kondisi klinis tertentu di mana pasien membutuhkan dialisis segera, urgent-start PD (dimulai dalam &lt;14 hari atau bahkan &lt;48 jam) menjadi alternatif yang baik untuk menghindari penggunakan kateter hemodialysis sementara. Pasien dengan break-in-period &lt; 7 hari memiliki risiko yang lebih tinggi terhadap komplikasi awal seperti kebocoran dialisat dan malposisi kateter. Namun, risiko tersebut tidak berkorelasi dengan penurunan kelangsungan hidup atau peningkatan risiko peritonitis jika dilakukan dengan protokol yang tepat. Pada kondisi urgent-start, risiko kebocoran dimitigasi dengan menggunakan volume pengisian rendah (10-20 ml/kg) dan posisi pasien supine untuk mengurangi tekanan intra-abdominal.[Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC3923692/) [Sumber 2](https://journals.plos.org/plosone/article?id=10.1371/journal.pone.0206426) [Sumber 3](https://www.sages.org/publications/guidelines/peritoneal-dialysis-access-guideline-update-2023/) [Sumber 4](https://www.frontiersin.org/journals/endocrinology/articles/10.3389/fendo.2022.936573/full) [Sumber 5](https://scholarlyexchange.childrensmercy.org/cgi/viewcontent.cgi?article=7522&amp;context=papers) [Sumber 6](https://pubmed.ncbi.nlm.nih.gov/33523772/) [Sumber 7](https://www.bcrenal.ca/resource-gallery/Documents/PD_Procedures-Exit_Site_Care-Post-Operative_PD_Catheter_Insertion.pdf) | Catheter Orientation: Posisi atau arah lubang keluar kateter (exit site) sangat memengaruhi risiko terjadinya infeksi. Data multisentrik dari SCOPE Collaborative menunjukkan bahwa orientasi kateter yang menghadap ke atas (Upward) dikaitkan dengan peningkatan risiko peritonitis hingga 4.2 kali lipat (Rate Ratio: 4.2; 95% CI: 1.49–11.89) dibandingkan orientasi lainnya. Secara anatomis, lubang keluar yang menghadap ke atas menciptakan bentuk cekungan yang dapat menampung keringat, air mandi, dan kotoran. Akibat gaya gravitasi, bakteri yang terkumpul di area ini akan mengendap dan bermigrasi ke dalam terowongan kateter. Oleh karena itu, lubang keluar kateter harus selalu diarahkan ke bawah (Downward) atau ke samping (Lateral) untuk mencegah penumpukan bakteri secara alami. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC5012476/) [Sumber 2](https://openurologyandnephrologyjournal.com/VOLUME/5/PAGE/4/) [Sumber 3](https://kidney.wiki/peritoneal-dialysis/pd-access/)</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>2026-05-19 12:45:15</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>18F27E0F</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>&lt;2 yo</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>&gt;12 mo</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>Fair/poor service</t>
+        </is>
+      </c>
+      <c r="I118" t="inlineStr">
+        <is>
+          <t>Poor/fair</t>
+        </is>
+      </c>
+      <c r="J118" t="inlineStr">
+        <is>
+          <t>Studies</t>
+        </is>
+      </c>
+      <c r="K118" t="inlineStr">
+        <is>
+          <t>ESI</t>
+        </is>
+      </c>
+      <c r="L118" t="inlineStr">
+        <is>
+          <t>Normal Nutrition</t>
+        </is>
+      </c>
+      <c r="M118" t="inlineStr">
+        <is>
+          <t>Non-glomerular</t>
+        </is>
+      </c>
+      <c r="N118" t="inlineStr">
+        <is>
+          <t>Coiled/swan neck</t>
+        </is>
+      </c>
+      <c r="O118" t="inlineStr">
+        <is>
+          <t>Single cuff</t>
+        </is>
+      </c>
+      <c r="P118" t="inlineStr">
+        <is>
+          <t>Laparoscopic</t>
+        </is>
+      </c>
+      <c r="Q118" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="R118" t="inlineStr">
+        <is>
+          <t>Parents/others</t>
+        </is>
+      </c>
+      <c r="S118" t="inlineStr"/>
+      <c r="T118" t="inlineStr">
+        <is>
+          <t>upward</t>
+        </is>
+      </c>
+      <c r="U118" t="inlineStr">
+        <is>
+          <t>No stunting</t>
+        </is>
+      </c>
+      <c r="V118" t="inlineStr"/>
+      <c r="W118" t="inlineStr"/>
+      <c r="X118" t="inlineStr"/>
+      <c r="Y118" t="inlineStr">
+        <is>
+          <t>Age*, Gender, Duration of PD*, Housing, Socioeconomic, Peritonitis in ESI*, Cause of ESRD*, Type of Catheter (Cuff), Catheter Placement, Gastrostomy/Intraperitoneal Device, Performed CAPD, Starting PD &lt;2 weeks after catheter placement, Catheter Orientation</t>
+        </is>
+      </c>
+      <c r="Z118" t="inlineStr">
+        <is>
+          <t>Housing: Lingkungan rumah harus diadaptasi untuk memenuhi standar prosedur medis. Ruangan yang digunakan untuk pertukaran cairan harus bersih dan bebas debu untuk meminimalkan risiko infeksi, sebab partikel debu dapat menjadi vektor bagi patogen udara yang dapat mengontaminasi set transfer saat prosedur koneksi atau diskoneksi. Penyediaan wastafel di dalam atau dekat ruangan dialisis diperlukan untuk memastikan kepatuhan protokol antiseptic tangan sehingga menurunkan insiden peritonitis akibat touch contamination. Pencahayaan yang optimal di dalam ruangan diperlukan agar caregiver dapat memantau kejernihan cairan efluen serta memeriksa kondisi tempat keluar kateter dengan teliti. Hewan peliharaan tidak boleh berada di area perawatan saat proses koneksi atau diskoneksi berlangsung karena risiko paparan bakteri seperti Pasteurella multocida atau kerusakan fisik pada selang dialisis akibat gigitan atau cakaran. Selain itu, caregiverharus ditekankan untuk selalu mencuci tangan setelah berinteraksi dengan hewan dan sebelum memulai prosedur dialisis. [Sumber 1](https://www.freseniuskidneycare.com/treatment/home-dialysis/getting-prepared) [Sumber 2](https://www.ouh.nhs.uk/media/agxhnni2/85713pdialysis.pdf) [Sumber 3](https://www.kidney.org/kidney-topics/preparing-home-dialysis) [Sumber 4](https://spnp-spp.pt/media/rqdpbrom/catheter-related-infections-and-peritonitis-in-pediatric-patients-receiving-peritoneal-dialysis-guideline-for-prevention-and-treatment-2012-1-_compressed-1.pdf) [Sumber 5](https://freseniusmedicalcare.com/content/dam/home-products-education/steps2home-pd/Preventing_Peritonitis.pdf) [Sumber 6](https://www.satellitehealthcare.com/blog/pets-and-peritoneal-dialysis-absolutely/) | Socioeconomic: Deprivasi sosioekonomi berdampak pada hasil treatment yang lebih buruk. Hal ini kemungkinan disebabkan oleh keterbatasan akses terhadap fasilitas sanitasi yang memadai, tekanan psikologis pada pengasuh, serta keterbatasan informasi medis. Strategi bisa dilakukan melalui program pelatihan bagi keluarga (caregiver) dari perawat dialisis yang berpengalaman. Bagi keluarga dengan keterbatasan pendidikan atau ekonomi, dukungan teknis telepon 24 jam dan kunjungan rumah secara berkala oleh tim medis sosial sangat efektif dalam memastikan kepatuhan terhadap prosedur aseptik. Pelatihan ulang sangat dianjurkan, terutama setelah terjadinya peritonitis, untuk mengidentifikasi adanya penyimpangan dalam teknik pertukaran cairan. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC11835194/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC4934433/) [Sumber 3](https://pubmed.ncbi.nlm.nih.gov/23226378/) [Sumber 4](https://pubmed.ncbi.nlm.nih.gov/16091376/) [Sumber 6](https://spnp-spp.pt/media/rqdpbrom/catheter-related-infections-and-peritonitis-in-pediatric-patients-receiving-peritoneal-dialysis-guideline-for-prevention-and-treatment-2012-1-_compressed-1.pdf) [Sumber 7](https://pmc.ncbi.nlm.nih.gov/articles/PMC5691857/) [Sumber 8](https://pmc.ncbi.nlm.nih.gov/articles/PMC4335934/) [Sumber 9](https://www.kidney.org/kidney-topics/preparing-home-dialysis) | Peritonitis in ESI: Penggunaan antibiotik topikal secara rutin pada tempat keluar kateter telat terbukti menurunkan angka infeksi. Aplikasi harian salep mupirocin atau gentamicin pada exit-site direkomendasikan untuk menekan kolonisasi Staphylococcus aureus dan Pseudomonas aeruginosa.Pembersihan area secara rutin dengan larutan antiseptik non-iritan (seperti chlorhexidine 0,05% atau sabun antibakteri ringan) juga merupakan bagian standar dari perawatan. Penilaian kondisi exit-site secara objektif menggunakan sistem skor (seperti Skor ISPD yang mencakup pembengkakan, kerak, kemerahan, nyeri, dan sekret) sangat membantu caregiver dalam mendeteksi infeksi secara dini. Immobilisasi kateter dengan menggunakan plester atau perangkat fiksasi sangat krusial karena trauma mekanis pada tempat keluar sering kali menjadi pintu masuk bagi bakteri. Jika ESI terjadi, terapi antibiotik oral atau intraperitoneal harus dimulai segera dan dilanjutkan selama minimal 2 minggu, atau 3 minggu jika disebabkan oleh Pseudomonas. Pengangkatan kateter mungkin diperlukan jika infeksi bersifat refrakter (tidak merespons pengobatan setelah 2 minggu) atau jika infeksi telah menyebar ke terowongan kateter (tunnel infection) yang menyebabkan peritonitis berulang. [Sumber 1](https://ispd.org/wp-content/uploads/2025/09/LI-ET-1.pdf) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC12640025/) [Sumber 3](https://pmc.ncbi.nlm.nih.gov/articles/PMC5033625/) [Sumber 4](https://www.chikd.org/journal/view.php?number=726) [Sumber 5](https://ispd.org/wp-content/uploads/ISPD-Catheter-related-Infection-Recommendations-2023-Update.pdf) [Sumber 6](https://www.bcrenal.ca/resource-gallery/Documents/PD_Procedures-Exit_Site_Care-Post-Operative_PD_Catheter_Insertion.pdf) [Sumber 7](https://davita.com/treatment-options/articles/preventing-catheter-infections-on-peritoneal-dialysis/) [Sumber 8](https://edren.org/ren/handbook/pd-handbook/protocol-for-the-management-of-pd-peritonitis-long-version/) | Type of Catheter (Cuff): Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff)untuk populasi anak secara umum. Deep cuff berfungsi untuk menjangkar kateter di otot rektus dan mencegah kebocoran, sementara superficial cuff bertindak sebagai penghalang fisik terhadap migrasi bakteri ke arah rongga peritoneum. Namun, pada neonatus atau bayi dengan dinding perut yang sangat tipis, kateter single-cuff sering kali lebih dipilih untuk mencegah ekstrusi manset ke permukaan kulit. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC10223083/) [Sumber 2](http://ispd.org/wp-content/uploads/7.-Dagmara-Borzych-Duzalka-Peritoneal-Dialysis-Catheters-Outcome-in-Children.-The-IPPN-Data.pdf) [Sumber 3](https://kidney.wiki/peritoneal-dialysis/pd-access/) | Catheter Placement: Pedoman klinis terbaru dari Society of American Gastrointestinal and Endoscopic Surgeons (SAGES) menyarankan penggunaan teknik laparoskopi tingkat lanjut (Laparoscopic) dibandingkan teknik bedah terbuka (Open) untuk pemasangan kateter pada populasi pediatrik. Laparoscopic menawarkan akurasi catheter placement yang jauh lebih tinggi di dalam rongga abdomen karena visualisasi langsung, serta meminimalkan trauma mekanis pada jaringan perut. Lebih lanjut, Laparoscopic memungkinkan dokter untuk melakukan prosedur profilaksis penting seperti omentektomi atau omentopeksi untuk meminimalkan risiko omental wrapping (penyumbatan kateter oleh omentum), yang merupakan salah satu penyebab utama kegagalan mekanis kateter pada anak-anak. Laparoscopic juga terbukti mempermudah penyelamatan (salvage) jika terjadi malposisi atau disfungsi kateter tanpa harus melakukan pembedahan ulang yang invasif. [Sumber 1](https://www.sages.org/publications/guidelines/peritoneal-dialysis-access-guideline-update-2023/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC10223083/) [[3]](https://kidney.wiki/peritoneal-dialysis/pd-access/) | Gastrostomy/Intraperitoneal Device:  | Performed CAPD: Tidak ada perbedaan yang signifikan dalam tingkat kelangsungan hidup teknik, kematian, maupun episode peritonitis antara dialisis yang dilakukan sendiri oleh pasien (self-care) dengan dialisis yang dibantu oleh keluarga atau pengasuh (assisted/home-care). Namun, pada populasi anak (khususnya balita atau anak dengan keterbatasan fisik/kognitif), peran orang tua (Parent/Others) sangat mutlak diperlukan. Bagi orang tua yang memiliki tingkat pendidikan rendah atau keterbatasan ekonomi, dialisis tetap dapat berhasil dengan baik tanpa komplikasi besar asalkan diberikan pelatihan intensif secara 1:1, dukungan telepon 24 jam, dan kunjungan rumah berkala oleh perawat dialisis berpengalaman. Di sisi lain, bagi pasien remaja yang melakukan dialisis secara mandiri (Patient), tantangan psikososial seperti kejenuhan (burnout), perasaan terkekang (slavery feeling), dan depresi sering kali muncul, sehingga membutuhkan pengawasan ketat dari tim medis agar kepatuhan terhadap prosedur aseptik tetap terjaga. [Sumber 1](https://pubmed.ncbi.nlm.nih.gov/29456210/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC4335934/) [Sumber 3](https://www.ispd.org/wp-content/uploads/2025/12/Assisted-PD-PP-2024-with-VA_formatted.pdf) | Starting PD &lt;2 weeks after catheter placement: Waktu antara pemasangan kateter dan dimulainya dialisis (break-in-period) merupakan faktor penting untuk mencegah komplikasi. Masa penyembuhan minimal 2 minggu sebelum dialysis dimulai. Namun, dalam kondisi klinis tertentu di mana pasien membutuhkan dialisis segera, urgent-start PD (dimulai dalam &lt;14 hari atau bahkan &lt;48 jam) menjadi alternatif yang baik untuk menghindari penggunakan kateter hemodialysis sementara. Pasien dengan break-in-period &lt; 7 hari memiliki risiko yang lebih tinggi terhadap komplikasi awal seperti kebocoran dialisat dan malposisi kateter. Namun, risiko tersebut tidak berkorelasi dengan penurunan kelangsungan hidup atau peningkatan risiko peritonitis jika dilakukan dengan protokol yang tepat. Pada kondisi urgent-start, risiko kebocoran dimitigasi dengan menggunakan volume pengisian rendah (10-20 ml/kg) dan posisi pasien supine untuk mengurangi tekanan intra-abdominal.[Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC3923692/) [Sumber 2](https://journals.plos.org/plosone/article?id=10.1371/journal.pone.0206426) [Sumber 3](https://www.sages.org/publications/guidelines/peritoneal-dialysis-access-guideline-update-2023/) [Sumber 4](https://www.frontiersin.org/journals/endocrinology/articles/10.3389/fendo.2022.936573/full) [Sumber 5](https://scholarlyexchange.childrensmercy.org/cgi/viewcontent.cgi?article=7522&amp;context=papers) [Sumber 6](https://pubmed.ncbi.nlm.nih.gov/33523772/) [Sumber 7](https://www.bcrenal.ca/resource-gallery/Documents/PD_Procedures-Exit_Site_Care-Post-Operative_PD_Catheter_Insertion.pdf) | Catheter Orientation: Posisi atau arah lubang keluar kateter (exit site) sangat memengaruhi risiko terjadinya infeksi. Data multisentrik dari SCOPE Collaborative menunjukkan bahwa orientasi kateter yang menghadap ke atas (Upward) dikaitkan dengan peningkatan risiko peritonitis hingga 4.2 kali lipat (Rate Ratio: 4.2; 95% CI: 1.49–11.89) dibandingkan orientasi lainnya. Secara anatomis, lubang keluar yang menghadap ke atas menciptakan bentuk cekungan yang dapat menampung keringat, air mandi, dan kotoran. Akibat gaya gravitasi, bakteri yang terkumpul di area ini akan mengendap dan bermigrasi ke dalam terowongan kateter. Oleh karena itu, lubang keluar kateter harus selalu diarahkan ke bawah (Downward) atau ke samping (Lateral) untuk mencegah penumpukan bakteri secara alami. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC5012476/) [Sumber 2](https://openurologyandnephrologyjournal.com/VOLUME/5/PAGE/4/) [Sumber 3](https://kidney.wiki/peritoneal-dialysis/pd-access/)</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>2026-05-19 12:45:18</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>18F27E0F</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>&lt;2 yo</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>&gt;12 mo</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>Fair/poor service</t>
+        </is>
+      </c>
+      <c r="I119" t="inlineStr">
+        <is>
+          <t>Poor/fair</t>
+        </is>
+      </c>
+      <c r="J119" t="inlineStr">
+        <is>
+          <t>Studies</t>
+        </is>
+      </c>
+      <c r="K119" t="inlineStr">
+        <is>
+          <t>ESI</t>
+        </is>
+      </c>
+      <c r="L119" t="inlineStr">
+        <is>
+          <t>Normal Nutrition</t>
+        </is>
+      </c>
+      <c r="M119" t="inlineStr">
+        <is>
+          <t>Non-glomerular</t>
+        </is>
+      </c>
+      <c r="N119" t="inlineStr">
+        <is>
+          <t>Coiled/swan neck</t>
+        </is>
+      </c>
+      <c r="O119" t="inlineStr">
+        <is>
+          <t>Single cuff</t>
+        </is>
+      </c>
+      <c r="P119" t="inlineStr">
+        <is>
+          <t>Laparoscopic</t>
+        </is>
+      </c>
+      <c r="Q119" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R119" t="inlineStr">
+        <is>
+          <t>Patients</t>
+        </is>
+      </c>
+      <c r="S119" t="inlineStr"/>
+      <c r="T119" t="inlineStr">
+        <is>
+          <t>upward</t>
+        </is>
+      </c>
+      <c r="U119" t="inlineStr">
+        <is>
+          <t>No stunting</t>
+        </is>
+      </c>
+      <c r="V119" t="inlineStr"/>
+      <c r="W119" t="inlineStr"/>
+      <c r="X119" t="inlineStr"/>
+      <c r="Y119" t="inlineStr">
+        <is>
+          <t>Age*, Gender, Duration of PD*, Housing, Socioeconomic, Peritonitis in ESI*, Cause of ESRD*, Type of Catheter (Cuff), Catheter Placement, Starting PD &lt;2 weeks after catheter placement, Catheter Orientation</t>
+        </is>
+      </c>
+      <c r="Z119" t="inlineStr">
+        <is>
+          <t>Housing: Lingkungan rumah harus diadaptasi untuk memenuhi standar prosedur medis. Ruangan yang digunakan untuk pertukaran cairan harus bersih dan bebas debu untuk meminimalkan risiko infeksi, sebab partikel debu dapat menjadi vektor bagi patogen udara yang dapat mengontaminasi set transfer saat prosedur koneksi atau diskoneksi. Penyediaan wastafel di dalam atau dekat ruangan dialisis diperlukan untuk memastikan kepatuhan protokol antiseptic tangan sehingga menurunkan insiden peritonitis akibat touch contamination. Pencahayaan yang optimal di dalam ruangan diperlukan agar caregiver dapat memantau kejernihan cairan efluen serta memeriksa kondisi tempat keluar kateter dengan teliti. Hewan peliharaan tidak boleh berada di area perawatan saat proses koneksi atau diskoneksi berlangsung karena risiko paparan bakteri seperti Pasteurella multocida atau kerusakan fisik pada selang dialisis akibat gigitan atau cakaran. Selain itu, caregiverharus ditekankan untuk selalu mencuci tangan setelah berinteraksi dengan hewan dan sebelum memulai prosedur dialisis. [Sumber 1](https://www.freseniuskidneycare.com/treatment/home-dialysis/getting-prepared) [Sumber 2](https://www.ouh.nhs.uk/media/agxhnni2/85713pdialysis.pdf) [Sumber 3](https://www.kidney.org/kidney-topics/preparing-home-dialysis) [Sumber 4](https://spnp-spp.pt/media/rqdpbrom/catheter-related-infections-and-peritonitis-in-pediatric-patients-receiving-peritoneal-dialysis-guideline-for-prevention-and-treatment-2012-1-_compressed-1.pdf) [Sumber 5](https://freseniusmedicalcare.com/content/dam/home-products-education/steps2home-pd/Preventing_Peritonitis.pdf) [Sumber 6](https://www.satellitehealthcare.com/blog/pets-and-peritoneal-dialysis-absolutely/) | Socioeconomic: Deprivasi sosioekonomi berdampak pada hasil treatment yang lebih buruk. Hal ini kemungkinan disebabkan oleh keterbatasan akses terhadap fasilitas sanitasi yang memadai, tekanan psikologis pada pengasuh, serta keterbatasan informasi medis. Strategi bisa dilakukan melalui program pelatihan bagi keluarga (caregiver) dari perawat dialisis yang berpengalaman. Bagi keluarga dengan keterbatasan pendidikan atau ekonomi, dukungan teknis telepon 24 jam dan kunjungan rumah secara berkala oleh tim medis sosial sangat efektif dalam memastikan kepatuhan terhadap prosedur aseptik. Pelatihan ulang sangat dianjurkan, terutama setelah terjadinya peritonitis, untuk mengidentifikasi adanya penyimpangan dalam teknik pertukaran cairan. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC11835194/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC4934433/) [Sumber 3](https://pubmed.ncbi.nlm.nih.gov/23226378/) [Sumber 4](https://pubmed.ncbi.nlm.nih.gov/16091376/) [Sumber 6](https://spnp-spp.pt/media/rqdpbrom/catheter-related-infections-and-peritonitis-in-pediatric-patients-receiving-peritoneal-dialysis-guideline-for-prevention-and-treatment-2012-1-_compressed-1.pdf) [Sumber 7](https://pmc.ncbi.nlm.nih.gov/articles/PMC5691857/) [Sumber 8](https://pmc.ncbi.nlm.nih.gov/articles/PMC4335934/) [Sumber 9](https://www.kidney.org/kidney-topics/preparing-home-dialysis) | Peritonitis in ESI: Penggunaan antibiotik topikal secara rutin pada tempat keluar kateter telat terbukti menurunkan angka infeksi. Aplikasi harian salep mupirocin atau gentamicin pada exit-site direkomendasikan untuk menekan kolonisasi Staphylococcus aureus dan Pseudomonas aeruginosa.Pembersihan area secara rutin dengan larutan antiseptik non-iritan (seperti chlorhexidine 0,05% atau sabun antibakteri ringan) juga merupakan bagian standar dari perawatan. Penilaian kondisi exit-site secara objektif menggunakan sistem skor (seperti Skor ISPD yang mencakup pembengkakan, kerak, kemerahan, nyeri, dan sekret) sangat membantu caregiver dalam mendeteksi infeksi secara dini. Immobilisasi kateter dengan menggunakan plester atau perangkat fiksasi sangat krusial karena trauma mekanis pada tempat keluar sering kali menjadi pintu masuk bagi bakteri. Jika ESI terjadi, terapi antibiotik oral atau intraperitoneal harus dimulai segera dan dilanjutkan selama minimal 2 minggu, atau 3 minggu jika disebabkan oleh Pseudomonas. Pengangkatan kateter mungkin diperlukan jika infeksi bersifat refrakter (tidak merespons pengobatan setelah 2 minggu) atau jika infeksi telah menyebar ke terowongan kateter (tunnel infection) yang menyebabkan peritonitis berulang. [Sumber 1](https://ispd.org/wp-content/uploads/2025/09/LI-ET-1.pdf) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC12640025/) [Sumber 3](https://pmc.ncbi.nlm.nih.gov/articles/PMC5033625/) [Sumber 4](https://www.chikd.org/journal/view.php?number=726) [Sumber 5](https://ispd.org/wp-content/uploads/ISPD-Catheter-related-Infection-Recommendations-2023-Update.pdf) [Sumber 6](https://www.bcrenal.ca/resource-gallery/Documents/PD_Procedures-Exit_Site_Care-Post-Operative_PD_Catheter_Insertion.pdf) [Sumber 7](https://davita.com/treatment-options/articles/preventing-catheter-infections-on-peritoneal-dialysis/) [Sumber 8](https://edren.org/ren/handbook/pd-handbook/protocol-for-the-management-of-pd-peritonitis-long-version/) | Type of Catheter (Cuff): Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff)untuk populasi anak secara umum. Deep cuff berfungsi untuk menjangkar kateter di otot rektus dan mencegah kebocoran, sementara superficial cuff bertindak sebagai penghalang fisik terhadap migrasi bakteri ke arah rongga peritoneum. Namun, pada neonatus atau bayi dengan dinding perut yang sangat tipis, kateter single-cuff sering kali lebih dipilih untuk mencegah ekstrusi manset ke permukaan kulit. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC10223083/) [Sumber 2](http://ispd.org/wp-content/uploads/7.-Dagmara-Borzych-Duzalka-Peritoneal-Dialysis-Catheters-Outcome-in-Children.-The-IPPN-Data.pdf) [Sumber 3](https://kidney.wiki/peritoneal-dialysis/pd-access/) | Catheter Placement: Pedoman klinis terbaru dari Society of American Gastrointestinal and Endoscopic Surgeons (SAGES) menyarankan penggunaan teknik laparoskopi tingkat lanjut (Laparoscopic) dibandingkan teknik bedah terbuka (Open) untuk pemasangan kateter pada populasi pediatrik. Laparoscopic menawarkan akurasi catheter placement yang jauh lebih tinggi di dalam rongga abdomen karena visualisasi langsung, serta meminimalkan trauma mekanis pada jaringan perut. Lebih lanjut, Laparoscopic memungkinkan dokter untuk melakukan prosedur profilaksis penting seperti omentektomi atau omentopeksi untuk meminimalkan risiko omental wrapping (penyumbatan kateter oleh omentum), yang merupakan salah satu penyebab utama kegagalan mekanis kateter pada anak-anak. Laparoscopic juga terbukti mempermudah penyelamatan (salvage) jika terjadi malposisi atau disfungsi kateter tanpa harus melakukan pembedahan ulang yang invasif. [Sumber 1](https://www.sages.org/publications/guidelines/peritoneal-dialysis-access-guideline-update-2023/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC10223083/) [[3]](https://kidney.wiki/peritoneal-dialysis/pd-access/) | Starting PD &lt;2 weeks after catheter placement: Waktu antara pemasangan kateter dan dimulainya dialisis (break-in-period) merupakan faktor penting untuk mencegah komplikasi. Masa penyembuhan minimal 2 minggu sebelum dialysis dimulai. Namun, dalam kondisi klinis tertentu di mana pasien membutuhkan dialisis segera, urgent-start PD (dimulai dalam &lt;14 hari atau bahkan &lt;48 jam) menjadi alternatif yang baik untuk menghindari penggunakan kateter hemodialysis sementara. Pasien dengan break-in-period &lt; 7 hari memiliki risiko yang lebih tinggi terhadap komplikasi awal seperti kebocoran dialisat dan malposisi kateter. Namun, risiko tersebut tidak berkorelasi dengan penurunan kelangsungan hidup atau peningkatan risiko peritonitis jika dilakukan dengan protokol yang tepat. Pada kondisi urgent-start, risiko kebocoran dimitigasi dengan menggunakan volume pengisian rendah (10-20 ml/kg) dan posisi pasien supine untuk mengurangi tekanan intra-abdominal.[Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC3923692/) [Sumber 2](https://journals.plos.org/plosone/article?id=10.1371/journal.pone.0206426) [Sumber 3](https://www.sages.org/publications/guidelines/peritoneal-dialysis-access-guideline-update-2023/) [Sumber 4](https://www.frontiersin.org/journals/endocrinology/articles/10.3389/fendo.2022.936573/full) [Sumber 5](https://scholarlyexchange.childrensmercy.org/cgi/viewcontent.cgi?article=7522&amp;context=papers) [Sumber 6](https://pubmed.ncbi.nlm.nih.gov/33523772/) [Sumber 7](https://www.bcrenal.ca/resource-gallery/Documents/PD_Procedures-Exit_Site_Care-Post-Operative_PD_Catheter_Insertion.pdf) | Catheter Orientation: Posisi atau arah lubang keluar kateter (exit site) sangat memengaruhi risiko terjadinya infeksi. Data multisentrik dari SCOPE Collaborative menunjukkan bahwa orientasi kateter yang menghadap ke atas (Upward) dikaitkan dengan peningkatan risiko peritonitis hingga 4.2 kali lipat (Rate Ratio: 4.2; 95% CI: 1.49–11.89) dibandingkan orientasi lainnya. Secara anatomis, lubang keluar yang menghadap ke atas menciptakan bentuk cekungan yang dapat menampung keringat, air mandi, dan kotoran. Akibat gaya gravitasi, bakteri yang terkumpul di area ini akan mengendap dan bermigrasi ke dalam terowongan kateter. Oleh karena itu, lubang keluar kateter harus selalu diarahkan ke bawah (Downward) atau ke samping (Lateral) untuk mencegah penumpukan bakteri secara alami. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC5012476/) [Sumber 2](https://openurologyandnephrologyjournal.com/VOLUME/5/PAGE/4/) [Sumber 3](https://kidney.wiki/peritoneal-dialysis/pd-access/)</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>2026-05-19 12:45:25</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>18F27E0F</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>&lt;2 yo</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>&gt;12 mo</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>Fair/poor service</t>
+        </is>
+      </c>
+      <c r="I120" t="inlineStr">
+        <is>
+          <t>Poor/fair</t>
+        </is>
+      </c>
+      <c r="J120" t="inlineStr">
+        <is>
+          <t>Studies</t>
+        </is>
+      </c>
+      <c r="K120" t="inlineStr">
+        <is>
+          <t>No ESI</t>
+        </is>
+      </c>
+      <c r="L120" t="inlineStr">
+        <is>
+          <t>Normal Nutrition</t>
+        </is>
+      </c>
+      <c r="M120" t="inlineStr">
+        <is>
+          <t>Non-glomerular</t>
+        </is>
+      </c>
+      <c r="N120" t="inlineStr">
+        <is>
+          <t>Coiled/swan neck</t>
+        </is>
+      </c>
+      <c r="O120" t="inlineStr">
+        <is>
+          <t>Single cuff</t>
+        </is>
+      </c>
+      <c r="P120" t="inlineStr">
+        <is>
+          <t>Laparoscopic</t>
+        </is>
+      </c>
+      <c r="Q120" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R120" t="inlineStr">
+        <is>
+          <t>Patients</t>
+        </is>
+      </c>
+      <c r="S120" t="inlineStr"/>
+      <c r="T120" t="inlineStr">
+        <is>
+          <t>upward</t>
+        </is>
+      </c>
+      <c r="U120" t="inlineStr">
+        <is>
+          <t>No stunting</t>
+        </is>
+      </c>
+      <c r="V120" t="inlineStr"/>
+      <c r="W120" t="inlineStr"/>
+      <c r="X120" t="inlineStr"/>
+      <c r="Y120" t="inlineStr">
+        <is>
+          <t>Age*, Gender, Duration of PD*, Housing, Socioeconomic, Cause of ESRD*, Type of Catheter (Cuff), Catheter Placement, Starting PD &lt;2 weeks after catheter placement, Catheter Orientation</t>
+        </is>
+      </c>
+      <c r="Z120" t="inlineStr">
+        <is>
+          <t>Housing: Lingkungan rumah harus diadaptasi untuk memenuhi standar prosedur medis. Ruangan yang digunakan untuk pertukaran cairan harus bersih dan bebas debu untuk meminimalkan risiko infeksi, sebab partikel debu dapat menjadi vektor bagi patogen udara yang dapat mengontaminasi set transfer saat prosedur koneksi atau diskoneksi. Penyediaan wastafel di dalam atau dekat ruangan dialisis diperlukan untuk memastikan kepatuhan protokol antiseptic tangan sehingga menurunkan insiden peritonitis akibat touch contamination. Pencahayaan yang optimal di dalam ruangan diperlukan agar caregiver dapat memantau kejernihan cairan efluen serta memeriksa kondisi tempat keluar kateter dengan teliti. Hewan peliharaan tidak boleh berada di area perawatan saat proses koneksi atau diskoneksi berlangsung karena risiko paparan bakteri seperti Pasteurella multocida atau kerusakan fisik pada selang dialisis akibat gigitan atau cakaran. Selain itu, caregiverharus ditekankan untuk selalu mencuci tangan setelah berinteraksi dengan hewan dan sebelum memulai prosedur dialisis. [Sumber 1](https://www.freseniuskidneycare.com/treatment/home-dialysis/getting-prepared) [Sumber 2](https://www.ouh.nhs.uk/media/agxhnni2/85713pdialysis.pdf) [Sumber 3](https://www.kidney.org/kidney-topics/preparing-home-dialysis) [Sumber 4](https://spnp-spp.pt/media/rqdpbrom/catheter-related-infections-and-peritonitis-in-pediatric-patients-receiving-peritoneal-dialysis-guideline-for-prevention-and-treatment-2012-1-_compressed-1.pdf) [Sumber 5](https://freseniusmedicalcare.com/content/dam/home-products-education/steps2home-pd/Preventing_Peritonitis.pdf) [Sumber 6](https://www.satellitehealthcare.com/blog/pets-and-peritoneal-dialysis-absolutely/) | Socioeconomic: Deprivasi sosioekonomi berdampak pada hasil treatment yang lebih buruk. Hal ini kemungkinan disebabkan oleh keterbatasan akses terhadap fasilitas sanitasi yang memadai, tekanan psikologis pada pengasuh, serta keterbatasan informasi medis. Strategi bisa dilakukan melalui program pelatihan bagi keluarga (caregiver) dari perawat dialisis yang berpengalaman. Bagi keluarga dengan keterbatasan pendidikan atau ekonomi, dukungan teknis telepon 24 jam dan kunjungan rumah secara berkala oleh tim medis sosial sangat efektif dalam memastikan kepatuhan terhadap prosedur aseptik. Pelatihan ulang sangat dianjurkan, terutama setelah terjadinya peritonitis, untuk mengidentifikasi adanya penyimpangan dalam teknik pertukaran cairan. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC11835194/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC4934433/) [Sumber 3](https://pubmed.ncbi.nlm.nih.gov/23226378/) [Sumber 4](https://pubmed.ncbi.nlm.nih.gov/16091376/) [Sumber 6](https://spnp-spp.pt/media/rqdpbrom/catheter-related-infections-and-peritonitis-in-pediatric-patients-receiving-peritoneal-dialysis-guideline-for-prevention-and-treatment-2012-1-_compressed-1.pdf) [Sumber 7](https://pmc.ncbi.nlm.nih.gov/articles/PMC5691857/) [Sumber 8](https://pmc.ncbi.nlm.nih.gov/articles/PMC4335934/) [Sumber 9](https://www.kidney.org/kidney-topics/preparing-home-dialysis) | Type of Catheter (Cuff): Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff)untuk populasi anak secara umum. Deep cuff berfungsi untuk menjangkar kateter di otot rektus dan mencegah kebocoran, sementara superficial cuff bertindak sebagai penghalang fisik terhadap migrasi bakteri ke arah rongga peritoneum. Namun, pada neonatus atau bayi dengan dinding perut yang sangat tipis, kateter single-cuff sering kali lebih dipilih untuk mencegah ekstrusi manset ke permukaan kulit. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC10223083/) [Sumber 2](http://ispd.org/wp-content/uploads/7.-Dagmara-Borzych-Duzalka-Peritoneal-Dialysis-Catheters-Outcome-in-Children.-The-IPPN-Data.pdf) [Sumber 3](https://kidney.wiki/peritoneal-dialysis/pd-access/) | Catheter Placement: Pedoman klinis terbaru dari Society of American Gastrointestinal and Endoscopic Surgeons (SAGES) menyarankan penggunaan teknik laparoskopi tingkat lanjut (Laparoscopic) dibandingkan teknik bedah terbuka (Open) untuk pemasangan kateter pada populasi pediatrik. Laparoscopic menawarkan akurasi catheter placement yang jauh lebih tinggi di dalam rongga abdomen karena visualisasi langsung, serta meminimalkan trauma mekanis pada jaringan perut. Lebih lanjut, Laparoscopic memungkinkan dokter untuk melakukan prosedur profilaksis penting seperti omentektomi atau omentopeksi untuk meminimalkan risiko omental wrapping (penyumbatan kateter oleh omentum), yang merupakan salah satu penyebab utama kegagalan mekanis kateter pada anak-anak. Laparoscopic juga terbukti mempermudah penyelamatan (salvage) jika terjadi malposisi atau disfungsi kateter tanpa harus melakukan pembedahan ulang yang invasif. [Sumber 1](https://www.sages.org/publications/guidelines/peritoneal-dialysis-access-guideline-update-2023/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC10223083/) [[3]](https://kidney.wiki/peritoneal-dialysis/pd-access/) | Starting PD &lt;2 weeks after catheter placement: Waktu antara pemasangan kateter dan dimulainya dialisis (break-in-period) merupakan faktor penting untuk mencegah komplikasi. Masa penyembuhan minimal 2 minggu sebelum dialysis dimulai. Namun, dalam kondisi klinis tertentu di mana pasien membutuhkan dialisis segera, urgent-start PD (dimulai dalam &lt;14 hari atau bahkan &lt;48 jam) menjadi alternatif yang baik untuk menghindari penggunakan kateter hemodialysis sementara. Pasien dengan break-in-period &lt; 7 hari memiliki risiko yang lebih tinggi terhadap komplikasi awal seperti kebocoran dialisat dan malposisi kateter. Namun, risiko tersebut tidak berkorelasi dengan penurunan kelangsungan hidup atau peningkatan risiko peritonitis jika dilakukan dengan protokol yang tepat. Pada kondisi urgent-start, risiko kebocoran dimitigasi dengan menggunakan volume pengisian rendah (10-20 ml/kg) dan posisi pasien supine untuk mengurangi tekanan intra-abdominal.[Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC3923692/) [Sumber 2](https://journals.plos.org/plosone/article?id=10.1371/journal.pone.0206426) [Sumber 3](https://www.sages.org/publications/guidelines/peritoneal-dialysis-access-guideline-update-2023/) [Sumber 4](https://www.frontiersin.org/journals/endocrinology/articles/10.3389/fendo.2022.936573/full) [Sumber 5](https://scholarlyexchange.childrensmercy.org/cgi/viewcontent.cgi?article=7522&amp;context=papers) [Sumber 6](https://pubmed.ncbi.nlm.nih.gov/33523772/) [Sumber 7](https://www.bcrenal.ca/resource-gallery/Documents/PD_Procedures-Exit_Site_Care-Post-Operative_PD_Catheter_Insertion.pdf) | Catheter Orientation: Posisi atau arah lubang keluar kateter (exit site) sangat memengaruhi risiko terjadinya infeksi. Data multisentrik dari SCOPE Collaborative menunjukkan bahwa orientasi kateter yang menghadap ke atas (Upward) dikaitkan dengan peningkatan risiko peritonitis hingga 4.2 kali lipat (Rate Ratio: 4.2; 95% CI: 1.49–11.89) dibandingkan orientasi lainnya. Secara anatomis, lubang keluar yang menghadap ke atas menciptakan bentuk cekungan yang dapat menampung keringat, air mandi, dan kotoran. Akibat gaya gravitasi, bakteri yang terkumpul di area ini akan mengendap dan bermigrasi ke dalam terowongan kateter. Oleh karena itu, lubang keluar kateter harus selalu diarahkan ke bawah (Downward) atau ke samping (Lateral) untuk mencegah penumpukan bakteri secara alami. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC5012476/) [Sumber 2](https://openurologyandnephrologyjournal.com/VOLUME/5/PAGE/4/) [Sumber 3](https://kidney.wiki/peritoneal-dialysis/pd-access/)</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>2026-05-19 12:45:29</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>18F27E0F</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>&gt;2 yo</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>&gt;12 mo</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>Fair/poor service</t>
+        </is>
+      </c>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>Poor/fair</t>
+        </is>
+      </c>
+      <c r="J121" t="inlineStr">
+        <is>
+          <t>Studies</t>
+        </is>
+      </c>
+      <c r="K121" t="inlineStr">
+        <is>
+          <t>No ESI</t>
+        </is>
+      </c>
+      <c r="L121" t="inlineStr">
+        <is>
+          <t>Normal Nutrition</t>
+        </is>
+      </c>
+      <c r="M121" t="inlineStr">
+        <is>
+          <t>Non-glomerular</t>
+        </is>
+      </c>
+      <c r="N121" t="inlineStr">
+        <is>
+          <t>Coiled/swan neck</t>
+        </is>
+      </c>
+      <c r="O121" t="inlineStr">
+        <is>
+          <t>Single cuff</t>
+        </is>
+      </c>
+      <c r="P121" t="inlineStr">
+        <is>
+          <t>Laparoscopic</t>
+        </is>
+      </c>
+      <c r="Q121" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R121" t="inlineStr">
+        <is>
+          <t>Patients</t>
+        </is>
+      </c>
+      <c r="S121" t="inlineStr"/>
+      <c r="T121" t="inlineStr">
+        <is>
+          <t>upward</t>
+        </is>
+      </c>
+      <c r="U121" t="inlineStr">
+        <is>
+          <t>No stunting</t>
+        </is>
+      </c>
+      <c r="V121" t="inlineStr"/>
+      <c r="W121" t="inlineStr"/>
+      <c r="X121" t="inlineStr"/>
+      <c r="Y121" t="inlineStr">
+        <is>
+          <t>Duration of PD*, Housing, Socioeconomic, Cause of ESRD*, Type of Catheter (Cuff), Catheter Placement, Starting PD &lt;2 weeks after catheter placement, Catheter Orientation</t>
+        </is>
+      </c>
+      <c r="Z121" t="inlineStr">
+        <is>
+          <t>Housing: Lingkungan rumah harus diadaptasi untuk memenuhi standar prosedur medis. Ruangan yang digunakan untuk pertukaran cairan harus bersih dan bebas debu untuk meminimalkan risiko infeksi, sebab partikel debu dapat menjadi vektor bagi patogen udara yang dapat mengontaminasi set transfer saat prosedur koneksi atau diskoneksi. Penyediaan wastafel di dalam atau dekat ruangan dialisis diperlukan untuk memastikan kepatuhan protokol antiseptic tangan sehingga menurunkan insiden peritonitis akibat touch contamination. Pencahayaan yang optimal di dalam ruangan diperlukan agar caregiver dapat memantau kejernihan cairan efluen serta memeriksa kondisi tempat keluar kateter dengan teliti. Hewan peliharaan tidak boleh berada di area perawatan saat proses koneksi atau diskoneksi berlangsung karena risiko paparan bakteri seperti Pasteurella multocida atau kerusakan fisik pada selang dialisis akibat gigitan atau cakaran. Selain itu, caregiverharus ditekankan untuk selalu mencuci tangan setelah berinteraksi dengan hewan dan sebelum memulai prosedur dialisis. [Sumber 1](https://www.freseniuskidneycare.com/treatment/home-dialysis/getting-prepared) [Sumber 2](https://www.ouh.nhs.uk/media/agxhnni2/85713pdialysis.pdf) [Sumber 3](https://www.kidney.org/kidney-topics/preparing-home-dialysis) [Sumber 4](https://spnp-spp.pt/media/rqdpbrom/catheter-related-infections-and-peritonitis-in-pediatric-patients-receiving-peritoneal-dialysis-guideline-for-prevention-and-treatment-2012-1-_compressed-1.pdf) [Sumber 5](https://freseniusmedicalcare.com/content/dam/home-products-education/steps2home-pd/Preventing_Peritonitis.pdf) [Sumber 6](https://www.satellitehealthcare.com/blog/pets-and-peritoneal-dialysis-absolutely/) | Socioeconomic: Deprivasi sosioekonomi berdampak pada hasil treatment yang lebih buruk. Hal ini kemungkinan disebabkan oleh keterbatasan akses terhadap fasilitas sanitasi yang memadai, tekanan psikologis pada pengasuh, serta keterbatasan informasi medis. Strategi bisa dilakukan melalui program pelatihan bagi keluarga (caregiver) dari perawat dialisis yang berpengalaman. Bagi keluarga dengan keterbatasan pendidikan atau ekonomi, dukungan teknis telepon 24 jam dan kunjungan rumah secara berkala oleh tim medis sosial sangat efektif dalam memastikan kepatuhan terhadap prosedur aseptik. Pelatihan ulang sangat dianjurkan, terutama setelah terjadinya peritonitis, untuk mengidentifikasi adanya penyimpangan dalam teknik pertukaran cairan. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC11835194/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC4934433/) [Sumber 3](https://pubmed.ncbi.nlm.nih.gov/23226378/) [Sumber 4](https://pubmed.ncbi.nlm.nih.gov/16091376/) [Sumber 6](https://spnp-spp.pt/media/rqdpbrom/catheter-related-infections-and-peritonitis-in-pediatric-patients-receiving-peritoneal-dialysis-guideline-for-prevention-and-treatment-2012-1-_compressed-1.pdf) [Sumber 7](https://pmc.ncbi.nlm.nih.gov/articles/PMC5691857/) [Sumber 8](https://pmc.ncbi.nlm.nih.gov/articles/PMC4335934/) [Sumber 9](https://www.kidney.org/kidney-topics/preparing-home-dialysis) | Type of Catheter (Cuff): Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff)untuk populasi anak secara umum. Deep cuff berfungsi untuk menjangkar kateter di otot rektus dan mencegah kebocoran, sementara superficial cuff bertindak sebagai penghalang fisik terhadap migrasi bakteri ke arah rongga peritoneum. Namun, pada neonatus atau bayi dengan dinding perut yang sangat tipis, kateter single-cuff sering kali lebih dipilih untuk mencegah ekstrusi manset ke permukaan kulit. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC10223083/) [Sumber 2](http://ispd.org/wp-content/uploads/7.-Dagmara-Borzych-Duzalka-Peritoneal-Dialysis-Catheters-Outcome-in-Children.-The-IPPN-Data.pdf) [Sumber 3](https://kidney.wiki/peritoneal-dialysis/pd-access/) | Catheter Placement: Pedoman klinis terbaru dari Society of American Gastrointestinal and Endoscopic Surgeons (SAGES) menyarankan penggunaan teknik laparoskopi tingkat lanjut (Laparoscopic) dibandingkan teknik bedah terbuka (Open) untuk pemasangan kateter pada populasi pediatrik. Laparoscopic menawarkan akurasi catheter placement yang jauh lebih tinggi di dalam rongga abdomen karena visualisasi langsung, serta meminimalkan trauma mekanis pada jaringan perut. Lebih lanjut, Laparoscopic memungkinkan dokter untuk melakukan prosedur profilaksis penting seperti omentektomi atau omentopeksi untuk meminimalkan risiko omental wrapping (penyumbatan kateter oleh omentum), yang merupakan salah satu penyebab utama kegagalan mekanis kateter pada anak-anak. Laparoscopic juga terbukti mempermudah penyelamatan (salvage) jika terjadi malposisi atau disfungsi kateter tanpa harus melakukan pembedahan ulang yang invasif. [Sumber 1](https://www.sages.org/publications/guidelines/peritoneal-dialysis-access-guideline-update-2023/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC10223083/) [[3]](https://kidney.wiki/peritoneal-dialysis/pd-access/) | Starting PD &lt;2 weeks after catheter placement: Waktu antara pemasangan kateter dan dimulainya dialisis (break-in-period) merupakan faktor penting untuk mencegah komplikasi. Masa penyembuhan minimal 2 minggu sebelum dialysis dimulai. Namun, dalam kondisi klinis tertentu di mana pasien membutuhkan dialisis segera, urgent-start PD (dimulai dalam &lt;14 hari atau bahkan &lt;48 jam) menjadi alternatif yang baik untuk menghindari penggunakan kateter hemodialysis sementara. Pasien dengan break-in-period &lt; 7 hari memiliki risiko yang lebih tinggi terhadap komplikasi awal seperti kebocoran dialisat dan malposisi kateter. Namun, risiko tersebut tidak berkorelasi dengan penurunan kelangsungan hidup atau peningkatan risiko peritonitis jika dilakukan dengan protokol yang tepat. Pada kondisi urgent-start, risiko kebocoran dimitigasi dengan menggunakan volume pengisian rendah (10-20 ml/kg) dan posisi pasien supine untuk mengurangi tekanan intra-abdominal.[Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC3923692/) [Sumber 2](https://journals.plos.org/plosone/article?id=10.1371/journal.pone.0206426) [Sumber 3](https://www.sages.org/publications/guidelines/peritoneal-dialysis-access-guideline-update-2023/) [Sumber 4](https://www.frontiersin.org/journals/endocrinology/articles/10.3389/fendo.2022.936573/full) [Sumber 5](https://scholarlyexchange.childrensmercy.org/cgi/viewcontent.cgi?article=7522&amp;context=papers) [Sumber 6](https://pubmed.ncbi.nlm.nih.gov/33523772/) [Sumber 7](https://www.bcrenal.ca/resource-gallery/Documents/PD_Procedures-Exit_Site_Care-Post-Operative_PD_Catheter_Insertion.pdf) | Catheter Orientation: Posisi atau arah lubang keluar kateter (exit site) sangat memengaruhi risiko terjadinya infeksi. Data multisentrik dari SCOPE Collaborative menunjukkan bahwa orientasi kateter yang menghadap ke atas (Upward) dikaitkan dengan peningkatan risiko peritonitis hingga 4.2 kali lipat (Rate Ratio: 4.2; 95% CI: 1.49–11.89) dibandingkan orientasi lainnya. Secara anatomis, lubang keluar yang menghadap ke atas menciptakan bentuk cekungan yang dapat menampung keringat, air mandi, dan kotoran. Akibat gaya gravitasi, bakteri yang terkumpul di area ini akan mengendap dan bermigrasi ke dalam terowongan kateter. Oleh karena itu, lubang keluar kateter harus selalu diarahkan ke bawah (Downward) atau ke samping (Lateral) untuk mencegah penumpukan bakteri secara alami. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC5012476/) [Sumber 2](https://openurologyandnephrologyjournal.com/VOLUME/5/PAGE/4/) [Sumber 3](https://kidney.wiki/peritoneal-dialysis/pd-access/)</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>2026-05-19 12:45:59</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>18F27E0F</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>&gt;2 yo</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>&gt;12 mo</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>Fair/poor service</t>
+        </is>
+      </c>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>Poor/fair</t>
+        </is>
+      </c>
+      <c r="J122" t="inlineStr">
+        <is>
+          <t>Studies</t>
+        </is>
+      </c>
+      <c r="K122" t="inlineStr">
+        <is>
+          <t>No ESI</t>
+        </is>
+      </c>
+      <c r="L122" t="inlineStr">
+        <is>
+          <t>Normal Nutrition</t>
+        </is>
+      </c>
+      <c r="M122" t="inlineStr">
+        <is>
+          <t>Non-glomerular</t>
+        </is>
+      </c>
+      <c r="N122" t="inlineStr">
+        <is>
+          <t>Coiled/swan neck</t>
+        </is>
+      </c>
+      <c r="O122" t="inlineStr">
+        <is>
+          <t>Single cuff</t>
+        </is>
+      </c>
+      <c r="P122" t="inlineStr">
+        <is>
+          <t>Laparoscopic</t>
+        </is>
+      </c>
+      <c r="Q122" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R122" t="inlineStr">
+        <is>
+          <t>Patients</t>
+        </is>
+      </c>
+      <c r="S122" t="inlineStr"/>
+      <c r="T122" t="inlineStr">
+        <is>
+          <t>upward</t>
+        </is>
+      </c>
+      <c r="U122" t="inlineStr">
+        <is>
+          <t>No stunting</t>
+        </is>
+      </c>
+      <c r="V122" t="inlineStr"/>
+      <c r="W122" t="inlineStr"/>
+      <c r="X122" t="inlineStr"/>
+      <c r="Y122" t="inlineStr">
+        <is>
+          <t>Duration of PD*, Housing, Socioeconomic, Cause of ESRD*, Type of Catheter (Cuff), Catheter Placement, Starting PD &lt;2 weeks after catheter placement, Catheter Orientation</t>
+        </is>
+      </c>
+      <c r="Z122" t="inlineStr">
+        <is>
+          <t>Housing: Lingkungan rumah harus diadaptasi untuk memenuhi standar prosedur medis. Ruangan yang digunakan untuk pertukaran cairan harus bersih dan bebas debu untuk meminimalkan risiko infeksi, sebab partikel debu dapat menjadi vektor bagi patogen udara yang dapat mengontaminasi set transfer saat prosedur koneksi atau diskoneksi. Penyediaan wastafel di dalam atau dekat ruangan dialisis diperlukan untuk memastikan kepatuhan protokol antiseptic tangan sehingga menurunkan insiden peritonitis akibat touch contamination. Pencahayaan yang optimal di dalam ruangan diperlukan agar caregiver dapat memantau kejernihan cairan efluen serta memeriksa kondisi tempat keluar kateter dengan teliti. Hewan peliharaan tidak boleh berada di area perawatan saat proses koneksi atau diskoneksi berlangsung karena risiko paparan bakteri seperti Pasteurella multocida atau kerusakan fisik pada selang dialisis akibat gigitan atau cakaran. Selain itu, caregiverharus ditekankan untuk selalu mencuci tangan setelah berinteraksi dengan hewan dan sebelum memulai prosedur dialisis. [Sumber 1](https://www.freseniuskidneycare.com/treatment/home-dialysis/getting-prepared) [Sumber 2](https://www.ouh.nhs.uk/media/agxhnni2/85713pdialysis.pdf) [Sumber 3](https://www.kidney.org/kidney-topics/preparing-home-dialysis) [Sumber 4](https://spnp-spp.pt/media/rqdpbrom/catheter-related-infections-and-peritonitis-in-pediatric-patients-receiving-peritoneal-dialysis-guideline-for-prevention-and-treatment-2012-1-_compressed-1.pdf) [Sumber 5](https://freseniusmedicalcare.com/content/dam/home-products-education/steps2home-pd/Preventing_Peritonitis.pdf) [Sumber 6](https://www.satellitehealthcare.com/blog/pets-and-peritoneal-dialysis-absolutely/) | Socioeconomic: Deprivasi sosioekonomi berdampak pada hasil treatment yang lebih buruk. Hal ini kemungkinan disebabkan oleh keterbatasan akses terhadap fasilitas sanitasi yang memadai, tekanan psikologis pada pengasuh, serta keterbatasan informasi medis. Strategi bisa dilakukan melalui program pelatihan bagi keluarga (caregiver) dari perawat dialisis yang berpengalaman. Bagi keluarga dengan keterbatasan pendidikan atau ekonomi, dukungan teknis telepon 24 jam dan kunjungan rumah secara berkala oleh tim medis sosial sangat efektif dalam memastikan kepatuhan terhadap prosedur aseptik. Pelatihan ulang sangat dianjurkan, terutama setelah terjadinya peritonitis, untuk mengidentifikasi adanya penyimpangan dalam teknik pertukaran cairan. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC11835194/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC4934433/) [Sumber 3](https://pubmed.ncbi.nlm.nih.gov/23226378/) [Sumber 4](https://pubmed.ncbi.nlm.nih.gov/16091376/) [Sumber 6](https://spnp-spp.pt/media/rqdpbrom/catheter-related-infections-and-peritonitis-in-pediatric-patients-receiving-peritoneal-dialysis-guideline-for-prevention-and-treatment-2012-1-_compressed-1.pdf) [Sumber 7](https://pmc.ncbi.nlm.nih.gov/articles/PMC5691857/) [Sumber 8](https://pmc.ncbi.nlm.nih.gov/articles/PMC4335934/) [Sumber 9](https://www.kidney.org/kidney-topics/preparing-home-dialysis) | Type of Catheter (Cuff): Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff)untuk populasi anak secara umum. Deep cuff berfungsi untuk menjangkar kateter di otot rektus dan mencegah kebocoran, sementara superficial cuff bertindak sebagai penghalang fisik terhadap migrasi bakteri ke arah rongga peritoneum. Namun, pada neonatus atau bayi dengan dinding perut yang sangat tipis, kateter single-cuff sering kali lebih dipilih untuk mencegah ekstrusi manset ke permukaan kulit. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC10223083/) [Sumber 2](http://ispd.org/wp-content/uploads/7.-Dagmara-Borzych-Duzalka-Peritoneal-Dialysis-Catheters-Outcome-in-Children.-The-IPPN-Data.pdf) [Sumber 3](https://kidney.wiki/peritoneal-dialysis/pd-access/) | Catheter Placement: Pedoman klinis terbaru dari Society of American Gastrointestinal and Endoscopic Surgeons (SAGES) menyarankan penggunaan teknik laparoskopi tingkat lanjut (Laparoscopic) dibandingkan teknik bedah terbuka (Open) untuk pemasangan kateter pada populasi pediatrik. Laparoscopic menawarkan akurasi catheter placement yang jauh lebih tinggi di dalam rongga abdomen karena visualisasi langsung, serta meminimalkan trauma mekanis pada jaringan perut. Lebih lanjut, Laparoscopic memungkinkan dokter untuk melakukan prosedur profilaksis penting seperti omentektomi atau omentopeksi untuk meminimalkan risiko omental wrapping (penyumbatan kateter oleh omentum), yang merupakan salah satu penyebab utama kegagalan mekanis kateter pada anak-anak. Laparoscopic juga terbukti mempermudah penyelamatan (salvage) jika terjadi malposisi atau disfungsi kateter tanpa harus melakukan pembedahan ulang yang invasif. [Sumber 1](https://www.sages.org/publications/guidelines/peritoneal-dialysis-access-guideline-update-2023/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC10223083/) [[3]](https://kidney.wiki/peritoneal-dialysis/pd-access/) | Starting PD &lt;2 weeks after catheter placement: Waktu antara pemasangan kateter dan dimulainya dialisis (break-in-period) merupakan faktor penting untuk mencegah komplikasi. Masa penyembuhan minimal 2 minggu sebelum dialysis dimulai. Namun, dalam kondisi klinis tertentu di mana pasien membutuhkan dialisis segera, urgent-start PD (dimulai dalam &lt;14 hari atau bahkan &lt;48 jam) menjadi alternatif yang baik untuk menghindari penggunakan kateter hemodialysis sementara. Pasien dengan break-in-period &lt; 7 hari memiliki risiko yang lebih tinggi terhadap komplikasi awal seperti kebocoran dialisat dan malposisi kateter. Namun, risiko tersebut tidak berkorelasi dengan penurunan kelangsungan hidup atau peningkatan risiko peritonitis jika dilakukan dengan protokol yang tepat. Pada kondisi urgent-start, risiko kebocoran dimitigasi dengan menggunakan volume pengisian rendah (10-20 ml/kg) dan posisi pasien supine untuk mengurangi tekanan intra-abdominal.[Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC3923692/) [Sumber 2](https://journals.plos.org/plosone/article?id=10.1371/journal.pone.0206426) [Sumber 3](https://www.sages.org/publications/guidelines/peritoneal-dialysis-access-guideline-update-2023/) [Sumber 4](https://www.frontiersin.org/journals/endocrinology/articles/10.3389/fendo.2022.936573/full) [Sumber 5](https://scholarlyexchange.childrensmercy.org/cgi/viewcontent.cgi?article=7522&amp;context=papers) [Sumber 6](https://pubmed.ncbi.nlm.nih.gov/33523772/) [Sumber 7](https://www.bcrenal.ca/resource-gallery/Documents/PD_Procedures-Exit_Site_Care-Post-Operative_PD_Catheter_Insertion.pdf) | Catheter Orientation: Posisi atau arah lubang keluar kateter (exit site) sangat memengaruhi risiko terjadinya infeksi. Data multisentrik dari SCOPE Collaborative menunjukkan bahwa orientasi kateter yang menghadap ke atas (Upward) dikaitkan dengan peningkatan risiko peritonitis hingga 4.2 kali lipat (Rate Ratio: 4.2; 95% CI: 1.49–11.89) dibandingkan orientasi lainnya. Secara anatomis, lubang keluar yang menghadap ke atas menciptakan bentuk cekungan yang dapat menampung keringat, air mandi, dan kotoran. Akibat gaya gravitasi, bakteri yang terkumpul di area ini akan mengendap dan bermigrasi ke dalam terowongan kateter. Oleh karena itu, lubang keluar kateter harus selalu diarahkan ke bawah (Downward) atau ke samping (Lateral) untuk mencegah penumpukan bakteri secara alami. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC5012476/) [Sumber 2](https://openurologyandnephrologyjournal.com/VOLUME/5/PAGE/4/) [Sumber 3](https://kidney.wiki/peritoneal-dialysis/pd-access/)</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>2026-05-19 12:46:18</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>18F27E0F</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>&gt;2 yo</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>&gt;12 mo</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>Fair/poor service</t>
+        </is>
+      </c>
+      <c r="I123" t="inlineStr">
+        <is>
+          <t>Poor/fair</t>
+        </is>
+      </c>
+      <c r="J123" t="inlineStr">
+        <is>
+          <t>Studies</t>
+        </is>
+      </c>
+      <c r="K123" t="inlineStr">
+        <is>
+          <t>No ESI</t>
+        </is>
+      </c>
+      <c r="L123" t="inlineStr">
+        <is>
+          <t>Normal Nutrition</t>
+        </is>
+      </c>
+      <c r="M123" t="inlineStr">
+        <is>
+          <t>Non-glomerular</t>
+        </is>
+      </c>
+      <c r="N123" t="inlineStr">
+        <is>
+          <t>Coiled/swan neck</t>
+        </is>
+      </c>
+      <c r="O123" t="inlineStr">
+        <is>
+          <t>Single cuff</t>
+        </is>
+      </c>
+      <c r="P123" t="inlineStr">
+        <is>
+          <t>Laparoscopic</t>
+        </is>
+      </c>
+      <c r="Q123" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R123" t="inlineStr">
+        <is>
+          <t>Patients</t>
+        </is>
+      </c>
+      <c r="S123" t="inlineStr"/>
+      <c r="T123" t="inlineStr">
+        <is>
+          <t>upward</t>
+        </is>
+      </c>
+      <c r="U123" t="inlineStr">
+        <is>
+          <t>No stunting</t>
+        </is>
+      </c>
+      <c r="V123" t="inlineStr"/>
+      <c r="W123" t="inlineStr"/>
+      <c r="X123" t="inlineStr"/>
+      <c r="Y123" t="inlineStr">
+        <is>
+          <t>Duration of PD*, Housing, Socioeconomic, Cause of ESRD*, Type of Catheter (Cuff), Catheter Placement, Starting PD &lt;2 weeks after catheter placement, Catheter Orientation</t>
+        </is>
+      </c>
+      <c r="Z123" t="inlineStr">
+        <is>
+          <t>Housing: Lingkungan rumah harus diadaptasi untuk memenuhi standar prosedur medis. Ruangan yang digunakan untuk pertukaran cairan harus bersih dan bebas debu untuk meminimalkan risiko infeksi, sebab partikel debu dapat menjadi vektor bagi patogen udara yang dapat mengontaminasi set transfer saat prosedur koneksi atau diskoneksi. Penyediaan wastafel di dalam atau dekat ruangan dialisis diperlukan untuk memastikan kepatuhan protokol antiseptic tangan sehingga menurunkan insiden peritonitis akibat touch contamination. Pencahayaan yang optimal di dalam ruangan diperlukan agar caregiver dapat memantau kejernihan cairan efluen serta memeriksa kondisi tempat keluar kateter dengan teliti. Hewan peliharaan tidak boleh berada di area perawatan saat proses koneksi atau diskoneksi berlangsung karena risiko paparan bakteri seperti Pasteurella multocida atau kerusakan fisik pada selang dialisis akibat gigitan atau cakaran. Selain itu, caregiverharus ditekankan untuk selalu mencuci tangan setelah berinteraksi dengan hewan dan sebelum memulai prosedur dialisis. [Sumber 1](https://www.freseniuskidneycare.com/treatment/home-dialysis/getting-prepared) [Sumber 2](https://www.ouh.nhs.uk/media/agxhnni2/85713pdialysis.pdf) [Sumber 3](https://www.kidney.org/kidney-topics/preparing-home-dialysis) [Sumber 4](https://spnp-spp.pt/media/rqdpbrom/catheter-related-infections-and-peritonitis-in-pediatric-patients-receiving-peritoneal-dialysis-guideline-for-prevention-and-treatment-2012-1-_compressed-1.pdf) [Sumber 5](https://freseniusmedicalcare.com/content/dam/home-products-education/steps2home-pd/Preventing_Peritonitis.pdf) [Sumber 6](https://www.satellitehealthcare.com/blog/pets-and-peritoneal-dialysis-absolutely/) | Socioeconomic: Deprivasi sosioekonomi berdampak pada hasil treatment yang lebih buruk. Hal ini kemungkinan disebabkan oleh keterbatasan akses terhadap fasilitas sanitasi yang memadai, tekanan psikologis pada pengasuh, serta keterbatasan informasi medis. Strategi bisa dilakukan melalui program pelatihan bagi keluarga (caregiver) dari perawat dialisis yang berpengalaman. Bagi keluarga dengan keterbatasan pendidikan atau ekonomi, dukungan teknis telepon 24 jam dan kunjungan rumah secara berkala oleh tim medis sosial sangat efektif dalam memastikan kepatuhan terhadap prosedur aseptik. Pelatihan ulang sangat dianjurkan, terutama setelah terjadinya peritonitis, untuk mengidentifikasi adanya penyimpangan dalam teknik pertukaran cairan. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC11835194/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC4934433/) [Sumber 3](https://pubmed.ncbi.nlm.nih.gov/23226378/) [Sumber 4](https://pubmed.ncbi.nlm.nih.gov/16091376/) [Sumber 6](https://spnp-spp.pt/media/rqdpbrom/catheter-related-infections-and-peritonitis-in-pediatric-patients-receiving-peritoneal-dialysis-guideline-for-prevention-and-treatment-2012-1-_compressed-1.pdf) [Sumber 7](https://pmc.ncbi.nlm.nih.gov/articles/PMC5691857/) [Sumber 8](https://pmc.ncbi.nlm.nih.gov/articles/PMC4335934/) [Sumber 9](https://www.kidney.org/kidney-topics/preparing-home-dialysis) | Type of Catheter (Cuff): Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff)untuk populasi anak secara umum. Deep cuff berfungsi untuk menjangkar kateter di otot rektus dan mencegah kebocoran, sementara superficial cuff bertindak sebagai penghalang fisik terhadap migrasi bakteri ke arah rongga peritoneum. Namun, pada neonatus atau bayi dengan dinding perut yang sangat tipis, kateter single-cuff sering kali lebih dipilih untuk mencegah ekstrusi manset ke permukaan kulit. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC10223083/) [Sumber 2](http://ispd.org/wp-content/uploads/7.-Dagmara-Borzych-Duzalka-Peritoneal-Dialysis-Catheters-Outcome-in-Children.-The-IPPN-Data.pdf) [Sumber 3](https://kidney.wiki/peritoneal-dialysis/pd-access/) | Catheter Placement: Pedoman klinis terbaru dari Society of American Gastrointestinal and Endoscopic Surgeons (SAGES) menyarankan penggunaan teknik laparoskopi tingkat lanjut (Laparoscopic) dibandingkan teknik bedah terbuka (Open) untuk pemasangan kateter pada populasi pediatrik. Laparoscopic menawarkan akurasi catheter placement yang jauh lebih tinggi di dalam rongga abdomen karena visualisasi langsung, serta meminimalkan trauma mekanis pada jaringan perut. Lebih lanjut, Laparoscopic memungkinkan dokter untuk melakukan prosedur profilaksis penting seperti omentektomi atau omentopeksi untuk meminimalkan risiko omental wrapping (penyumbatan kateter oleh omentum), yang merupakan salah satu penyebab utama kegagalan mekanis kateter pada anak-anak. Laparoscopic juga terbukti mempermudah penyelamatan (salvage) jika terjadi malposisi atau disfungsi kateter tanpa harus melakukan pembedahan ulang yang invasif. [Sumber 1](https://www.sages.org/publications/guidelines/peritoneal-dialysis-access-guideline-update-2023/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC10223083/) [[3]](https://kidney.wiki/peritoneal-dialysis/pd-access/) | Starting PD &lt;2 weeks after catheter placement: Waktu antara pemasangan kateter dan dimulainya dialisis (break-in-period) merupakan faktor penting untuk mencegah komplikasi. Masa penyembuhan minimal 2 minggu sebelum dialysis dimulai. Namun, dalam kondisi klinis tertentu di mana pasien membutuhkan dialisis segera, urgent-start PD (dimulai dalam &lt;14 hari atau bahkan &lt;48 jam) menjadi alternatif yang baik untuk menghindari penggunakan kateter hemodialysis sementara. Pasien dengan break-in-period &lt; 7 hari memiliki risiko yang lebih tinggi terhadap komplikasi awal seperti kebocoran dialisat dan malposisi kateter. Namun, risiko tersebut tidak berkorelasi dengan penurunan kelangsungan hidup atau peningkatan risiko peritonitis jika dilakukan dengan protokol yang tepat. Pada kondisi urgent-start, risiko kebocoran dimitigasi dengan menggunakan volume pengisian rendah (10-20 ml/kg) dan posisi pasien supine untuk mengurangi tekanan intra-abdominal.[Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC3923692/) [Sumber 2](https://journals.plos.org/plosone/article?id=10.1371/journal.pone.0206426) [Sumber 3](https://www.sages.org/publications/guidelines/peritoneal-dialysis-access-guideline-update-2023/) [Sumber 4](https://www.frontiersin.org/journals/endocrinology/articles/10.3389/fendo.2022.936573/full) [Sumber 5](https://scholarlyexchange.childrensmercy.org/cgi/viewcontent.cgi?article=7522&amp;context=papers) [Sumber 6](https://pubmed.ncbi.nlm.nih.gov/33523772/) [Sumber 7](https://www.bcrenal.ca/resource-gallery/Documents/PD_Procedures-Exit_Site_Care-Post-Operative_PD_Catheter_Insertion.pdf) | Catheter Orientation: Posisi atau arah lubang keluar kateter (exit site) sangat memengaruhi risiko terjadinya infeksi. Data multisentrik dari SCOPE Collaborative menunjukkan bahwa orientasi kateter yang menghadap ke atas (Upward) dikaitkan dengan peningkatan risiko peritonitis hingga 4.2 kali lipat (Rate Ratio: 4.2; 95% CI: 1.49–11.89) dibandingkan orientasi lainnya. Secara anatomis, lubang keluar yang menghadap ke atas menciptakan bentuk cekungan yang dapat menampung keringat, air mandi, dan kotoran. Akibat gaya gravitasi, bakteri yang terkumpul di area ini akan mengendap dan bermigrasi ke dalam terowongan kateter. Oleh karena itu, lubang keluar kateter harus selalu diarahkan ke bawah (Downward) atau ke samping (Lateral) untuk mencegah penumpukan bakteri secara alami. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC5012476/) [Sumber 2](https://openurologyandnephrologyjournal.com/VOLUME/5/PAGE/4/) [Sumber 3](https://kidney.wiki/peritoneal-dialysis/pd-access/)</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>2026-05-19 12:46:44</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>18F27E0F</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>&gt;2 yo</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>&gt;12 mo</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>Fair/poor service</t>
+        </is>
+      </c>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>Poor/fair</t>
+        </is>
+      </c>
+      <c r="J124" t="inlineStr">
+        <is>
+          <t>Studies</t>
+        </is>
+      </c>
+      <c r="K124" t="inlineStr">
+        <is>
+          <t>No ESI</t>
+        </is>
+      </c>
+      <c r="L124" t="inlineStr">
+        <is>
+          <t>Normal Nutrition</t>
+        </is>
+      </c>
+      <c r="M124" t="inlineStr">
+        <is>
+          <t>Non-glomerular</t>
+        </is>
+      </c>
+      <c r="N124" t="inlineStr">
+        <is>
+          <t>Coiled/swan neck</t>
+        </is>
+      </c>
+      <c r="O124" t="inlineStr">
+        <is>
+          <t>Single cuff</t>
+        </is>
+      </c>
+      <c r="P124" t="inlineStr">
+        <is>
+          <t>Laparoscopic</t>
+        </is>
+      </c>
+      <c r="Q124" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R124" t="inlineStr">
+        <is>
+          <t>Patients</t>
+        </is>
+      </c>
+      <c r="S124" t="inlineStr"/>
+      <c r="T124" t="inlineStr">
+        <is>
+          <t>upward</t>
+        </is>
+      </c>
+      <c r="U124" t="inlineStr">
+        <is>
+          <t>No stunting</t>
+        </is>
+      </c>
+      <c r="V124" t="inlineStr"/>
+      <c r="W124" t="inlineStr"/>
+      <c r="X124" t="inlineStr"/>
+      <c r="Y124" t="inlineStr">
+        <is>
+          <t>Duration of PD*, Housing, Socioeconomic, Cause of ESRD*, Type of Catheter (Cuff), Catheter Placement, Starting PD &lt;2 weeks after catheter placement, Catheter Orientation</t>
+        </is>
+      </c>
+      <c r="Z124" t="inlineStr">
+        <is>
+          <t>Housing: Lingkungan rumah harus diadaptasi untuk memenuhi standar prosedur medis. Ruangan yang digunakan untuk pertukaran cairan harus bersih dan bebas debu untuk meminimalkan risiko infeksi, sebab partikel debu dapat menjadi vektor bagi patogen udara yang dapat mengontaminasi set transfer saat prosedur koneksi atau diskoneksi. Penyediaan wastafel di dalam atau dekat ruangan dialisis diperlukan untuk memastikan kepatuhan protokol antiseptic tangan sehingga menurunkan insiden peritonitis akibat touch contamination. Pencahayaan yang optimal di dalam ruangan diperlukan agar caregiver dapat memantau kejernihan cairan efluen serta memeriksa kondisi tempat keluar kateter dengan teliti. Hewan peliharaan tidak boleh berada di area perawatan saat proses koneksi atau diskoneksi berlangsung karena risiko paparan bakteri seperti Pasteurella multocida atau kerusakan fisik pada selang dialisis akibat gigitan atau cakaran. Selain itu, caregiverharus ditekankan untuk selalu mencuci tangan setelah berinteraksi dengan hewan dan sebelum memulai prosedur dialisis. [Sumber 1](https://www.freseniuskidneycare.com/treatment/home-dialysis/getting-prepared) [Sumber 2](https://www.ouh.nhs.uk/media/agxhnni2/85713pdialysis.pdf) [Sumber 3](https://www.kidney.org/kidney-topics/preparing-home-dialysis) [Sumber 4](https://spnp-spp.pt/media/rqdpbrom/catheter-related-infections-and-peritonitis-in-pediatric-patients-receiving-peritoneal-dialysis-guideline-for-prevention-and-treatment-2012-1-_compressed-1.pdf) [Sumber 5](https://freseniusmedicalcare.com/content/dam/home-products-education/steps2home-pd/Preventing_Peritonitis.pdf) [Sumber 6](https://www.satellitehealthcare.com/blog/pets-and-peritoneal-dialysis-absolutely/) | Socioeconomic: Deprivasi sosioekonomi berdampak pada hasil treatment yang lebih buruk. Hal ini kemungkinan disebabkan oleh keterbatasan akses terhadap fasilitas sanitasi yang memadai, tekanan psikologis pada pengasuh, serta keterbatasan informasi medis. Strategi bisa dilakukan melalui program pelatihan bagi keluarga (caregiver) dari perawat dialisis yang berpengalaman. Bagi keluarga dengan keterbatasan pendidikan atau ekonomi, dukungan teknis telepon 24 jam dan kunjungan rumah secara berkala oleh tim medis sosial sangat efektif dalam memastikan kepatuhan terhadap prosedur aseptik. Pelatihan ulang sangat dianjurkan, terutama setelah terjadinya peritonitis, untuk mengidentifikasi adanya penyimpangan dalam teknik pertukaran cairan. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC11835194/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC4934433/) [Sumber 3](https://pubmed.ncbi.nlm.nih.gov/23226378/) [Sumber 4](https://pubmed.ncbi.nlm.nih.gov/16091376/) [Sumber 6](https://spnp-spp.pt/media/rqdpbrom/catheter-related-infections-and-peritonitis-in-pediatric-patients-receiving-peritoneal-dialysis-guideline-for-prevention-and-treatment-2012-1-_compressed-1.pdf) [Sumber 7](https://pmc.ncbi.nlm.nih.gov/articles/PMC5691857/) [Sumber 8](https://pmc.ncbi.nlm.nih.gov/articles/PMC4335934/) [Sumber 9](https://www.kidney.org/kidney-topics/preparing-home-dialysis) | Type of Catheter (Cuff): Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff)untuk populasi anak secara umum. Deep cuff berfungsi untuk menjangkar kateter di otot rektus dan mencegah kebocoran, sementara superficial cuff bertindak sebagai penghalang fisik terhadap migrasi bakteri ke arah rongga peritoneum. Namun, pada neonatus atau bayi dengan dinding perut yang sangat tipis, kateter single-cuff sering kali lebih dipilih untuk mencegah ekstrusi manset ke permukaan kulit. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC10223083/) [Sumber 2](http://ispd.org/wp-content/uploads/7.-Dagmara-Borzych-Duzalka-Peritoneal-Dialysis-Catheters-Outcome-in-Children.-The-IPPN-Data.pdf) [Sumber 3](https://kidney.wiki/peritoneal-dialysis/pd-access/) | Catheter Placement: Pedoman klinis terbaru dari Society of American Gastrointestinal and Endoscopic Surgeons (SAGES) menyarankan penggunaan teknik laparoskopi tingkat lanjut (Laparoscopic) dibandingkan teknik bedah terbuka (Open) untuk pemasangan kateter pada populasi pediatrik. Laparoscopic menawarkan akurasi catheter placement yang jauh lebih tinggi di dalam rongga abdomen karena visualisasi langsung, serta meminimalkan trauma mekanis pada jaringan perut. Lebih lanjut, Laparoscopic memungkinkan dokter untuk melakukan prosedur profilaksis penting seperti omentektomi atau omentopeksi untuk meminimalkan risiko omental wrapping (penyumbatan kateter oleh omentum), yang merupakan salah satu penyebab utama kegagalan mekanis kateter pada anak-anak. Laparoscopic juga terbukti mempermudah penyelamatan (salvage) jika terjadi malposisi atau disfungsi kateter tanpa harus melakukan pembedahan ulang yang invasif. [Sumber 1](https://www.sages.org/publications/guidelines/peritoneal-dialysis-access-guideline-update-2023/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC10223083/) [[3]](https://kidney.wiki/peritoneal-dialysis/pd-access/) | Starting PD &lt;2 weeks after catheter placement: Waktu antara pemasangan kateter dan dimulainya dialisis (break-in-period) merupakan faktor penting untuk mencegah komplikasi. Masa penyembuhan minimal 2 minggu sebelum dialysis dimulai. Namun, dalam kondisi klinis tertentu di mana pasien membutuhkan dialisis segera, urgent-start PD (dimulai dalam &lt;14 hari atau bahkan &lt;48 jam) menjadi alternatif yang baik untuk menghindari penggunakan kateter hemodialysis sementara. Pasien dengan break-in-period &lt; 7 hari memiliki risiko yang lebih tinggi terhadap komplikasi awal seperti kebocoran dialisat dan malposisi kateter. Namun, risiko tersebut tidak berkorelasi dengan penurunan kelangsungan hidup atau peningkatan risiko peritonitis jika dilakukan dengan protokol yang tepat. Pada kondisi urgent-start, risiko kebocoran dimitigasi dengan menggunakan volume pengisian rendah (10-20 ml/kg) dan posisi pasien supine untuk mengurangi tekanan intra-abdominal.[Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC3923692/) [Sumber 2](https://journals.plos.org/plosone/article?id=10.1371/journal.pone.0206426) [Sumber 3](https://www.sages.org/publications/guidelines/peritoneal-dialysis-access-guideline-update-2023/) [Sumber 4](https://www.frontiersin.org/journals/endocrinology/articles/10.3389/fendo.2022.936573/full) [Sumber 5](https://scholarlyexchange.childrensmercy.org/cgi/viewcontent.cgi?article=7522&amp;context=papers) [Sumber 6](https://pubmed.ncbi.nlm.nih.gov/33523772/) [Sumber 7](https://www.bcrenal.ca/resource-gallery/Documents/PD_Procedures-Exit_Site_Care-Post-Operative_PD_Catheter_Insertion.pdf) | Catheter Orientation: Posisi atau arah lubang keluar kateter (exit site) sangat memengaruhi risiko terjadinya infeksi. Data multisentrik dari SCOPE Collaborative menunjukkan bahwa orientasi kateter yang menghadap ke atas (Upward) dikaitkan dengan peningkatan risiko peritonitis hingga 4.2 kali lipat (Rate Ratio: 4.2; 95% CI: 1.49–11.89) dibandingkan orientasi lainnya. Secara anatomis, lubang keluar yang menghadap ke atas menciptakan bentuk cekungan yang dapat menampung keringat, air mandi, dan kotoran. Akibat gaya gravitasi, bakteri yang terkumpul di area ini akan mengendap dan bermigrasi ke dalam terowongan kateter. Oleh karena itu, lubang keluar kateter harus selalu diarahkan ke bawah (Downward) atau ke samping (Lateral) untuk mencegah penumpukan bakteri secara alami. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC5012476/) [Sumber 2](https://openurologyandnephrologyjournal.com/VOLUME/5/PAGE/4/) [Sumber 3](https://kidney.wiki/peritoneal-dialysis/pd-access/)</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>2026-05-19 12:49:13</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>18F27E0F</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>&gt;2 yo</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>&gt;12 mo</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>Fair/poor service</t>
+        </is>
+      </c>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>Poor/fair</t>
+        </is>
+      </c>
+      <c r="J125" t="inlineStr">
+        <is>
+          <t>Studies</t>
+        </is>
+      </c>
+      <c r="K125" t="inlineStr">
+        <is>
+          <t>No ESI</t>
+        </is>
+      </c>
+      <c r="L125" t="inlineStr">
+        <is>
+          <t>Normal Nutrition</t>
+        </is>
+      </c>
+      <c r="M125" t="inlineStr">
+        <is>
+          <t>Non-glomerular</t>
+        </is>
+      </c>
+      <c r="N125" t="inlineStr">
+        <is>
+          <t>Coiled/swan neck</t>
+        </is>
+      </c>
+      <c r="O125" t="inlineStr">
+        <is>
+          <t>Single cuff</t>
+        </is>
+      </c>
+      <c r="P125" t="inlineStr">
+        <is>
+          <t>Laparoscopic</t>
+        </is>
+      </c>
+      <c r="Q125" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R125" t="inlineStr">
+        <is>
+          <t>Patients</t>
+        </is>
+      </c>
+      <c r="S125" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="T125" t="inlineStr">
+        <is>
+          <t>upward</t>
+        </is>
+      </c>
+      <c r="U125" t="inlineStr">
+        <is>
+          <t>No stunting</t>
+        </is>
+      </c>
+      <c r="V125" t="inlineStr">
+        <is>
+          <t>45.45%</t>
+        </is>
+      </c>
+      <c r="W125" t="inlineStr">
+        <is>
+          <t>Berisiko Rendah Peritonitis</t>
+        </is>
+      </c>
+      <c r="X125" t="inlineStr">
+        <is>
+          <t>Age*, Gender, Place of Residence, Education, Peritonitis in ESI*, Nutrition, Type of Catheter (Shape), Gastrostomy/Intraperitoneal Device, Performed CAPD, Stunting</t>
+        </is>
+      </c>
+      <c r="Y125" t="inlineStr">
+        <is>
+          <t>Duration of PD*, Housing, Socioeconomic, Cause of ESRD*, Type of Catheter (Cuff), Catheter Placement, Starting PD &lt;2 weeks after catheter placement, Catheter Orientation</t>
+        </is>
+      </c>
+      <c r="Z125" t="inlineStr">
+        <is>
+          <t>Housing: Lingkungan rumah harus diadaptasi untuk memenuhi standar prosedur medis. Ruangan yang digunakan untuk pertukaran cairan harus bersih dan bebas debu untuk meminimalkan risiko infeksi, sebab partikel debu dapat menjadi vektor bagi patogen udara yang dapat mengontaminasi set transfer saat prosedur koneksi atau diskoneksi. Penyediaan wastafel di dalam atau dekat ruangan dialisis diperlukan untuk memastikan kepatuhan protokol antiseptic tangan sehingga menurunkan insiden peritonitis akibat touch contamination. Pencahayaan yang optimal di dalam ruangan diperlukan agar caregiver dapat memantau kejernihan cairan efluen serta memeriksa kondisi tempat keluar kateter dengan teliti. Hewan peliharaan tidak boleh berada di area perawatan saat proses koneksi atau diskoneksi berlangsung karena risiko paparan bakteri seperti Pasteurella multocida atau kerusakan fisik pada selang dialisis akibat gigitan atau cakaran. Selain itu, caregiverharus ditekankan untuk selalu mencuci tangan setelah berinteraksi dengan hewan dan sebelum memulai prosedur dialisis. [Sumber 1](https://www.freseniuskidneycare.com/treatment/home-dialysis/getting-prepared) [Sumber 2](https://www.ouh.nhs.uk/media/agxhnni2/85713pdialysis.pdf) [Sumber 3](https://www.kidney.org/kidney-topics/preparing-home-dialysis) [Sumber 4](https://spnp-spp.pt/media/rqdpbrom/catheter-related-infections-and-peritonitis-in-pediatric-patients-receiving-peritoneal-dialysis-guideline-for-prevention-and-treatment-2012-1-_compressed-1.pdf) [Sumber 5](https://freseniusmedicalcare.com/content/dam/home-products-education/steps2home-pd/Preventing_Peritonitis.pdf) [Sumber 6](https://www.satellitehealthcare.com/blog/pets-and-peritoneal-dialysis-absolutely/) | Socioeconomic: Deprivasi sosioekonomi berdampak pada hasil treatment yang lebih buruk. Hal ini kemungkinan disebabkan oleh keterbatasan akses terhadap fasilitas sanitasi yang memadai, tekanan psikologis pada pengasuh, serta keterbatasan informasi medis. Strategi bisa dilakukan melalui program pelatihan bagi keluarga (caregiver) dari perawat dialisis yang berpengalaman. Bagi keluarga dengan keterbatasan pendidikan atau ekonomi, dukungan teknis telepon 24 jam dan kunjungan rumah secara berkala oleh tim medis sosial sangat efektif dalam memastikan kepatuhan terhadap prosedur aseptik. Pelatihan ulang sangat dianjurkan, terutama setelah terjadinya peritonitis, untuk mengidentifikasi adanya penyimpangan dalam teknik pertukaran cairan. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC11835194/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC4934433/) [Sumber 3](https://pubmed.ncbi.nlm.nih.gov/23226378/) [Sumber 4](https://pubmed.ncbi.nlm.nih.gov/16091376/) [Sumber 6](https://spnp-spp.pt/media/rqdpbrom/catheter-related-infections-and-peritonitis-in-pediatric-patients-receiving-peritoneal-dialysis-guideline-for-prevention-and-treatment-2012-1-_compressed-1.pdf) [Sumber 7](https://pmc.ncbi.nlm.nih.gov/articles/PMC5691857/) [Sumber 8](https://pmc.ncbi.nlm.nih.gov/articles/PMC4335934/) [Sumber 9](https://www.kidney.org/kidney-topics/preparing-home-dialysis) | Type of Catheter (Cuff): Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff)untuk populasi anak secara umum. Deep cuff berfungsi untuk menjangkar kateter di otot rektus dan mencegah kebocoran, sementara superficial cuff bertindak sebagai penghalang fisik terhadap migrasi bakteri ke arah rongga peritoneum. Namun, pada neonatus atau bayi dengan dinding perut yang sangat tipis, kateter single-cuff sering kali lebih dipilih untuk mencegah ekstrusi manset ke permukaan kulit. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC10223083/) [Sumber 2](http://ispd.org/wp-content/uploads/7.-Dagmara-Borzych-Duzalka-Peritoneal-Dialysis-Catheters-Outcome-in-Children.-The-IPPN-Data.pdf) [Sumber 3](https://kidney.wiki/peritoneal-dialysis/pd-access/) | Catheter Placement: Pedoman klinis terbaru dari Society of American Gastrointestinal and Endoscopic Surgeons (SAGES) menyarankan penggunaan teknik laparoskopi tingkat lanjut (Laparoscopic) dibandingkan teknik bedah terbuka (Open) untuk pemasangan kateter pada populasi pediatrik. Laparoscopic menawarkan akurasi catheter placement yang jauh lebih tinggi di dalam rongga abdomen karena visualisasi langsung, serta meminimalkan trauma mekanis pada jaringan perut. Lebih lanjut, Laparoscopic memungkinkan dokter untuk melakukan prosedur profilaksis penting seperti omentektomi atau omentopeksi untuk meminimalkan risiko omental wrapping (penyumbatan kateter oleh omentum), yang merupakan salah satu penyebab utama kegagalan mekanis kateter pada anak-anak. Laparoscopic juga terbukti mempermudah penyelamatan (salvage) jika terjadi malposisi atau disfungsi kateter tanpa harus melakukan pembedahan ulang yang invasif. [Sumber 1](https://www.sages.org/publications/guidelines/peritoneal-dialysis-access-guideline-update-2023/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC10223083/) [[3]](https://kidney.wiki/peritoneal-dialysis/pd-access/) | Starting PD &lt;2 weeks after catheter placement: Waktu antara pemasangan kateter dan dimulainya dialisis (break-in-period) merupakan faktor penting untuk mencegah komplikasi. Masa penyembuhan minimal 2 minggu sebelum dialysis dimulai. Namun, dalam kondisi klinis tertentu di mana pasien membutuhkan dialisis segera, urgent-start PD (dimulai dalam &lt;14 hari atau bahkan &lt;48 jam) menjadi alternatif yang baik untuk menghindari penggunakan kateter hemodialysis sementara. Pasien dengan break-in-period &lt; 7 hari memiliki risiko yang lebih tinggi terhadap komplikasi awal seperti kebocoran dialisat dan malposisi kateter. Namun, risiko tersebut tidak berkorelasi dengan penurunan kelangsungan hidup atau peningkatan risiko peritonitis jika dilakukan dengan protokol yang tepat. Pada kondisi urgent-start, risiko kebocoran dimitigasi dengan menggunakan volume pengisian rendah (10-20 ml/kg) dan posisi pasien supine untuk mengurangi tekanan intra-abdominal.[Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC3923692/) [Sumber 2](https://journals.plos.org/plosone/article?id=10.1371/journal.pone.0206426) [Sumber 3](https://www.sages.org/publications/guidelines/peritoneal-dialysis-access-guideline-update-2023/) [Sumber 4](https://www.frontiersin.org/journals/endocrinology/articles/10.3389/fendo.2022.936573/full) [Sumber 5](https://scholarlyexchange.childrensmercy.org/cgi/viewcontent.cgi?article=7522&amp;context=papers) [Sumber 6](https://pubmed.ncbi.nlm.nih.gov/33523772/) [Sumber 7](https://www.bcrenal.ca/resource-gallery/Documents/PD_Procedures-Exit_Site_Care-Post-Operative_PD_Catheter_Insertion.pdf) | Catheter Orientation: Posisi atau arah lubang keluar kateter (exit site) sangat memengaruhi risiko terjadinya infeksi. Data multisentrik dari SCOPE Collaborative menunjukkan bahwa orientasi kateter yang menghadap ke atas (Upward) dikaitkan dengan peningkatan risiko peritonitis hingga 4.2 kali lipat (Rate Ratio: 4.2; 95% CI: 1.49–11.89) dibandingkan orientasi lainnya. Secara anatomis, lubang keluar yang menghadap ke atas menciptakan bentuk cekungan yang dapat menampung keringat, air mandi, dan kotoran. Akibat gaya gravitasi, bakteri yang terkumpul di area ini akan mengendap dan bermigrasi ke dalam terowongan kateter. Oleh karena itu, lubang keluar kateter harus selalu diarahkan ke bawah (Downward) atau ke samping (Lateral) untuk mencegah penumpukan bakteri secara alami. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC5012476/) [Sumber 2](https://openurologyandnephrologyjournal.com/VOLUME/5/PAGE/4/) [Sumber 3](https://kidney.wiki/peritoneal-dialysis/pd-access/)</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>2026-05-19 12:50:33</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>18F27E0F</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>&gt;2 yo</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>&gt;12 mo</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>Fair/poor service</t>
+        </is>
+      </c>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>Poor/fair</t>
+        </is>
+      </c>
+      <c r="J126" t="inlineStr">
+        <is>
+          <t>Studies</t>
+        </is>
+      </c>
+      <c r="K126" t="inlineStr">
+        <is>
+          <t>No ESI</t>
+        </is>
+      </c>
+      <c r="L126" t="inlineStr">
+        <is>
+          <t>Normal Nutrition</t>
+        </is>
+      </c>
+      <c r="M126" t="inlineStr">
+        <is>
+          <t>Non-glomerular</t>
+        </is>
+      </c>
+      <c r="N126" t="inlineStr">
+        <is>
+          <t>Coiled/swan neck</t>
+        </is>
+      </c>
+      <c r="O126" t="inlineStr">
+        <is>
+          <t>Single cuff</t>
+        </is>
+      </c>
+      <c r="P126" t="inlineStr">
+        <is>
+          <t>Laparoscopic</t>
+        </is>
+      </c>
+      <c r="Q126" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R126" t="inlineStr">
+        <is>
+          <t>Patients</t>
+        </is>
+      </c>
+      <c r="S126" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="T126" t="inlineStr">
+        <is>
+          <t>upward</t>
+        </is>
+      </c>
+      <c r="U126" t="inlineStr">
+        <is>
+          <t>Stunting</t>
+        </is>
+      </c>
+      <c r="V126" t="inlineStr">
+        <is>
+          <t>50.00%</t>
+        </is>
+      </c>
+      <c r="W126" t="inlineStr">
+        <is>
+          <t>Berisiko Tinggi Peritonitis</t>
+        </is>
+      </c>
+      <c r="X126" t="inlineStr">
+        <is>
+          <t>Age*, Gender, Place of Residence, Education, Peritonitis in ESI*, Nutrition, Type of Catheter (Shape), Gastrostomy/Intraperitoneal Device, Performed CAPD</t>
+        </is>
+      </c>
+      <c r="Y126" t="inlineStr">
+        <is>
+          <t>Duration of PD*, Housing, Socioeconomic, Cause of ESRD*, Type of Catheter (Cuff), Catheter Placement, Starting PD &lt;2 weeks after catheter placement, Catheter Orientation, Stunting</t>
+        </is>
+      </c>
+      <c r="Z126" t="inlineStr">
+        <is>
+          <t>Housing: Lingkungan rumah harus diadaptasi untuk memenuhi standar prosedur medis. Ruangan yang digunakan untuk pertukaran cairan harus bersih dan bebas debu untuk meminimalkan risiko infeksi, sebab partikel debu dapat menjadi vektor bagi patogen udara yang dapat mengontaminasi set transfer saat prosedur koneksi atau diskoneksi. Penyediaan wastafel di dalam atau dekat ruangan dialisis diperlukan untuk memastikan kepatuhan protokol antiseptic tangan sehingga menurunkan insiden peritonitis akibat touch contamination. Pencahayaan yang optimal di dalam ruangan diperlukan agar caregiver dapat memantau kejernihan cairan efluen serta memeriksa kondisi tempat keluar kateter dengan teliti. Hewan peliharaan tidak boleh berada di area perawatan saat proses koneksi atau diskoneksi berlangsung karena risiko paparan bakteri seperti Pasteurella multocida atau kerusakan fisik pada selang dialisis akibat gigitan atau cakaran. Selain itu, caregiverharus ditekankan untuk selalu mencuci tangan setelah berinteraksi dengan hewan dan sebelum memulai prosedur dialisis. [Sumber 1](https://www.freseniuskidneycare.com/treatment/home-dialysis/getting-prepared) [Sumber 2](https://www.ouh.nhs.uk/media/agxhnni2/85713pdialysis.pdf) [Sumber 3](https://www.kidney.org/kidney-topics/preparing-home-dialysis) [Sumber 4](https://spnp-spp.pt/media/rqdpbrom/catheter-related-infections-and-peritonitis-in-pediatric-patients-receiving-peritoneal-dialysis-guideline-for-prevention-and-treatment-2012-1-_compressed-1.pdf) [Sumber 5](https://freseniusmedicalcare.com/content/dam/home-products-education/steps2home-pd/Preventing_Peritonitis.pdf) [Sumber 6](https://www.satellitehealthcare.com/blog/pets-and-peritoneal-dialysis-absolutely/) | Socioeconomic: Deprivasi sosioekonomi berdampak pada hasil treatment yang lebih buruk. Hal ini kemungkinan disebabkan oleh keterbatasan akses terhadap fasilitas sanitasi yang memadai, tekanan psikologis pada pengasuh, serta keterbatasan informasi medis. Strategi bisa dilakukan melalui program pelatihan bagi keluarga (caregiver) dari perawat dialisis yang berpengalaman. Bagi keluarga dengan keterbatasan pendidikan atau ekonomi, dukungan teknis telepon 24 jam dan kunjungan rumah secara berkala oleh tim medis sosial sangat efektif dalam memastikan kepatuhan terhadap prosedur aseptik. Pelatihan ulang sangat dianjurkan, terutama setelah terjadinya peritonitis, untuk mengidentifikasi adanya penyimpangan dalam teknik pertukaran cairan. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC11835194/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC4934433/) [Sumber 3](https://pubmed.ncbi.nlm.nih.gov/23226378/) [Sumber 4](https://pubmed.ncbi.nlm.nih.gov/16091376/) [Sumber 6](https://spnp-spp.pt/media/rqdpbrom/catheter-related-infections-and-peritonitis-in-pediatric-patients-receiving-peritoneal-dialysis-guideline-for-prevention-and-treatment-2012-1-_compressed-1.pdf) [Sumber 7](https://pmc.ncbi.nlm.nih.gov/articles/PMC5691857/) [Sumber 8](https://pmc.ncbi.nlm.nih.gov/articles/PMC4335934/) [Sumber 9](https://www.kidney.org/kidney-topics/preparing-home-dialysis) | Type of Catheter (Cuff): Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff)untuk populasi anak secara umum. Deep cuff berfungsi untuk menjangkar kateter di otot rektus dan mencegah kebocoran, sementara superficial cuff bertindak sebagai penghalang fisik terhadap migrasi bakteri ke arah rongga peritoneum. Namun, pada neonatus atau bayi dengan dinding perut yang sangat tipis, kateter single-cuff sering kali lebih dipilih untuk mencegah ekstrusi manset ke permukaan kulit. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC10223083/) [Sumber 2](http://ispd.org/wp-content/uploads/7.-Dagmara-Borzych-Duzalka-Peritoneal-Dialysis-Catheters-Outcome-in-Children.-The-IPPN-Data.pdf) [Sumber 3](https://kidney.wiki/peritoneal-dialysis/pd-access/) | Catheter Placement: Pedoman klinis terbaru dari Society of American Gastrointestinal and Endoscopic Surgeons (SAGES) menyarankan penggunaan teknik laparoskopi tingkat lanjut (Laparoscopic) dibandingkan teknik bedah terbuka (Open) untuk pemasangan kateter pada populasi pediatrik. Laparoscopic menawarkan akurasi catheter placement yang jauh lebih tinggi di dalam rongga abdomen karena visualisasi langsung, serta meminimalkan trauma mekanis pada jaringan perut. Lebih lanjut, Laparoscopic memungkinkan dokter untuk melakukan prosedur profilaksis penting seperti omentektomi atau omentopeksi untuk meminimalkan risiko omental wrapping (penyumbatan kateter oleh omentum), yang merupakan salah satu penyebab utama kegagalan mekanis kateter pada anak-anak. Laparoscopic juga terbukti mempermudah penyelamatan (salvage) jika terjadi malposisi atau disfungsi kateter tanpa harus melakukan pembedahan ulang yang invasif. [Sumber 1](https://www.sages.org/publications/guidelines/peritoneal-dialysis-access-guideline-update-2023/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC10223083/) [[3]](https://kidney.wiki/peritoneal-dialysis/pd-access/) | Starting PD &lt;2 weeks after catheter placement: Waktu antara pemasangan kateter dan dimulainya dialisis (break-in-period) merupakan faktor penting untuk mencegah komplikasi. Masa penyembuhan minimal 2 minggu sebelum dialysis dimulai. Namun, dalam kondisi klinis tertentu di mana pasien membutuhkan dialisis segera, urgent-start PD (dimulai dalam &lt;14 hari atau bahkan &lt;48 jam) menjadi alternatif yang baik untuk menghindari penggunakan kateter hemodialysis sementara. Pasien dengan break-in-period &lt; 7 hari memiliki risiko yang lebih tinggi terhadap komplikasi awal seperti kebocoran dialisat dan malposisi kateter. Namun, risiko tersebut tidak berkorelasi dengan penurunan kelangsungan hidup atau peningkatan risiko peritonitis jika dilakukan dengan protokol yang tepat. Pada kondisi urgent-start, risiko kebocoran dimitigasi dengan menggunakan volume pengisian rendah (10-20 ml/kg) dan posisi pasien supine untuk mengurangi tekanan intra-abdominal.[Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC3923692/) [Sumber 2](https://journals.plos.org/plosone/article?id=10.1371/journal.pone.0206426) [Sumber 3](https://www.sages.org/publications/guidelines/peritoneal-dialysis-access-guideline-update-2023/) [Sumber 4](https://www.frontiersin.org/journals/endocrinology/articles/10.3389/fendo.2022.936573/full) [Sumber 5](https://scholarlyexchange.childrensmercy.org/cgi/viewcontent.cgi?article=7522&amp;context=papers) [Sumber 6](https://pubmed.ncbi.nlm.nih.gov/33523772/) [Sumber 7](https://www.bcrenal.ca/resource-gallery/Documents/PD_Procedures-Exit_Site_Care-Post-Operative_PD_Catheter_Insertion.pdf) | Catheter Orientation: Posisi atau arah lubang keluar kateter (exit site) sangat memengaruhi risiko terjadinya infeksi. Data multisentrik dari SCOPE Collaborative menunjukkan bahwa orientasi kateter yang menghadap ke atas (Upward) dikaitkan dengan peningkatan risiko peritonitis hingga 4.2 kali lipat (Rate Ratio: 4.2; 95% CI: 1.49–11.89) dibandingkan orientasi lainnya. Secara anatomis, lubang keluar yang menghadap ke atas menciptakan bentuk cekungan yang dapat menampung keringat, air mandi, dan kotoran. Akibat gaya gravitasi, bakteri yang terkumpul di area ini akan mengendap dan bermigrasi ke dalam terowongan kateter. Oleh karena itu, lubang keluar kateter harus selalu diarahkan ke bawah (Downward) atau ke samping (Lateral) untuk mencegah penumpukan bakteri secara alami. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC5012476/) [Sumber 2](https://openurologyandnephrologyjournal.com/VOLUME/5/PAGE/4/) [Sumber 3](https://kidney.wiki/peritoneal-dialysis/pd-access/) | Stunting: Stunting pada anak dialisis bukan hanya disebabkan oleh asupan kalori yang rendah, tetapi juga oleh asidosis metabolik, anemia, osteodistrofi ginjal, dan resistensi terhadap hormon pertumbuhan. Intervensi pertama adalah memastikan kecukupan dialisis dan koreksi parameter metabolik seperti asidosis dan hiperparatiroidisme.Jika pertumbuhan masih belum optimal meskipun parameter metabolik telah terkendali dan asupan nutrisi sudah mencapai target, terapi dengan hormon pertumbuhan manusia rekombinan (rhGH) dapat dipertimbangkan. Selain itu, dukungan nutrisi intensif dan klirens dialisis yang adekuat pada pasien prepubertal dapat mempromosikan pertumbuhan normal tanpa selalu memerlukan rhGH. Pada anak yang mengalami stunting (tinggi badan &lt; persentil ke-2), perhitungan kebutuhan energi dan mikronutrien harus didasarkan pada height-age pasien, bukan chronological age-nya, untuk memberikan dukungan yang sesuai dengan ukuran tubuh aktualnya. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/)</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>2026-05-19 13:07:54</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>18F27E0F</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>&gt;2 yo</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>&gt;12 mo</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>Good service</t>
+        </is>
+      </c>
+      <c r="I127" t="inlineStr">
+        <is>
+          <t>Poor/fair</t>
+        </is>
+      </c>
+      <c r="J127" t="inlineStr">
+        <is>
+          <t>Studies</t>
+        </is>
+      </c>
+      <c r="K127" t="inlineStr">
+        <is>
+          <t>No ESI</t>
+        </is>
+      </c>
+      <c r="L127" t="inlineStr">
+        <is>
+          <t>Normal Nutrition</t>
+        </is>
+      </c>
+      <c r="M127" t="inlineStr">
+        <is>
+          <t>Non-glomerular</t>
+        </is>
+      </c>
+      <c r="N127" t="inlineStr">
+        <is>
+          <t>Coiled/swan neck</t>
+        </is>
+      </c>
+      <c r="O127" t="inlineStr">
+        <is>
+          <t>Single cuff</t>
+        </is>
+      </c>
+      <c r="P127" t="inlineStr">
+        <is>
+          <t>Laparoscopic</t>
+        </is>
+      </c>
+      <c r="Q127" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R127" t="inlineStr">
+        <is>
+          <t>Patients</t>
+        </is>
+      </c>
+      <c r="S127" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="T127" t="inlineStr">
+        <is>
+          <t>upward</t>
+        </is>
+      </c>
+      <c r="U127" t="inlineStr">
+        <is>
+          <t>Stunting</t>
+        </is>
+      </c>
+      <c r="V127" t="inlineStr">
+        <is>
+          <t>45.45%</t>
+        </is>
+      </c>
+      <c r="W127" t="inlineStr">
+        <is>
+          <t>Berisiko Rendah Peritonitis</t>
+        </is>
+      </c>
+      <c r="X127" t="inlineStr">
+        <is>
+          <t>Age*, Gender, Place of Residence, Housing, Education, Peritonitis in ESI*, Nutrition, Type of Catheter (Shape), Gastrostomy/Intraperitoneal Device, Performed CAPD</t>
+        </is>
+      </c>
+      <c r="Y127" t="inlineStr">
+        <is>
+          <t>Duration of PD*, Socioeconomic, Cause of ESRD*, Type of Catheter (Cuff), Catheter Placement, Starting PD &lt;2 weeks after catheter placement, Catheter Orientation, Stunting</t>
+        </is>
+      </c>
+      <c r="Z127" t="inlineStr">
+        <is>
+          <t>Socioeconomic: Deprivasi sosioekonomi berdampak pada hasil treatment yang lebih buruk. Hal ini kemungkinan disebabkan oleh keterbatasan akses terhadap fasilitas sanitasi yang memadai, tekanan psikologis pada pengasuh, serta keterbatasan informasi medis. Strategi bisa dilakukan melalui program pelatihan bagi keluarga (caregiver) dari perawat dialisis yang berpengalaman. Bagi keluarga dengan keterbatasan pendidikan atau ekonomi, dukungan teknis telepon 24 jam dan kunjungan rumah secara berkala oleh tim medis sosial sangat efektif dalam memastikan kepatuhan terhadap prosedur aseptik. Pelatihan ulang sangat dianjurkan, terutama setelah terjadinya peritonitis, untuk mengidentifikasi adanya penyimpangan dalam teknik pertukaran cairan. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC11835194/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC4934433/) [Sumber 3](https://pubmed.ncbi.nlm.nih.gov/23226378/) [Sumber 4](https://pubmed.ncbi.nlm.nih.gov/16091376/) [Sumber 6](https://spnp-spp.pt/media/rqdpbrom/catheter-related-infections-and-peritonitis-in-pediatric-patients-receiving-peritoneal-dialysis-guideline-for-prevention-and-treatment-2012-1-_compressed-1.pdf) [Sumber 7](https://pmc.ncbi.nlm.nih.gov/articles/PMC5691857/) [Sumber 8](https://pmc.ncbi.nlm.nih.gov/articles/PMC4335934/) [Sumber 9](https://www.kidney.org/kidney-topics/preparing-home-dialysis) | Type of Catheter (Cuff): Penggunaan kateter dengan double-cuff lebih disarankan daripada single-cuff)untuk populasi anak secara umum. Deep cuff berfungsi untuk menjangkar kateter di otot rektus dan mencegah kebocoran, sementara superficial cuff bertindak sebagai penghalang fisik terhadap migrasi bakteri ke arah rongga peritoneum. Namun, pada neonatus atau bayi dengan dinding perut yang sangat tipis, kateter single-cuff sering kali lebih dipilih untuk mencegah ekstrusi manset ke permukaan kulit. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC10223083/) [Sumber 2](http://ispd.org/wp-content/uploads/7.-Dagmara-Borzych-Duzalka-Peritoneal-Dialysis-Catheters-Outcome-in-Children.-The-IPPN-Data.pdf) [Sumber 3](https://kidney.wiki/peritoneal-dialysis/pd-access/) | Catheter Placement: Pedoman klinis terbaru dari Society of American Gastrointestinal and Endoscopic Surgeons (SAGES) menyarankan penggunaan teknik laparoskopi tingkat lanjut (Laparoscopic) dibandingkan teknik bedah terbuka (Open) untuk pemasangan kateter pada populasi pediatrik. Laparoscopic menawarkan akurasi catheter placement yang jauh lebih tinggi di dalam rongga abdomen karena visualisasi langsung, serta meminimalkan trauma mekanis pada jaringan perut. Lebih lanjut, Laparoscopic memungkinkan dokter untuk melakukan prosedur profilaksis penting seperti omentektomi atau omentopeksi untuk meminimalkan risiko omental wrapping (penyumbatan kateter oleh omentum), yang merupakan salah satu penyebab utama kegagalan mekanis kateter pada anak-anak. Laparoscopic juga terbukti mempermudah penyelamatan (salvage) jika terjadi malposisi atau disfungsi kateter tanpa harus melakukan pembedahan ulang yang invasif. [Sumber 1](https://www.sages.org/publications/guidelines/peritoneal-dialysis-access-guideline-update-2023/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC10223083/) [[3]](https://kidney.wiki/peritoneal-dialysis/pd-access/) | Starting PD &lt;2 weeks after catheter placement: Waktu antara pemasangan kateter dan dimulainya dialisis (break-in-period) merupakan faktor penting untuk mencegah komplikasi. Masa penyembuhan minimal 2 minggu sebelum dialysis dimulai. Namun, dalam kondisi klinis tertentu di mana pasien membutuhkan dialisis segera, urgent-start PD (dimulai dalam &lt;14 hari atau bahkan &lt;48 jam) menjadi alternatif yang baik untuk menghindari penggunakan kateter hemodialysis sementara. Pasien dengan break-in-period &lt; 7 hari memiliki risiko yang lebih tinggi terhadap komplikasi awal seperti kebocoran dialisat dan malposisi kateter. Namun, risiko tersebut tidak berkorelasi dengan penurunan kelangsungan hidup atau peningkatan risiko peritonitis jika dilakukan dengan protokol yang tepat. Pada kondisi urgent-start, risiko kebocoran dimitigasi dengan menggunakan volume pengisian rendah (10-20 ml/kg) dan posisi pasien supine untuk mengurangi tekanan intra-abdominal.[Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC3923692/) [Sumber 2](https://journals.plos.org/plosone/article?id=10.1371/journal.pone.0206426) [Sumber 3](https://www.sages.org/publications/guidelines/peritoneal-dialysis-access-guideline-update-2023/) [Sumber 4](https://www.frontiersin.org/journals/endocrinology/articles/10.3389/fendo.2022.936573/full) [Sumber 5](https://scholarlyexchange.childrensmercy.org/cgi/viewcontent.cgi?article=7522&amp;context=papers) [Sumber 6](https://pubmed.ncbi.nlm.nih.gov/33523772/) [Sumber 7](https://www.bcrenal.ca/resource-gallery/Documents/PD_Procedures-Exit_Site_Care-Post-Operative_PD_Catheter_Insertion.pdf) | Catheter Orientation: Posisi atau arah lubang keluar kateter (exit site) sangat memengaruhi risiko terjadinya infeksi. Data multisentrik dari SCOPE Collaborative menunjukkan bahwa orientasi kateter yang menghadap ke atas (Upward) dikaitkan dengan peningkatan risiko peritonitis hingga 4.2 kali lipat (Rate Ratio: 4.2; 95% CI: 1.49–11.89) dibandingkan orientasi lainnya. Secara anatomis, lubang keluar yang menghadap ke atas menciptakan bentuk cekungan yang dapat menampung keringat, air mandi, dan kotoran. Akibat gaya gravitasi, bakteri yang terkumpul di area ini akan mengendap dan bermigrasi ke dalam terowongan kateter. Oleh karena itu, lubang keluar kateter harus selalu diarahkan ke bawah (Downward) atau ke samping (Lateral) untuk mencegah penumpukan bakteri secara alami. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC5012476/) [Sumber 2](https://openurologyandnephrologyjournal.com/VOLUME/5/PAGE/4/) [Sumber 3](https://kidney.wiki/peritoneal-dialysis/pd-access/) | Stunting: Stunting pada anak dialisis bukan hanya disebabkan oleh asupan kalori yang rendah, tetapi juga oleh asidosis metabolik, anemia, osteodistrofi ginjal, dan resistensi terhadap hormon pertumbuhan. Intervensi pertama adalah memastikan kecukupan dialisis dan koreksi parameter metabolik seperti asidosis dan hiperparatiroidisme.Jika pertumbuhan masih belum optimal meskipun parameter metabolik telah terkendali dan asupan nutrisi sudah mencapai target, terapi dengan hormon pertumbuhan manusia rekombinan (rhGH) dapat dipertimbangkan. Selain itu, dukungan nutrisi intensif dan klirens dialisis yang adekuat pada pasien prepubertal dapat mempromosikan pertumbuhan normal tanpa selalu memerlukan rhGH. Pada anak yang mengalami stunting (tinggi badan &lt; persentil ke-2), perhitungan kebutuhan energi dan mikronutrien harus didasarkan pada height-age pasien, bukan chronological age-nya, untuk memberikan dukungan yang sesuai dengan ukuran tubuh aktualnya. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC6904418/)</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>2026-05-19 13:09:47</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>E84BB22D</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>&gt;2 yo</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>&lt;12 mo</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="H128" t="inlineStr">
+        <is>
+          <t>Good service</t>
+        </is>
+      </c>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="J128" t="inlineStr">
+        <is>
+          <t>Studies</t>
+        </is>
+      </c>
+      <c r="K128" t="inlineStr">
+        <is>
+          <t>No ESI</t>
+        </is>
+      </c>
+      <c r="L128" t="inlineStr">
+        <is>
+          <t>Normal Nutrition</t>
+        </is>
+      </c>
+      <c r="M128" t="inlineStr">
+        <is>
+          <t>Glomerular</t>
+        </is>
+      </c>
+      <c r="N128" t="inlineStr">
+        <is>
+          <t>Coiled/swan neck</t>
+        </is>
+      </c>
+      <c r="O128" t="inlineStr">
+        <is>
+          <t>Double</t>
+        </is>
+      </c>
+      <c r="P128" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="Q128" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R128" t="inlineStr">
+        <is>
+          <t>Patients</t>
+        </is>
+      </c>
+      <c r="S128" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T128" t="inlineStr">
+        <is>
+          <t>Lateral/downward</t>
+        </is>
+      </c>
+      <c r="U128" t="inlineStr">
+        <is>
+          <t>No stunting</t>
+        </is>
+      </c>
+      <c r="V128" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="W128" t="inlineStr">
+        <is>
+          <t>Berisiko Rendah Peritonitis</t>
+        </is>
+      </c>
+      <c r="X128" t="inlineStr">
+        <is>
+          <t>Age*, Gender, Duration of PD*, Place of Residence, Housing, Socioeconomic, Education, Peritonitis in ESI*, Nutrition, Cause of ESRD*, Type of Catheter (Shape), Type of Catheter (Cuff), Catheter Placement, Gastrostomy/Intraperitoneal Device, Performed CAPD, Starting PD &lt;2 weeks after catheter placement, Catheter Orientation, Stunting</t>
+        </is>
+      </c>
+      <c r="Y128" t="inlineStr"/>
+      <c r="Z128" t="inlineStr"/>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>2026-05-19 13:09:57</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>E84BB22D</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>&gt;2 yo</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>&lt;12 mo</t>
+        </is>
+      </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>Urban</t>
+        </is>
+      </c>
+      <c r="H129" t="inlineStr">
+        <is>
+          <t>Good service</t>
+        </is>
+      </c>
+      <c r="I129" t="inlineStr">
+        <is>
+          <t>Poor/fair</t>
+        </is>
+      </c>
+      <c r="J129" t="inlineStr">
+        <is>
+          <t>Studies</t>
+        </is>
+      </c>
+      <c r="K129" t="inlineStr">
+        <is>
+          <t>No ESI</t>
+        </is>
+      </c>
+      <c r="L129" t="inlineStr">
+        <is>
+          <t>Normal Nutrition</t>
+        </is>
+      </c>
+      <c r="M129" t="inlineStr">
+        <is>
+          <t>Glomerular</t>
+        </is>
+      </c>
+      <c r="N129" t="inlineStr">
+        <is>
+          <t>Coiled/swan neck</t>
+        </is>
+      </c>
+      <c r="O129" t="inlineStr">
+        <is>
+          <t>Double</t>
+        </is>
+      </c>
+      <c r="P129" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="Q129" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R129" t="inlineStr">
+        <is>
+          <t>Patients</t>
+        </is>
+      </c>
+      <c r="S129" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="T129" t="inlineStr">
+        <is>
+          <t>Lateral/downward</t>
+        </is>
+      </c>
+      <c r="U129" t="inlineStr">
+        <is>
+          <t>No stunting</t>
+        </is>
+      </c>
+      <c r="V129" t="inlineStr">
+        <is>
+          <t>13.64%</t>
+        </is>
+      </c>
+      <c r="W129" t="inlineStr">
+        <is>
+          <t>Berisiko Rendah Peritonitis</t>
+        </is>
+      </c>
+      <c r="X129" t="inlineStr">
+        <is>
+          <t>Age*, Gender, Duration of PD*, Housing, Education, Peritonitis in ESI*, Nutrition, Cause of ESRD*, Type of Catheter (Shape), Type of Catheter (Cuff), Catheter Placement, Gastrostomy/Intraperitoneal Device, Performed CAPD, Catheter Orientation, Stunting</t>
+        </is>
+      </c>
+      <c r="Y129" t="inlineStr">
+        <is>
+          <t>Place of Residence, Socioeconomic, Starting PD &lt;2 weeks after catheter placement</t>
+        </is>
+      </c>
+      <c r="Z129" t="inlineStr">
+        <is>
+          <t>Socioeconomic: Deprivasi sosioekonomi berdampak pada hasil treatment yang lebih buruk. Hal ini kemungkinan disebabkan oleh keterbatasan akses terhadap fasilitas sanitasi yang memadai, tekanan psikologis pada pengasuh, serta keterbatasan informasi medis. Strategi bisa dilakukan melalui program pelatihan bagi keluarga (caregiver) dari perawat dialisis yang berpengalaman. Bagi keluarga dengan keterbatasan pendidikan atau ekonomi, dukungan teknis telepon 24 jam dan kunjungan rumah secara berkala oleh tim medis sosial sangat efektif dalam memastikan kepatuhan terhadap prosedur aseptik. Pelatihan ulang sangat dianjurkan, terutama setelah terjadinya peritonitis, untuk mengidentifikasi adanya penyimpangan dalam teknik pertukaran cairan. [Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC11835194/) [Sumber 2](https://pmc.ncbi.nlm.nih.gov/articles/PMC4934433/) [Sumber 3](https://pubmed.ncbi.nlm.nih.gov/23226378/) [Sumber 4](https://pubmed.ncbi.nlm.nih.gov/16091376/) [Sumber 6](https://spnp-spp.pt/media/rqdpbrom/catheter-related-infections-and-peritonitis-in-pediatric-patients-receiving-peritoneal-dialysis-guideline-for-prevention-and-treatment-2012-1-_compressed-1.pdf) [Sumber 7](https://pmc.ncbi.nlm.nih.gov/articles/PMC5691857/) [Sumber 8](https://pmc.ncbi.nlm.nih.gov/articles/PMC4335934/) [Sumber 9](https://www.kidney.org/kidney-topics/preparing-home-dialysis) | Starting PD &lt;2 weeks after catheter placement: Waktu antara pemasangan kateter dan dimulainya dialisis (break-in-period) merupakan faktor penting untuk mencegah komplikasi. Masa penyembuhan minimal 2 minggu sebelum dialysis dimulai. Namun, dalam kondisi klinis tertentu di mana pasien membutuhkan dialisis segera, urgent-start PD (dimulai dalam &lt;14 hari atau bahkan &lt;48 jam) menjadi alternatif yang baik untuk menghindari penggunakan kateter hemodialysis sementara. Pasien dengan break-in-period &lt; 7 hari memiliki risiko yang lebih tinggi terhadap komplikasi awal seperti kebocoran dialisat dan malposisi kateter. Namun, risiko tersebut tidak berkorelasi dengan penurunan kelangsungan hidup atau peningkatan risiko peritonitis jika dilakukan dengan protokol yang tepat. Pada kondisi urgent-start, risiko kebocoran dimitigasi dengan menggunakan volume pengisian rendah (10-20 ml/kg) dan posisi pasien supine untuk mengurangi tekanan intra-abdominal.[Sumber 1](https://pmc.ncbi.nlm.nih.gov/articles/PMC3923692/) [Sumber 2](https://journals.plos.org/plosone/article?id=10.1371/journal.pone.0206426) [Sumber 3](https://www.sages.org/publications/guidelines/peritoneal-dialysis-access-guideline-update-2023/) [Sumber 4](https://www.frontiersin.org/journals/endocrinology/articles/10.3389/fendo.2022.936573/full) [Sumber 5](https://scholarlyexchange.childrensmercy.org/cgi/viewcontent.cgi?article=7522&amp;context=papers) [Sumber 6](https://pubmed.ncbi.nlm.nih.gov/33523772/) [Sumber 7](https://www.bcrenal.ca/resource-gallery/Documents/PD_Procedures-Exit_Site_Care-Post-Operative_PD_Catheter_Insertion.pdf)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
v2 11 Juni 2026 - FINAL (login form)
</commit_message>
<xml_diff>
--- a/peritonitis-prediction/PeritonitisPrediction_Database.xlsx
+++ b/peritonitis-prediction/PeritonitisPrediction_Database.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF318"/>
+  <dimension ref="A1:AF319"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -43752,6 +43752,152 @@
         </is>
       </c>
     </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
+          <t>Peritonitis</t>
+        </is>
+      </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>2026-06-11 10:43:27</t>
+        </is>
+      </c>
+      <c r="C319" t="inlineStr">
+        <is>
+          <t>132E80D3</t>
+        </is>
+      </c>
+      <c r="D319" t="inlineStr">
+        <is>
+          <t>&lt;2 yo</t>
+        </is>
+      </c>
+      <c r="E319" t="inlineStr">
+        <is>
+          <t>Tidak Diketahui</t>
+        </is>
+      </c>
+      <c r="F319" t="inlineStr">
+        <is>
+          <t>Tidak Diketahui</t>
+        </is>
+      </c>
+      <c r="G319" t="inlineStr">
+        <is>
+          <t>Tidak Diketahui</t>
+        </is>
+      </c>
+      <c r="H319" t="inlineStr">
+        <is>
+          <t>Tidak Diketahui</t>
+        </is>
+      </c>
+      <c r="I319" t="inlineStr">
+        <is>
+          <t>Tidak Diketahui</t>
+        </is>
+      </c>
+      <c r="J319" t="inlineStr">
+        <is>
+          <t>Tidak Diketahui</t>
+        </is>
+      </c>
+      <c r="K319" t="inlineStr">
+        <is>
+          <t>Tidak Diketahui</t>
+        </is>
+      </c>
+      <c r="L319" t="inlineStr">
+        <is>
+          <t>Tidak Diketahui</t>
+        </is>
+      </c>
+      <c r="M319" t="inlineStr">
+        <is>
+          <t>Tidak Diketahui</t>
+        </is>
+      </c>
+      <c r="N319" t="inlineStr">
+        <is>
+          <t>Tidak Diketahui</t>
+        </is>
+      </c>
+      <c r="O319" t="inlineStr">
+        <is>
+          <t>Tidak Diketahui</t>
+        </is>
+      </c>
+      <c r="P319" t="inlineStr">
+        <is>
+          <t>Tidak Diketahui</t>
+        </is>
+      </c>
+      <c r="Q319" t="inlineStr">
+        <is>
+          <t>Tidak Diketahui</t>
+        </is>
+      </c>
+      <c r="R319" t="inlineStr">
+        <is>
+          <t>Tidak Diketahui</t>
+        </is>
+      </c>
+      <c r="S319" t="inlineStr"/>
+      <c r="T319" t="inlineStr">
+        <is>
+          <t>Tidak Diketahui</t>
+        </is>
+      </c>
+      <c r="U319" t="inlineStr">
+        <is>
+          <t>Tidak Diketahui</t>
+        </is>
+      </c>
+      <c r="V319" t="inlineStr"/>
+      <c r="W319" t="inlineStr"/>
+      <c r="X319" t="inlineStr"/>
+      <c r="Y319" t="inlineStr">
+        <is>
+          <t>Age*</t>
+        </is>
+      </c>
+      <c r="Z319" t="inlineStr">
+        <is>
+          <t>Tidak ada intervensi MRF aktif.</t>
+        </is>
+      </c>
+      <c r="AA319" t="inlineStr">
+        <is>
+          <t>Tidak Diketahui</t>
+        </is>
+      </c>
+      <c r="AB319" t="inlineStr">
+        <is>
+          <t>BERISIKO RENDAH PERITONITIS</t>
+        </is>
+      </c>
+      <c r="AC319" t="inlineStr">
+        <is>
+          <t>1.40%</t>
+        </is>
+      </c>
+      <c r="AD319" t="inlineStr">
+        <is>
+          <t>1.42%</t>
+        </is>
+      </c>
+      <c r="AE319" t="inlineStr">
+        <is>
+          <t>9.09%</t>
+        </is>
+      </c>
+      <c r="AF319" t="inlineStr">
+        <is>
+          <t>9.52%</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>